<commit_message>
RPA datasets push 2024-08-14
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="132">
   <si>
     <t>상장일</t>
   </si>
@@ -69,6 +69,9 @@
     <t>총기관배정수량</t>
   </si>
   <si>
+    <t>2024-08-13</t>
+  </si>
+  <si>
     <t>2024-08-12</t>
   </si>
   <si>
@@ -117,174 +120,165 @@
     <t>2024-06-24</t>
   </si>
   <si>
+    <t>2024-07-01</t>
+  </si>
+  <si>
+    <t>교보16호스팩</t>
+  </si>
+  <si>
+    <t>뱅크웨어글로벌</t>
+  </si>
+  <si>
+    <t>아이빔테크놀로지</t>
+  </si>
+  <si>
+    <t>피앤에스미캐닉스</t>
+  </si>
+  <si>
+    <t>산일전기</t>
+  </si>
+  <si>
+    <t>엔에이치스팩31호</t>
+  </si>
+  <si>
+    <t>SK증권제13호스팩</t>
+  </si>
+  <si>
+    <t>엑셀세라퓨틱스</t>
+  </si>
+  <si>
+    <t>시프트업</t>
+  </si>
+  <si>
+    <t>이베스트스팩6호</t>
+  </si>
+  <si>
+    <t>하스</t>
+  </si>
+  <si>
+    <t>이노스페이스</t>
+  </si>
+  <si>
+    <t>에이치브이엠</t>
+  </si>
+  <si>
+    <t>하이젠알앤엠</t>
+  </si>
+  <si>
+    <t>한국제15호스팩</t>
+  </si>
+  <si>
+    <t>에스오에스랩</t>
+  </si>
+  <si>
+    <t>미래에셋비전스팩6호</t>
+  </si>
+  <si>
+    <t>신한글로벌액티브리츠</t>
+  </si>
+  <si>
+    <t>코스닥</t>
+  </si>
+  <si>
+    <t>코스피</t>
+  </si>
+  <si>
+    <t>교보</t>
+  </si>
+  <si>
+    <t>미래</t>
+  </si>
+  <si>
+    <t>삼성</t>
+  </si>
+  <si>
+    <t>키움</t>
+  </si>
+  <si>
+    <t>NH</t>
+  </si>
+  <si>
+    <t>SK</t>
+  </si>
+  <si>
+    <t>대신</t>
+  </si>
+  <si>
+    <t>한국</t>
+  </si>
+  <si>
+    <t>제이피모간회사</t>
+  </si>
+  <si>
+    <t>신한</t>
+  </si>
+  <si>
+    <t>LS</t>
+  </si>
+  <si>
+    <t>BNK</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>대표</t>
+  </si>
+  <si>
+    <t>인수</t>
+  </si>
+  <si>
+    <t>공동대표</t>
+  </si>
+  <si>
+    <t>2024-08-01</t>
+  </si>
+  <si>
+    <t>2024-07-22</t>
+  </si>
+  <si>
+    <t>2024-07-18</t>
+  </si>
+  <si>
+    <t>2024-07-16</t>
+  </si>
+  <si>
+    <t>2024-06-20</t>
+  </si>
+  <si>
+    <t>2024-06-19</t>
+  </si>
+  <si>
+    <t>2024-06-18</t>
+  </si>
+  <si>
+    <t>2024-06-17</t>
+  </si>
+  <si>
+    <t>2024-06-14</t>
+  </si>
+  <si>
+    <t>2024-06-13</t>
+  </si>
+  <si>
+    <t>2024-07-30</t>
+  </si>
+  <si>
+    <t>2024-07-23</t>
+  </si>
+  <si>
+    <t>2024-07-19</t>
+  </si>
+  <si>
+    <t>2024-07-08</t>
+  </si>
+  <si>
+    <t>2024-07-05</t>
+  </si>
+  <si>
     <t>2024-06-21</t>
   </si>
   <si>
-    <t>2024-07-01</t>
-  </si>
-  <si>
-    <t>뱅크웨어글로벌</t>
-  </si>
-  <si>
-    <t>아이빔테크놀로지</t>
-  </si>
-  <si>
-    <t>피앤에스미캐닉스</t>
-  </si>
-  <si>
-    <t>산일전기</t>
-  </si>
-  <si>
-    <t>엔에이치스팩31호</t>
-  </si>
-  <si>
-    <t>SK증권제13호스팩</t>
-  </si>
-  <si>
-    <t>엑셀세라퓨틱스</t>
-  </si>
-  <si>
-    <t>시프트업</t>
-  </si>
-  <si>
-    <t>이베스트스팩6호</t>
-  </si>
-  <si>
-    <t>하스</t>
-  </si>
-  <si>
-    <t>이노스페이스</t>
-  </si>
-  <si>
-    <t>에이치브이엠</t>
-  </si>
-  <si>
-    <t>하이젠알앤엠</t>
-  </si>
-  <si>
-    <t>한국제15호스팩</t>
-  </si>
-  <si>
-    <t>에스오에스랩</t>
-  </si>
-  <si>
-    <t>미래에셋비전스팩6호</t>
-  </si>
-  <si>
-    <t>KB제29호스팩</t>
-  </si>
-  <si>
-    <t>에이치엠씨제7호스팩</t>
-  </si>
-  <si>
-    <t>신한글로벌액티브리츠</t>
-  </si>
-  <si>
-    <t>코스닥</t>
-  </si>
-  <si>
-    <t>코스피</t>
-  </si>
-  <si>
-    <t>미래</t>
-  </si>
-  <si>
-    <t>삼성</t>
-  </si>
-  <si>
-    <t>키움</t>
-  </si>
-  <si>
-    <t>NH</t>
-  </si>
-  <si>
-    <t>SK</t>
-  </si>
-  <si>
-    <t>대신</t>
-  </si>
-  <si>
-    <t>한국</t>
-  </si>
-  <si>
-    <t>제이피모간회사</t>
-  </si>
-  <si>
-    <t>신한</t>
-  </si>
-  <si>
-    <t>LS</t>
-  </si>
-  <si>
-    <t>BNK</t>
-  </si>
-  <si>
-    <t>KB</t>
-  </si>
-  <si>
-    <t>현대차</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>대표</t>
-  </si>
-  <si>
-    <t>인수</t>
-  </si>
-  <si>
-    <t>공동대표</t>
-  </si>
-  <si>
-    <t>2024-08-01</t>
-  </si>
-  <si>
-    <t>2024-07-22</t>
-  </si>
-  <si>
-    <t>2024-07-18</t>
-  </si>
-  <si>
-    <t>2024-07-16</t>
-  </si>
-  <si>
-    <t>2024-06-20</t>
-  </si>
-  <si>
-    <t>2024-06-19</t>
-  </si>
-  <si>
-    <t>2024-06-18</t>
-  </si>
-  <si>
-    <t>2024-06-17</t>
-  </si>
-  <si>
-    <t>2024-06-14</t>
-  </si>
-  <si>
-    <t>2024-06-13</t>
-  </si>
-  <si>
-    <t>2024-06-11</t>
-  </si>
-  <si>
-    <t>2024-07-30</t>
-  </si>
-  <si>
-    <t>2024-07-23</t>
-  </si>
-  <si>
-    <t>2024-07-19</t>
-  </si>
-  <si>
-    <t>2024-07-08</t>
-  </si>
-  <si>
-    <t>2024-07-05</t>
-  </si>
-  <si>
     <t>회사명</t>
   </si>
   <si>
@@ -345,6 +339,9 @@
     <t>신한, 한국</t>
   </si>
   <si>
+    <t>330.1 : 1</t>
+  </si>
+  <si>
     <t>239.19 : 1</t>
   </si>
   <si>
@@ -393,12 +390,6 @@
     <t>607 : 1</t>
   </si>
   <si>
-    <t>408 : 1</t>
-  </si>
-  <si>
-    <t>205.26 : 1</t>
-  </si>
-  <si>
     <t>120.3 : 1</t>
   </si>
   <si>
@@ -417,10 +408,10 @@
     <t>한국, 제이피모간회사 서울지점, NH, 신한</t>
   </si>
   <si>
+    <t>미래, 삼성</t>
+  </si>
+  <si>
     <t>미래, 신한</t>
-  </si>
-  <si>
-    <t>미래, 삼성</t>
   </si>
 </sst>
 </file>
@@ -778,7 +769,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -842,49 +833,49 @@
         <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D2">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="E2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F2">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="G2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M2">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N2">
         <v>100</v>
       </c>
       <c r="O2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="P2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q2">
-        <v>1050000</v>
+        <v>4350000</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -895,49 +886,49 @@
         <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D3">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="E3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F3">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="G3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M3">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="N3">
         <v>100</v>
       </c>
       <c r="O3" t="s">
-        <v>22</v>
+        <v>71</v>
       </c>
       <c r="P3" t="s">
-        <v>84</v>
+        <v>19</v>
       </c>
       <c r="Q3">
-        <v>1675500</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -948,49 +939,49 @@
         <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D4">
-        <v>297</v>
+        <v>223.4</v>
       </c>
       <c r="E4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F4">
-        <v>297</v>
+        <v>223.4</v>
       </c>
       <c r="G4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M4">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="N4">
         <v>100</v>
       </c>
       <c r="O4" t="s">
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="P4" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="Q4">
-        <v>1012500</v>
+        <v>1675500</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -1001,99 +992,99 @@
         <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D5">
-        <v>2660</v>
+        <v>297</v>
       </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F5">
-        <v>2553.6</v>
+        <v>297</v>
       </c>
       <c r="G5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M5">
-        <v>35000</v>
+        <v>22000</v>
       </c>
       <c r="N5">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="O5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="P5" t="s">
-        <v>85</v>
+        <v>23</v>
       </c>
       <c r="Q5">
-        <v>9340690</v>
+        <v>1012500</v>
       </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D6">
         <v>2660</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F6">
-        <v>106.4</v>
+        <v>2553.6</v>
       </c>
       <c r="G6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="L6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M6">
         <v>35000</v>
       </c>
       <c r="N6">
-        <v>4</v>
+        <v>96</v>
       </c>
       <c r="O6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="P6" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="Q6">
         <v>9340690</v>
@@ -1110,46 +1101,46 @@
         <v>54</v>
       </c>
       <c r="D7">
-        <v>120</v>
+        <v>2660</v>
       </c>
       <c r="E7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F7">
-        <v>120</v>
+        <v>106.4</v>
       </c>
       <c r="G7" t="s">
+        <v>67</v>
+      </c>
+      <c r="H7" t="s">
+        <v>67</v>
+      </c>
+      <c r="I7" t="s">
+        <v>67</v>
+      </c>
+      <c r="J7" t="s">
+        <v>67</v>
+      </c>
+      <c r="K7" t="s">
         <v>69</v>
       </c>
-      <c r="H7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I7" t="s">
-        <v>69</v>
-      </c>
-      <c r="J7" t="s">
-        <v>69</v>
-      </c>
-      <c r="K7" t="s">
-        <v>70</v>
-      </c>
       <c r="L7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M7">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="N7">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="O7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P7" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="Q7">
-        <v>4500000</v>
+        <v>9340690</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -1160,34 +1151,34 @@
         <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D8">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F8">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="G8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M8">
         <v>2000</v>
@@ -1196,13 +1187,13 @@
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>23</v>
+        <v>74</v>
       </c>
       <c r="P8" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="Q8">
-        <v>3000000</v>
+        <v>4500000</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -1213,49 +1204,49 @@
         <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D9">
-        <v>161.8</v>
+        <v>80</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F9">
-        <v>161.8</v>
+        <v>80</v>
       </c>
       <c r="G9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M9">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="N9">
         <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="P9" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="Q9">
-        <v>1187900</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -1266,87 +1257,87 @@
         <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D10">
-        <v>4350</v>
+        <v>161.8</v>
       </c>
       <c r="E10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F10">
-        <v>1435.5</v>
+        <v>161.8</v>
       </c>
       <c r="G10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M10">
-        <v>60000</v>
+        <v>10000</v>
       </c>
       <c r="N10">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="O10" t="s">
         <v>27</v>
       </c>
       <c r="P10" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Q10">
-        <v>21750000</v>
+        <v>1187900</v>
       </c>
     </row>
     <row r="11" spans="1:17">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D11">
         <v>4350</v>
       </c>
       <c r="E11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F11">
         <v>1435.5</v>
       </c>
       <c r="G11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K11" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M11">
         <v>60000</v>
@@ -1355,10 +1346,10 @@
         <v>33</v>
       </c>
       <c r="O11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P11" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="Q11">
         <v>21750000</v>
@@ -1366,52 +1357,52 @@
     </row>
     <row r="12" spans="1:17">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D12">
         <v>4350</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F12">
-        <v>1305</v>
+        <v>1435.5</v>
       </c>
       <c r="G12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M12">
         <v>60000</v>
       </c>
       <c r="N12">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="O12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P12" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="Q12">
         <v>21750000</v>
@@ -1419,52 +1410,52 @@
     </row>
     <row r="13" spans="1:17">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D13">
         <v>4350</v>
       </c>
       <c r="E13" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="F13">
-        <v>174</v>
+        <v>1305</v>
       </c>
       <c r="G13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K13" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="L13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M13">
         <v>60000</v>
       </c>
       <c r="N13">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="O13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P13" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="Q13">
         <v>21750000</v>
@@ -1481,46 +1472,46 @@
         <v>54</v>
       </c>
       <c r="D14">
-        <v>80</v>
+        <v>4350</v>
       </c>
       <c r="E14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F14">
-        <v>80</v>
+        <v>174</v>
       </c>
       <c r="G14" t="s">
+        <v>67</v>
+      </c>
+      <c r="H14" t="s">
+        <v>67</v>
+      </c>
+      <c r="I14" t="s">
+        <v>67</v>
+      </c>
+      <c r="J14" t="s">
+        <v>67</v>
+      </c>
+      <c r="K14" t="s">
         <v>69</v>
       </c>
-      <c r="H14" t="s">
-        <v>69</v>
-      </c>
-      <c r="I14" t="s">
-        <v>69</v>
-      </c>
-      <c r="J14" t="s">
-        <v>69</v>
-      </c>
-      <c r="K14" t="s">
-        <v>70</v>
-      </c>
       <c r="L14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M14">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="N14">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="O14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P14" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="Q14">
-        <v>3000000</v>
+        <v>21750000</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1531,49 +1522,49 @@
         <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D15">
-        <v>289.6</v>
+        <v>80</v>
       </c>
       <c r="E15" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="F15">
-        <v>289.6</v>
+        <v>80</v>
       </c>
       <c r="G15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M15">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N15">
         <v>100</v>
       </c>
       <c r="O15" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="P15" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="Q15">
-        <v>1357500</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -1584,99 +1575,99 @@
         <v>45</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D16">
-        <v>575.89</v>
+        <v>289.6</v>
       </c>
       <c r="E16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F16">
-        <v>541.3366</v>
+        <v>289.6</v>
       </c>
       <c r="G16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K16" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M16">
-        <v>43300</v>
+        <v>16000</v>
       </c>
       <c r="N16">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="O16" t="s">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="P16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Q16">
-        <v>1906400</v>
+        <v>1357500</v>
       </c>
     </row>
     <row r="17" spans="1:17">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D17">
         <v>575.89</v>
       </c>
       <c r="E17" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="F17">
-        <v>34.5534</v>
+        <v>541.3366</v>
       </c>
       <c r="G17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K17" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="L17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M17">
         <v>43300</v>
       </c>
       <c r="N17">
-        <v>6</v>
+        <v>94</v>
       </c>
       <c r="O17" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="P17" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="Q17">
         <v>1906400</v>
@@ -1690,49 +1681,49 @@
         <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D18">
-        <v>432</v>
+        <v>575.89</v>
       </c>
       <c r="E18" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="F18">
-        <v>432</v>
+        <v>34.5534</v>
       </c>
       <c r="G18" t="s">
+        <v>67</v>
+      </c>
+      <c r="H18" t="s">
+        <v>67</v>
+      </c>
+      <c r="I18" t="s">
+        <v>67</v>
+      </c>
+      <c r="J18" t="s">
+        <v>67</v>
+      </c>
+      <c r="K18" t="s">
         <v>69</v>
       </c>
-      <c r="H18" t="s">
-        <v>69</v>
-      </c>
-      <c r="I18" t="s">
-        <v>69</v>
-      </c>
-      <c r="J18" t="s">
-        <v>69</v>
-      </c>
-      <c r="K18" t="s">
-        <v>70</v>
-      </c>
       <c r="L18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M18">
-        <v>18000</v>
+        <v>43300</v>
       </c>
       <c r="N18">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="O18" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="P18" t="s">
         <v>32</v>
       </c>
       <c r="Q18">
-        <v>1758600</v>
+        <v>1906400</v>
       </c>
     </row>
     <row r="19" spans="1:17">
@@ -1743,49 +1734,49 @@
         <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D19">
-        <v>238</v>
+        <v>432</v>
       </c>
       <c r="E19" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F19">
-        <v>238</v>
+        <v>432</v>
       </c>
       <c r="G19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K19" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M19">
-        <v>7000</v>
+        <v>18000</v>
       </c>
       <c r="N19">
         <v>100</v>
       </c>
       <c r="O19" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="P19" t="s">
         <v>33</v>
       </c>
       <c r="Q19">
-        <v>2350000</v>
+        <v>1758600</v>
       </c>
     </row>
     <row r="20" spans="1:17">
@@ -1796,49 +1787,49 @@
         <v>48</v>
       </c>
       <c r="C20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D20">
-        <v>125</v>
+        <v>238</v>
       </c>
       <c r="E20" t="s">
         <v>62</v>
       </c>
       <c r="F20">
-        <v>125</v>
+        <v>238</v>
       </c>
       <c r="G20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K20" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M20">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="N20">
         <v>100</v>
       </c>
       <c r="O20" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="P20" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="Q20">
-        <v>4687500</v>
+        <v>2350000</v>
       </c>
     </row>
     <row r="21" spans="1:17">
@@ -1849,99 +1840,99 @@
         <v>49</v>
       </c>
       <c r="C21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D21">
-        <v>230</v>
+        <v>125</v>
       </c>
       <c r="E21" t="s">
         <v>62</v>
       </c>
       <c r="F21">
-        <v>218.5</v>
+        <v>125</v>
       </c>
       <c r="G21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K21" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M21">
-        <v>11500</v>
+        <v>2000</v>
       </c>
       <c r="N21">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O21" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="P21" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="Q21">
-        <v>3000000</v>
+        <v>4687500</v>
       </c>
     </row>
     <row r="22" spans="1:17">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D22">
         <v>230</v>
       </c>
       <c r="E22" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F22">
-        <v>11.5</v>
+        <v>218.5</v>
       </c>
       <c r="G22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K22" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="L22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M22">
         <v>11500</v>
       </c>
       <c r="N22">
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="O22" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="P22" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="Q22">
         <v>3000000</v>
@@ -1955,49 +1946,49 @@
         <v>50</v>
       </c>
       <c r="C23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D23">
-        <v>129</v>
+        <v>230</v>
       </c>
       <c r="E23" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="F23">
-        <v>129</v>
+        <v>11.5</v>
       </c>
       <c r="G23" t="s">
+        <v>67</v>
+      </c>
+      <c r="H23" t="s">
+        <v>67</v>
+      </c>
+      <c r="I23" t="s">
+        <v>67</v>
+      </c>
+      <c r="J23" t="s">
+        <v>67</v>
+      </c>
+      <c r="K23" t="s">
         <v>69</v>
       </c>
-      <c r="H23" t="s">
-        <v>69</v>
-      </c>
-      <c r="I23" t="s">
-        <v>69</v>
-      </c>
-      <c r="J23" t="s">
-        <v>69</v>
-      </c>
-      <c r="K23" t="s">
-        <v>70</v>
-      </c>
       <c r="L23" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M23">
-        <v>2000</v>
+        <v>11500</v>
       </c>
       <c r="N23">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="O23" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="P23" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="Q23">
-        <v>4837500</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="24" spans="1:17">
@@ -2008,34 +1999,34 @@
         <v>51</v>
       </c>
       <c r="C24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D24">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="E24" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="F24">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="G24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K24" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M24">
         <v>2000</v>
@@ -2044,18 +2035,18 @@
         <v>100</v>
       </c>
       <c r="O24" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="P24" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="Q24">
-        <v>4500000</v>
+        <v>4837500</v>
       </c>
     </row>
     <row r="25" spans="1:17">
       <c r="A25" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B25" t="s">
         <v>52</v>
@@ -2064,46 +2055,46 @@
         <v>54</v>
       </c>
       <c r="D25">
-        <v>140</v>
+        <v>700.0000199999999</v>
       </c>
       <c r="E25" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F25">
-        <v>140</v>
+        <v>350.00001</v>
       </c>
       <c r="G25" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H25" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I25" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J25" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K25" t="s">
         <v>70</v>
       </c>
       <c r="L25" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M25">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="N25">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="O25" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="P25" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="Q25">
-        <v>5250000</v>
+        <v>32666668</v>
       </c>
     </row>
     <row r="26" spans="1:17">
@@ -2111,37 +2102,37 @@
         <v>34</v>
       </c>
       <c r="B26" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D26">
         <v>700.0000199999999</v>
       </c>
       <c r="E26" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F26">
         <v>350.00001</v>
       </c>
       <c r="G26" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H26" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I26" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J26" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K26" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="L26" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M26">
         <v>3000</v>
@@ -2150,65 +2141,12 @@
         <v>50</v>
       </c>
       <c r="O26" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="P26" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="Q26">
-        <v>32666668</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17">
-      <c r="A27" t="s">
-        <v>34</v>
-      </c>
-      <c r="B27" t="s">
-        <v>53</v>
-      </c>
-      <c r="C27" t="s">
-        <v>55</v>
-      </c>
-      <c r="D27">
-        <v>700.0000199999999</v>
-      </c>
-      <c r="E27" t="s">
-        <v>62</v>
-      </c>
-      <c r="F27">
-        <v>350.00001</v>
-      </c>
-      <c r="G27" t="s">
-        <v>69</v>
-      </c>
-      <c r="H27" t="s">
-        <v>69</v>
-      </c>
-      <c r="I27" t="s">
-        <v>69</v>
-      </c>
-      <c r="J27" t="s">
-        <v>69</v>
-      </c>
-      <c r="K27" t="s">
-        <v>72</v>
-      </c>
-      <c r="L27" t="s">
-        <v>69</v>
-      </c>
-      <c r="M27">
-        <v>3000</v>
-      </c>
-      <c r="N27">
-        <v>50</v>
-      </c>
-      <c r="O27" t="s">
-        <v>82</v>
-      </c>
-      <c r="P27" t="s">
-        <v>79</v>
-      </c>
-      <c r="Q27">
         <v>32666668</v>
       </c>
     </row>
@@ -2219,7 +2157,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -2227,10 +2165,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -2239,385 +2177,385 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B2" t="s">
         <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
       </c>
       <c r="F2">
-        <v>22400000</v>
+        <v>11600000</v>
       </c>
       <c r="G2">
-        <v>1400000</v>
+        <v>5800000</v>
       </c>
       <c r="H2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I2">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="J2">
-        <v>19000</v>
+        <v>2000</v>
       </c>
       <c r="K2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L2">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="M2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="S2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>71</v>
       </c>
       <c r="B3" t="s">
         <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D3" t="s">
-        <v>84</v>
+        <v>19</v>
       </c>
       <c r="E3" t="s">
         <v>18</v>
       </c>
       <c r="F3">
-        <v>22340000</v>
+        <v>22400000</v>
       </c>
       <c r="G3">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="H3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I3">
-        <v>7300</v>
+        <v>16000</v>
       </c>
       <c r="J3">
-        <v>8500</v>
+        <v>19000</v>
       </c>
       <c r="K3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L3">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="M3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="S3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
         <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="E4" t="s">
         <v>19</v>
       </c>
       <c r="F4">
-        <v>29700000</v>
+        <v>22340000</v>
       </c>
       <c r="G4">
-        <v>1350000</v>
+        <v>2234000</v>
       </c>
       <c r="H4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I4">
-        <v>14000</v>
+        <v>7300</v>
       </c>
       <c r="J4">
-        <v>17000</v>
+        <v>8500</v>
       </c>
       <c r="K4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L4">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="M4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="S4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B5" t="s">
         <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>85</v>
+        <v>23</v>
       </c>
       <c r="E5" t="s">
         <v>20</v>
       </c>
       <c r="F5">
-        <v>266000000</v>
+        <v>29700000</v>
       </c>
       <c r="G5">
-        <v>7600000</v>
+        <v>1350000</v>
       </c>
       <c r="H5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I5">
-        <v>24000</v>
+        <v>14000</v>
       </c>
       <c r="J5">
-        <v>30000</v>
+        <v>17000</v>
       </c>
       <c r="K5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L5">
-        <v>35000</v>
+        <v>22000</v>
       </c>
       <c r="M5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O5">
-        <v>14.47368421052632</v>
+        <v>0</v>
       </c>
       <c r="P5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="S5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B6" t="s">
         <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D6" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E6" t="s">
         <v>21</v>
       </c>
       <c r="F6">
-        <v>12000000</v>
+        <v>266000000</v>
       </c>
       <c r="G6">
-        <v>6000000</v>
+        <v>7600000</v>
       </c>
       <c r="H6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I6">
-        <v>2000</v>
+        <v>24000</v>
       </c>
       <c r="J6">
-        <v>2000</v>
+        <v>30000</v>
       </c>
       <c r="K6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L6">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="M6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>14.47368421052632</v>
       </c>
       <c r="P6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R6" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="S6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>74</v>
       </c>
       <c r="B7" t="s">
         <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E7" t="s">
         <v>22</v>
       </c>
       <c r="F7">
-        <v>8000000</v>
+        <v>12000000</v>
       </c>
       <c r="G7">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="H7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I7">
         <v>2000</v>
@@ -2626,96 +2564,96 @@
         <v>2000</v>
       </c>
       <c r="K7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L7">
         <v>2000</v>
       </c>
       <c r="M7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="S7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s">
         <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="E8" t="s">
         <v>23</v>
       </c>
       <c r="F8">
-        <v>16180000</v>
+        <v>8000000</v>
       </c>
       <c r="G8">
-        <v>1618000</v>
+        <v>4000000</v>
       </c>
       <c r="H8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I8">
-        <v>6200</v>
+        <v>2000</v>
       </c>
       <c r="J8">
-        <v>7700</v>
+        <v>2000</v>
       </c>
       <c r="K8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L8">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="M8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R8" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="S8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -2726,255 +2664,255 @@
         <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E9" t="s">
         <v>24</v>
       </c>
       <c r="F9">
-        <v>435000000</v>
+        <v>16180000</v>
       </c>
       <c r="G9">
-        <v>7250000</v>
+        <v>1618000</v>
       </c>
       <c r="H9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I9">
-        <v>47000</v>
+        <v>6200</v>
       </c>
       <c r="J9">
-        <v>60000</v>
+        <v>7700</v>
       </c>
       <c r="K9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L9">
-        <v>60000</v>
+        <v>10000</v>
       </c>
       <c r="M9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O9">
         <v>0</v>
       </c>
       <c r="P9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R9" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="S9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
         <v>43</v>
       </c>
       <c r="C10" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D10" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E10" t="s">
         <v>25</v>
       </c>
       <c r="F10">
-        <v>8000000</v>
+        <v>435000000</v>
       </c>
       <c r="G10">
-        <v>4000000</v>
+        <v>7250000</v>
       </c>
       <c r="H10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I10">
-        <v>2000</v>
+        <v>47000</v>
       </c>
       <c r="J10">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="K10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L10">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="M10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O10">
         <v>0</v>
       </c>
       <c r="P10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="S10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
         <v>44</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>105</v>
       </c>
       <c r="D11" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="E11" t="s">
         <v>26</v>
       </c>
       <c r="F11">
-        <v>28960000</v>
+        <v>8000000</v>
       </c>
       <c r="G11">
-        <v>1810000</v>
+        <v>4000000</v>
       </c>
       <c r="H11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I11">
-        <v>9000</v>
+        <v>2000</v>
       </c>
       <c r="J11">
-        <v>12000</v>
+        <v>2000</v>
       </c>
       <c r="K11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L11">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="M11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O11">
         <v>0</v>
       </c>
       <c r="P11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="S11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="B12" t="s">
         <v>45</v>
       </c>
       <c r="C12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E12" t="s">
         <v>27</v>
       </c>
       <c r="F12">
-        <v>57589000</v>
+        <v>28960000</v>
       </c>
       <c r="G12">
-        <v>1330000</v>
+        <v>1810000</v>
       </c>
       <c r="H12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I12">
-        <v>36400</v>
+        <v>9000</v>
       </c>
       <c r="J12">
-        <v>43300</v>
+        <v>12000</v>
       </c>
       <c r="K12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L12">
-        <v>43300</v>
+        <v>16000</v>
       </c>
       <c r="M12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O12">
         <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R12" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="S12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
         <v>46</v>
       </c>
       <c r="C13" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D13" t="s">
         <v>32</v>
@@ -2983,60 +2921,60 @@
         <v>28</v>
       </c>
       <c r="F13">
-        <v>43200000</v>
+        <v>57589000</v>
       </c>
       <c r="G13">
-        <v>2400000</v>
+        <v>1330000</v>
       </c>
       <c r="H13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I13">
-        <v>11000</v>
+        <v>36400</v>
       </c>
       <c r="J13">
-        <v>14200</v>
+        <v>43300</v>
       </c>
       <c r="K13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L13">
-        <v>18000</v>
+        <v>43300</v>
       </c>
       <c r="M13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O13">
         <v>0</v>
       </c>
       <c r="P13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="S13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
         <v>47</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D14" t="s">
         <v>33</v>
@@ -3045,54 +2983,54 @@
         <v>29</v>
       </c>
       <c r="F14">
-        <v>23800000</v>
+        <v>43200000</v>
       </c>
       <c r="G14">
-        <v>3400000</v>
+        <v>2400000</v>
       </c>
       <c r="H14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I14">
-        <v>4500</v>
+        <v>11000</v>
       </c>
       <c r="J14">
-        <v>5500</v>
+        <v>14200</v>
       </c>
       <c r="K14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L14">
-        <v>7000</v>
+        <v>18000</v>
       </c>
       <c r="M14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O14">
         <v>0</v>
       </c>
       <c r="P14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="S14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B15" t="s">
         <v>48</v>
@@ -3101,60 +3039,60 @@
         <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="E15" t="s">
         <v>30</v>
       </c>
       <c r="F15">
-        <v>12500000</v>
+        <v>23800000</v>
       </c>
       <c r="G15">
-        <v>6250000</v>
+        <v>3400000</v>
       </c>
       <c r="H15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I15">
-        <v>2000</v>
+        <v>4500</v>
       </c>
       <c r="J15">
-        <v>2000</v>
+        <v>5500</v>
       </c>
       <c r="K15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L15">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="M15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O15">
         <v>0</v>
       </c>
       <c r="P15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R15" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="S15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:20">
       <c r="A16" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
         <v>49</v>
@@ -3163,143 +3101,143 @@
         <v>62</v>
       </c>
       <c r="D16" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E16" t="s">
         <v>31</v>
       </c>
       <c r="F16">
-        <v>23000000</v>
+        <v>12500000</v>
       </c>
       <c r="G16">
-        <v>2000000</v>
+        <v>6250000</v>
       </c>
       <c r="H16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I16">
-        <v>7500</v>
+        <v>2000</v>
       </c>
       <c r="J16">
-        <v>9000</v>
+        <v>2000</v>
       </c>
       <c r="K16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L16">
-        <v>11500</v>
+        <v>2000</v>
       </c>
       <c r="M16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O16">
         <v>0</v>
       </c>
       <c r="P16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R16" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="S16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:20">
       <c r="A17" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
         <v>50</v>
       </c>
       <c r="C17" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E17" t="s">
         <v>32</v>
       </c>
       <c r="F17">
-        <v>12900000</v>
+        <v>23000000</v>
       </c>
       <c r="G17">
-        <v>6450000</v>
+        <v>2000000</v>
       </c>
       <c r="H17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I17">
-        <v>2000</v>
+        <v>7500</v>
       </c>
       <c r="J17">
-        <v>2000</v>
+        <v>9000</v>
       </c>
       <c r="K17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L17">
-        <v>2000</v>
+        <v>11500</v>
       </c>
       <c r="M17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O17">
         <v>0</v>
       </c>
       <c r="P17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R17" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="S17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:20">
       <c r="A18" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s">
         <v>51</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="D18" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E18" t="s">
         <v>33</v>
       </c>
       <c r="F18">
-        <v>12000000</v>
+        <v>12900000</v>
       </c>
       <c r="G18">
-        <v>6000000</v>
+        <v>6450000</v>
       </c>
       <c r="H18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I18">
         <v>2000</v>
@@ -3308,158 +3246,96 @@
         <v>2000</v>
       </c>
       <c r="K18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L18">
         <v>2000</v>
       </c>
       <c r="M18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O18">
         <v>0</v>
       </c>
       <c r="P18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R18" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="S18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:20">
       <c r="A19" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B19" t="s">
         <v>52</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
+        <v>106</v>
       </c>
       <c r="D19" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F19">
-        <v>14000000</v>
+        <v>70000002</v>
       </c>
       <c r="G19">
-        <v>7000000</v>
+        <v>23333334</v>
       </c>
       <c r="H19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I19">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="J19">
-        <v>2000</v>
+        <v>3800</v>
       </c>
       <c r="K19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L19">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="M19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O19">
         <v>0</v>
       </c>
       <c r="P19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R19" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="S19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T19" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20">
-      <c r="A20" t="s">
-        <v>82</v>
-      </c>
-      <c r="B20" t="s">
-        <v>53</v>
-      </c>
-      <c r="C20" t="s">
-        <v>108</v>
-      </c>
-      <c r="D20" t="s">
-        <v>79</v>
-      </c>
-      <c r="E20" t="s">
-        <v>34</v>
-      </c>
-      <c r="F20">
-        <v>70000002</v>
-      </c>
-      <c r="G20">
-        <v>23333334</v>
-      </c>
-      <c r="H20" t="s">
-        <v>69</v>
-      </c>
-      <c r="I20">
-        <v>3000</v>
-      </c>
-      <c r="J20">
-        <v>3800</v>
-      </c>
-      <c r="K20" t="s">
-        <v>69</v>
-      </c>
-      <c r="L20">
-        <v>3000</v>
-      </c>
-      <c r="M20" t="s">
-        <v>69</v>
-      </c>
-      <c r="N20" t="s">
-        <v>69</v>
-      </c>
-      <c r="O20">
-        <v>0</v>
-      </c>
-      <c r="P20" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>69</v>
-      </c>
-      <c r="R20" t="s">
-        <v>127</v>
-      </c>
-      <c r="S20" t="s">
-        <v>69</v>
-      </c>
-      <c r="T20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -3469,21 +3345,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -3495,10 +3371,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -3507,7 +3383,7 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -3515,22 +3391,22 @@
         <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D2" t="s">
         <v>62</v>
       </c>
       <c r="E2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="F2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H2">
         <v>1150</v>
@@ -3550,31 +3426,31 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>83</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="F3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="H3">
-        <v>12000</v>
+        <v>8000</v>
       </c>
       <c r="I3">
-        <v>6000000</v>
+        <v>4000000</v>
       </c>
       <c r="J3">
         <v>2000</v>
@@ -3588,31 +3464,31 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D4" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="E4" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="F4" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="G4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H4">
-        <v>8000</v>
+        <v>12000</v>
       </c>
       <c r="I4">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="J4">
         <v>2000</v>
@@ -3629,10 +3505,10 @@
         <v>59</v>
       </c>
       <c r="B5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D5" t="s">
         <v>59</v>
@@ -3641,10 +3517,10 @@
         <v>59</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H5">
         <v>43200</v>
@@ -3667,104 +3543,104 @@
         <v>59</v>
       </c>
       <c r="B6" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D6" t="s">
-        <v>59</v>
+        <v>104</v>
       </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>129</v>
       </c>
       <c r="F6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H6">
-        <v>12000</v>
+        <v>130500</v>
       </c>
       <c r="I6">
-        <v>6000000</v>
+        <v>7250000</v>
       </c>
       <c r="J6">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="K6">
         <v>0</v>
       </c>
       <c r="L6">
-        <v>100</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>106</v>
+        <v>60</v>
       </c>
       <c r="E7" t="s">
-        <v>132</v>
+        <v>60</v>
       </c>
       <c r="F7" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="G7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H7">
-        <v>130500</v>
+        <v>8000</v>
       </c>
       <c r="I7">
-        <v>7250000</v>
+        <v>4000000</v>
       </c>
       <c r="J7">
-        <v>60000</v>
+        <v>2000</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7">
-        <v>30</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F8" t="s">
-        <v>75</v>
+        <v>19</v>
       </c>
       <c r="G8" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="H8">
-        <v>8000</v>
+        <v>11600</v>
       </c>
       <c r="I8">
-        <v>4000000</v>
+        <v>5800000</v>
       </c>
       <c r="J8">
         <v>2000</v>
@@ -3781,10 +3657,10 @@
         <v>61</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
         <v>61</v>
@@ -3793,10 +3669,10 @@
         <v>61</v>
       </c>
       <c r="F9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="G9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H9">
         <v>16180</v>
@@ -3819,10 +3695,10 @@
         <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="D10" t="s">
         <v>56</v>
@@ -3831,19 +3707,19 @@
         <v>56</v>
       </c>
       <c r="F10" t="s">
-        <v>79</v>
+        <v>19</v>
       </c>
       <c r="G10" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="H10">
-        <v>12900</v>
+        <v>22400</v>
       </c>
       <c r="I10">
-        <v>6450000</v>
+        <v>1400000</v>
       </c>
       <c r="J10">
-        <v>2000</v>
+        <v>16000</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -3857,37 +3733,37 @@
         <v>56</v>
       </c>
       <c r="B11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="D11" t="s">
         <v>56</v>
       </c>
       <c r="E11" t="s">
-        <v>133</v>
+        <v>56</v>
       </c>
       <c r="F11" t="s">
-        <v>31</v>
+        <v>77</v>
       </c>
       <c r="G11" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="H11">
-        <v>54133.66</v>
+        <v>12900</v>
       </c>
       <c r="I11">
-        <v>1330000</v>
+        <v>6450000</v>
       </c>
       <c r="J11">
-        <v>43300</v>
+        <v>2000</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -3898,34 +3774,34 @@
         <v>73</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D12" t="s">
         <v>56</v>
       </c>
       <c r="E12" t="s">
-        <v>56</v>
+        <v>130</v>
       </c>
       <c r="F12" t="s">
-        <v>18</v>
+        <v>82</v>
       </c>
       <c r="G12" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="H12">
-        <v>22400</v>
+        <v>255360</v>
       </c>
       <c r="I12">
-        <v>1400000</v>
+        <v>7600000</v>
       </c>
       <c r="J12">
-        <v>16000</v>
+        <v>35000</v>
       </c>
       <c r="K12">
         <v>0</v>
       </c>
       <c r="L12">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -3936,34 +3812,34 @@
         <v>75</v>
       </c>
       <c r="C13" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D13" t="s">
         <v>56</v>
       </c>
       <c r="E13" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="F13" t="s">
-        <v>85</v>
+        <v>32</v>
       </c>
       <c r="G13" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="H13">
-        <v>255360</v>
+        <v>54133.66</v>
       </c>
       <c r="I13">
-        <v>7600000</v>
+        <v>1330000</v>
       </c>
       <c r="J13">
-        <v>35000</v>
+        <v>43300</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -3971,10 +3847,10 @@
         <v>57</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="D14" t="s">
         <v>57</v>
@@ -3983,19 +3859,19 @@
         <v>57</v>
       </c>
       <c r="F14" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="G14" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="H14">
-        <v>28960</v>
+        <v>22340</v>
       </c>
       <c r="I14">
-        <v>1810000</v>
+        <v>2234000</v>
       </c>
       <c r="J14">
-        <v>16000</v>
+        <v>10000</v>
       </c>
       <c r="K14">
         <v>0</v>
@@ -4009,22 +3885,22 @@
         <v>57</v>
       </c>
       <c r="B15" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D15" t="s">
         <v>56</v>
       </c>
       <c r="E15" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H15">
         <v>10640</v>
@@ -4047,10 +3923,10 @@
         <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C16" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="D16" t="s">
         <v>57</v>
@@ -4059,19 +3935,19 @@
         <v>57</v>
       </c>
       <c r="F16" t="s">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="G16" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="H16">
-        <v>22340</v>
+        <v>28960</v>
       </c>
       <c r="I16">
-        <v>2234000</v>
+        <v>1810000</v>
       </c>
       <c r="J16">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="K16">
         <v>0</v>
@@ -4085,37 +3961,37 @@
         <v>64</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="C17" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D17" t="s">
-        <v>106</v>
+        <v>56</v>
       </c>
       <c r="E17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F17" t="s">
-        <v>88</v>
+        <v>32</v>
       </c>
       <c r="G17" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="H17">
-        <v>17400</v>
+        <v>3455.34</v>
       </c>
       <c r="I17">
-        <v>7250000</v>
+        <v>1330000</v>
       </c>
       <c r="J17">
-        <v>60000</v>
+        <v>43300</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
       <c r="L17">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -4123,37 +3999,37 @@
         <v>64</v>
       </c>
       <c r="B18" t="s">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="D18" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E18" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="F18" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G18" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="H18">
-        <v>35000.001</v>
+        <v>17400</v>
       </c>
       <c r="I18">
-        <v>23333334</v>
+        <v>7250000</v>
       </c>
       <c r="J18">
-        <v>3000</v>
+        <v>60000</v>
       </c>
       <c r="K18">
         <v>0</v>
       </c>
       <c r="L18">
-        <v>50</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -4161,37 +4037,37 @@
         <v>64</v>
       </c>
       <c r="B19" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" t="s">
+        <v>106</v>
+      </c>
+      <c r="E19" t="s">
+        <v>106</v>
+      </c>
+      <c r="F19" t="s">
         <v>77</v>
       </c>
-      <c r="C19" t="s">
-        <v>45</v>
-      </c>
-      <c r="D19" t="s">
-        <v>56</v>
-      </c>
-      <c r="E19" t="s">
-        <v>133</v>
-      </c>
-      <c r="F19" t="s">
-        <v>31</v>
-      </c>
       <c r="G19" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="H19">
-        <v>3455.34</v>
+        <v>35000.001</v>
       </c>
       <c r="I19">
-        <v>1330000</v>
+        <v>23333334</v>
       </c>
       <c r="J19">
-        <v>43300</v>
+        <v>3000</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>6</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -4199,22 +4075,22 @@
         <v>63</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D20" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E20" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F20" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="G20" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H20">
         <v>143550</v>
@@ -4237,10 +4113,10 @@
         <v>58</v>
       </c>
       <c r="B21" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C21" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D21" t="s">
         <v>58</v>
@@ -4249,10 +4125,10 @@
         <v>58</v>
       </c>
       <c r="F21" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G21" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H21">
         <v>29700</v>
@@ -4275,37 +4151,37 @@
         <v>62</v>
       </c>
       <c r="B22" t="s">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="C22" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D22" t="s">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="E22" t="s">
-        <v>132</v>
+        <v>62</v>
       </c>
       <c r="F22" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G22" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="H22">
-        <v>143550</v>
+        <v>23800</v>
       </c>
       <c r="I22">
-        <v>7250000</v>
+        <v>3400000</v>
       </c>
       <c r="J22">
-        <v>60000</v>
+        <v>7000</v>
       </c>
       <c r="K22">
         <v>0</v>
       </c>
       <c r="L22">
-        <v>33</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -4313,10 +4189,10 @@
         <v>62</v>
       </c>
       <c r="B23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D23" t="s">
         <v>62</v>
@@ -4325,19 +4201,19 @@
         <v>62</v>
       </c>
       <c r="F23" t="s">
-        <v>33</v>
+        <v>75</v>
       </c>
       <c r="G23" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H23">
-        <v>23800</v>
+        <v>12500</v>
       </c>
       <c r="I23">
-        <v>3400000</v>
+        <v>6250000</v>
       </c>
       <c r="J23">
-        <v>7000</v>
+        <v>2000</v>
       </c>
       <c r="K23">
         <v>0</v>
@@ -4351,37 +4227,37 @@
         <v>62</v>
       </c>
       <c r="B24" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C24" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D24" t="s">
         <v>62</v>
       </c>
       <c r="E24" t="s">
-        <v>62</v>
+        <v>128</v>
       </c>
       <c r="F24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G24" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H24">
-        <v>12500</v>
+        <v>21850</v>
       </c>
       <c r="I24">
-        <v>6250000</v>
+        <v>2000000</v>
       </c>
       <c r="J24">
-        <v>2000</v>
+        <v>11500</v>
       </c>
       <c r="K24">
         <v>0</v>
       </c>
       <c r="L24">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -4389,37 +4265,37 @@
         <v>62</v>
       </c>
       <c r="B25" t="s">
-        <v>81</v>
+        <v>28</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="D25" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="E25" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F25" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="G25" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="H25">
-        <v>21850</v>
+        <v>143550</v>
       </c>
       <c r="I25">
-        <v>2000000</v>
+        <v>7250000</v>
       </c>
       <c r="J25">
-        <v>11500</v>
+        <v>60000</v>
       </c>
       <c r="K25">
         <v>0</v>
       </c>
       <c r="L25">
-        <v>95</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -4427,19 +4303,19 @@
         <v>62</v>
       </c>
       <c r="B26" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C26" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D26" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E26" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F26" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G26" t="s">
         <v>34</v>
@@ -4458,44 +4334,6 @@
       </c>
       <c r="L26">
         <v>50</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12">
-      <c r="A27" t="s">
-        <v>68</v>
-      </c>
-      <c r="B27" t="s">
-        <v>83</v>
-      </c>
-      <c r="C27" t="s">
-        <v>52</v>
-      </c>
-      <c r="D27" t="s">
-        <v>68</v>
-      </c>
-      <c r="E27" t="s">
-        <v>68</v>
-      </c>
-      <c r="F27" t="s">
-        <v>81</v>
-      </c>
-      <c r="G27" t="s">
-        <v>32</v>
-      </c>
-      <c r="H27">
-        <v>14000</v>
-      </c>
-      <c r="I27">
-        <v>7000000</v>
-      </c>
-      <c r="J27">
-        <v>2000</v>
-      </c>
-      <c r="K27">
-        <v>0</v>
-      </c>
-      <c r="L27">
-        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-08-22
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="130">
   <si>
     <t>상장일</t>
   </si>
@@ -69,6 +69,9 @@
     <t>총기관배정수량</t>
   </si>
   <si>
+    <t>2024-08-21</t>
+  </si>
+  <si>
     <t>2024-08-19</t>
   </si>
   <si>
@@ -117,6 +120,9 @@
     <t>2024-06-28</t>
   </si>
   <si>
+    <t>티디에스팜</t>
+  </si>
+  <si>
     <t>전진건설로봇</t>
   </si>
   <si>
@@ -168,10 +174,13 @@
     <t>에이치브이엠</t>
   </si>
   <si>
+    <t>코스닥</t>
+  </si>
+  <si>
     <t>코스피</t>
   </si>
   <si>
-    <t>코스닥</t>
+    <t>한국</t>
   </si>
   <si>
     <t>미래</t>
@@ -180,9 +189,6 @@
     <t>하나</t>
   </si>
   <si>
-    <t>한국</t>
-  </si>
-  <si>
     <t>키움</t>
   </si>
   <si>
@@ -219,6 +225,9 @@
     <t>인수</t>
   </si>
   <si>
+    <t>2024-08-09</t>
+  </si>
+  <si>
     <t>2024-08-08</t>
   </si>
   <si>
@@ -246,7 +255,7 @@
     <t>2024-06-19</t>
   </si>
   <si>
-    <t>2024-08-09</t>
+    <t>2024-08-14</t>
   </si>
   <si>
     <t>2024-07-30</t>
@@ -327,6 +336,9 @@
     <t>엘에스</t>
   </si>
   <si>
+    <t>1608.17 : 1</t>
+  </si>
+  <si>
     <t>1087.3 : 1</t>
   </si>
   <si>
@@ -390,10 +402,10 @@
     <t>한국, 제이피모간회사 서울지점, NH, 신한</t>
   </si>
   <si>
+    <t>미래, 신한</t>
+  </si>
+  <si>
     <t>미래, 삼성</t>
-  </si>
-  <si>
-    <t>미래, 신한</t>
   </si>
 </sst>
 </file>
@@ -751,7 +763,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -812,52 +824,52 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D2">
-        <v>507.81225</v>
+        <v>130</v>
       </c>
       <c r="E2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F2">
-        <v>507.81225</v>
+        <v>130</v>
       </c>
       <c r="G2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M2">
-        <v>16500</v>
+        <v>13000</v>
       </c>
       <c r="N2">
         <v>100</v>
       </c>
       <c r="O2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="P2" t="s">
-        <v>20</v>
+        <v>79</v>
       </c>
       <c r="Q2">
-        <v>2078175</v>
+        <v>723700</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -865,105 +877,105 @@
         <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D3">
-        <v>217</v>
+        <v>507.81225</v>
       </c>
       <c r="E3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F3">
-        <v>217</v>
+        <v>507.81225</v>
       </c>
       <c r="G3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M3">
-        <v>15500</v>
+        <v>16500</v>
       </c>
       <c r="N3">
         <v>100</v>
       </c>
       <c r="O3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="P3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Q3">
-        <v>1050000</v>
+        <v>2078175</v>
       </c>
     </row>
     <row r="4" spans="1:17">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D4">
-        <v>290</v>
+        <v>217</v>
       </c>
       <c r="E4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F4">
-        <v>290</v>
+        <v>217</v>
       </c>
       <c r="G4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M4">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="N4">
         <v>100</v>
       </c>
       <c r="O4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="P4" t="s">
         <v>21</v>
       </c>
       <c r="Q4">
-        <v>720000</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -971,52 +983,52 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D5">
-        <v>157.71</v>
+        <v>290</v>
       </c>
       <c r="E5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F5">
-        <v>157.71</v>
+        <v>290</v>
       </c>
       <c r="G5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M5">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="N5">
         <v>100</v>
       </c>
       <c r="O5" t="s">
+        <v>71</v>
+      </c>
+      <c r="P5" t="s">
         <v>22</v>
       </c>
-      <c r="P5" t="s">
-        <v>76</v>
-      </c>
       <c r="Q5">
-        <v>540250</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -1024,52 +1036,52 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D6">
-        <v>116</v>
+        <v>157.71</v>
       </c>
       <c r="E6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F6">
-        <v>116</v>
+        <v>157.71</v>
       </c>
       <c r="G6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M6">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="N6">
         <v>100</v>
       </c>
       <c r="O6" t="s">
+        <v>23</v>
+      </c>
+      <c r="P6" t="s">
         <v>69</v>
       </c>
-      <c r="P6" t="s">
-        <v>22</v>
-      </c>
       <c r="Q6">
-        <v>4350000</v>
+        <v>540250</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -1077,52 +1089,52 @@
         <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D7">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="E7" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="F7">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="G7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M7">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N7">
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="P7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q7">
-        <v>1050000</v>
+        <v>4350000</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -1130,52 +1142,52 @@
         <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D8">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="E8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F8">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="G8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M8">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="N8">
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="P8" t="s">
-        <v>77</v>
+        <v>23</v>
       </c>
       <c r="Q8">
-        <v>1675500</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -1183,52 +1195,52 @@
         <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D9">
-        <v>297</v>
+        <v>223.4</v>
       </c>
       <c r="E9" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F9">
-        <v>297</v>
+        <v>223.4</v>
       </c>
       <c r="G9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M9">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="N9">
         <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="P9" t="s">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="Q9">
-        <v>1012500</v>
+        <v>1675500</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -1236,102 +1248,102 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D10">
-        <v>2660</v>
+        <v>297</v>
       </c>
       <c r="E10" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F10">
-        <v>2553.6</v>
+        <v>297</v>
       </c>
       <c r="G10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M10">
-        <v>35000</v>
+        <v>22000</v>
       </c>
       <c r="N10">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="O10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="P10" t="s">
-        <v>78</v>
+        <v>27</v>
       </c>
       <c r="Q10">
-        <v>9340690</v>
+        <v>1012500</v>
       </c>
     </row>
     <row r="11" spans="1:17">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D11">
         <v>2660</v>
       </c>
       <c r="E11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F11">
-        <v>106.4</v>
+        <v>2553.6</v>
       </c>
       <c r="G11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="L11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M11">
         <v>35000</v>
       </c>
       <c r="N11">
-        <v>4</v>
+        <v>96</v>
       </c>
       <c r="O11" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="P11" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="Q11">
         <v>9340690</v>
@@ -1342,52 +1354,52 @@
         <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D12">
-        <v>120</v>
+        <v>2660</v>
       </c>
       <c r="E12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F12">
-        <v>120</v>
+        <v>106.4</v>
       </c>
       <c r="G12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K12" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="L12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M12">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="N12">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="O12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="P12" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="Q12">
-        <v>4500000</v>
+        <v>9340690</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -1395,37 +1407,37 @@
         <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D13">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="E13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F13">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="G13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M13">
         <v>2000</v>
@@ -1434,13 +1446,13 @@
         <v>100</v>
       </c>
       <c r="O13" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="P13" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="Q13">
-        <v>3000000</v>
+        <v>4500000</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1448,52 +1460,52 @@
         <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D14">
-        <v>161.8</v>
+        <v>80</v>
       </c>
       <c r="E14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F14">
-        <v>161.8</v>
+        <v>80</v>
       </c>
       <c r="G14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K14" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M14">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="N14">
         <v>100</v>
       </c>
       <c r="O14" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="P14" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="Q14">
-        <v>1187900</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1501,90 +1513,90 @@
         <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C15" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D15">
-        <v>4350</v>
+        <v>161.8</v>
       </c>
       <c r="E15" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F15">
-        <v>1435.5</v>
+        <v>161.8</v>
       </c>
       <c r="G15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M15">
-        <v>60000</v>
+        <v>10000</v>
       </c>
       <c r="N15">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="O15" t="s">
         <v>31</v>
       </c>
       <c r="P15" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="Q15">
-        <v>21750000</v>
+        <v>1187900</v>
       </c>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D16">
         <v>4350</v>
       </c>
       <c r="E16" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F16">
         <v>1435.5</v>
       </c>
       <c r="G16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M16">
         <v>60000</v>
@@ -1593,10 +1605,10 @@
         <v>33</v>
       </c>
       <c r="O16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P16" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="Q16">
         <v>21750000</v>
@@ -1604,52 +1616,52 @@
     </row>
     <row r="17" spans="1:17">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D17">
         <v>4350</v>
       </c>
       <c r="E17" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="F17">
-        <v>1305</v>
+        <v>1435.5</v>
       </c>
       <c r="G17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K17" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M17">
         <v>60000</v>
       </c>
       <c r="N17">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="O17" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P17" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="Q17">
         <v>21750000</v>
@@ -1657,52 +1669,52 @@
     </row>
     <row r="18" spans="1:17">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C18" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D18">
         <v>4350</v>
       </c>
       <c r="E18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F18">
-        <v>174</v>
+        <v>1305</v>
       </c>
       <c r="G18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="L18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M18">
         <v>60000</v>
       </c>
       <c r="N18">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="O18" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P18" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="Q18">
         <v>21750000</v>
@@ -1713,52 +1725,52 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D19">
-        <v>80</v>
+        <v>4350</v>
       </c>
       <c r="E19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F19">
-        <v>80</v>
+        <v>174</v>
       </c>
       <c r="G19" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H19" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I19" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J19" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K19" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="L19" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M19">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="N19">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="O19" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P19" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="Q19">
-        <v>3000000</v>
+        <v>21750000</v>
       </c>
     </row>
     <row r="20" spans="1:17">
@@ -1766,52 +1778,52 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C20" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D20">
-        <v>289.6</v>
+        <v>80</v>
       </c>
       <c r="E20" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="F20">
-        <v>289.6</v>
+        <v>80</v>
       </c>
       <c r="G20" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H20" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I20" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J20" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L20" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M20">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N20">
         <v>100</v>
       </c>
       <c r="O20" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="P20" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q20">
-        <v>1357500</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="21" spans="1:17">
@@ -1819,102 +1831,102 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C21" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D21">
-        <v>575.89</v>
+        <v>289.6</v>
       </c>
       <c r="E21" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="F21">
-        <v>541.3366</v>
+        <v>289.6</v>
       </c>
       <c r="G21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K21" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M21">
-        <v>43300</v>
+        <v>16000</v>
       </c>
       <c r="N21">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="O21" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P21" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="Q21">
-        <v>1906400</v>
+        <v>1357500</v>
       </c>
     </row>
     <row r="22" spans="1:17">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C22" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D22">
         <v>575.89</v>
       </c>
       <c r="E22" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="F22">
-        <v>34.5534</v>
+        <v>541.3366</v>
       </c>
       <c r="G22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K22" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="L22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M22">
         <v>43300</v>
       </c>
       <c r="N22">
-        <v>6</v>
+        <v>94</v>
       </c>
       <c r="O22" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="P22" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="Q22">
         <v>1906400</v>
@@ -1925,51 +1937,104 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C23" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23">
+        <v>575.89</v>
+      </c>
+      <c r="E23" t="s">
+        <v>64</v>
+      </c>
+      <c r="F23">
+        <v>34.5534</v>
+      </c>
+      <c r="G23" t="s">
+        <v>66</v>
+      </c>
+      <c r="H23" t="s">
+        <v>66</v>
+      </c>
+      <c r="I23" t="s">
+        <v>66</v>
+      </c>
+      <c r="J23" t="s">
+        <v>66</v>
+      </c>
+      <c r="K23" t="s">
+        <v>68</v>
+      </c>
+      <c r="L23" t="s">
+        <v>66</v>
+      </c>
+      <c r="M23">
+        <v>43300</v>
+      </c>
+      <c r="N23">
+        <v>6</v>
+      </c>
+      <c r="O23" t="s">
+        <v>77</v>
+      </c>
+      <c r="P23" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q23">
+        <v>1906400</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17">
+      <c r="A24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" t="s">
         <v>51</v>
       </c>
-      <c r="D23">
+      <c r="C24" t="s">
+        <v>52</v>
+      </c>
+      <c r="D24">
         <v>432</v>
       </c>
-      <c r="E23" t="s">
-        <v>58</v>
-      </c>
-      <c r="F23">
+      <c r="E24" t="s">
+        <v>60</v>
+      </c>
+      <c r="F24">
         <v>432</v>
       </c>
-      <c r="G23" t="s">
-        <v>64</v>
-      </c>
-      <c r="H23" t="s">
-        <v>64</v>
-      </c>
-      <c r="I23" t="s">
-        <v>64</v>
-      </c>
-      <c r="J23" t="s">
-        <v>64</v>
-      </c>
-      <c r="K23" t="s">
-        <v>65</v>
-      </c>
-      <c r="L23" t="s">
-        <v>64</v>
-      </c>
-      <c r="M23">
+      <c r="G24" t="s">
+        <v>66</v>
+      </c>
+      <c r="H24" t="s">
+        <v>66</v>
+      </c>
+      <c r="I24" t="s">
+        <v>66</v>
+      </c>
+      <c r="J24" t="s">
+        <v>66</v>
+      </c>
+      <c r="K24" t="s">
+        <v>67</v>
+      </c>
+      <c r="L24" t="s">
+        <v>66</v>
+      </c>
+      <c r="M24">
         <v>18000</v>
       </c>
-      <c r="N23">
+      <c r="N24">
         <v>100</v>
       </c>
-      <c r="O23" t="s">
-        <v>75</v>
-      </c>
-      <c r="P23" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q23">
+      <c r="O24" t="s">
+        <v>78</v>
+      </c>
+      <c r="P24" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q24">
         <v>1758600</v>
       </c>
     </row>
@@ -1980,7 +2045,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T18"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -1988,10 +2053,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -2000,695 +2065,695 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D2" t="s">
-        <v>20</v>
+        <v>79</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
       </c>
       <c r="F2">
-        <v>50781225</v>
+        <v>13000000</v>
       </c>
       <c r="G2">
-        <v>3077650</v>
+        <v>1000000</v>
       </c>
       <c r="H2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I2">
-        <v>13800</v>
+        <v>9500</v>
       </c>
       <c r="J2">
-        <v>15700</v>
+        <v>10700</v>
       </c>
       <c r="K2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L2">
-        <v>16500</v>
+        <v>13000</v>
       </c>
       <c r="M2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O2">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="P2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="S2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" t="s">
         <v>18</v>
       </c>
       <c r="F3">
-        <v>21700000</v>
+        <v>50781225</v>
       </c>
       <c r="G3">
-        <v>1400000</v>
+        <v>3077650</v>
       </c>
       <c r="H3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I3">
-        <v>12500</v>
+        <v>13800</v>
       </c>
       <c r="J3">
-        <v>15500</v>
+        <v>15700</v>
       </c>
       <c r="K3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L3">
-        <v>15500</v>
+        <v>16500</v>
       </c>
       <c r="M3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O3">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="S3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D4" t="s">
         <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F4">
-        <v>29000000</v>
+        <v>21700000</v>
       </c>
       <c r="G4">
-        <v>1000000</v>
+        <v>1400000</v>
       </c>
       <c r="H4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I4">
-        <v>24000</v>
+        <v>12500</v>
       </c>
       <c r="J4">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="K4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L4">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="M4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R4" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="S4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" t="s">
         <v>22</v>
-      </c>
-      <c r="B5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D5" t="s">
-        <v>76</v>
       </c>
       <c r="E5" t="s">
         <v>19</v>
       </c>
       <c r="F5">
-        <v>15771000</v>
+        <v>29000000</v>
       </c>
       <c r="G5">
-        <v>751000</v>
+        <v>1000000</v>
       </c>
       <c r="H5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I5">
-        <v>18000</v>
+        <v>24000</v>
       </c>
       <c r="J5">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="K5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L5">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="M5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O5">
-        <v>72.87616511318242</v>
+        <v>0</v>
       </c>
       <c r="P5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="S5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" t="s">
         <v>69</v>
-      </c>
-      <c r="B6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D6" t="s">
-        <v>22</v>
       </c>
       <c r="E6" t="s">
         <v>20</v>
       </c>
       <c r="F6">
-        <v>11600000</v>
+        <v>15771000</v>
       </c>
       <c r="G6">
-        <v>5800000</v>
+        <v>751000</v>
       </c>
       <c r="H6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I6">
-        <v>2000</v>
+        <v>18000</v>
       </c>
       <c r="J6">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="K6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L6">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="M6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>72.87616511318242</v>
       </c>
       <c r="P6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R6" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="S6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E7" t="s">
         <v>21</v>
       </c>
       <c r="F7">
-        <v>22400000</v>
+        <v>11600000</v>
       </c>
       <c r="G7">
-        <v>1400000</v>
+        <v>5800000</v>
       </c>
       <c r="H7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I7">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="J7">
-        <v>19000</v>
+        <v>2000</v>
       </c>
       <c r="K7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L7">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="M7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="S7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D8" t="s">
-        <v>77</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s">
         <v>22</v>
       </c>
       <c r="F8">
-        <v>22340000</v>
+        <v>22400000</v>
       </c>
       <c r="G8">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="H8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I8">
-        <v>7300</v>
+        <v>16000</v>
       </c>
       <c r="J8">
-        <v>8500</v>
+        <v>19000</v>
       </c>
       <c r="K8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L8">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="M8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R8" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="S8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="E9" t="s">
         <v>23</v>
       </c>
       <c r="F9">
-        <v>29700000</v>
+        <v>22340000</v>
       </c>
       <c r="G9">
-        <v>1350000</v>
+        <v>2234000</v>
       </c>
       <c r="H9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I9">
-        <v>14000</v>
+        <v>7300</v>
       </c>
       <c r="J9">
-        <v>17000</v>
+        <v>8500</v>
       </c>
       <c r="K9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L9">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="M9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O9">
         <v>0</v>
       </c>
       <c r="P9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R9" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="S9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D10" t="s">
-        <v>78</v>
+        <v>27</v>
       </c>
       <c r="E10" t="s">
         <v>24</v>
       </c>
       <c r="F10">
-        <v>266000000</v>
+        <v>29700000</v>
       </c>
       <c r="G10">
-        <v>7600000</v>
+        <v>1350000</v>
       </c>
       <c r="H10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I10">
-        <v>24000</v>
+        <v>14000</v>
       </c>
       <c r="J10">
-        <v>30000</v>
+        <v>17000</v>
       </c>
       <c r="K10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L10">
-        <v>35000</v>
+        <v>22000</v>
       </c>
       <c r="M10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O10">
-        <v>14.47368421052632</v>
+        <v>0</v>
       </c>
       <c r="P10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R10" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="S10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E11" t="s">
         <v>25</v>
       </c>
       <c r="F11">
-        <v>12000000</v>
+        <v>266000000</v>
       </c>
       <c r="G11">
-        <v>6000000</v>
+        <v>7600000</v>
       </c>
       <c r="H11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I11">
-        <v>2000</v>
+        <v>24000</v>
       </c>
       <c r="J11">
-        <v>2000</v>
+        <v>30000</v>
       </c>
       <c r="K11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L11">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="M11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O11">
-        <v>0</v>
+        <v>14.47368421052632</v>
       </c>
       <c r="P11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R11" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="S11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D12" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="E12" t="s">
         <v>26</v>
       </c>
       <c r="F12">
-        <v>8000000</v>
+        <v>12000000</v>
       </c>
       <c r="G12">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="H12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I12">
         <v>2000</v>
@@ -2697,96 +2762,96 @@
         <v>2000</v>
       </c>
       <c r="K12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L12">
         <v>2000</v>
       </c>
       <c r="M12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O12">
         <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R12" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="S12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E13" t="s">
         <v>27</v>
       </c>
       <c r="F13">
-        <v>16180000</v>
+        <v>8000000</v>
       </c>
       <c r="G13">
-        <v>1618000</v>
+        <v>4000000</v>
       </c>
       <c r="H13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I13">
-        <v>6200</v>
+        <v>2000</v>
       </c>
       <c r="J13">
-        <v>7700</v>
+        <v>2000</v>
       </c>
       <c r="K13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L13">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="M13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O13">
         <v>0</v>
       </c>
       <c r="P13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R13" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="S13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -2794,309 +2859,371 @@
         <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C14" t="s">
-        <v>101</v>
+        <v>62</v>
       </c>
       <c r="D14" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E14" t="s">
         <v>28</v>
       </c>
       <c r="F14">
-        <v>435000000</v>
+        <v>16180000</v>
       </c>
       <c r="G14">
-        <v>7250000</v>
+        <v>1618000</v>
       </c>
       <c r="H14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I14">
-        <v>47000</v>
+        <v>6200</v>
       </c>
       <c r="J14">
-        <v>60000</v>
+        <v>7700</v>
       </c>
       <c r="K14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L14">
-        <v>60000</v>
+        <v>10000</v>
       </c>
       <c r="M14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O14">
         <v>0</v>
       </c>
       <c r="P14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R14" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="S14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C15" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D15" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E15" t="s">
         <v>29</v>
       </c>
       <c r="F15">
-        <v>8000000</v>
+        <v>435000000</v>
       </c>
       <c r="G15">
-        <v>4000000</v>
+        <v>7250000</v>
       </c>
       <c r="H15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I15">
-        <v>2000</v>
+        <v>47000</v>
       </c>
       <c r="J15">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="K15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L15">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="M15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O15">
         <v>0</v>
       </c>
       <c r="P15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R15" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="S15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:20">
       <c r="A16" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C16" t="s">
-        <v>57</v>
+        <v>105</v>
       </c>
       <c r="D16" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E16" t="s">
         <v>30</v>
       </c>
       <c r="F16">
-        <v>28960000</v>
+        <v>8000000</v>
       </c>
       <c r="G16">
-        <v>1810000</v>
+        <v>4000000</v>
       </c>
       <c r="H16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I16">
-        <v>9000</v>
+        <v>2000</v>
       </c>
       <c r="J16">
-        <v>12000</v>
+        <v>2000</v>
       </c>
       <c r="K16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L16">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="M16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O16">
         <v>0</v>
       </c>
       <c r="P16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R16" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="S16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:20">
       <c r="A17" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="D17" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E17" t="s">
         <v>31</v>
       </c>
       <c r="F17">
-        <v>57589000</v>
+        <v>28960000</v>
       </c>
       <c r="G17">
-        <v>1330000</v>
+        <v>1810000</v>
       </c>
       <c r="H17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I17">
-        <v>36400</v>
+        <v>9000</v>
       </c>
       <c r="J17">
-        <v>43300</v>
+        <v>12000</v>
       </c>
       <c r="K17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L17">
-        <v>43300</v>
+        <v>16000</v>
       </c>
       <c r="M17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O17">
         <v>0</v>
       </c>
       <c r="P17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R17" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="S17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:20">
       <c r="A18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C18" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D18" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="E18" t="s">
         <v>32</v>
       </c>
       <c r="F18">
-        <v>43200000</v>
+        <v>57589000</v>
       </c>
       <c r="G18">
-        <v>2400000</v>
+        <v>1330000</v>
       </c>
       <c r="H18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I18">
-        <v>11000</v>
+        <v>36400</v>
       </c>
       <c r="J18">
-        <v>14200</v>
+        <v>43300</v>
       </c>
       <c r="K18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L18">
-        <v>18000</v>
+        <v>43300</v>
       </c>
       <c r="M18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O18">
         <v>0</v>
       </c>
       <c r="P18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Q18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R18" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="S18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="T18" t="s">
-        <v>64</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20">
+      <c r="A19" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" t="s">
+        <v>76</v>
+      </c>
+      <c r="E19" t="s">
+        <v>33</v>
+      </c>
+      <c r="F19">
+        <v>43200000</v>
+      </c>
+      <c r="G19">
+        <v>2400000</v>
+      </c>
+      <c r="H19" t="s">
+        <v>66</v>
+      </c>
+      <c r="I19">
+        <v>11000</v>
+      </c>
+      <c r="J19">
+        <v>14200</v>
+      </c>
+      <c r="K19" t="s">
+        <v>66</v>
+      </c>
+      <c r="L19">
+        <v>18000</v>
+      </c>
+      <c r="M19" t="s">
+        <v>66</v>
+      </c>
+      <c r="N19" t="s">
+        <v>66</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>66</v>
+      </c>
+      <c r="R19" t="s">
+        <v>123</v>
+      </c>
+      <c r="S19" t="s">
+        <v>66</v>
+      </c>
+      <c r="T19" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -3106,21 +3233,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -3132,10 +3259,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -3144,30 +3271,30 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D2" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E2" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F2" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H2">
         <v>8000</v>
@@ -3187,25 +3314,25 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H3">
         <v>12000</v>
@@ -3225,25 +3352,25 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D4" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E4" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="F4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H4">
         <v>130500</v>
@@ -3263,25 +3390,25 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H5">
         <v>43200</v>
@@ -3301,25 +3428,25 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F6" t="s">
+        <v>74</v>
+      </c>
+      <c r="G6" t="s">
         <v>27</v>
-      </c>
-      <c r="C6" t="s">
-        <v>43</v>
-      </c>
-      <c r="D6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F6" t="s">
-        <v>71</v>
-      </c>
-      <c r="G6" t="s">
-        <v>26</v>
       </c>
       <c r="H6">
         <v>8000</v>
@@ -3339,25 +3466,25 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H7">
         <v>11600</v>
@@ -3377,25 +3504,25 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F8" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H8">
         <v>16180</v>
@@ -3415,139 +3542,139 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E9" t="s">
-        <v>124</v>
+        <v>55</v>
       </c>
       <c r="F9" t="s">
-        <v>78</v>
+        <v>23</v>
       </c>
       <c r="G9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H9">
-        <v>255360</v>
+        <v>22400</v>
       </c>
       <c r="I9">
-        <v>7600000</v>
+        <v>1400000</v>
       </c>
       <c r="J9">
-        <v>35000</v>
+        <v>16000</v>
       </c>
       <c r="K9">
         <v>0</v>
       </c>
       <c r="L9">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B10" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E10" t="s">
-        <v>52</v>
+        <v>128</v>
       </c>
       <c r="F10" t="s">
-        <v>22</v>
+        <v>86</v>
       </c>
       <c r="G10" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="H10">
-        <v>22400</v>
+        <v>54133.66</v>
       </c>
       <c r="I10">
-        <v>1400000</v>
+        <v>1330000</v>
       </c>
       <c r="J10">
-        <v>16000</v>
+        <v>43300</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>100</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B11" t="s">
         <v>74</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E11" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="F11" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G11" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="H11">
-        <v>54133.66</v>
+        <v>255360</v>
       </c>
       <c r="I11">
-        <v>1330000</v>
+        <v>7600000</v>
       </c>
       <c r="J11">
-        <v>43300</v>
+        <v>35000</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C12" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H12">
         <v>50781.225</v>
@@ -3567,110 +3694,110 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B13" t="s">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
         <v>41</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E13" t="s">
-        <v>124</v>
+        <v>59</v>
       </c>
       <c r="F13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H13">
-        <v>10640</v>
+        <v>22340</v>
       </c>
       <c r="I13">
-        <v>7600000</v>
+        <v>2234000</v>
       </c>
       <c r="J13">
-        <v>35000</v>
+        <v>10000</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
-        <v>4</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C14" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E14" t="s">
-        <v>57</v>
+        <v>129</v>
       </c>
       <c r="F14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G14" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H14">
-        <v>28960</v>
+        <v>10640</v>
       </c>
       <c r="I14">
-        <v>1810000</v>
+        <v>7600000</v>
       </c>
       <c r="J14">
-        <v>16000</v>
+        <v>35000</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>76</v>
       </c>
       <c r="C15" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F15" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="G15" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="H15">
-        <v>22340</v>
+        <v>28960</v>
       </c>
       <c r="I15">
-        <v>2234000</v>
+        <v>1810000</v>
       </c>
       <c r="J15">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="K15">
         <v>0</v>
@@ -3681,25 +3808,25 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B16" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C16" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D16" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F16" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="G16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H16">
         <v>3455.34</v>
@@ -3719,25 +3846,25 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D17" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E17" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="F17" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H17">
         <v>17400</v>
@@ -3757,25 +3884,25 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B18" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D18" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E18" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="F18" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H18">
         <v>143550</v>
@@ -3795,34 +3922,34 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B19" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="C19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D19" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E19" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F19" t="s">
-        <v>26</v>
+        <v>69</v>
       </c>
       <c r="G19" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H19">
-        <v>29700</v>
+        <v>15771</v>
       </c>
       <c r="I19">
-        <v>1350000</v>
+        <v>751000</v>
       </c>
       <c r="J19">
-        <v>22000</v>
+        <v>21000</v>
       </c>
       <c r="K19">
         <v>0</v>
@@ -3833,34 +3960,34 @@
     </row>
     <row r="20" spans="1:12">
       <c r="A20" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B20" t="s">
-        <v>22</v>
+        <v>73</v>
       </c>
       <c r="C20" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D20" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E20" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F20" t="s">
-        <v>76</v>
+        <v>27</v>
       </c>
       <c r="G20" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="H20">
-        <v>15771</v>
+        <v>29700</v>
       </c>
       <c r="I20">
-        <v>751000</v>
+        <v>1350000</v>
       </c>
       <c r="J20">
-        <v>21000</v>
+        <v>22000</v>
       </c>
       <c r="K20">
         <v>0</v>
@@ -3871,25 +3998,25 @@
     </row>
     <row r="21" spans="1:12">
       <c r="A21" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B21" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C21" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D21" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E21" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F21" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G21" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H21">
         <v>21700</v>
@@ -3912,22 +4039,22 @@
         <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C22" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D22" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E22" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="F22" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H22">
         <v>143550</v>
@@ -3950,10 +4077,10 @@
         <v>54</v>
       </c>
       <c r="B23" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C23" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D23" t="s">
         <v>54</v>
@@ -3962,10 +4089,10 @@
         <v>54</v>
       </c>
       <c r="F23" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G23" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H23">
         <v>29000</v>
@@ -3980,6 +4107,44 @@
         <v>0</v>
       </c>
       <c r="L23">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" t="s">
+        <v>69</v>
+      </c>
+      <c r="C24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" t="s">
+        <v>54</v>
+      </c>
+      <c r="E24" t="s">
+        <v>54</v>
+      </c>
+      <c r="F24" t="s">
+        <v>79</v>
+      </c>
+      <c r="G24" t="s">
+        <v>17</v>
+      </c>
+      <c r="H24">
+        <v>13000</v>
+      </c>
+      <c r="I24">
+        <v>1000000</v>
+      </c>
+      <c r="J24">
+        <v>13000</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RPA datasets push 2024-08-23
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="138">
   <si>
     <t>상장일</t>
   </si>
@@ -69,6 +69,9 @@
     <t>총기관배정수량</t>
   </si>
   <si>
+    <t>2024-08-22</t>
+  </si>
+  <si>
     <t>2024-08-21</t>
   </si>
   <si>
@@ -120,9 +123,15 @@
     <t>2024-06-28</t>
   </si>
   <si>
+    <t>M83</t>
+  </si>
+  <si>
     <t>티디에스팜</t>
   </si>
   <si>
+    <t>대신밸런스제18호스팩</t>
+  </si>
+  <si>
     <t>전진건설로봇</t>
   </si>
   <si>
@@ -180,9 +189,18 @@
     <t>코스피</t>
   </si>
   <si>
+    <t>신영</t>
+  </si>
+  <si>
+    <t>유진</t>
+  </si>
+  <si>
     <t>한국</t>
   </si>
   <si>
+    <t>대신</t>
+  </si>
+  <si>
     <t>미래</t>
   </si>
   <si>
@@ -204,9 +222,6 @@
     <t>SK</t>
   </si>
   <si>
-    <t>대신</t>
-  </si>
-  <si>
     <t>제이피모간회사</t>
   </si>
   <si>
@@ -336,9 +351,15 @@
     <t>엘에스</t>
   </si>
   <si>
+    <t>638.07 : 1</t>
+  </si>
+  <si>
     <t>1608.17 : 1</t>
   </si>
   <si>
+    <t>135.53 : 1</t>
+  </si>
+  <si>
     <t>1087.3 : 1</t>
   </si>
   <si>
@@ -406,6 +427,9 @@
   </si>
   <si>
     <t>미래, 삼성</t>
+  </si>
+  <si>
+    <t>신영, 유진</t>
   </si>
 </sst>
 </file>
@@ -763,7 +787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -824,847 +848,847 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D2">
-        <v>130</v>
+        <v>240</v>
       </c>
       <c r="E2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F2">
-        <v>130</v>
+        <v>228</v>
       </c>
       <c r="G2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K2" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M2">
-        <v>13000</v>
+        <v>16000</v>
       </c>
       <c r="N2">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="O2" t="s">
-        <v>69</v>
+        <v>23</v>
       </c>
       <c r="P2" t="s">
-        <v>79</v>
+        <v>21</v>
       </c>
       <c r="Q2">
-        <v>723700</v>
+        <v>2100000</v>
       </c>
     </row>
     <row r="3" spans="1:17">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
         <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D3">
-        <v>507.81225</v>
+        <v>240</v>
       </c>
       <c r="E3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F3">
-        <v>507.81225</v>
+        <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K3" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="L3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M3">
-        <v>16500</v>
+        <v>16000</v>
       </c>
       <c r="N3">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="O3" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="P3" t="s">
         <v>21</v>
       </c>
       <c r="Q3">
-        <v>2078175</v>
+        <v>2100000</v>
       </c>
     </row>
     <row r="4" spans="1:17">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D4">
-        <v>217</v>
+        <v>130</v>
       </c>
       <c r="E4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F4">
-        <v>217</v>
+        <v>130</v>
       </c>
       <c r="G4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K4" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M4">
-        <v>15500</v>
+        <v>13000</v>
       </c>
       <c r="N4">
         <v>100</v>
       </c>
       <c r="O4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="P4" t="s">
-        <v>21</v>
+        <v>84</v>
       </c>
       <c r="Q4">
-        <v>1050000</v>
+        <v>723700</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
         <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D5">
-        <v>290</v>
+        <v>130</v>
       </c>
       <c r="E5" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="F5">
-        <v>290</v>
+        <v>130</v>
       </c>
       <c r="G5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K5" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M5">
-        <v>29000</v>
+        <v>2000</v>
       </c>
       <c r="N5">
         <v>100</v>
       </c>
       <c r="O5" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="P5" t="s">
-        <v>22</v>
+        <v>84</v>
       </c>
       <c r="Q5">
-        <v>720000</v>
+        <v>4875000</v>
       </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D6">
-        <v>157.71</v>
+        <v>507.81225</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F6">
-        <v>157.71</v>
+        <v>507.81225</v>
       </c>
       <c r="G6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K6" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M6">
-        <v>21000</v>
+        <v>16500</v>
       </c>
       <c r="N6">
         <v>100</v>
       </c>
       <c r="O6" t="s">
-        <v>23</v>
+        <v>75</v>
       </c>
       <c r="P6" t="s">
-        <v>69</v>
+        <v>22</v>
       </c>
       <c r="Q6">
-        <v>540250</v>
+        <v>2078175</v>
       </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D7">
-        <v>116</v>
+        <v>217</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F7">
-        <v>116</v>
+        <v>217</v>
       </c>
       <c r="G7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K7" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M7">
-        <v>2000</v>
+        <v>15500</v>
       </c>
       <c r="N7">
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="P7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q7">
-        <v>4350000</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
         <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D8">
-        <v>224</v>
+        <v>290</v>
       </c>
       <c r="E8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F8">
-        <v>224</v>
+        <v>290</v>
       </c>
       <c r="G8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K8" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M8">
-        <v>16000</v>
+        <v>29000</v>
       </c>
       <c r="N8">
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="P8" t="s">
         <v>23</v>
       </c>
       <c r="Q8">
-        <v>1050000</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="9" spans="1:17">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
         <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D9">
-        <v>223.4</v>
+        <v>157.71</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F9">
-        <v>223.4</v>
+        <v>157.71</v>
       </c>
       <c r="G9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K9" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M9">
-        <v>10000</v>
+        <v>21000</v>
       </c>
       <c r="N9">
         <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="P9" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="Q9">
-        <v>1675500</v>
+        <v>540250</v>
       </c>
     </row>
     <row r="10" spans="1:17">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B10" t="s">
         <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D10">
-        <v>297</v>
+        <v>116</v>
       </c>
       <c r="E10" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F10">
-        <v>297</v>
+        <v>116</v>
       </c>
       <c r="G10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K10" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M10">
-        <v>22000</v>
+        <v>2000</v>
       </c>
       <c r="N10">
         <v>100</v>
       </c>
       <c r="O10" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="P10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="Q10">
-        <v>1012500</v>
+        <v>4350000</v>
       </c>
     </row>
     <row r="11" spans="1:17">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B11" t="s">
         <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D11">
-        <v>2660</v>
+        <v>224</v>
       </c>
       <c r="E11" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="F11">
-        <v>2553.6</v>
+        <v>224</v>
       </c>
       <c r="G11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K11" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M11">
-        <v>35000</v>
+        <v>16000</v>
       </c>
       <c r="N11">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="O11" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="P11" t="s">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="Q11">
-        <v>9340690</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="12" spans="1:17">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D12">
-        <v>2660</v>
+        <v>223.4</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F12">
-        <v>106.4</v>
+        <v>223.4</v>
       </c>
       <c r="G12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K12" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="L12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M12">
-        <v>35000</v>
+        <v>10000</v>
       </c>
       <c r="N12">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="O12" t="s">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="P12" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="Q12">
-        <v>9340690</v>
+        <v>1675500</v>
       </c>
     </row>
     <row r="13" spans="1:17">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D13">
-        <v>120</v>
+        <v>297</v>
       </c>
       <c r="E13" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F13">
-        <v>120</v>
+        <v>297</v>
       </c>
       <c r="G13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K13" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M13">
-        <v>2000</v>
+        <v>22000</v>
       </c>
       <c r="N13">
         <v>100</v>
       </c>
       <c r="O13" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="P13" t="s">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="Q13">
-        <v>4500000</v>
+        <v>1012500</v>
       </c>
     </row>
     <row r="14" spans="1:17">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D14">
-        <v>80</v>
+        <v>2660</v>
       </c>
       <c r="E14" t="s">
         <v>61</v>
       </c>
       <c r="F14">
-        <v>80</v>
+        <v>2553.6</v>
       </c>
       <c r="G14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K14" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M14">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="N14">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="O14" t="s">
-        <v>28</v>
+        <v>79</v>
       </c>
       <c r="P14" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="Q14">
-        <v>3000000</v>
+        <v>9340690</v>
       </c>
     </row>
     <row r="15" spans="1:17">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B15" t="s">
         <v>46</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D15">
-        <v>161.8</v>
+        <v>2660</v>
       </c>
       <c r="E15" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F15">
-        <v>161.8</v>
+        <v>106.4</v>
       </c>
       <c r="G15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K15" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="L15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M15">
-        <v>10000</v>
+        <v>35000</v>
       </c>
       <c r="N15">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="O15" t="s">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="P15" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="Q15">
-        <v>1187900</v>
+        <v>9340690</v>
       </c>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
         <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D16">
-        <v>4350</v>
+        <v>120</v>
       </c>
       <c r="E16" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="F16">
-        <v>1435.5</v>
+        <v>120</v>
       </c>
       <c r="G16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K16" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M16">
-        <v>60000</v>
+        <v>2000</v>
       </c>
       <c r="N16">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="O16" t="s">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="P16" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="Q16">
-        <v>21750000</v>
+        <v>4500000</v>
       </c>
     </row>
     <row r="17" spans="1:17">
       <c r="A17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17">
+        <v>80</v>
+      </c>
+      <c r="E17" t="s">
+        <v>67</v>
+      </c>
+      <c r="F17">
+        <v>80</v>
+      </c>
+      <c r="G17" t="s">
+        <v>71</v>
+      </c>
+      <c r="H17" t="s">
+        <v>71</v>
+      </c>
+      <c r="I17" t="s">
+        <v>71</v>
+      </c>
+      <c r="J17" t="s">
+        <v>71</v>
+      </c>
+      <c r="K17" t="s">
+        <v>72</v>
+      </c>
+      <c r="L17" t="s">
+        <v>71</v>
+      </c>
+      <c r="M17">
+        <v>2000</v>
+      </c>
+      <c r="N17">
+        <v>100</v>
+      </c>
+      <c r="O17" t="s">
         <v>29</v>
       </c>
-      <c r="B17" t="s">
-        <v>47</v>
-      </c>
-      <c r="C17" t="s">
-        <v>53</v>
-      </c>
-      <c r="D17">
-        <v>4350</v>
-      </c>
-      <c r="E17" t="s">
-        <v>63</v>
-      </c>
-      <c r="F17">
-        <v>1435.5</v>
-      </c>
-      <c r="G17" t="s">
-        <v>66</v>
-      </c>
-      <c r="H17" t="s">
-        <v>66</v>
-      </c>
-      <c r="I17" t="s">
-        <v>66</v>
-      </c>
-      <c r="J17" t="s">
-        <v>66</v>
-      </c>
-      <c r="K17" t="s">
-        <v>67</v>
-      </c>
-      <c r="L17" t="s">
-        <v>66</v>
-      </c>
-      <c r="M17">
-        <v>60000</v>
-      </c>
-      <c r="N17">
-        <v>33</v>
-      </c>
-      <c r="O17" t="s">
-        <v>32</v>
-      </c>
       <c r="P17" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="Q17">
-        <v>21750000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="18" spans="1:17">
@@ -1672,102 +1696,102 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D18">
-        <v>4350</v>
+        <v>161.8</v>
       </c>
       <c r="E18" t="s">
         <v>60</v>
       </c>
       <c r="F18">
-        <v>1305</v>
+        <v>161.8</v>
       </c>
       <c r="G18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K18" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M18">
-        <v>60000</v>
+        <v>10000</v>
       </c>
       <c r="N18">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="O18" t="s">
         <v>32</v>
       </c>
       <c r="P18" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="Q18">
-        <v>21750000</v>
+        <v>1187900</v>
       </c>
     </row>
     <row r="19" spans="1:17">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D19">
         <v>4350</v>
       </c>
       <c r="E19" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="F19">
-        <v>174</v>
+        <v>1435.5</v>
       </c>
       <c r="G19" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H19" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I19" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J19" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K19" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="L19" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M19">
         <v>60000</v>
       </c>
       <c r="N19">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="O19" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P19" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="Q19">
         <v>21750000</v>
@@ -1778,263 +1802,422 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D20">
-        <v>80</v>
+        <v>4350</v>
       </c>
       <c r="E20" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F20">
-        <v>80</v>
+        <v>1435.5</v>
       </c>
       <c r="G20" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H20" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I20" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J20" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K20" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L20" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M20">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="N20">
-        <v>100</v>
+        <v>33</v>
       </c>
       <c r="O20" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P20" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="Q20">
-        <v>3000000</v>
+        <v>21750000</v>
       </c>
     </row>
     <row r="21" spans="1:17">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C21" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D21">
-        <v>289.6</v>
+        <v>4350</v>
       </c>
       <c r="E21" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F21">
-        <v>289.6</v>
+        <v>1305</v>
       </c>
       <c r="G21" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H21" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I21" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J21" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K21" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L21" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M21">
-        <v>16000</v>
+        <v>60000</v>
       </c>
       <c r="N21">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="O21" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="P21" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="Q21">
-        <v>1357500</v>
+        <v>21750000</v>
       </c>
     </row>
     <row r="22" spans="1:17">
       <c r="A22" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B22" t="s">
         <v>50</v>
       </c>
       <c r="C22" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D22">
-        <v>575.89</v>
+        <v>4350</v>
       </c>
       <c r="E22" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="F22">
-        <v>541.3366</v>
+        <v>174</v>
       </c>
       <c r="G22" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H22" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I22" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J22" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K22" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="L22" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M22">
-        <v>43300</v>
+        <v>60000</v>
       </c>
       <c r="N22">
-        <v>94</v>
+        <v>4</v>
       </c>
       <c r="O22" t="s">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="P22" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="Q22">
-        <v>1906400</v>
+        <v>21750000</v>
       </c>
     </row>
     <row r="23" spans="1:17">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C23" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D23">
-        <v>575.89</v>
+        <v>80</v>
       </c>
       <c r="E23" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F23">
-        <v>34.5534</v>
+        <v>80</v>
       </c>
       <c r="G23" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H23" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I23" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J23" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K23" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="L23" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M23">
-        <v>43300</v>
+        <v>2000</v>
       </c>
       <c r="N23">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="O23" t="s">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="P23" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="Q23">
-        <v>1906400</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="24" spans="1:17">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C24" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D24">
-        <v>432</v>
+        <v>289.6</v>
       </c>
       <c r="E24" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="F24">
-        <v>432</v>
+        <v>289.6</v>
       </c>
       <c r="G24" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H24" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I24" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J24" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K24" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L24" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M24">
-        <v>18000</v>
+        <v>16000</v>
       </c>
       <c r="N24">
         <v>100</v>
       </c>
       <c r="O24" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="P24" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="Q24">
+        <v>1357500</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17">
+      <c r="A25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25">
+        <v>575.89</v>
+      </c>
+      <c r="E25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F25">
+        <v>541.3366</v>
+      </c>
+      <c r="G25" t="s">
+        <v>71</v>
+      </c>
+      <c r="H25" t="s">
+        <v>71</v>
+      </c>
+      <c r="I25" t="s">
+        <v>71</v>
+      </c>
+      <c r="J25" t="s">
+        <v>71</v>
+      </c>
+      <c r="K25" t="s">
+        <v>72</v>
+      </c>
+      <c r="L25" t="s">
+        <v>71</v>
+      </c>
+      <c r="M25">
+        <v>43300</v>
+      </c>
+      <c r="N25">
+        <v>94</v>
+      </c>
+      <c r="O25" t="s">
+        <v>82</v>
+      </c>
+      <c r="P25" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q25">
+        <v>1906400</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17">
+      <c r="A26" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" t="s">
+        <v>53</v>
+      </c>
+      <c r="C26" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26">
+        <v>575.89</v>
+      </c>
+      <c r="E26" t="s">
+        <v>69</v>
+      </c>
+      <c r="F26">
+        <v>34.5534</v>
+      </c>
+      <c r="G26" t="s">
+        <v>71</v>
+      </c>
+      <c r="H26" t="s">
+        <v>71</v>
+      </c>
+      <c r="I26" t="s">
+        <v>71</v>
+      </c>
+      <c r="J26" t="s">
+        <v>71</v>
+      </c>
+      <c r="K26" t="s">
+        <v>73</v>
+      </c>
+      <c r="L26" t="s">
+        <v>71</v>
+      </c>
+      <c r="M26">
+        <v>43300</v>
+      </c>
+      <c r="N26">
+        <v>6</v>
+      </c>
+      <c r="O26" t="s">
+        <v>82</v>
+      </c>
+      <c r="P26" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q26">
+        <v>1906400</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17">
+      <c r="A27" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" t="s">
+        <v>55</v>
+      </c>
+      <c r="D27">
+        <v>432</v>
+      </c>
+      <c r="E27" t="s">
+        <v>66</v>
+      </c>
+      <c r="F27">
+        <v>432</v>
+      </c>
+      <c r="G27" t="s">
+        <v>71</v>
+      </c>
+      <c r="H27" t="s">
+        <v>71</v>
+      </c>
+      <c r="I27" t="s">
+        <v>71</v>
+      </c>
+      <c r="J27" t="s">
+        <v>71</v>
+      </c>
+      <c r="K27" t="s">
+        <v>72</v>
+      </c>
+      <c r="L27" t="s">
+        <v>71</v>
+      </c>
+      <c r="M27">
+        <v>18000</v>
+      </c>
+      <c r="N27">
+        <v>100</v>
+      </c>
+      <c r="O27" t="s">
+        <v>83</v>
+      </c>
+      <c r="P27" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q27">
         <v>1758600</v>
       </c>
     </row>
@@ -2045,7 +2228,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T19"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -2053,10 +2236,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -2065,246 +2248,246 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>69</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D2" t="s">
-        <v>79</v>
+        <v>21</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
       </c>
       <c r="F2">
-        <v>13000000</v>
+        <v>24000000</v>
       </c>
       <c r="G2">
-        <v>1000000</v>
+        <v>1500000</v>
       </c>
       <c r="H2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I2">
-        <v>9500</v>
+        <v>11000</v>
       </c>
       <c r="J2">
-        <v>10700</v>
+        <v>13000</v>
       </c>
       <c r="K2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L2">
-        <v>13000</v>
+        <v>16000</v>
       </c>
       <c r="M2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O2">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="S2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>84</v>
       </c>
       <c r="E3" t="s">
         <v>18</v>
       </c>
       <c r="F3">
-        <v>50781225</v>
+        <v>13000000</v>
       </c>
       <c r="G3">
-        <v>3077650</v>
+        <v>1000000</v>
       </c>
       <c r="H3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I3">
-        <v>13800</v>
+        <v>9500</v>
       </c>
       <c r="J3">
-        <v>15700</v>
+        <v>10700</v>
       </c>
       <c r="K3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L3">
-        <v>16500</v>
+        <v>13000</v>
       </c>
       <c r="M3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O3">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="P3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="S3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>84</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F4">
-        <v>21700000</v>
+        <v>13000000</v>
       </c>
       <c r="G4">
-        <v>1400000</v>
+        <v>6500000</v>
       </c>
       <c r="H4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I4">
-        <v>12500</v>
+        <v>2000</v>
       </c>
       <c r="J4">
-        <v>15500</v>
+        <v>2000</v>
       </c>
       <c r="K4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L4">
-        <v>15500</v>
+        <v>2000</v>
       </c>
       <c r="M4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R4" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="S4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
         <v>22</v>
@@ -2313,669 +2496,669 @@
         <v>19</v>
       </c>
       <c r="F5">
-        <v>29000000</v>
+        <v>50781225</v>
       </c>
       <c r="G5">
-        <v>1000000</v>
+        <v>3077650</v>
       </c>
       <c r="H5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I5">
-        <v>24000</v>
+        <v>13800</v>
       </c>
       <c r="J5">
-        <v>29000</v>
+        <v>15700</v>
       </c>
       <c r="K5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L5">
-        <v>29000</v>
+        <v>16500</v>
       </c>
       <c r="M5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R5" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="S5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>75</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D6" t="s">
-        <v>69</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
         <v>20</v>
       </c>
       <c r="F6">
-        <v>15771000</v>
+        <v>21700000</v>
       </c>
       <c r="G6">
-        <v>751000</v>
+        <v>1400000</v>
       </c>
       <c r="H6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I6">
-        <v>18000</v>
+        <v>12500</v>
       </c>
       <c r="J6">
-        <v>21000</v>
+        <v>15500</v>
       </c>
       <c r="K6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L6">
-        <v>21000</v>
+        <v>15500</v>
       </c>
       <c r="M6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O6">
-        <v>72.87616511318242</v>
+        <v>0</v>
       </c>
       <c r="P6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R6" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="S6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
         <v>23</v>
       </c>
       <c r="E7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F7">
-        <v>11600000</v>
+        <v>29000000</v>
       </c>
       <c r="G7">
-        <v>5800000</v>
+        <v>1000000</v>
       </c>
       <c r="H7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I7">
-        <v>2000</v>
+        <v>24000</v>
       </c>
       <c r="J7">
-        <v>2000</v>
+        <v>29000</v>
       </c>
       <c r="K7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L7">
-        <v>2000</v>
+        <v>29000</v>
       </c>
       <c r="M7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R7" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="S7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>74</v>
       </c>
       <c r="E8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F8">
-        <v>22400000</v>
+        <v>15771000</v>
       </c>
       <c r="G8">
-        <v>1400000</v>
+        <v>751000</v>
       </c>
       <c r="H8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I8">
-        <v>16000</v>
+        <v>18000</v>
       </c>
       <c r="J8">
-        <v>19000</v>
+        <v>21000</v>
       </c>
       <c r="K8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L8">
-        <v>16000</v>
+        <v>21000</v>
       </c>
       <c r="M8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>72.87616511318242</v>
       </c>
       <c r="P8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R8" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="S8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D9" t="s">
-        <v>80</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F9">
-        <v>22340000</v>
+        <v>11600000</v>
       </c>
       <c r="G9">
-        <v>2234000</v>
+        <v>5800000</v>
       </c>
       <c r="H9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I9">
-        <v>7300</v>
+        <v>2000</v>
       </c>
       <c r="J9">
-        <v>8500</v>
+        <v>2000</v>
       </c>
       <c r="K9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L9">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="M9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O9">
         <v>0</v>
       </c>
       <c r="P9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R9" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="S9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F10">
-        <v>29700000</v>
+        <v>22400000</v>
       </c>
       <c r="G10">
-        <v>1350000</v>
+        <v>1400000</v>
       </c>
       <c r="H10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I10">
-        <v>14000</v>
+        <v>16000</v>
       </c>
       <c r="J10">
-        <v>17000</v>
+        <v>19000</v>
       </c>
       <c r="K10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L10">
-        <v>22000</v>
+        <v>16000</v>
       </c>
       <c r="M10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O10">
         <v>0</v>
       </c>
       <c r="P10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R10" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="S10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="D11" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="E11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F11">
-        <v>266000000</v>
+        <v>22340000</v>
       </c>
       <c r="G11">
-        <v>7600000</v>
+        <v>2234000</v>
       </c>
       <c r="H11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I11">
-        <v>24000</v>
+        <v>7300</v>
       </c>
       <c r="J11">
-        <v>30000</v>
+        <v>8500</v>
       </c>
       <c r="K11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L11">
-        <v>35000</v>
+        <v>10000</v>
       </c>
       <c r="M11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O11">
-        <v>14.47368421052632</v>
+        <v>0</v>
       </c>
       <c r="P11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R11" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="S11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D12" t="s">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F12">
-        <v>12000000</v>
+        <v>29700000</v>
       </c>
       <c r="G12">
-        <v>6000000</v>
+        <v>1350000</v>
       </c>
       <c r="H12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I12">
-        <v>2000</v>
+        <v>14000</v>
       </c>
       <c r="J12">
-        <v>2000</v>
+        <v>17000</v>
       </c>
       <c r="K12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L12">
-        <v>2000</v>
+        <v>22000</v>
       </c>
       <c r="M12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O12">
         <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R12" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="S12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T12" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>79</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C13" t="s">
         <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="E13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F13">
-        <v>8000000</v>
+        <v>266000000</v>
       </c>
       <c r="G13">
-        <v>4000000</v>
+        <v>7600000</v>
       </c>
       <c r="H13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I13">
-        <v>2000</v>
+        <v>24000</v>
       </c>
       <c r="J13">
-        <v>2000</v>
+        <v>30000</v>
       </c>
       <c r="K13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L13">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="M13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O13">
-        <v>0</v>
+        <v>14.47368421052632</v>
       </c>
       <c r="P13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R13" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="S13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>80</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D14" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F14">
-        <v>16180000</v>
+        <v>12000000</v>
       </c>
       <c r="G14">
-        <v>1618000</v>
+        <v>6000000</v>
       </c>
       <c r="H14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I14">
-        <v>6200</v>
+        <v>2000</v>
       </c>
       <c r="J14">
-        <v>7700</v>
+        <v>2000</v>
       </c>
       <c r="K14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L14">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="M14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O14">
         <v>0</v>
       </c>
       <c r="P14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R14" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="S14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B15" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C15" t="s">
-        <v>104</v>
+        <v>67</v>
       </c>
       <c r="D15" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F15">
-        <v>435000000</v>
+        <v>8000000</v>
       </c>
       <c r="G15">
-        <v>7250000</v>
+        <v>4000000</v>
       </c>
       <c r="H15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I15">
-        <v>47000</v>
+        <v>2000</v>
       </c>
       <c r="J15">
-        <v>60000</v>
+        <v>2000</v>
       </c>
       <c r="K15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L15">
-        <v>60000</v>
+        <v>2000</v>
       </c>
       <c r="M15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O15">
         <v>0</v>
       </c>
       <c r="P15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R15" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="S15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -2983,247 +3166,371 @@
         <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C16" t="s">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="D16" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F16">
-        <v>8000000</v>
+        <v>16180000</v>
       </c>
       <c r="G16">
-        <v>4000000</v>
+        <v>1618000</v>
       </c>
       <c r="H16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I16">
-        <v>2000</v>
+        <v>6200</v>
       </c>
       <c r="J16">
-        <v>2000</v>
+        <v>7700</v>
       </c>
       <c r="K16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L16">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="M16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O16">
         <v>0</v>
       </c>
       <c r="P16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R16" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="S16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" spans="1:20">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C17" t="s">
-        <v>59</v>
+        <v>109</v>
       </c>
       <c r="D17" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="E17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F17">
-        <v>28960000</v>
+        <v>435000000</v>
       </c>
       <c r="G17">
-        <v>1810000</v>
+        <v>7250000</v>
       </c>
       <c r="H17" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I17">
-        <v>9000</v>
+        <v>47000</v>
       </c>
       <c r="J17">
-        <v>12000</v>
+        <v>60000</v>
       </c>
       <c r="K17" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L17">
-        <v>16000</v>
+        <v>60000</v>
       </c>
       <c r="M17" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N17" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O17">
         <v>0</v>
       </c>
       <c r="P17" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q17" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R17" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="S17" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T17" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:20">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C18" t="s">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="D18" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F18">
-        <v>57589000</v>
+        <v>8000000</v>
       </c>
       <c r="G18">
-        <v>1330000</v>
+        <v>4000000</v>
       </c>
       <c r="H18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I18">
-        <v>36400</v>
+        <v>2000</v>
       </c>
       <c r="J18">
-        <v>43300</v>
+        <v>2000</v>
       </c>
       <c r="K18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L18">
-        <v>43300</v>
+        <v>2000</v>
       </c>
       <c r="M18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O18">
         <v>0</v>
       </c>
       <c r="P18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="Q18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="R18" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="S18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="T18" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:20">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C19" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D19" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="E19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F19">
-        <v>43200000</v>
+        <v>28960000</v>
       </c>
       <c r="G19">
-        <v>2400000</v>
+        <v>1810000</v>
       </c>
       <c r="H19" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I19">
-        <v>11000</v>
+        <v>9000</v>
       </c>
       <c r="J19">
-        <v>14200</v>
+        <v>12000</v>
       </c>
       <c r="K19" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L19">
-        <v>18000</v>
+        <v>16000</v>
       </c>
       <c r="M19" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="N19" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="O19">
         <v>0</v>
       </c>
       <c r="P19" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>71</v>
+      </c>
+      <c r="R19" t="s">
+        <v>128</v>
+      </c>
+      <c r="S19" t="s">
+        <v>71</v>
+      </c>
+      <c r="T19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20">
+      <c r="A20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" t="s">
+        <v>91</v>
+      </c>
+      <c r="E20" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20">
+        <v>57589000</v>
+      </c>
+      <c r="G20">
+        <v>1330000</v>
+      </c>
+      <c r="H20" t="s">
+        <v>71</v>
+      </c>
+      <c r="I20">
+        <v>36400</v>
+      </c>
+      <c r="J20">
+        <v>43300</v>
+      </c>
+      <c r="K20" t="s">
+        <v>71</v>
+      </c>
+      <c r="L20">
+        <v>43300</v>
+      </c>
+      <c r="M20" t="s">
+        <v>71</v>
+      </c>
+      <c r="N20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>71</v>
+      </c>
+      <c r="R20" t="s">
+        <v>129</v>
+      </c>
+      <c r="S20" t="s">
+        <v>71</v>
+      </c>
+      <c r="T20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20">
+      <c r="A21" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" t="s">
         <v>66</v>
       </c>
-      <c r="Q19" t="s">
-        <v>66</v>
-      </c>
-      <c r="R19" t="s">
-        <v>123</v>
-      </c>
-      <c r="S19" t="s">
-        <v>66</v>
-      </c>
-      <c r="T19" t="s">
-        <v>66</v>
+      <c r="D21" t="s">
+        <v>81</v>
+      </c>
+      <c r="E21" t="s">
+        <v>34</v>
+      </c>
+      <c r="F21">
+        <v>43200000</v>
+      </c>
+      <c r="G21">
+        <v>2400000</v>
+      </c>
+      <c r="H21" t="s">
+        <v>71</v>
+      </c>
+      <c r="I21">
+        <v>11000</v>
+      </c>
+      <c r="J21">
+        <v>14200</v>
+      </c>
+      <c r="K21" t="s">
+        <v>71</v>
+      </c>
+      <c r="L21">
+        <v>18000</v>
+      </c>
+      <c r="M21" t="s">
+        <v>71</v>
+      </c>
+      <c r="N21" t="s">
+        <v>71</v>
+      </c>
+      <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="P21" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>71</v>
+      </c>
+      <c r="R21" t="s">
+        <v>130</v>
+      </c>
+      <c r="S21" t="s">
+        <v>71</v>
+      </c>
+      <c r="T21" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -3233,21 +3540,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -3259,10 +3566,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -3271,30 +3578,30 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D2" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="E2" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="F2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="G2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H2">
         <v>8000</v>
@@ -3314,34 +3621,34 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B3" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="D3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="E3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="H3">
-        <v>12000</v>
+        <v>43200</v>
       </c>
       <c r="I3">
-        <v>6000000</v>
+        <v>2400000</v>
       </c>
       <c r="J3">
-        <v>2000</v>
+        <v>18000</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -3352,25 +3659,25 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D4" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E4" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="F4" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="G4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H4">
         <v>130500</v>
@@ -3390,34 +3697,34 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D5" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F5" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="G5" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="H5">
-        <v>43200</v>
+        <v>12000</v>
       </c>
       <c r="I5">
-        <v>2400000</v>
+        <v>6000000</v>
       </c>
       <c r="J5">
-        <v>18000</v>
+        <v>2000</v>
       </c>
       <c r="K5">
         <v>0</v>
@@ -3428,25 +3735,25 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F6" t="s">
+        <v>79</v>
+      </c>
+      <c r="G6" t="s">
         <v>28</v>
-      </c>
-      <c r="C6" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" t="s">
-        <v>61</v>
-      </c>
-      <c r="E6" t="s">
-        <v>61</v>
-      </c>
-      <c r="F6" t="s">
-        <v>74</v>
-      </c>
-      <c r="G6" t="s">
-        <v>27</v>
       </c>
       <c r="H6">
         <v>8000</v>
@@ -3466,25 +3773,25 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B7" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H7">
         <v>11600</v>
@@ -3504,34 +3811,34 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>74</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G8" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="H8">
-        <v>16180</v>
+        <v>13000</v>
       </c>
       <c r="I8">
-        <v>1618000</v>
+        <v>6500000</v>
       </c>
       <c r="J8">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -3542,34 +3849,34 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E9" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="F9" t="s">
-        <v>23</v>
+        <v>88</v>
       </c>
       <c r="G9" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="H9">
-        <v>22400</v>
+        <v>16180</v>
       </c>
       <c r="I9">
-        <v>1400000</v>
+        <v>1618000</v>
       </c>
       <c r="J9">
-        <v>16000</v>
+        <v>10000</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -3580,25 +3887,25 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B10" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E10" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="F10" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H10">
         <v>54133.66</v>
@@ -3618,25 +3925,25 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B11" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E11" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="F11" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="G11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H11">
         <v>255360</v>
@@ -3656,25 +3963,25 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B12" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E12" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="F12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H12">
         <v>50781.225</v>
@@ -3694,34 +4001,34 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="C13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D13" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E13" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F13" t="s">
-        <v>80</v>
+        <v>24</v>
       </c>
       <c r="G13" t="s">
         <v>23</v>
       </c>
       <c r="H13">
-        <v>22340</v>
+        <v>22400</v>
       </c>
       <c r="I13">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="J13">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -3732,376 +4039,376 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B14" t="s">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="E14" t="s">
-        <v>129</v>
+        <v>65</v>
       </c>
       <c r="F14" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H14">
-        <v>10640</v>
+        <v>22340</v>
       </c>
       <c r="I14">
-        <v>7600000</v>
+        <v>2234000</v>
       </c>
       <c r="J14">
-        <v>35000</v>
+        <v>10000</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14">
-        <v>4</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B15" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D15" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E15" t="s">
-        <v>59</v>
+        <v>136</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G15" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="H15">
-        <v>28960</v>
+        <v>10640</v>
       </c>
       <c r="I15">
-        <v>1810000</v>
+        <v>7600000</v>
       </c>
       <c r="J15">
-        <v>16000</v>
+        <v>35000</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B16" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C16" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="E16" t="s">
-        <v>128</v>
+        <v>65</v>
       </c>
       <c r="F16" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G16" t="s">
         <v>32</v>
       </c>
       <c r="H16">
-        <v>3455.34</v>
+        <v>28960</v>
       </c>
       <c r="I16">
-        <v>1330000</v>
+        <v>1810000</v>
       </c>
       <c r="J16">
-        <v>43300</v>
+        <v>16000</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16">
-        <v>6</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>104</v>
+        <v>57</v>
       </c>
       <c r="E17" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="F17" t="s">
-        <v>84</v>
+        <v>21</v>
       </c>
       <c r="G17" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="H17">
-        <v>17400</v>
+        <v>22800</v>
       </c>
       <c r="I17">
-        <v>7250000</v>
+        <v>1500000</v>
       </c>
       <c r="J17">
-        <v>60000</v>
+        <v>16000</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
       <c r="L17">
-        <v>4</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>82</v>
       </c>
       <c r="C18" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="D18" t="s">
-        <v>104</v>
+        <v>61</v>
       </c>
       <c r="E18" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="F18" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="G18" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="H18">
-        <v>143550</v>
+        <v>3455.34</v>
       </c>
       <c r="I18">
-        <v>7250000</v>
+        <v>1330000</v>
       </c>
       <c r="J18">
-        <v>60000</v>
+        <v>43300</v>
       </c>
       <c r="K18">
         <v>0</v>
       </c>
       <c r="L18">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D19" t="s">
-        <v>57</v>
+        <v>109</v>
       </c>
       <c r="E19" t="s">
-        <v>57</v>
+        <v>134</v>
       </c>
       <c r="F19" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="G19" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H19">
-        <v>15771</v>
+        <v>17400</v>
       </c>
       <c r="I19">
-        <v>751000</v>
+        <v>7250000</v>
       </c>
       <c r="J19">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
+        <v>23</v>
       </c>
       <c r="C20" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="D20" t="s">
         <v>57</v>
       </c>
       <c r="E20" t="s">
-        <v>57</v>
+        <v>137</v>
       </c>
       <c r="F20" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G20" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="H20">
-        <v>29700</v>
+        <v>1200</v>
       </c>
       <c r="I20">
-        <v>1350000</v>
+        <v>1500000</v>
       </c>
       <c r="J20">
-        <v>22000</v>
+        <v>16000</v>
       </c>
       <c r="K20">
         <v>0</v>
       </c>
       <c r="L20">
-        <v>100</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:12">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>33</v>
       </c>
       <c r="C21" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="D21" t="s">
-        <v>56</v>
+        <v>109</v>
       </c>
       <c r="E21" t="s">
-        <v>56</v>
+        <v>134</v>
       </c>
       <c r="F21" t="s">
-        <v>21</v>
+        <v>89</v>
       </c>
       <c r="G21" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="H21">
-        <v>21700</v>
+        <v>143550</v>
       </c>
       <c r="I21">
-        <v>1400000</v>
+        <v>7250000</v>
       </c>
       <c r="J21">
-        <v>15500</v>
+        <v>60000</v>
       </c>
       <c r="K21">
         <v>0</v>
       </c>
       <c r="L21">
-        <v>100</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:12">
       <c r="A22" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="B22" t="s">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="C22" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D22" t="s">
-        <v>104</v>
+        <v>63</v>
       </c>
       <c r="E22" t="s">
-        <v>127</v>
+        <v>63</v>
       </c>
       <c r="F22" t="s">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="G22" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="H22">
-        <v>143550</v>
+        <v>29700</v>
       </c>
       <c r="I22">
-        <v>7250000</v>
+        <v>1350000</v>
       </c>
       <c r="J22">
-        <v>60000</v>
+        <v>22000</v>
       </c>
       <c r="K22">
         <v>0</v>
       </c>
       <c r="L22">
-        <v>33</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:12">
       <c r="A23" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="B23" t="s">
-        <v>71</v>
+        <v>24</v>
       </c>
       <c r="C23" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D23" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="E23" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="F23" t="s">
-        <v>22</v>
+        <v>74</v>
       </c>
       <c r="G23" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H23">
-        <v>29000</v>
+        <v>15771</v>
       </c>
       <c r="I23">
-        <v>1000000</v>
+        <v>751000</v>
       </c>
       <c r="J23">
-        <v>29000</v>
+        <v>21000</v>
       </c>
       <c r="K23">
         <v>0</v>
@@ -4112,39 +4419,153 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B24" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C24" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="D24" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="E24" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F24" t="s">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="G24" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H24">
-        <v>13000</v>
+        <v>21700</v>
       </c>
       <c r="I24">
-        <v>1000000</v>
+        <v>1400000</v>
       </c>
       <c r="J24">
-        <v>13000</v>
+        <v>15500</v>
       </c>
       <c r="K24">
         <v>0</v>
       </c>
       <c r="L24">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" t="s">
+        <v>59</v>
+      </c>
+      <c r="B25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D25" t="s">
+        <v>59</v>
+      </c>
+      <c r="E25" t="s">
+        <v>59</v>
+      </c>
+      <c r="F25" t="s">
+        <v>23</v>
+      </c>
+      <c r="G25" t="s">
+        <v>20</v>
+      </c>
+      <c r="H25">
+        <v>29000</v>
+      </c>
+      <c r="I25">
+        <v>1000000</v>
+      </c>
+      <c r="J25">
+        <v>29000</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" t="s">
+        <v>59</v>
+      </c>
+      <c r="B26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" t="s">
+        <v>50</v>
+      </c>
+      <c r="D26" t="s">
+        <v>109</v>
+      </c>
+      <c r="E26" t="s">
+        <v>134</v>
+      </c>
+      <c r="F26" t="s">
+        <v>89</v>
+      </c>
+      <c r="G26" t="s">
+        <v>30</v>
+      </c>
+      <c r="H26">
+        <v>143550</v>
+      </c>
+      <c r="I26">
+        <v>7250000</v>
+      </c>
+      <c r="J26">
+        <v>60000</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="L26">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B27" t="s">
+        <v>74</v>
+      </c>
+      <c r="C27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D27" t="s">
+        <v>59</v>
+      </c>
+      <c r="E27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F27" t="s">
+        <v>84</v>
+      </c>
+      <c r="G27" t="s">
+        <v>18</v>
+      </c>
+      <c r="H27">
+        <v>13000</v>
+      </c>
+      <c r="I27">
+        <v>1000000</v>
+      </c>
+      <c r="J27">
+        <v>13000</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RPA datasets push 2024-08-24
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="141">
   <si>
     <t>상장일</t>
   </si>
@@ -72,6 +72,9 @@
     <t>2024-08-22</t>
   </si>
   <si>
+    <t>2024-08-23</t>
+  </si>
+  <si>
     <t>2024-08-21</t>
   </si>
   <si>
@@ -126,6 +129,9 @@
     <t>M83</t>
   </si>
   <si>
+    <t>이엔셀</t>
+  </si>
+  <si>
     <t>티디에스팜</t>
   </si>
   <si>
@@ -195,6 +201,9 @@
     <t>유진</t>
   </si>
   <si>
+    <t>NH</t>
+  </si>
+  <si>
     <t>한국</t>
   </si>
   <si>
@@ -216,9 +225,6 @@
     <t>삼성</t>
   </si>
   <si>
-    <t>NH</t>
-  </si>
-  <si>
     <t>SK</t>
   </si>
   <si>
@@ -352,6 +358,9 @@
   </si>
   <si>
     <t>638.07 : 1</t>
+  </si>
+  <si>
+    <t>928.06 : 1</t>
   </si>
   <si>
     <t>1608.17 : 1</t>
@@ -787,7 +796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -848,37 +857,37 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D2">
         <v>240</v>
       </c>
       <c r="E2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F2">
         <v>228</v>
       </c>
       <c r="G2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M2">
         <v>16000</v>
@@ -887,10 +896,10 @@
         <v>95</v>
       </c>
       <c r="O2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q2">
         <v>2100000</v>
@@ -901,37 +910,37 @@
         <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D3">
         <v>240</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F3">
         <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="L3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M3">
         <v>16000</v>
@@ -940,10 +949,10 @@
         <v>5</v>
       </c>
       <c r="O3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q3">
         <v>2100000</v>
@@ -954,158 +963,158 @@
         <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D4">
-        <v>130</v>
+        <v>239.7204</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F4">
-        <v>130</v>
+        <v>239.7204</v>
       </c>
       <c r="G4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M4">
-        <v>13000</v>
+        <v>15300</v>
       </c>
       <c r="N4">
         <v>100</v>
       </c>
       <c r="O4" t="s">
-        <v>74</v>
+        <v>24</v>
       </c>
       <c r="P4" t="s">
-        <v>84</v>
+        <v>22</v>
       </c>
       <c r="Q4">
-        <v>723700</v>
+        <v>1156798</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D5">
         <v>130</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F5">
         <v>130</v>
       </c>
       <c r="G5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M5">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="N5">
         <v>100</v>
       </c>
       <c r="O5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="Q5">
-        <v>4875000</v>
+        <v>723700</v>
       </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D6">
-        <v>507.81225</v>
+        <v>130</v>
       </c>
       <c r="E6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F6">
-        <v>507.81225</v>
+        <v>130</v>
       </c>
       <c r="G6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M6">
-        <v>16500</v>
+        <v>2000</v>
       </c>
       <c r="N6">
         <v>100</v>
       </c>
       <c r="O6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="P6" t="s">
-        <v>22</v>
+        <v>86</v>
       </c>
       <c r="Q6">
-        <v>2078175</v>
+        <v>4875000</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -1113,105 +1122,105 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D7">
-        <v>217</v>
+        <v>507.81225</v>
       </c>
       <c r="E7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F7">
-        <v>217</v>
+        <v>507.81225</v>
       </c>
       <c r="G7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M7">
-        <v>15500</v>
+        <v>16500</v>
       </c>
       <c r="N7">
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="P7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q7">
-        <v>1050000</v>
+        <v>2078175</v>
       </c>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D8">
-        <v>290</v>
+        <v>217</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F8">
-        <v>290</v>
+        <v>217</v>
       </c>
       <c r="G8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M8">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="N8">
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="P8" t="s">
         <v>23</v>
       </c>
       <c r="Q8">
-        <v>720000</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -1219,52 +1228,52 @@
         <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D9">
-        <v>157.71</v>
+        <v>290</v>
       </c>
       <c r="E9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F9">
-        <v>157.71</v>
+        <v>290</v>
       </c>
       <c r="G9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M9">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="N9">
         <v>100</v>
       </c>
       <c r="O9" t="s">
+        <v>78</v>
+      </c>
+      <c r="P9" t="s">
         <v>24</v>
       </c>
-      <c r="P9" t="s">
-        <v>74</v>
-      </c>
       <c r="Q9">
-        <v>540250</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -1272,52 +1281,52 @@
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D10">
-        <v>116</v>
+        <v>157.71</v>
       </c>
       <c r="E10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F10">
-        <v>116</v>
+        <v>157.71</v>
       </c>
       <c r="G10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M10">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="N10">
         <v>100</v>
       </c>
       <c r="O10" t="s">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="P10" t="s">
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="Q10">
-        <v>4350000</v>
+        <v>540250</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -1325,52 +1334,52 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D11">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="E11" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F11">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="G11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M11">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N11">
         <v>100</v>
       </c>
       <c r="O11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="P11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q11">
-        <v>1050000</v>
+        <v>4350000</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -1378,52 +1387,52 @@
         <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D12">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="E12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F12">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="G12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M12">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="N12">
         <v>100</v>
       </c>
       <c r="O12" t="s">
-        <v>28</v>
+        <v>79</v>
       </c>
       <c r="P12" t="s">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="Q12">
-        <v>1675500</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -1431,52 +1440,52 @@
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D13">
-        <v>297</v>
+        <v>223.4</v>
       </c>
       <c r="E13" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="F13">
-        <v>297</v>
+        <v>223.4</v>
       </c>
       <c r="G13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M13">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="N13">
         <v>100</v>
       </c>
       <c r="O13" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="P13" t="s">
-        <v>28</v>
+        <v>87</v>
       </c>
       <c r="Q13">
-        <v>1012500</v>
+        <v>1675500</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1484,102 +1493,102 @@
         <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D14">
-        <v>2660</v>
+        <v>297</v>
       </c>
       <c r="E14" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="F14">
-        <v>2553.6</v>
+        <v>297</v>
       </c>
       <c r="G14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K14" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M14">
-        <v>35000</v>
+        <v>22000</v>
       </c>
       <c r="N14">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="O14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="P14" t="s">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="Q14">
-        <v>9340690</v>
+        <v>1012500</v>
       </c>
     </row>
     <row r="15" spans="1:17">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D15">
         <v>2660</v>
       </c>
       <c r="E15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F15">
-        <v>106.4</v>
+        <v>2553.6</v>
       </c>
       <c r="G15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="L15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M15">
         <v>35000</v>
       </c>
       <c r="N15">
-        <v>4</v>
+        <v>96</v>
       </c>
       <c r="O15" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="P15" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="Q15">
         <v>9340690</v>
@@ -1590,52 +1599,52 @@
         <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C16" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D16">
-        <v>120</v>
+        <v>2660</v>
       </c>
       <c r="E16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F16">
-        <v>120</v>
+        <v>106.4</v>
       </c>
       <c r="G16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K16" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="L16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M16">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="N16">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="O16" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="P16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q16">
-        <v>4500000</v>
+        <v>9340690</v>
       </c>
     </row>
     <row r="17" spans="1:17">
@@ -1643,37 +1652,37 @@
         <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D17">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="E17" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="F17">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="G17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K17" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M17">
         <v>2000</v>
@@ -1682,13 +1691,13 @@
         <v>100</v>
       </c>
       <c r="O17" t="s">
-        <v>29</v>
+        <v>82</v>
       </c>
       <c r="P17" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="Q17">
-        <v>3000000</v>
+        <v>4500000</v>
       </c>
     </row>
     <row r="18" spans="1:17">
@@ -1696,52 +1705,52 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C18" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D18">
-        <v>161.8</v>
+        <v>80</v>
       </c>
       <c r="E18" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="F18">
-        <v>161.8</v>
+        <v>80</v>
       </c>
       <c r="G18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M18">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="N18">
         <v>100</v>
       </c>
       <c r="O18" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="P18" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="Q18">
-        <v>1187900</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="19" spans="1:17">
@@ -1749,90 +1758,90 @@
         <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D19">
-        <v>4350</v>
+        <v>161.8</v>
       </c>
       <c r="E19" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F19">
-        <v>1435.5</v>
+        <v>161.8</v>
       </c>
       <c r="G19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M19">
-        <v>60000</v>
+        <v>10000</v>
       </c>
       <c r="N19">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="O19" t="s">
         <v>33</v>
       </c>
       <c r="P19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q19">
-        <v>21750000</v>
+        <v>1187900</v>
       </c>
     </row>
     <row r="20" spans="1:17">
       <c r="A20" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C20" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D20">
         <v>4350</v>
       </c>
       <c r="E20" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F20">
         <v>1435.5</v>
       </c>
       <c r="G20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K20" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M20">
         <v>60000</v>
@@ -1841,10 +1850,10 @@
         <v>33</v>
       </c>
       <c r="O20" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P20" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="Q20">
         <v>21750000</v>
@@ -1852,52 +1861,52 @@
     </row>
     <row r="21" spans="1:17">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D21">
         <v>4350</v>
       </c>
       <c r="E21" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="F21">
-        <v>1305</v>
+        <v>1435.5</v>
       </c>
       <c r="G21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M21">
         <v>60000</v>
       </c>
       <c r="N21">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="O21" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P21" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="Q21">
         <v>21750000</v>
@@ -1905,52 +1914,52 @@
     </row>
     <row r="22" spans="1:17">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C22" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D22">
         <v>4350</v>
       </c>
       <c r="E22" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="F22">
-        <v>174</v>
+        <v>1305</v>
       </c>
       <c r="G22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K22" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="L22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M22">
         <v>60000</v>
       </c>
       <c r="N22">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="O22" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P22" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="Q22">
         <v>21750000</v>
@@ -1961,52 +1970,52 @@
         <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C23" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D23">
-        <v>80</v>
+        <v>4350</v>
       </c>
       <c r="E23" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F23">
-        <v>80</v>
+        <v>174</v>
       </c>
       <c r="G23" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H23" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I23" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J23" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K23" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="L23" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M23">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="N23">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="O23" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P23" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="Q23">
-        <v>3000000</v>
+        <v>21750000</v>
       </c>
     </row>
     <row r="24" spans="1:17">
@@ -2014,52 +2023,52 @@
         <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C24" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D24">
-        <v>289.6</v>
+        <v>80</v>
       </c>
       <c r="E24" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="F24">
-        <v>289.6</v>
+        <v>80</v>
       </c>
       <c r="G24" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H24" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I24" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J24" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K24" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L24" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M24">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N24">
         <v>100</v>
       </c>
       <c r="O24" t="s">
-        <v>81</v>
+        <v>34</v>
       </c>
       <c r="P24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q24">
-        <v>1357500</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="25" spans="1:17">
@@ -2067,102 +2076,102 @@
         <v>33</v>
       </c>
       <c r="B25" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C25" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D25">
-        <v>575.89</v>
+        <v>289.6</v>
       </c>
       <c r="E25" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="F25">
-        <v>541.3366</v>
+        <v>289.6</v>
       </c>
       <c r="G25" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H25" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I25" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J25" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L25" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M25">
-        <v>43300</v>
+        <v>16000</v>
       </c>
       <c r="N25">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="O25" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="P25" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q25">
-        <v>1906400</v>
+        <v>1357500</v>
       </c>
     </row>
     <row r="26" spans="1:17">
       <c r="A26" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B26" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C26" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D26">
         <v>575.89</v>
       </c>
       <c r="E26" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="F26">
-        <v>34.5534</v>
+        <v>541.3366</v>
       </c>
       <c r="G26" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H26" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I26" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J26" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K26" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="L26" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="M26">
         <v>43300</v>
       </c>
       <c r="N26">
-        <v>6</v>
+        <v>94</v>
       </c>
       <c r="O26" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P26" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Q26">
         <v>1906400</v>
@@ -2173,51 +2182,104 @@
         <v>34</v>
       </c>
       <c r="B27" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C27" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D27">
+        <v>575.89</v>
+      </c>
+      <c r="E27" t="s">
+        <v>71</v>
+      </c>
+      <c r="F27">
+        <v>34.5534</v>
+      </c>
+      <c r="G27" t="s">
+        <v>73</v>
+      </c>
+      <c r="H27" t="s">
+        <v>73</v>
+      </c>
+      <c r="I27" t="s">
+        <v>73</v>
+      </c>
+      <c r="J27" t="s">
+        <v>73</v>
+      </c>
+      <c r="K27" t="s">
+        <v>75</v>
+      </c>
+      <c r="L27" t="s">
+        <v>73</v>
+      </c>
+      <c r="M27">
+        <v>43300</v>
+      </c>
+      <c r="N27">
+        <v>6</v>
+      </c>
+      <c r="O27" t="s">
+        <v>84</v>
+      </c>
+      <c r="P27" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q27">
+        <v>1906400</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17">
+      <c r="A28" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" t="s">
+        <v>57</v>
+      </c>
+      <c r="D28">
         <v>432</v>
       </c>
-      <c r="E27" t="s">
-        <v>66</v>
-      </c>
-      <c r="F27">
+      <c r="E28" t="s">
+        <v>61</v>
+      </c>
+      <c r="F28">
         <v>432</v>
       </c>
-      <c r="G27" t="s">
-        <v>71</v>
-      </c>
-      <c r="H27" t="s">
-        <v>71</v>
-      </c>
-      <c r="I27" t="s">
-        <v>71</v>
-      </c>
-      <c r="J27" t="s">
-        <v>71</v>
-      </c>
-      <c r="K27" t="s">
-        <v>72</v>
-      </c>
-      <c r="L27" t="s">
-        <v>71</v>
-      </c>
-      <c r="M27">
+      <c r="G28" t="s">
+        <v>73</v>
+      </c>
+      <c r="H28" t="s">
+        <v>73</v>
+      </c>
+      <c r="I28" t="s">
+        <v>73</v>
+      </c>
+      <c r="J28" t="s">
+        <v>73</v>
+      </c>
+      <c r="K28" t="s">
+        <v>74</v>
+      </c>
+      <c r="L28" t="s">
+        <v>73</v>
+      </c>
+      <c r="M28">
         <v>18000</v>
       </c>
-      <c r="N27">
+      <c r="N28">
         <v>100</v>
       </c>
-      <c r="O27" t="s">
+      <c r="O28" t="s">
+        <v>85</v>
+      </c>
+      <c r="P28" t="s">
         <v>83</v>
       </c>
-      <c r="P27" t="s">
-        <v>81</v>
-      </c>
-      <c r="Q27">
+      <c r="Q28">
         <v>1758600</v>
       </c>
     </row>
@@ -2228,7 +2290,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T21"/>
+  <dimension ref="A1:T22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -2236,10 +2298,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -2248,63 +2310,63 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
@@ -2316,7 +2378,7 @@
         <v>1500000</v>
       </c>
       <c r="H2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I2">
         <v>11000</v>
@@ -2325,804 +2387,804 @@
         <v>13000</v>
       </c>
       <c r="K2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L2">
         <v>16000</v>
       </c>
       <c r="M2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="S2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D3" t="s">
-        <v>84</v>
+        <v>22</v>
       </c>
       <c r="E3" t="s">
         <v>18</v>
       </c>
       <c r="F3">
-        <v>13000000</v>
+        <v>23972040</v>
       </c>
       <c r="G3">
-        <v>1000000</v>
+        <v>1566800</v>
       </c>
       <c r="H3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I3">
-        <v>9500</v>
+        <v>13600</v>
       </c>
       <c r="J3">
-        <v>10700</v>
+        <v>15300</v>
       </c>
       <c r="K3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L3">
-        <v>13000</v>
+        <v>15300</v>
       </c>
       <c r="M3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O3">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="S3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F4">
         <v>13000000</v>
       </c>
       <c r="G4">
-        <v>6500000</v>
+        <v>1000000</v>
       </c>
       <c r="H4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I4">
-        <v>2000</v>
+        <v>9500</v>
       </c>
       <c r="J4">
-        <v>2000</v>
+        <v>10700</v>
       </c>
       <c r="K4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L4">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="M4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="P4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="S4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>86</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F5">
-        <v>50781225</v>
+        <v>13000000</v>
       </c>
       <c r="G5">
-        <v>3077650</v>
+        <v>6500000</v>
       </c>
       <c r="H5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I5">
-        <v>13800</v>
+        <v>2000</v>
       </c>
       <c r="J5">
-        <v>15700</v>
+        <v>2000</v>
       </c>
       <c r="K5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L5">
-        <v>16500</v>
+        <v>2000</v>
       </c>
       <c r="M5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O5">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="S5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E6" t="s">
         <v>20</v>
       </c>
       <c r="F6">
-        <v>21700000</v>
+        <v>50781225</v>
       </c>
       <c r="G6">
-        <v>1400000</v>
+        <v>3077650</v>
       </c>
       <c r="H6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I6">
-        <v>12500</v>
+        <v>13800</v>
       </c>
       <c r="J6">
-        <v>15500</v>
+        <v>15700</v>
       </c>
       <c r="K6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L6">
-        <v>15500</v>
+        <v>16500</v>
       </c>
       <c r="M6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="S6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D7" t="s">
         <v>23</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F7">
-        <v>29000000</v>
+        <v>21700000</v>
       </c>
       <c r="G7">
-        <v>1000000</v>
+        <v>1400000</v>
       </c>
       <c r="H7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I7">
-        <v>24000</v>
+        <v>12500</v>
       </c>
       <c r="J7">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="K7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L7">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="M7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="S7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" t="s">
         <v>24</v>
-      </c>
-      <c r="B8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" t="s">
-        <v>63</v>
-      </c>
-      <c r="D8" t="s">
-        <v>74</v>
       </c>
       <c r="E8" t="s">
         <v>21</v>
       </c>
       <c r="F8">
-        <v>15771000</v>
+        <v>29000000</v>
       </c>
       <c r="G8">
-        <v>751000</v>
+        <v>1000000</v>
       </c>
       <c r="H8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I8">
-        <v>18000</v>
+        <v>24000</v>
       </c>
       <c r="J8">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="K8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L8">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="M8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O8">
-        <v>72.87616511318242</v>
+        <v>0</v>
       </c>
       <c r="P8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="S8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="E9" t="s">
         <v>22</v>
       </c>
       <c r="F9">
-        <v>11600000</v>
+        <v>15771000</v>
       </c>
       <c r="G9">
-        <v>5800000</v>
+        <v>751000</v>
       </c>
       <c r="H9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I9">
-        <v>2000</v>
+        <v>18000</v>
       </c>
       <c r="J9">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="K9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L9">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="M9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O9">
-        <v>0</v>
+        <v>72.87616511318242</v>
       </c>
       <c r="P9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R9" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="S9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
         <v>23</v>
       </c>
       <c r="F10">
-        <v>22400000</v>
+        <v>11600000</v>
       </c>
       <c r="G10">
-        <v>1400000</v>
+        <v>5800000</v>
       </c>
       <c r="H10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I10">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="J10">
-        <v>19000</v>
+        <v>2000</v>
       </c>
       <c r="K10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L10">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="M10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O10">
         <v>0</v>
       </c>
       <c r="P10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R10" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="S10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>79</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="E11" t="s">
         <v>24</v>
       </c>
       <c r="F11">
-        <v>22340000</v>
+        <v>22400000</v>
       </c>
       <c r="G11">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="H11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I11">
-        <v>7300</v>
+        <v>16000</v>
       </c>
       <c r="J11">
-        <v>8500</v>
+        <v>19000</v>
       </c>
       <c r="K11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L11">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="M11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O11">
         <v>0</v>
       </c>
       <c r="P11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="S11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>87</v>
       </c>
       <c r="E12" t="s">
         <v>25</v>
       </c>
       <c r="F12">
-        <v>29700000</v>
+        <v>22340000</v>
       </c>
       <c r="G12">
-        <v>1350000</v>
+        <v>2234000</v>
       </c>
       <c r="H12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I12">
-        <v>14000</v>
+        <v>7300</v>
       </c>
       <c r="J12">
-        <v>17000</v>
+        <v>8500</v>
       </c>
       <c r="K12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L12">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="M12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O12">
         <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R12" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="S12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C13" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D13" t="s">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="E13" t="s">
         <v>26</v>
       </c>
       <c r="F13">
-        <v>266000000</v>
+        <v>29700000</v>
       </c>
       <c r="G13">
-        <v>7600000</v>
+        <v>1350000</v>
       </c>
       <c r="H13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I13">
-        <v>24000</v>
+        <v>14000</v>
       </c>
       <c r="J13">
-        <v>30000</v>
+        <v>17000</v>
       </c>
       <c r="K13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L13">
-        <v>35000</v>
+        <v>22000</v>
       </c>
       <c r="M13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O13">
-        <v>14.47368421052632</v>
+        <v>0</v>
       </c>
       <c r="P13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R13" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="S13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C14" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E14" t="s">
         <v>27</v>
       </c>
       <c r="F14">
-        <v>12000000</v>
+        <v>266000000</v>
       </c>
       <c r="G14">
-        <v>6000000</v>
+        <v>7600000</v>
       </c>
       <c r="H14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I14">
-        <v>2000</v>
+        <v>24000</v>
       </c>
       <c r="J14">
-        <v>2000</v>
+        <v>30000</v>
       </c>
       <c r="K14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L14">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="M14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O14">
-        <v>0</v>
+        <v>14.47368421052632</v>
       </c>
       <c r="P14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R14" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="S14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>82</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="E15" t="s">
         <v>28</v>
       </c>
       <c r="F15">
-        <v>8000000</v>
+        <v>12000000</v>
       </c>
       <c r="G15">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="H15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I15">
         <v>2000</v>
@@ -3131,96 +3193,96 @@
         <v>2000</v>
       </c>
       <c r="K15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L15">
         <v>2000</v>
       </c>
       <c r="M15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O15">
         <v>0</v>
       </c>
       <c r="P15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R15" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="S15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:20">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C16" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D16" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
       </c>
       <c r="F16">
-        <v>16180000</v>
+        <v>8000000</v>
       </c>
       <c r="G16">
-        <v>1618000</v>
+        <v>4000000</v>
       </c>
       <c r="H16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I16">
-        <v>6200</v>
+        <v>2000</v>
       </c>
       <c r="J16">
-        <v>7700</v>
+        <v>2000</v>
       </c>
       <c r="K16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L16">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="M16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O16">
         <v>0</v>
       </c>
       <c r="P16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R16" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="S16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:20">
@@ -3228,309 +3290,371 @@
         <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C17" t="s">
-        <v>109</v>
+        <v>63</v>
       </c>
       <c r="D17" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E17" t="s">
         <v>30</v>
       </c>
       <c r="F17">
-        <v>435000000</v>
+        <v>16180000</v>
       </c>
       <c r="G17">
-        <v>7250000</v>
+        <v>1618000</v>
       </c>
       <c r="H17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I17">
-        <v>47000</v>
+        <v>6200</v>
       </c>
       <c r="J17">
-        <v>60000</v>
+        <v>7700</v>
       </c>
       <c r="K17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L17">
-        <v>60000</v>
+        <v>10000</v>
       </c>
       <c r="M17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O17">
         <v>0</v>
       </c>
       <c r="P17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R17" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="S17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:20">
       <c r="A18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E18" t="s">
         <v>31</v>
       </c>
       <c r="F18">
-        <v>8000000</v>
+        <v>435000000</v>
       </c>
       <c r="G18">
-        <v>4000000</v>
+        <v>7250000</v>
       </c>
       <c r="H18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I18">
-        <v>2000</v>
+        <v>47000</v>
       </c>
       <c r="J18">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="K18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L18">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="M18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O18">
         <v>0</v>
       </c>
       <c r="P18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R18" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="S18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="1:20">
       <c r="A19" t="s">
-        <v>81</v>
+        <v>34</v>
       </c>
       <c r="B19" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C19" t="s">
-        <v>65</v>
+        <v>112</v>
       </c>
       <c r="D19" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E19" t="s">
         <v>32</v>
       </c>
       <c r="F19">
-        <v>28960000</v>
+        <v>8000000</v>
       </c>
       <c r="G19">
-        <v>1810000</v>
+        <v>4000000</v>
       </c>
       <c r="H19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I19">
-        <v>9000</v>
+        <v>2000</v>
       </c>
       <c r="J19">
-        <v>12000</v>
+        <v>2000</v>
       </c>
       <c r="K19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L19">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="M19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O19">
         <v>0</v>
       </c>
       <c r="P19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R19" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="S19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:20">
       <c r="A20" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B20" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C20" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="D20" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E20" t="s">
         <v>33</v>
       </c>
       <c r="F20">
-        <v>57589000</v>
+        <v>28960000</v>
       </c>
       <c r="G20">
-        <v>1330000</v>
+        <v>1810000</v>
       </c>
       <c r="H20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I20">
-        <v>36400</v>
+        <v>9000</v>
       </c>
       <c r="J20">
-        <v>43300</v>
+        <v>12000</v>
       </c>
       <c r="K20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L20">
-        <v>43300</v>
+        <v>16000</v>
       </c>
       <c r="M20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O20">
         <v>0</v>
       </c>
       <c r="P20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R20" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="S20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:20">
       <c r="A21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C21" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="E21" t="s">
         <v>34</v>
       </c>
       <c r="F21">
-        <v>43200000</v>
+        <v>57589000</v>
       </c>
       <c r="G21">
-        <v>2400000</v>
+        <v>1330000</v>
       </c>
       <c r="H21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I21">
-        <v>11000</v>
+        <v>36400</v>
       </c>
       <c r="J21">
-        <v>14200</v>
+        <v>43300</v>
       </c>
       <c r="K21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L21">
-        <v>18000</v>
+        <v>43300</v>
       </c>
       <c r="M21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O21">
         <v>0</v>
       </c>
       <c r="P21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R21" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="S21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="T21" t="s">
-        <v>71</v>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20">
+      <c r="A22" t="s">
+        <v>85</v>
+      </c>
+      <c r="B22" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" t="s">
+        <v>61</v>
+      </c>
+      <c r="D22" t="s">
+        <v>83</v>
+      </c>
+      <c r="E22" t="s">
+        <v>35</v>
+      </c>
+      <c r="F22">
+        <v>43200000</v>
+      </c>
+      <c r="G22">
+        <v>2400000</v>
+      </c>
+      <c r="H22" t="s">
+        <v>73</v>
+      </c>
+      <c r="I22">
+        <v>11000</v>
+      </c>
+      <c r="J22">
+        <v>14200</v>
+      </c>
+      <c r="K22" t="s">
+        <v>73</v>
+      </c>
+      <c r="L22">
+        <v>18000</v>
+      </c>
+      <c r="M22" t="s">
+        <v>73</v>
+      </c>
+      <c r="N22" t="s">
+        <v>73</v>
+      </c>
+      <c r="O22">
+        <v>0</v>
+      </c>
+      <c r="P22" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>73</v>
+      </c>
+      <c r="R22" t="s">
+        <v>133</v>
+      </c>
+      <c r="S22" t="s">
+        <v>73</v>
+      </c>
+      <c r="T22" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -3540,21 +3664,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -3566,10 +3690,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -3578,30 +3702,30 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H2">
         <v>8000</v>
@@ -3621,25 +3745,25 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F3" t="s">
         <v>83</v>
       </c>
-      <c r="C3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F3" t="s">
-        <v>81</v>
-      </c>
       <c r="G3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H3">
         <v>43200</v>
@@ -3659,107 +3783,107 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>109</v>
+        <v>61</v>
       </c>
       <c r="E4" t="s">
-        <v>134</v>
+        <v>61</v>
       </c>
       <c r="F4" t="s">
-        <v>89</v>
+        <v>22</v>
       </c>
       <c r="G4" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="H4">
-        <v>130500</v>
+        <v>23972.04</v>
       </c>
       <c r="I4">
-        <v>7250000</v>
+        <v>1566800</v>
       </c>
       <c r="J4">
-        <v>60000</v>
+        <v>15300</v>
       </c>
       <c r="K4">
         <v>0</v>
       </c>
       <c r="L4">
-        <v>30</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D5" t="s">
-        <v>66</v>
+        <v>111</v>
       </c>
       <c r="E5" t="s">
-        <v>66</v>
+        <v>137</v>
       </c>
       <c r="F5" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="G5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="H5">
-        <v>12000</v>
+        <v>130500</v>
       </c>
       <c r="I5">
-        <v>6000000</v>
+        <v>7250000</v>
       </c>
       <c r="J5">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="K5">
         <v>0</v>
       </c>
       <c r="L5">
-        <v>100</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>82</v>
       </c>
       <c r="C6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D6" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E6" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="F6" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G6" t="s">
         <v>28</v>
       </c>
       <c r="H6">
-        <v>8000</v>
+        <v>12000</v>
       </c>
       <c r="I6">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="J6">
         <v>2000</v>
@@ -3773,31 +3897,31 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="D7" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E7" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="F7" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="H7">
-        <v>11600</v>
+        <v>8000</v>
       </c>
       <c r="I7">
-        <v>5800000</v>
+        <v>4000000</v>
       </c>
       <c r="J7">
         <v>2000</v>
@@ -3811,31 +3935,31 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="F8" t="s">
-        <v>84</v>
+        <v>25</v>
       </c>
       <c r="G8" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="H8">
-        <v>13000</v>
+        <v>11600</v>
       </c>
       <c r="I8">
-        <v>6500000</v>
+        <v>5800000</v>
       </c>
       <c r="J8">
         <v>2000</v>
@@ -3849,34 +3973,34 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G9" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="H9">
-        <v>16180</v>
+        <v>13000</v>
       </c>
       <c r="I9">
-        <v>1618000</v>
+        <v>6500000</v>
       </c>
       <c r="J9">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -3887,148 +4011,148 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>82</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E10" t="s">
-        <v>135</v>
+        <v>63</v>
       </c>
       <c r="F10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G10" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H10">
-        <v>54133.66</v>
+        <v>16180</v>
       </c>
       <c r="I10">
-        <v>1330000</v>
+        <v>1618000</v>
       </c>
       <c r="J10">
-        <v>43300</v>
+        <v>10000</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B11" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C11" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="D11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F11" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="G11" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="H11">
-        <v>255360</v>
+        <v>54133.66</v>
       </c>
       <c r="I11">
-        <v>7600000</v>
+        <v>1330000</v>
       </c>
       <c r="J11">
-        <v>35000</v>
+        <v>43300</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="D12" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E12" t="s">
-        <v>61</v>
+        <v>139</v>
       </c>
       <c r="F12" t="s">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="G12" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="H12">
-        <v>50781.225</v>
+        <v>255360</v>
       </c>
       <c r="I12">
-        <v>3077650</v>
+        <v>7600000</v>
       </c>
       <c r="J12">
-        <v>16500</v>
+        <v>35000</v>
       </c>
       <c r="K12">
         <v>0</v>
       </c>
       <c r="L12">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B13" t="s">
         <v>77</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D13" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E13" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G13" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H13">
-        <v>22400</v>
+        <v>50781.225</v>
       </c>
       <c r="I13">
-        <v>1400000</v>
+        <v>3077650</v>
       </c>
       <c r="J13">
-        <v>16000</v>
+        <v>16500</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -4039,34 +4163,34 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>79</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F14" t="s">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="G14" t="s">
         <v>24</v>
       </c>
       <c r="H14">
-        <v>22340</v>
+        <v>22400</v>
       </c>
       <c r="I14">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="J14">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="K14">
         <v>0</v>
@@ -4077,107 +4201,107 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B15" t="s">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
         <v>46</v>
       </c>
       <c r="D15" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="E15" t="s">
-        <v>136</v>
+        <v>68</v>
       </c>
       <c r="F15" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H15">
-        <v>10640</v>
+        <v>22340</v>
       </c>
       <c r="I15">
-        <v>7600000</v>
+        <v>2234000</v>
       </c>
       <c r="J15">
-        <v>35000</v>
+        <v>10000</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>4</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B16" t="s">
         <v>81</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E16" t="s">
-        <v>65</v>
+        <v>139</v>
       </c>
       <c r="F16" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G16" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="H16">
-        <v>28960</v>
+        <v>10640</v>
       </c>
       <c r="I16">
-        <v>1810000</v>
+        <v>7600000</v>
       </c>
       <c r="J16">
-        <v>16000</v>
+        <v>35000</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="B17" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="C17" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="D17" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="E17" t="s">
-        <v>137</v>
+        <v>68</v>
       </c>
       <c r="F17" t="s">
-        <v>21</v>
+        <v>92</v>
       </c>
       <c r="G17" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="H17">
-        <v>22800</v>
+        <v>28960</v>
       </c>
       <c r="I17">
-        <v>1500000</v>
+        <v>1810000</v>
       </c>
       <c r="J17">
         <v>16000</v>
@@ -4186,229 +4310,229 @@
         <v>0</v>
       </c>
       <c r="L17">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="B18" t="s">
-        <v>82</v>
+        <v>24</v>
       </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="D18" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E18" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F18" t="s">
-        <v>91</v>
+        <v>22</v>
       </c>
       <c r="G18" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="H18">
-        <v>3455.34</v>
+        <v>22800</v>
       </c>
       <c r="I18">
-        <v>1330000</v>
+        <v>1500000</v>
       </c>
       <c r="J18">
-        <v>43300</v>
+        <v>16000</v>
       </c>
       <c r="K18">
         <v>0</v>
       </c>
       <c r="L18">
-        <v>6</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D19" t="s">
-        <v>109</v>
+        <v>64</v>
       </c>
       <c r="E19" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="F19" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G19" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="H19">
-        <v>17400</v>
+        <v>3455.34</v>
       </c>
       <c r="I19">
-        <v>7250000</v>
+        <v>1330000</v>
       </c>
       <c r="J19">
-        <v>60000</v>
+        <v>43300</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="B20" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="C20" t="s">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="D20" t="s">
-        <v>57</v>
+        <v>111</v>
       </c>
       <c r="E20" t="s">
         <v>137</v>
       </c>
       <c r="F20" t="s">
-        <v>21</v>
+        <v>91</v>
       </c>
       <c r="G20" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="H20">
-        <v>1200</v>
+        <v>17400</v>
       </c>
       <c r="I20">
-        <v>1500000</v>
+        <v>7250000</v>
       </c>
       <c r="J20">
-        <v>16000</v>
+        <v>60000</v>
       </c>
       <c r="K20">
         <v>0</v>
       </c>
       <c r="L20">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:12">
       <c r="A21" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="B21" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C21" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="D21" t="s">
-        <v>109</v>
+        <v>59</v>
       </c>
       <c r="E21" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="F21" t="s">
-        <v>89</v>
+        <v>22</v>
       </c>
       <c r="G21" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="H21">
-        <v>143550</v>
+        <v>1200</v>
       </c>
       <c r="I21">
-        <v>7250000</v>
+        <v>1500000</v>
       </c>
       <c r="J21">
-        <v>60000</v>
+        <v>16000</v>
       </c>
       <c r="K21">
         <v>0</v>
       </c>
       <c r="L21">
-        <v>33</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:12">
       <c r="A22" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B22" t="s">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="C22" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="D22" t="s">
-        <v>63</v>
+        <v>111</v>
       </c>
       <c r="E22" t="s">
-        <v>63</v>
+        <v>137</v>
       </c>
       <c r="F22" t="s">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="G22" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="H22">
-        <v>29700</v>
+        <v>143550</v>
       </c>
       <c r="I22">
-        <v>1350000</v>
+        <v>7250000</v>
       </c>
       <c r="J22">
-        <v>22000</v>
+        <v>60000</v>
       </c>
       <c r="K22">
         <v>0</v>
       </c>
       <c r="L22">
-        <v>100</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:12">
       <c r="A23" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B23" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="C23" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="D23" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E23" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F23" t="s">
-        <v>74</v>
+        <v>29</v>
       </c>
       <c r="G23" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="H23">
-        <v>15771</v>
+        <v>29700</v>
       </c>
       <c r="I23">
-        <v>751000</v>
+        <v>1350000</v>
       </c>
       <c r="J23">
-        <v>21000</v>
+        <v>22000</v>
       </c>
       <c r="K23">
         <v>0</v>
@@ -4419,34 +4543,34 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B24" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="C24" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D24" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E24" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F24" t="s">
+        <v>76</v>
+      </c>
+      <c r="G24" t="s">
         <v>22</v>
       </c>
-      <c r="G24" t="s">
-        <v>20</v>
-      </c>
       <c r="H24">
-        <v>21700</v>
+        <v>15771</v>
       </c>
       <c r="I24">
-        <v>1400000</v>
+        <v>751000</v>
       </c>
       <c r="J24">
-        <v>15500</v>
+        <v>21000</v>
       </c>
       <c r="K24">
         <v>0</v>
@@ -4457,34 +4581,34 @@
     </row>
     <row r="25" spans="1:12">
       <c r="A25" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B25" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C25" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D25" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="E25" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F25" t="s">
         <v>23</v>
       </c>
       <c r="G25" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H25">
-        <v>29000</v>
+        <v>21700</v>
       </c>
       <c r="I25">
-        <v>1000000</v>
+        <v>1400000</v>
       </c>
       <c r="J25">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="K25">
         <v>0</v>
@@ -4495,77 +4619,115 @@
     </row>
     <row r="26" spans="1:12">
       <c r="A26" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B26" t="s">
-        <v>33</v>
+        <v>78</v>
       </c>
       <c r="C26" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="D26" t="s">
-        <v>109</v>
+        <v>62</v>
       </c>
       <c r="E26" t="s">
-        <v>134</v>
+        <v>62</v>
       </c>
       <c r="F26" t="s">
-        <v>89</v>
+        <v>24</v>
       </c>
       <c r="G26" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="H26">
-        <v>143550</v>
+        <v>29000</v>
       </c>
       <c r="I26">
-        <v>7250000</v>
+        <v>1000000</v>
       </c>
       <c r="J26">
-        <v>60000</v>
+        <v>29000</v>
       </c>
       <c r="K26">
         <v>0</v>
       </c>
       <c r="L26">
-        <v>33</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:12">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B27" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="C27" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D27" t="s">
-        <v>59</v>
+        <v>111</v>
       </c>
       <c r="E27" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="F27" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="G27" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="H27">
-        <v>13000</v>
+        <v>143550</v>
       </c>
       <c r="I27">
-        <v>1000000</v>
+        <v>7250000</v>
       </c>
       <c r="J27">
-        <v>13000</v>
+        <v>60000</v>
       </c>
       <c r="K27">
         <v>0</v>
       </c>
       <c r="L27">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" t="s">
+        <v>62</v>
+      </c>
+      <c r="B28" t="s">
+        <v>76</v>
+      </c>
+      <c r="C28" t="s">
+        <v>38</v>
+      </c>
+      <c r="D28" t="s">
+        <v>62</v>
+      </c>
+      <c r="E28" t="s">
+        <v>62</v>
+      </c>
+      <c r="F28" t="s">
+        <v>86</v>
+      </c>
+      <c r="G28" t="s">
+        <v>19</v>
+      </c>
+      <c r="H28">
+        <v>13000</v>
+      </c>
+      <c r="I28">
+        <v>1000000</v>
+      </c>
+      <c r="J28">
+        <v>13000</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+      <c r="L28">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RPA datasets push 2024-08-25
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="132">
   <si>
     <t>상장일</t>
   </si>
@@ -120,162 +120,147 @@
     <t>2024-07-03</t>
   </si>
   <si>
+    <t>M83</t>
+  </si>
+  <si>
+    <t>이엔셀</t>
+  </si>
+  <si>
+    <t>티디에스팜</t>
+  </si>
+  <si>
+    <t>대신밸런스제18호스팩</t>
+  </si>
+  <si>
+    <t>전진건설로봇</t>
+  </si>
+  <si>
+    <t>케이쓰리아이</t>
+  </si>
+  <si>
+    <t>넥스트바이오메디컬</t>
+  </si>
+  <si>
+    <t>유라클</t>
+  </si>
+  <si>
+    <t>교보16호스팩</t>
+  </si>
+  <si>
+    <t>뱅크웨어글로벌</t>
+  </si>
+  <si>
+    <t>아이빔테크놀로지</t>
+  </si>
+  <si>
+    <t>피앤에스미캐닉스</t>
+  </si>
+  <si>
+    <t>산일전기</t>
+  </si>
+  <si>
+    <t>엔에이치스팩31호</t>
+  </si>
+  <si>
+    <t>SK증권제13호스팩</t>
+  </si>
+  <si>
+    <t>엑셀세라퓨틱스</t>
+  </si>
+  <si>
+    <t>시프트업</t>
+  </si>
+  <si>
+    <t>이베스트스팩6호</t>
+  </si>
+  <si>
+    <t>하스</t>
+  </si>
+  <si>
+    <t>코스닥</t>
+  </si>
+  <si>
+    <t>코스피</t>
+  </si>
+  <si>
+    <t>신영</t>
+  </si>
+  <si>
+    <t>유진</t>
+  </si>
+  <si>
+    <t>NH</t>
+  </si>
+  <si>
+    <t>한국</t>
+  </si>
+  <si>
+    <t>대신</t>
+  </si>
+  <si>
+    <t>미래</t>
+  </si>
+  <si>
+    <t>하나</t>
+  </si>
+  <si>
+    <t>키움</t>
+  </si>
+  <si>
+    <t>교보</t>
+  </si>
+  <si>
+    <t>삼성</t>
+  </si>
+  <si>
+    <t>SK</t>
+  </si>
+  <si>
+    <t>제이피모간회사</t>
+  </si>
+  <si>
+    <t>신한</t>
+  </si>
+  <si>
+    <t>LS</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>대표</t>
+  </si>
+  <si>
+    <t>인수</t>
+  </si>
+  <si>
+    <t>2024-08-09</t>
+  </si>
+  <si>
+    <t>2024-08-08</t>
+  </si>
+  <si>
+    <t>2024-08-07</t>
+  </si>
+  <si>
+    <t>2024-08-01</t>
+  </si>
+  <si>
+    <t>2024-07-22</t>
+  </si>
+  <si>
+    <t>2024-07-18</t>
+  </si>
+  <si>
+    <t>2024-07-16</t>
+  </si>
+  <si>
     <t>2024-07-02</t>
   </si>
   <si>
-    <t>2024-06-28</t>
-  </si>
-  <si>
-    <t>M83</t>
-  </si>
-  <si>
-    <t>이엔셀</t>
-  </si>
-  <si>
-    <t>티디에스팜</t>
-  </si>
-  <si>
-    <t>대신밸런스제18호스팩</t>
-  </si>
-  <si>
-    <t>전진건설로봇</t>
-  </si>
-  <si>
-    <t>케이쓰리아이</t>
-  </si>
-  <si>
-    <t>넥스트바이오메디컬</t>
-  </si>
-  <si>
-    <t>유라클</t>
-  </si>
-  <si>
-    <t>교보16호스팩</t>
-  </si>
-  <si>
-    <t>뱅크웨어글로벌</t>
-  </si>
-  <si>
-    <t>아이빔테크놀로지</t>
-  </si>
-  <si>
-    <t>피앤에스미캐닉스</t>
-  </si>
-  <si>
-    <t>산일전기</t>
-  </si>
-  <si>
-    <t>엔에이치스팩31호</t>
-  </si>
-  <si>
-    <t>SK증권제13호스팩</t>
-  </si>
-  <si>
-    <t>엑셀세라퓨틱스</t>
-  </si>
-  <si>
-    <t>시프트업</t>
-  </si>
-  <si>
-    <t>이베스트스팩6호</t>
-  </si>
-  <si>
-    <t>하스</t>
-  </si>
-  <si>
-    <t>이노스페이스</t>
-  </si>
-  <si>
-    <t>에이치브이엠</t>
-  </si>
-  <si>
-    <t>코스닥</t>
-  </si>
-  <si>
-    <t>코스피</t>
-  </si>
-  <si>
-    <t>신영</t>
-  </si>
-  <si>
-    <t>유진</t>
-  </si>
-  <si>
-    <t>NH</t>
-  </si>
-  <si>
-    <t>한국</t>
-  </si>
-  <si>
-    <t>대신</t>
-  </si>
-  <si>
-    <t>미래</t>
-  </si>
-  <si>
-    <t>하나</t>
-  </si>
-  <si>
-    <t>키움</t>
-  </si>
-  <si>
-    <t>교보</t>
-  </si>
-  <si>
-    <t>삼성</t>
-  </si>
-  <si>
-    <t>SK</t>
-  </si>
-  <si>
-    <t>제이피모간회사</t>
-  </si>
-  <si>
-    <t>신한</t>
-  </si>
-  <si>
-    <t>LS</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>대표</t>
-  </si>
-  <si>
-    <t>인수</t>
-  </si>
-  <si>
-    <t>2024-08-09</t>
-  </si>
-  <si>
-    <t>2024-08-08</t>
-  </si>
-  <si>
-    <t>2024-08-07</t>
-  </si>
-  <si>
-    <t>2024-08-01</t>
-  </si>
-  <si>
-    <t>2024-07-22</t>
-  </si>
-  <si>
-    <t>2024-07-18</t>
-  </si>
-  <si>
-    <t>2024-07-16</t>
-  </si>
-  <si>
     <t>2024-06-24</t>
   </si>
   <si>
-    <t>2024-06-20</t>
-  </si>
-  <si>
-    <t>2024-06-19</t>
-  </si>
-  <si>
     <t>2024-08-14</t>
   </si>
   <si>
@@ -297,9 +282,6 @@
     <t>2024-06-27</t>
   </si>
   <si>
-    <t>2024-06-25</t>
-  </si>
-  <si>
     <t>회사명</t>
   </si>
   <si>
@@ -414,12 +396,6 @@
     <t>2126.46 : 1</t>
   </si>
   <si>
-    <t>1150.72 : 1</t>
-  </si>
-  <si>
-    <t>960.3509 : 1</t>
-  </si>
-  <si>
     <t>인수기관</t>
   </si>
   <si>
@@ -430,9 +406,6 @@
   </si>
   <si>
     <t>한국, 제이피모간회사 서울지점, NH, 신한</t>
-  </si>
-  <si>
-    <t>미래, 신한</t>
   </si>
   <si>
     <t>미래, 삼성</t>
@@ -796,7 +769,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q28"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -857,37 +830,37 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D2">
         <v>240</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F2">
         <v>228</v>
       </c>
       <c r="G2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K2" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M2">
         <v>16000</v>
@@ -910,37 +883,37 @@
         <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D3">
         <v>240</v>
       </c>
       <c r="E3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F3">
         <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="L3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M3">
         <v>16000</v>
@@ -963,37 +936,37 @@
         <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D4">
         <v>239.7204</v>
       </c>
       <c r="E4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F4">
         <v>239.7204</v>
       </c>
       <c r="G4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M4">
         <v>15300</v>
@@ -1016,37 +989,37 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D5">
         <v>130</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F5">
         <v>130</v>
       </c>
       <c r="G5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K5" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M5">
         <v>13000</v>
@@ -1055,10 +1028,10 @@
         <v>100</v>
       </c>
       <c r="O5" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="P5" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="Q5">
         <v>723700</v>
@@ -1069,37 +1042,37 @@
         <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D6">
         <v>130</v>
       </c>
       <c r="E6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F6">
         <v>130</v>
       </c>
       <c r="G6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K6" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M6">
         <v>2000</v>
@@ -1108,10 +1081,10 @@
         <v>100</v>
       </c>
       <c r="O6" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="P6" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="Q6">
         <v>4875000</v>
@@ -1122,37 +1095,37 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D7">
         <v>507.81225</v>
       </c>
       <c r="E7" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F7">
         <v>507.81225</v>
       </c>
       <c r="G7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K7" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M7">
         <v>16500</v>
@@ -1161,7 +1134,7 @@
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="P7" t="s">
         <v>23</v>
@@ -1175,37 +1148,37 @@
         <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D8">
         <v>217</v>
       </c>
       <c r="E8" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F8">
         <v>217</v>
       </c>
       <c r="G8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K8" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M8">
         <v>15500</v>
@@ -1214,7 +1187,7 @@
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="P8" t="s">
         <v>23</v>
@@ -1228,37 +1201,37 @@
         <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D9">
         <v>290</v>
       </c>
       <c r="E9" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F9">
         <v>290</v>
       </c>
       <c r="G9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K9" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M9">
         <v>29000</v>
@@ -1267,7 +1240,7 @@
         <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="P9" t="s">
         <v>24</v>
@@ -1281,37 +1254,37 @@
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D10">
         <v>157.71</v>
       </c>
       <c r="E10" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F10">
         <v>157.71</v>
       </c>
       <c r="G10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K10" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M10">
         <v>21000</v>
@@ -1323,7 +1296,7 @@
         <v>25</v>
       </c>
       <c r="P10" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="Q10">
         <v>540250</v>
@@ -1334,37 +1307,37 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D11">
         <v>116</v>
       </c>
       <c r="E11" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F11">
         <v>116</v>
       </c>
       <c r="G11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K11" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M11">
         <v>2000</v>
@@ -1373,7 +1346,7 @@
         <v>100</v>
       </c>
       <c r="O11" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="P11" t="s">
         <v>25</v>
@@ -1387,37 +1360,37 @@
         <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D12">
         <v>224</v>
       </c>
       <c r="E12" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F12">
         <v>224</v>
       </c>
       <c r="G12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K12" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M12">
         <v>16000</v>
@@ -1426,7 +1399,7 @@
         <v>100</v>
       </c>
       <c r="O12" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="P12" t="s">
         <v>25</v>
@@ -1440,37 +1413,37 @@
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D13">
         <v>223.4</v>
       </c>
       <c r="E13" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F13">
         <v>223.4</v>
       </c>
       <c r="G13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M13">
         <v>10000</v>
@@ -1482,7 +1455,7 @@
         <v>29</v>
       </c>
       <c r="P13" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="Q13">
         <v>1675500</v>
@@ -1493,37 +1466,37 @@
         <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D14">
         <v>297</v>
       </c>
       <c r="E14" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F14">
         <v>297</v>
       </c>
       <c r="G14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K14" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M14">
         <v>22000</v>
@@ -1532,7 +1505,7 @@
         <v>100</v>
       </c>
       <c r="O14" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="P14" t="s">
         <v>29</v>
@@ -1546,37 +1519,37 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D15">
         <v>2660</v>
       </c>
       <c r="E15" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F15">
         <v>2553.6</v>
       </c>
       <c r="G15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K15" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M15">
         <v>35000</v>
@@ -1585,10 +1558,10 @@
         <v>96</v>
       </c>
       <c r="O15" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="P15" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="Q15">
         <v>9340690</v>
@@ -1599,37 +1572,37 @@
         <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D16">
         <v>2660</v>
       </c>
       <c r="E16" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F16">
         <v>106.4</v>
       </c>
       <c r="G16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K16" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="L16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M16">
         <v>35000</v>
@@ -1638,10 +1611,10 @@
         <v>4</v>
       </c>
       <c r="O16" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="P16" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="Q16">
         <v>9340690</v>
@@ -1652,37 +1625,37 @@
         <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D17">
         <v>120</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F17">
         <v>120</v>
       </c>
       <c r="G17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K17" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M17">
         <v>2000</v>
@@ -1691,10 +1664,10 @@
         <v>100</v>
       </c>
       <c r="O17" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="P17" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="Q17">
         <v>4500000</v>
@@ -1705,37 +1678,37 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C18" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D18">
         <v>80</v>
       </c>
       <c r="E18" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F18">
         <v>80</v>
       </c>
       <c r="G18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K18" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M18">
         <v>2000</v>
@@ -1747,7 +1720,7 @@
         <v>30</v>
       </c>
       <c r="P18" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="Q18">
         <v>3000000</v>
@@ -1758,37 +1731,37 @@
         <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D19">
         <v>161.8</v>
       </c>
       <c r="E19" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F19">
         <v>161.8</v>
       </c>
       <c r="G19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K19" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M19">
         <v>10000</v>
@@ -1800,7 +1773,7 @@
         <v>33</v>
       </c>
       <c r="P19" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="Q19">
         <v>1187900</v>
@@ -1811,37 +1784,37 @@
         <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C20" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D20">
         <v>4350</v>
       </c>
       <c r="E20" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F20">
         <v>1435.5</v>
       </c>
       <c r="G20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K20" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M20">
         <v>60000</v>
@@ -1850,10 +1823,10 @@
         <v>33</v>
       </c>
       <c r="O20" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="P20" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="Q20">
         <v>21750000</v>
@@ -1864,37 +1837,37 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C21" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D21">
         <v>4350</v>
       </c>
       <c r="E21" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F21">
         <v>1435.5</v>
       </c>
       <c r="G21" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H21" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I21" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J21" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K21" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L21" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M21">
         <v>60000</v>
@@ -1903,10 +1876,10 @@
         <v>33</v>
       </c>
       <c r="O21" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="P21" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="Q21">
         <v>21750000</v>
@@ -1917,37 +1890,37 @@
         <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C22" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D22">
         <v>4350</v>
       </c>
       <c r="E22" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F22">
         <v>1305</v>
       </c>
       <c r="G22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K22" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M22">
         <v>60000</v>
@@ -1956,10 +1929,10 @@
         <v>30</v>
       </c>
       <c r="O22" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="P22" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="Q22">
         <v>21750000</v>
@@ -1970,37 +1943,37 @@
         <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C23" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D23">
         <v>4350</v>
       </c>
       <c r="E23" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F23">
         <v>174</v>
       </c>
       <c r="G23" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H23" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I23" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J23" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K23" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="L23" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M23">
         <v>60000</v>
@@ -2009,10 +1982,10 @@
         <v>4</v>
       </c>
       <c r="O23" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="P23" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="Q23">
         <v>21750000</v>
@@ -2023,37 +1996,37 @@
         <v>32</v>
       </c>
       <c r="B24" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" t="s">
         <v>53</v>
-      </c>
-      <c r="C24" t="s">
-        <v>57</v>
       </c>
       <c r="D24">
         <v>80</v>
       </c>
       <c r="E24" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F24">
         <v>80</v>
       </c>
       <c r="G24" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H24" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I24" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J24" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K24" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L24" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M24">
         <v>2000</v>
@@ -2062,10 +2035,10 @@
         <v>100</v>
       </c>
       <c r="O24" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="P24" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="Q24">
         <v>3000000</v>
@@ -2076,37 +2049,37 @@
         <v>33</v>
       </c>
       <c r="B25" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C25" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D25">
         <v>289.6</v>
       </c>
       <c r="E25" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F25">
         <v>289.6</v>
       </c>
       <c r="G25" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H25" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I25" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J25" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K25" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L25" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M25">
         <v>16000</v>
@@ -2115,172 +2088,13 @@
         <v>100</v>
       </c>
       <c r="O25" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="P25" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="Q25">
         <v>1357500</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17">
-      <c r="A26" t="s">
-        <v>34</v>
-      </c>
-      <c r="B26" t="s">
-        <v>55</v>
-      </c>
-      <c r="C26" t="s">
-        <v>57</v>
-      </c>
-      <c r="D26">
-        <v>575.89</v>
-      </c>
-      <c r="E26" t="s">
-        <v>64</v>
-      </c>
-      <c r="F26">
-        <v>541.3366</v>
-      </c>
-      <c r="G26" t="s">
-        <v>73</v>
-      </c>
-      <c r="H26" t="s">
-        <v>73</v>
-      </c>
-      <c r="I26" t="s">
-        <v>73</v>
-      </c>
-      <c r="J26" t="s">
-        <v>73</v>
-      </c>
-      <c r="K26" t="s">
-        <v>74</v>
-      </c>
-      <c r="L26" t="s">
-        <v>73</v>
-      </c>
-      <c r="M26">
-        <v>43300</v>
-      </c>
-      <c r="N26">
-        <v>94</v>
-      </c>
-      <c r="O26" t="s">
-        <v>84</v>
-      </c>
-      <c r="P26" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q26">
-        <v>1906400</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17">
-      <c r="A27" t="s">
-        <v>34</v>
-      </c>
-      <c r="B27" t="s">
-        <v>55</v>
-      </c>
-      <c r="C27" t="s">
-        <v>57</v>
-      </c>
-      <c r="D27">
-        <v>575.89</v>
-      </c>
-      <c r="E27" t="s">
-        <v>71</v>
-      </c>
-      <c r="F27">
-        <v>34.5534</v>
-      </c>
-      <c r="G27" t="s">
-        <v>73</v>
-      </c>
-      <c r="H27" t="s">
-        <v>73</v>
-      </c>
-      <c r="I27" t="s">
-        <v>73</v>
-      </c>
-      <c r="J27" t="s">
-        <v>73</v>
-      </c>
-      <c r="K27" t="s">
-        <v>75</v>
-      </c>
-      <c r="L27" t="s">
-        <v>73</v>
-      </c>
-      <c r="M27">
-        <v>43300</v>
-      </c>
-      <c r="N27">
-        <v>6</v>
-      </c>
-      <c r="O27" t="s">
-        <v>84</v>
-      </c>
-      <c r="P27" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q27">
-        <v>1906400</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17">
-      <c r="A28" t="s">
-        <v>35</v>
-      </c>
-      <c r="B28" t="s">
-        <v>56</v>
-      </c>
-      <c r="C28" t="s">
-        <v>57</v>
-      </c>
-      <c r="D28">
-        <v>432</v>
-      </c>
-      <c r="E28" t="s">
-        <v>61</v>
-      </c>
-      <c r="F28">
-        <v>432</v>
-      </c>
-      <c r="G28" t="s">
-        <v>73</v>
-      </c>
-      <c r="H28" t="s">
-        <v>73</v>
-      </c>
-      <c r="I28" t="s">
-        <v>73</v>
-      </c>
-      <c r="J28" t="s">
-        <v>73</v>
-      </c>
-      <c r="K28" t="s">
-        <v>74</v>
-      </c>
-      <c r="L28" t="s">
-        <v>73</v>
-      </c>
-      <c r="M28">
-        <v>18000</v>
-      </c>
-      <c r="N28">
-        <v>100</v>
-      </c>
-      <c r="O28" t="s">
-        <v>85</v>
-      </c>
-      <c r="P28" t="s">
-        <v>83</v>
-      </c>
-      <c r="Q28">
-        <v>1758600</v>
       </c>
     </row>
   </sheetData>
@@ -2290,7 +2104,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T22"/>
+  <dimension ref="A1:T20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -2298,10 +2112,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -2310,49 +2124,49 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:20">
@@ -2360,10 +2174,10 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D2" t="s">
         <v>22</v>
@@ -2378,7 +2192,7 @@
         <v>1500000</v>
       </c>
       <c r="H2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I2">
         <v>11000</v>
@@ -2387,34 +2201,34 @@
         <v>13000</v>
       </c>
       <c r="K2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L2">
         <v>16000</v>
       </c>
       <c r="M2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="S2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -2422,10 +2236,10 @@
         <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D3" t="s">
         <v>22</v>
@@ -2440,7 +2254,7 @@
         <v>1566800</v>
       </c>
       <c r="H3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I3">
         <v>13600</v>
@@ -2449,48 +2263,48 @@
         <v>15300</v>
       </c>
       <c r="K3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L3">
         <v>15300</v>
       </c>
       <c r="M3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R3" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="S3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E4" t="s">
         <v>19</v>
@@ -2502,7 +2316,7 @@
         <v>1000000</v>
       </c>
       <c r="H4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I4">
         <v>9500</v>
@@ -2511,48 +2325,48 @@
         <v>10700</v>
       </c>
       <c r="K4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L4">
         <v>13000</v>
       </c>
       <c r="M4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O4">
         <v>50</v>
       </c>
       <c r="P4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R4" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="S4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E5" t="s">
         <v>17</v>
@@ -2564,7 +2378,7 @@
         <v>6500000</v>
       </c>
       <c r="H5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I5">
         <v>2000</v>
@@ -2573,45 +2387,45 @@
         <v>2000</v>
       </c>
       <c r="K5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L5">
         <v>2000</v>
       </c>
       <c r="M5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R5" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="S5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D6" t="s">
         <v>23</v>
@@ -2626,7 +2440,7 @@
         <v>3077650</v>
       </c>
       <c r="H6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I6">
         <v>13800</v>
@@ -2635,45 +2449,45 @@
         <v>15700</v>
       </c>
       <c r="K6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L6">
         <v>16500</v>
       </c>
       <c r="M6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O6">
         <v>100</v>
       </c>
       <c r="P6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R6" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="S6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
         <v>23</v>
@@ -2688,7 +2502,7 @@
         <v>1400000</v>
       </c>
       <c r="H7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I7">
         <v>12500</v>
@@ -2697,45 +2511,45 @@
         <v>15500</v>
       </c>
       <c r="K7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L7">
         <v>15500</v>
       </c>
       <c r="M7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R7" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="S7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D8" t="s">
         <v>24</v>
@@ -2750,7 +2564,7 @@
         <v>1000000</v>
       </c>
       <c r="H8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I8">
         <v>24000</v>
@@ -2759,34 +2573,34 @@
         <v>29000</v>
       </c>
       <c r="K8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L8">
         <v>29000</v>
       </c>
       <c r="M8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R8" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="S8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -2794,13 +2608,13 @@
         <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D9" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E9" t="s">
         <v>22</v>
@@ -2812,7 +2626,7 @@
         <v>751000</v>
       </c>
       <c r="H9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I9">
         <v>18000</v>
@@ -2821,45 +2635,45 @@
         <v>21000</v>
       </c>
       <c r="K9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L9">
         <v>21000</v>
       </c>
       <c r="M9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O9">
         <v>72.87616511318242</v>
       </c>
       <c r="P9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R9" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="S9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D10" t="s">
         <v>25</v>
@@ -2874,7 +2688,7 @@
         <v>5800000</v>
       </c>
       <c r="H10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I10">
         <v>2000</v>
@@ -2883,45 +2697,45 @@
         <v>2000</v>
       </c>
       <c r="K10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L10">
         <v>2000</v>
       </c>
       <c r="M10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O10">
         <v>0</v>
       </c>
       <c r="P10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R10" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="S10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D11" t="s">
         <v>25</v>
@@ -2936,7 +2750,7 @@
         <v>1400000</v>
       </c>
       <c r="H11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I11">
         <v>16000</v>
@@ -2945,34 +2759,34 @@
         <v>19000</v>
       </c>
       <c r="K11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L11">
         <v>16000</v>
       </c>
       <c r="M11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O11">
         <v>0</v>
       </c>
       <c r="P11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R11" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="S11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -2980,13 +2794,13 @@
         <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D12" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E12" t="s">
         <v>25</v>
@@ -2998,7 +2812,7 @@
         <v>2234000</v>
       </c>
       <c r="H12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I12">
         <v>7300</v>
@@ -3007,45 +2821,45 @@
         <v>8500</v>
       </c>
       <c r="K12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L12">
         <v>10000</v>
       </c>
       <c r="M12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O12">
         <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R12" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="S12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D13" t="s">
         <v>29</v>
@@ -3060,7 +2874,7 @@
         <v>1350000</v>
       </c>
       <c r="H13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I13">
         <v>14000</v>
@@ -3069,48 +2883,48 @@
         <v>17000</v>
       </c>
       <c r="K13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L13">
         <v>22000</v>
       </c>
       <c r="M13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O13">
         <v>0</v>
       </c>
       <c r="P13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R13" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="S13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C14" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="E14" t="s">
         <v>27</v>
@@ -3122,7 +2936,7 @@
         <v>7600000</v>
       </c>
       <c r="H14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I14">
         <v>24000</v>
@@ -3131,48 +2945,48 @@
         <v>30000</v>
       </c>
       <c r="K14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L14">
         <v>35000</v>
       </c>
       <c r="M14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O14">
         <v>14.47368421052632</v>
       </c>
       <c r="P14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R14" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="S14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D15" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E15" t="s">
         <v>28</v>
@@ -3184,7 +2998,7 @@
         <v>6000000</v>
       </c>
       <c r="H15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I15">
         <v>2000</v>
@@ -3193,34 +3007,34 @@
         <v>2000</v>
       </c>
       <c r="K15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L15">
         <v>2000</v>
       </c>
       <c r="M15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O15">
         <v>0</v>
       </c>
       <c r="P15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R15" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="S15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -3228,13 +3042,13 @@
         <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C16" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D16" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
@@ -3246,7 +3060,7 @@
         <v>4000000</v>
       </c>
       <c r="H16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I16">
         <v>2000</v>
@@ -3255,34 +3069,34 @@
         <v>2000</v>
       </c>
       <c r="K16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L16">
         <v>2000</v>
       </c>
       <c r="M16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O16">
         <v>0</v>
       </c>
       <c r="P16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R16" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="S16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:20">
@@ -3290,13 +3104,13 @@
         <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D17" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E17" t="s">
         <v>30</v>
@@ -3308,7 +3122,7 @@
         <v>1618000</v>
       </c>
       <c r="H17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I17">
         <v>6200</v>
@@ -3317,48 +3131,48 @@
         <v>7700</v>
       </c>
       <c r="K17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L17">
         <v>10000</v>
       </c>
       <c r="M17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O17">
         <v>0</v>
       </c>
       <c r="P17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R17" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="S17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:20">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="B18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C18" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D18" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E18" t="s">
         <v>31</v>
@@ -3370,7 +3184,7 @@
         <v>7250000</v>
       </c>
       <c r="H18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I18">
         <v>47000</v>
@@ -3379,48 +3193,48 @@
         <v>60000</v>
       </c>
       <c r="K18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L18">
         <v>60000</v>
       </c>
       <c r="M18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O18">
         <v>0</v>
       </c>
       <c r="P18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R18" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="S18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:20">
       <c r="A19" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C19" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="D19" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E19" t="s">
         <v>32</v>
@@ -3432,7 +3246,7 @@
         <v>4000000</v>
       </c>
       <c r="H19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I19">
         <v>2000</v>
@@ -3441,48 +3255,48 @@
         <v>2000</v>
       </c>
       <c r="K19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L19">
         <v>2000</v>
       </c>
       <c r="M19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O19">
         <v>0</v>
       </c>
       <c r="P19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R19" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="S19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:20">
       <c r="A20" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D20" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E20" t="s">
         <v>33</v>
@@ -3494,7 +3308,7 @@
         <v>1810000</v>
       </c>
       <c r="H20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I20">
         <v>9000</v>
@@ -3503,158 +3317,34 @@
         <v>12000</v>
       </c>
       <c r="K20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L20">
         <v>16000</v>
       </c>
       <c r="M20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="O20">
         <v>0</v>
       </c>
       <c r="P20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="R20" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="S20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T20" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20">
-      <c r="A21" t="s">
-        <v>84</v>
-      </c>
-      <c r="B21" t="s">
-        <v>55</v>
-      </c>
-      <c r="C21" t="s">
-        <v>64</v>
-      </c>
-      <c r="D21" t="s">
-        <v>93</v>
-      </c>
-      <c r="E21" t="s">
-        <v>34</v>
-      </c>
-      <c r="F21">
-        <v>57589000</v>
-      </c>
-      <c r="G21">
-        <v>1330000</v>
-      </c>
-      <c r="H21" t="s">
-        <v>73</v>
-      </c>
-      <c r="I21">
-        <v>36400</v>
-      </c>
-      <c r="J21">
-        <v>43300</v>
-      </c>
-      <c r="K21" t="s">
-        <v>73</v>
-      </c>
-      <c r="L21">
-        <v>43300</v>
-      </c>
-      <c r="M21" t="s">
-        <v>73</v>
-      </c>
-      <c r="N21" t="s">
-        <v>73</v>
-      </c>
-      <c r="O21">
-        <v>0</v>
-      </c>
-      <c r="P21" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>73</v>
-      </c>
-      <c r="R21" t="s">
-        <v>132</v>
-      </c>
-      <c r="S21" t="s">
-        <v>73</v>
-      </c>
-      <c r="T21" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="22" spans="1:20">
-      <c r="A22" t="s">
-        <v>85</v>
-      </c>
-      <c r="B22" t="s">
-        <v>56</v>
-      </c>
-      <c r="C22" t="s">
-        <v>61</v>
-      </c>
-      <c r="D22" t="s">
-        <v>83</v>
-      </c>
-      <c r="E22" t="s">
-        <v>35</v>
-      </c>
-      <c r="F22">
-        <v>43200000</v>
-      </c>
-      <c r="G22">
-        <v>2400000</v>
-      </c>
-      <c r="H22" t="s">
-        <v>73</v>
-      </c>
-      <c r="I22">
-        <v>11000</v>
-      </c>
-      <c r="J22">
-        <v>14200</v>
-      </c>
-      <c r="K22" t="s">
-        <v>73</v>
-      </c>
-      <c r="L22">
-        <v>18000</v>
-      </c>
-      <c r="M22" t="s">
-        <v>73</v>
-      </c>
-      <c r="N22" t="s">
-        <v>73</v>
-      </c>
-      <c r="O22">
-        <v>0</v>
-      </c>
-      <c r="P22" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q22" t="s">
-        <v>73</v>
-      </c>
-      <c r="R22" t="s">
-        <v>133</v>
-      </c>
-      <c r="S22" t="s">
-        <v>73</v>
-      </c>
-      <c r="T22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -3664,21 +3354,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -3690,10 +3380,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -3702,27 +3392,27 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="E2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="F2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="G2" t="s">
         <v>32</v>
@@ -3745,57 +3435,57 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C3" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>105</v>
       </c>
       <c r="E3" t="s">
-        <v>61</v>
+        <v>129</v>
       </c>
       <c r="F3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="G3" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H3">
-        <v>43200</v>
+        <v>130500</v>
       </c>
       <c r="I3">
-        <v>2400000</v>
+        <v>7250000</v>
       </c>
       <c r="J3">
-        <v>18000</v>
+        <v>60000</v>
       </c>
       <c r="K3">
         <v>0</v>
       </c>
       <c r="L3">
-        <v>100</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
         <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F4" t="s">
         <v>22</v>
@@ -3821,69 +3511,69 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D5" t="s">
-        <v>111</v>
+        <v>57</v>
       </c>
       <c r="E5" t="s">
-        <v>137</v>
+        <v>57</v>
       </c>
       <c r="F5" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="G5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H5">
-        <v>130500</v>
+        <v>12000</v>
       </c>
       <c r="I5">
-        <v>7250000</v>
+        <v>6000000</v>
       </c>
       <c r="J5">
-        <v>60000</v>
+        <v>2000</v>
       </c>
       <c r="K5">
         <v>0</v>
       </c>
       <c r="L5">
-        <v>30</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D6" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E6" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F6" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="G6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H6">
-        <v>12000</v>
+        <v>8000</v>
       </c>
       <c r="I6">
-        <v>6000000</v>
+        <v>4000000</v>
       </c>
       <c r="J6">
         <v>2000</v>
@@ -3897,31 +3587,31 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="C7" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="E7" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="F7" t="s">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="G7" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="H7">
-        <v>8000</v>
+        <v>11600</v>
       </c>
       <c r="I7">
-        <v>4000000</v>
+        <v>5800000</v>
       </c>
       <c r="J7">
         <v>2000</v>
@@ -3935,34 +3625,34 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B8" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="E8" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="F8" t="s">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="G8" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H8">
-        <v>11600</v>
+        <v>16180</v>
       </c>
       <c r="I8">
-        <v>5800000</v>
+        <v>1618000</v>
       </c>
       <c r="J8">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -3973,22 +3663,22 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F9" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="G9" t="s">
         <v>17</v>
@@ -4011,34 +3701,34 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>73</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="D10" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E10" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F10" t="s">
-        <v>90</v>
+        <v>23</v>
       </c>
       <c r="G10" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H10">
-        <v>16180</v>
+        <v>50781.225</v>
       </c>
       <c r="I10">
-        <v>1618000</v>
+        <v>3077650</v>
       </c>
       <c r="J10">
-        <v>10000</v>
+        <v>16500</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -4049,60 +3739,60 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B11" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E11" t="s">
-        <v>138</v>
+        <v>60</v>
       </c>
       <c r="F11" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="G11" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="H11">
-        <v>54133.66</v>
+        <v>22400</v>
       </c>
       <c r="I11">
-        <v>1330000</v>
+        <v>1400000</v>
       </c>
       <c r="J11">
-        <v>43300</v>
+        <v>16000</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B12" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E12" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="F12" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="G12" t="s">
         <v>27</v>
@@ -4128,10 +3818,10 @@
         <v>64</v>
       </c>
       <c r="B13" t="s">
-        <v>77</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D13" t="s">
         <v>64</v>
@@ -4140,19 +3830,19 @@
         <v>64</v>
       </c>
       <c r="F13" t="s">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="G13" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H13">
-        <v>50781.225</v>
+        <v>22340</v>
       </c>
       <c r="I13">
-        <v>3077650</v>
+        <v>2234000</v>
       </c>
       <c r="J13">
-        <v>16500</v>
+        <v>10000</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -4166,69 +3856,69 @@
         <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E14" t="s">
-        <v>64</v>
+        <v>130</v>
       </c>
       <c r="F14" t="s">
-        <v>25</v>
+        <v>83</v>
       </c>
       <c r="G14" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="H14">
-        <v>22400</v>
+        <v>10640</v>
       </c>
       <c r="I14">
-        <v>1400000</v>
+        <v>7600000</v>
       </c>
       <c r="J14">
-        <v>16000</v>
+        <v>35000</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="C15" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="D15" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E15" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F15" t="s">
         <v>87</v>
       </c>
       <c r="G15" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="H15">
-        <v>22340</v>
+        <v>28960</v>
       </c>
       <c r="I15">
-        <v>2234000</v>
+        <v>1810000</v>
       </c>
       <c r="J15">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="K15">
         <v>0</v>
@@ -4239,95 +3929,95 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="B16" t="s">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="C16" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="D16" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="E16" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="F16" t="s">
-        <v>88</v>
+        <v>22</v>
       </c>
       <c r="G16" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="H16">
-        <v>10640</v>
+        <v>22800</v>
       </c>
       <c r="I16">
-        <v>7600000</v>
+        <v>1500000</v>
       </c>
       <c r="J16">
-        <v>35000</v>
+        <v>16000</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16">
-        <v>4</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B17" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C17" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D17" t="s">
-        <v>68</v>
+        <v>105</v>
       </c>
       <c r="E17" t="s">
-        <v>68</v>
+        <v>129</v>
       </c>
       <c r="F17" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="G17" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="H17">
-        <v>28960</v>
+        <v>17400</v>
       </c>
       <c r="I17">
-        <v>1810000</v>
+        <v>7250000</v>
       </c>
       <c r="J17">
-        <v>16000</v>
+        <v>60000</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
       <c r="L17">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B18" t="s">
         <v>24</v>
       </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E18" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="F18" t="s">
         <v>22</v>
@@ -4336,7 +4026,7 @@
         <v>17</v>
       </c>
       <c r="H18">
-        <v>22800</v>
+        <v>1200</v>
       </c>
       <c r="I18">
         <v>1500000</v>
@@ -4348,191 +4038,191 @@
         <v>0</v>
       </c>
       <c r="L18">
-        <v>95</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B19" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C19" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D19" t="s">
-        <v>64</v>
+        <v>105</v>
       </c>
       <c r="E19" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="F19" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="G19" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H19">
-        <v>3455.34</v>
+        <v>143550</v>
       </c>
       <c r="I19">
-        <v>1330000</v>
+        <v>7250000</v>
       </c>
       <c r="J19">
-        <v>43300</v>
+        <v>60000</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="B20" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="D20" t="s">
-        <v>111</v>
+        <v>62</v>
       </c>
       <c r="E20" t="s">
-        <v>137</v>
+        <v>62</v>
       </c>
       <c r="F20" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="G20" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="H20">
-        <v>17400</v>
+        <v>15771</v>
       </c>
       <c r="I20">
-        <v>7250000</v>
+        <v>751000</v>
       </c>
       <c r="J20">
-        <v>60000</v>
+        <v>21000</v>
       </c>
       <c r="K20">
         <v>0</v>
       </c>
       <c r="L20">
-        <v>4</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" spans="1:12">
       <c r="A21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="C21" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="D21" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E21" t="s">
-        <v>140</v>
+        <v>62</v>
       </c>
       <c r="F21" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="G21" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="H21">
-        <v>1200</v>
+        <v>29700</v>
       </c>
       <c r="I21">
-        <v>1500000</v>
+        <v>1350000</v>
       </c>
       <c r="J21">
-        <v>16000</v>
+        <v>22000</v>
       </c>
       <c r="K21">
         <v>0</v>
       </c>
       <c r="L21">
-        <v>5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:12">
       <c r="A22" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="B22" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="C22" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="D22" t="s">
-        <v>111</v>
+        <v>61</v>
       </c>
       <c r="E22" t="s">
-        <v>137</v>
+        <v>61</v>
       </c>
       <c r="F22" t="s">
-        <v>91</v>
+        <v>23</v>
       </c>
       <c r="G22" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H22">
-        <v>143550</v>
+        <v>21700</v>
       </c>
       <c r="I22">
-        <v>7250000</v>
+        <v>1400000</v>
       </c>
       <c r="J22">
-        <v>60000</v>
+        <v>15500</v>
       </c>
       <c r="K22">
         <v>0</v>
       </c>
       <c r="L22">
-        <v>33</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:12">
       <c r="A23" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B23" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C23" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="D23" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="E23" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="F23" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="G23" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="H23">
-        <v>29700</v>
+        <v>29000</v>
       </c>
       <c r="I23">
-        <v>1350000</v>
+        <v>1000000</v>
       </c>
       <c r="J23">
-        <v>22000</v>
+        <v>29000</v>
       </c>
       <c r="K23">
         <v>0</v>
@@ -4543,34 +4233,34 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B24" t="s">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="C24" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D24" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="E24" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="F24" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G24" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H24">
-        <v>15771</v>
+        <v>13000</v>
       </c>
       <c r="I24">
-        <v>751000</v>
+        <v>1000000</v>
       </c>
       <c r="J24">
-        <v>21000</v>
+        <v>13000</v>
       </c>
       <c r="K24">
         <v>0</v>
@@ -4581,154 +4271,40 @@
     </row>
     <row r="25" spans="1:12">
       <c r="A25" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="B25" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C25" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="D25" t="s">
-        <v>65</v>
+        <v>105</v>
       </c>
       <c r="E25" t="s">
-        <v>65</v>
+        <v>129</v>
       </c>
       <c r="F25" t="s">
-        <v>23</v>
+        <v>86</v>
       </c>
       <c r="G25" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="H25">
-        <v>21700</v>
+        <v>143550</v>
       </c>
       <c r="I25">
-        <v>1400000</v>
+        <v>7250000</v>
       </c>
       <c r="J25">
-        <v>15500</v>
+        <v>60000</v>
       </c>
       <c r="K25">
         <v>0</v>
       </c>
       <c r="L25">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12">
-      <c r="A26" t="s">
-        <v>62</v>
-      </c>
-      <c r="B26" t="s">
-        <v>78</v>
-      </c>
-      <c r="C26" t="s">
-        <v>42</v>
-      </c>
-      <c r="D26" t="s">
-        <v>62</v>
-      </c>
-      <c r="E26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F26" t="s">
-        <v>24</v>
-      </c>
-      <c r="G26" t="s">
-        <v>21</v>
-      </c>
-      <c r="H26">
-        <v>29000</v>
-      </c>
-      <c r="I26">
-        <v>1000000</v>
-      </c>
-      <c r="J26">
-        <v>29000</v>
-      </c>
-      <c r="K26">
-        <v>0</v>
-      </c>
-      <c r="L26">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12">
-      <c r="A27" t="s">
-        <v>62</v>
-      </c>
-      <c r="B27" t="s">
-        <v>34</v>
-      </c>
-      <c r="C27" t="s">
-        <v>52</v>
-      </c>
-      <c r="D27" t="s">
-        <v>111</v>
-      </c>
-      <c r="E27" t="s">
-        <v>137</v>
-      </c>
-      <c r="F27" t="s">
-        <v>91</v>
-      </c>
-      <c r="G27" t="s">
-        <v>31</v>
-      </c>
-      <c r="H27">
-        <v>143550</v>
-      </c>
-      <c r="I27">
-        <v>7250000</v>
-      </c>
-      <c r="J27">
-        <v>60000</v>
-      </c>
-      <c r="K27">
-        <v>0</v>
-      </c>
-      <c r="L27">
         <v>33</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12">
-      <c r="A28" t="s">
-        <v>62</v>
-      </c>
-      <c r="B28" t="s">
-        <v>76</v>
-      </c>
-      <c r="C28" t="s">
-        <v>38</v>
-      </c>
-      <c r="D28" t="s">
-        <v>62</v>
-      </c>
-      <c r="E28" t="s">
-        <v>62</v>
-      </c>
-      <c r="F28" t="s">
-        <v>86</v>
-      </c>
-      <c r="G28" t="s">
-        <v>19</v>
-      </c>
-      <c r="H28">
-        <v>13000</v>
-      </c>
-      <c r="I28">
-        <v>1000000</v>
-      </c>
-      <c r="J28">
-        <v>13000</v>
-      </c>
-      <c r="K28">
-        <v>0</v>
-      </c>
-      <c r="L28">
-        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-08-27
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="128">
   <si>
     <t>상장일</t>
   </si>
@@ -117,150 +117,144 @@
     <t>2024-07-12</t>
   </si>
   <si>
+    <t>M83</t>
+  </si>
+  <si>
+    <t>이엔셀</t>
+  </si>
+  <si>
+    <t>티디에스팜</t>
+  </si>
+  <si>
+    <t>대신밸런스제18호스팩</t>
+  </si>
+  <si>
+    <t>전진건설로봇</t>
+  </si>
+  <si>
+    <t>케이쓰리아이</t>
+  </si>
+  <si>
+    <t>넥스트바이오메디컬</t>
+  </si>
+  <si>
+    <t>유라클</t>
+  </si>
+  <si>
+    <t>교보16호스팩</t>
+  </si>
+  <si>
+    <t>뱅크웨어글로벌</t>
+  </si>
+  <si>
+    <t>아이빔테크놀로지</t>
+  </si>
+  <si>
+    <t>피앤에스미캐닉스</t>
+  </si>
+  <si>
+    <t>산일전기</t>
+  </si>
+  <si>
+    <t>엔에이치스팩31호</t>
+  </si>
+  <si>
+    <t>SK증권제13호스팩</t>
+  </si>
+  <si>
+    <t>엑셀세라퓨틱스</t>
+  </si>
+  <si>
+    <t>시프트업</t>
+  </si>
+  <si>
+    <t>이베스트스팩6호</t>
+  </si>
+  <si>
+    <t>코스닥</t>
+  </si>
+  <si>
+    <t>코스피</t>
+  </si>
+  <si>
+    <t>신영</t>
+  </si>
+  <si>
+    <t>유진</t>
+  </si>
+  <si>
+    <t>NH</t>
+  </si>
+  <si>
+    <t>한국</t>
+  </si>
+  <si>
+    <t>대신</t>
+  </si>
+  <si>
+    <t>미래</t>
+  </si>
+  <si>
+    <t>하나</t>
+  </si>
+  <si>
+    <t>키움</t>
+  </si>
+  <si>
+    <t>교보</t>
+  </si>
+  <si>
+    <t>삼성</t>
+  </si>
+  <si>
+    <t>SK</t>
+  </si>
+  <si>
+    <t>제이피모간회사</t>
+  </si>
+  <si>
+    <t>신한</t>
+  </si>
+  <si>
+    <t>LS</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>대표</t>
+  </si>
+  <si>
+    <t>인수</t>
+  </si>
+  <si>
+    <t>2024-08-09</t>
+  </si>
+  <si>
+    <t>2024-08-08</t>
+  </si>
+  <si>
+    <t>2024-08-07</t>
+  </si>
+  <si>
+    <t>2024-08-01</t>
+  </si>
+  <si>
+    <t>2024-07-22</t>
+  </si>
+  <si>
+    <t>2024-07-18</t>
+  </si>
+  <si>
+    <t>2024-07-16</t>
+  </si>
+  <si>
     <t>2024-07-03</t>
   </si>
   <si>
-    <t>M83</t>
-  </si>
-  <si>
-    <t>이엔셀</t>
-  </si>
-  <si>
-    <t>티디에스팜</t>
-  </si>
-  <si>
-    <t>대신밸런스제18호스팩</t>
-  </si>
-  <si>
-    <t>전진건설로봇</t>
-  </si>
-  <si>
-    <t>케이쓰리아이</t>
-  </si>
-  <si>
-    <t>넥스트바이오메디컬</t>
-  </si>
-  <si>
-    <t>유라클</t>
-  </si>
-  <si>
-    <t>교보16호스팩</t>
-  </si>
-  <si>
-    <t>뱅크웨어글로벌</t>
-  </si>
-  <si>
-    <t>아이빔테크놀로지</t>
-  </si>
-  <si>
-    <t>피앤에스미캐닉스</t>
-  </si>
-  <si>
-    <t>산일전기</t>
-  </si>
-  <si>
-    <t>엔에이치스팩31호</t>
-  </si>
-  <si>
-    <t>SK증권제13호스팩</t>
-  </si>
-  <si>
-    <t>엑셀세라퓨틱스</t>
-  </si>
-  <si>
-    <t>시프트업</t>
-  </si>
-  <si>
-    <t>이베스트스팩6호</t>
-  </si>
-  <si>
-    <t>하스</t>
-  </si>
-  <si>
-    <t>코스닥</t>
-  </si>
-  <si>
-    <t>코스피</t>
-  </si>
-  <si>
-    <t>신영</t>
-  </si>
-  <si>
-    <t>유진</t>
-  </si>
-  <si>
-    <t>NH</t>
-  </si>
-  <si>
-    <t>한국</t>
-  </si>
-  <si>
-    <t>대신</t>
-  </si>
-  <si>
-    <t>미래</t>
-  </si>
-  <si>
-    <t>하나</t>
-  </si>
-  <si>
-    <t>키움</t>
-  </si>
-  <si>
-    <t>교보</t>
-  </si>
-  <si>
-    <t>삼성</t>
-  </si>
-  <si>
-    <t>SK</t>
-  </si>
-  <si>
-    <t>제이피모간회사</t>
-  </si>
-  <si>
-    <t>신한</t>
-  </si>
-  <si>
-    <t>LS</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>대표</t>
-  </si>
-  <si>
-    <t>인수</t>
-  </si>
-  <si>
-    <t>2024-08-09</t>
-  </si>
-  <si>
-    <t>2024-08-08</t>
-  </si>
-  <si>
-    <t>2024-08-07</t>
-  </si>
-  <si>
-    <t>2024-08-01</t>
-  </si>
-  <si>
-    <t>2024-07-22</t>
-  </si>
-  <si>
-    <t>2024-07-18</t>
-  </si>
-  <si>
-    <t>2024-07-16</t>
-  </si>
-  <si>
     <t>2024-07-02</t>
   </si>
   <si>
-    <t>2024-06-24</t>
-  </si>
-  <si>
     <t>2024-08-14</t>
   </si>
   <si>
@@ -279,9 +273,6 @@
     <t>2024-07-05</t>
   </si>
   <si>
-    <t>2024-06-27</t>
-  </si>
-  <si>
     <t>회사명</t>
   </si>
   <si>
@@ -391,9 +382,6 @@
   </si>
   <si>
     <t>107.32 : 1</t>
-  </si>
-  <si>
-    <t>2126.46 : 1</t>
   </si>
   <si>
     <t>인수기관</t>
@@ -769,7 +757,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -830,37 +818,37 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D2">
         <v>240</v>
       </c>
       <c r="E2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F2">
         <v>228</v>
       </c>
       <c r="G2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M2">
         <v>16000</v>
@@ -883,37 +871,37 @@
         <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D3">
         <v>240</v>
       </c>
       <c r="E3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F3">
         <v>12</v>
       </c>
       <c r="G3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I3" t="s">
+        <v>67</v>
+      </c>
+      <c r="J3" t="s">
+        <v>67</v>
+      </c>
+      <c r="K3" t="s">
         <v>69</v>
       </c>
-      <c r="H3" t="s">
-        <v>69</v>
-      </c>
-      <c r="I3" t="s">
-        <v>69</v>
-      </c>
-      <c r="J3" t="s">
-        <v>69</v>
-      </c>
-      <c r="K3" t="s">
-        <v>71</v>
-      </c>
       <c r="L3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M3">
         <v>16000</v>
@@ -936,37 +924,37 @@
         <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D4">
         <v>239.7204</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F4">
         <v>239.7204</v>
       </c>
       <c r="G4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M4">
         <v>15300</v>
@@ -989,37 +977,37 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D5">
         <v>130</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F5">
         <v>130</v>
       </c>
       <c r="G5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M5">
         <v>13000</v>
@@ -1028,10 +1016,10 @@
         <v>100</v>
       </c>
       <c r="O5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="P5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="Q5">
         <v>723700</v>
@@ -1042,37 +1030,37 @@
         <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D6">
         <v>130</v>
       </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F6">
         <v>130</v>
       </c>
       <c r="G6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M6">
         <v>2000</v>
@@ -1081,10 +1069,10 @@
         <v>100</v>
       </c>
       <c r="O6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="P6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="Q6">
         <v>4875000</v>
@@ -1095,37 +1083,37 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D7">
         <v>507.81225</v>
       </c>
       <c r="E7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F7">
         <v>507.81225</v>
       </c>
       <c r="G7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M7">
         <v>16500</v>
@@ -1134,7 +1122,7 @@
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="P7" t="s">
         <v>23</v>
@@ -1148,37 +1136,37 @@
         <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D8">
         <v>217</v>
       </c>
       <c r="E8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F8">
         <v>217</v>
       </c>
       <c r="G8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M8">
         <v>15500</v>
@@ -1187,7 +1175,7 @@
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="P8" t="s">
         <v>23</v>
@@ -1201,37 +1189,37 @@
         <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D9">
         <v>290</v>
       </c>
       <c r="E9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F9">
         <v>290</v>
       </c>
       <c r="G9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M9">
         <v>29000</v>
@@ -1240,7 +1228,7 @@
         <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="P9" t="s">
         <v>24</v>
@@ -1254,37 +1242,37 @@
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D10">
         <v>157.71</v>
       </c>
       <c r="E10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F10">
         <v>157.71</v>
       </c>
       <c r="G10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M10">
         <v>21000</v>
@@ -1296,7 +1284,7 @@
         <v>25</v>
       </c>
       <c r="P10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="Q10">
         <v>540250</v>
@@ -1307,37 +1295,37 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D11">
         <v>116</v>
       </c>
       <c r="E11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F11">
         <v>116</v>
       </c>
       <c r="G11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K11" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M11">
         <v>2000</v>
@@ -1346,7 +1334,7 @@
         <v>100</v>
       </c>
       <c r="O11" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="P11" t="s">
         <v>25</v>
@@ -1360,37 +1348,37 @@
         <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D12">
         <v>224</v>
       </c>
       <c r="E12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F12">
         <v>224</v>
       </c>
       <c r="G12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M12">
         <v>16000</v>
@@ -1399,7 +1387,7 @@
         <v>100</v>
       </c>
       <c r="O12" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="P12" t="s">
         <v>25</v>
@@ -1413,37 +1401,37 @@
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D13">
         <v>223.4</v>
       </c>
       <c r="E13" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F13">
         <v>223.4</v>
       </c>
       <c r="G13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K13" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M13">
         <v>10000</v>
@@ -1455,7 +1443,7 @@
         <v>29</v>
       </c>
       <c r="P13" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q13">
         <v>1675500</v>
@@ -1466,37 +1454,37 @@
         <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D14">
         <v>297</v>
       </c>
       <c r="E14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F14">
         <v>297</v>
       </c>
       <c r="G14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M14">
         <v>22000</v>
@@ -1505,7 +1493,7 @@
         <v>100</v>
       </c>
       <c r="O14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="P14" t="s">
         <v>29</v>
@@ -1519,37 +1507,37 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D15">
         <v>2660</v>
       </c>
       <c r="E15" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F15">
         <v>2553.6</v>
       </c>
       <c r="G15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M15">
         <v>35000</v>
@@ -1558,10 +1546,10 @@
         <v>96</v>
       </c>
       <c r="O15" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="P15" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="Q15">
         <v>9340690</v>
@@ -1572,37 +1560,37 @@
         <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D16">
         <v>2660</v>
       </c>
       <c r="E16" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F16">
         <v>106.4</v>
       </c>
       <c r="G16" t="s">
+        <v>67</v>
+      </c>
+      <c r="H16" t="s">
+        <v>67</v>
+      </c>
+      <c r="I16" t="s">
+        <v>67</v>
+      </c>
+      <c r="J16" t="s">
+        <v>67</v>
+      </c>
+      <c r="K16" t="s">
         <v>69</v>
       </c>
-      <c r="H16" t="s">
-        <v>69</v>
-      </c>
-      <c r="I16" t="s">
-        <v>69</v>
-      </c>
-      <c r="J16" t="s">
-        <v>69</v>
-      </c>
-      <c r="K16" t="s">
-        <v>71</v>
-      </c>
       <c r="L16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M16">
         <v>35000</v>
@@ -1611,10 +1599,10 @@
         <v>4</v>
       </c>
       <c r="O16" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="P16" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="Q16">
         <v>9340690</v>
@@ -1625,37 +1613,37 @@
         <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C17" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D17">
         <v>120</v>
       </c>
       <c r="E17" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F17">
         <v>120</v>
       </c>
       <c r="G17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K17" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M17">
         <v>2000</v>
@@ -1664,10 +1652,10 @@
         <v>100</v>
       </c>
       <c r="O17" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="P17" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="Q17">
         <v>4500000</v>
@@ -1678,37 +1666,37 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D18">
         <v>80</v>
       </c>
       <c r="E18" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F18">
         <v>80</v>
       </c>
       <c r="G18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M18">
         <v>2000</v>
@@ -1720,7 +1708,7 @@
         <v>30</v>
       </c>
       <c r="P18" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="Q18">
         <v>3000000</v>
@@ -1731,37 +1719,37 @@
         <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D19">
         <v>161.8</v>
       </c>
       <c r="E19" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F19">
         <v>161.8</v>
       </c>
       <c r="G19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K19" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M19">
         <v>10000</v>
@@ -1770,10 +1758,10 @@
         <v>100</v>
       </c>
       <c r="O19" t="s">
-        <v>33</v>
+        <v>77</v>
       </c>
       <c r="P19" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="Q19">
         <v>1187900</v>
@@ -1784,37 +1772,37 @@
         <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D20">
         <v>4350</v>
       </c>
       <c r="E20" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F20">
         <v>1435.5</v>
       </c>
       <c r="G20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K20" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M20">
         <v>60000</v>
@@ -1823,10 +1811,10 @@
         <v>33</v>
       </c>
       <c r="O20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P20" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="Q20">
         <v>21750000</v>
@@ -1837,37 +1825,37 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C21" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D21">
         <v>4350</v>
       </c>
       <c r="E21" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F21">
         <v>1435.5</v>
       </c>
       <c r="G21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K21" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M21">
         <v>60000</v>
@@ -1876,10 +1864,10 @@
         <v>33</v>
       </c>
       <c r="O21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P21" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="Q21">
         <v>21750000</v>
@@ -1890,37 +1878,37 @@
         <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C22" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D22">
         <v>4350</v>
       </c>
       <c r="E22" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F22">
         <v>1305</v>
       </c>
       <c r="G22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K22" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M22">
         <v>60000</v>
@@ -1929,10 +1917,10 @@
         <v>30</v>
       </c>
       <c r="O22" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P22" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="Q22">
         <v>21750000</v>
@@ -1943,37 +1931,37 @@
         <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C23" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D23">
         <v>4350</v>
       </c>
       <c r="E23" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F23">
         <v>174</v>
       </c>
       <c r="G23" t="s">
+        <v>67</v>
+      </c>
+      <c r="H23" t="s">
+        <v>67</v>
+      </c>
+      <c r="I23" t="s">
+        <v>67</v>
+      </c>
+      <c r="J23" t="s">
+        <v>67</v>
+      </c>
+      <c r="K23" t="s">
         <v>69</v>
       </c>
-      <c r="H23" t="s">
-        <v>69</v>
-      </c>
-      <c r="I23" t="s">
-        <v>69</v>
-      </c>
-      <c r="J23" t="s">
-        <v>69</v>
-      </c>
-      <c r="K23" t="s">
-        <v>71</v>
-      </c>
       <c r="L23" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M23">
         <v>60000</v>
@@ -1982,10 +1970,10 @@
         <v>4</v>
       </c>
       <c r="O23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="Q23">
         <v>21750000</v>
@@ -1996,37 +1984,37 @@
         <v>32</v>
       </c>
       <c r="B24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24" t="s">
         <v>51</v>
-      </c>
-      <c r="C24" t="s">
-        <v>53</v>
       </c>
       <c r="D24">
         <v>80</v>
       </c>
       <c r="E24" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F24">
         <v>80</v>
       </c>
       <c r="G24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K24" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M24">
         <v>2000</v>
@@ -2035,66 +2023,13 @@
         <v>100</v>
       </c>
       <c r="O24" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P24" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="Q24">
         <v>3000000</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17">
-      <c r="A25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B25" t="s">
-        <v>52</v>
-      </c>
-      <c r="C25" t="s">
-        <v>53</v>
-      </c>
-      <c r="D25">
-        <v>289.6</v>
-      </c>
-      <c r="E25" t="s">
-        <v>64</v>
-      </c>
-      <c r="F25">
-        <v>289.6</v>
-      </c>
-      <c r="G25" t="s">
-        <v>69</v>
-      </c>
-      <c r="H25" t="s">
-        <v>69</v>
-      </c>
-      <c r="I25" t="s">
-        <v>69</v>
-      </c>
-      <c r="J25" t="s">
-        <v>69</v>
-      </c>
-      <c r="K25" t="s">
-        <v>70</v>
-      </c>
-      <c r="L25" t="s">
-        <v>69</v>
-      </c>
-      <c r="M25">
-        <v>16000</v>
-      </c>
-      <c r="N25">
-        <v>100</v>
-      </c>
-      <c r="O25" t="s">
-        <v>80</v>
-      </c>
-      <c r="P25" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q25">
-        <v>1357500</v>
       </c>
     </row>
   </sheetData>
@@ -2104,7 +2039,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -2112,10 +2047,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -2124,49 +2059,49 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:20">
@@ -2174,10 +2109,10 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D2" t="s">
         <v>22</v>
@@ -2192,7 +2127,7 @@
         <v>1500000</v>
       </c>
       <c r="H2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I2">
         <v>11000</v>
@@ -2201,34 +2136,34 @@
         <v>13000</v>
       </c>
       <c r="K2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L2">
         <v>16000</v>
       </c>
       <c r="M2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="S2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -2236,10 +2171,10 @@
         <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D3" t="s">
         <v>22</v>
@@ -2254,7 +2189,7 @@
         <v>1566800</v>
       </c>
       <c r="H3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I3">
         <v>13600</v>
@@ -2263,48 +2198,48 @@
         <v>15300</v>
       </c>
       <c r="K3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L3">
         <v>15300</v>
       </c>
       <c r="M3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="S3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E4" t="s">
         <v>19</v>
@@ -2316,7 +2251,7 @@
         <v>1000000</v>
       </c>
       <c r="H4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I4">
         <v>9500</v>
@@ -2325,48 +2260,48 @@
         <v>10700</v>
       </c>
       <c r="K4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L4">
         <v>13000</v>
       </c>
       <c r="M4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O4">
         <v>50</v>
       </c>
       <c r="P4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="S4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E5" t="s">
         <v>17</v>
@@ -2378,7 +2313,7 @@
         <v>6500000</v>
       </c>
       <c r="H5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I5">
         <v>2000</v>
@@ -2387,45 +2322,45 @@
         <v>2000</v>
       </c>
       <c r="K5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L5">
         <v>2000</v>
       </c>
       <c r="M5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R5" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="S5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D6" t="s">
         <v>23</v>
@@ -2440,7 +2375,7 @@
         <v>3077650</v>
       </c>
       <c r="H6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I6">
         <v>13800</v>
@@ -2449,45 +2384,45 @@
         <v>15700</v>
       </c>
       <c r="K6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L6">
         <v>16500</v>
       </c>
       <c r="M6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O6">
         <v>100</v>
       </c>
       <c r="P6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R6" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="S6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
         <v>23</v>
@@ -2502,7 +2437,7 @@
         <v>1400000</v>
       </c>
       <c r="H7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I7">
         <v>12500</v>
@@ -2511,45 +2446,45 @@
         <v>15500</v>
       </c>
       <c r="K7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L7">
         <v>15500</v>
       </c>
       <c r="M7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R7" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="S7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D8" t="s">
         <v>24</v>
@@ -2564,7 +2499,7 @@
         <v>1000000</v>
       </c>
       <c r="H8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I8">
         <v>24000</v>
@@ -2573,34 +2508,34 @@
         <v>29000</v>
       </c>
       <c r="K8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L8">
         <v>29000</v>
       </c>
       <c r="M8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R8" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="S8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -2608,13 +2543,13 @@
         <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E9" t="s">
         <v>22</v>
@@ -2626,7 +2561,7 @@
         <v>751000</v>
       </c>
       <c r="H9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I9">
         <v>18000</v>
@@ -2635,45 +2570,45 @@
         <v>21000</v>
       </c>
       <c r="K9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L9">
         <v>21000</v>
       </c>
       <c r="M9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O9">
         <v>72.87616511318242</v>
       </c>
       <c r="P9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R9" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="S9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s">
         <v>25</v>
@@ -2688,7 +2623,7 @@
         <v>5800000</v>
       </c>
       <c r="H10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I10">
         <v>2000</v>
@@ -2697,45 +2632,45 @@
         <v>2000</v>
       </c>
       <c r="K10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L10">
         <v>2000</v>
       </c>
       <c r="M10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O10">
         <v>0</v>
       </c>
       <c r="P10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R10" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="S10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D11" t="s">
         <v>25</v>
@@ -2750,7 +2685,7 @@
         <v>1400000</v>
       </c>
       <c r="H11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I11">
         <v>16000</v>
@@ -2759,34 +2694,34 @@
         <v>19000</v>
       </c>
       <c r="K11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L11">
         <v>16000</v>
       </c>
       <c r="M11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O11">
         <v>0</v>
       </c>
       <c r="P11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R11" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="S11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -2794,13 +2729,13 @@
         <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E12" t="s">
         <v>25</v>
@@ -2812,7 +2747,7 @@
         <v>2234000</v>
       </c>
       <c r="H12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I12">
         <v>7300</v>
@@ -2821,45 +2756,45 @@
         <v>8500</v>
       </c>
       <c r="K12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L12">
         <v>10000</v>
       </c>
       <c r="M12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O12">
         <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R12" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="S12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D13" t="s">
         <v>29</v>
@@ -2874,7 +2809,7 @@
         <v>1350000</v>
       </c>
       <c r="H13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I13">
         <v>14000</v>
@@ -2883,48 +2818,48 @@
         <v>17000</v>
       </c>
       <c r="K13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L13">
         <v>22000</v>
       </c>
       <c r="M13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O13">
         <v>0</v>
       </c>
       <c r="P13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R13" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="S13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D14" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E14" t="s">
         <v>27</v>
@@ -2936,7 +2871,7 @@
         <v>7600000</v>
       </c>
       <c r="H14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I14">
         <v>24000</v>
@@ -2945,48 +2880,48 @@
         <v>30000</v>
       </c>
       <c r="K14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L14">
         <v>35000</v>
       </c>
       <c r="M14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O14">
         <v>14.47368421052632</v>
       </c>
       <c r="P14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R14" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="S14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D15" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E15" t="s">
         <v>28</v>
@@ -2998,7 +2933,7 @@
         <v>6000000</v>
       </c>
       <c r="H15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I15">
         <v>2000</v>
@@ -3007,34 +2942,34 @@
         <v>2000</v>
       </c>
       <c r="K15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L15">
         <v>2000</v>
       </c>
       <c r="M15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O15">
         <v>0</v>
       </c>
       <c r="P15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R15" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="S15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -3042,13 +2977,13 @@
         <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D16" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
@@ -3060,7 +2995,7 @@
         <v>4000000</v>
       </c>
       <c r="H16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I16">
         <v>2000</v>
@@ -3069,48 +3004,48 @@
         <v>2000</v>
       </c>
       <c r="K16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L16">
         <v>2000</v>
       </c>
       <c r="M16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O16">
         <v>0</v>
       </c>
       <c r="P16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R16" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="S16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:20">
       <c r="A17" t="s">
-        <v>33</v>
+        <v>77</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D17" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E17" t="s">
         <v>30</v>
@@ -3122,7 +3057,7 @@
         <v>1618000</v>
       </c>
       <c r="H17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I17">
         <v>6200</v>
@@ -3131,48 +3066,48 @@
         <v>7700</v>
       </c>
       <c r="K17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L17">
         <v>10000</v>
       </c>
       <c r="M17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O17">
         <v>0</v>
       </c>
       <c r="P17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R17" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="S17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:20">
       <c r="A18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C18" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D18" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E18" t="s">
         <v>31</v>
@@ -3184,7 +3119,7 @@
         <v>7250000</v>
       </c>
       <c r="H18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I18">
         <v>47000</v>
@@ -3193,48 +3128,48 @@
         <v>60000</v>
       </c>
       <c r="K18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L18">
         <v>60000</v>
       </c>
       <c r="M18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O18">
         <v>0</v>
       </c>
       <c r="P18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R18" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="S18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:20">
       <c r="A19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C19" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D19" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E19" t="s">
         <v>32</v>
@@ -3246,7 +3181,7 @@
         <v>4000000</v>
       </c>
       <c r="H19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I19">
         <v>2000</v>
@@ -3255,96 +3190,34 @@
         <v>2000</v>
       </c>
       <c r="K19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L19">
         <v>2000</v>
       </c>
       <c r="M19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O19">
         <v>0</v>
       </c>
       <c r="P19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="R19" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="S19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T19" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20">
-      <c r="A20" t="s">
-        <v>80</v>
-      </c>
-      <c r="B20" t="s">
-        <v>52</v>
-      </c>
-      <c r="C20" t="s">
-        <v>64</v>
-      </c>
-      <c r="D20" t="s">
-        <v>87</v>
-      </c>
-      <c r="E20" t="s">
-        <v>33</v>
-      </c>
-      <c r="F20">
-        <v>28960000</v>
-      </c>
-      <c r="G20">
-        <v>1810000</v>
-      </c>
-      <c r="H20" t="s">
-        <v>69</v>
-      </c>
-      <c r="I20">
-        <v>9000</v>
-      </c>
-      <c r="J20">
-        <v>12000</v>
-      </c>
-      <c r="K20" t="s">
-        <v>69</v>
-      </c>
-      <c r="L20">
-        <v>16000</v>
-      </c>
-      <c r="M20" t="s">
-        <v>69</v>
-      </c>
-      <c r="N20" t="s">
-        <v>69</v>
-      </c>
-      <c r="O20">
-        <v>0</v>
-      </c>
-      <c r="P20" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>69</v>
-      </c>
-      <c r="R20" t="s">
-        <v>125</v>
-      </c>
-      <c r="S20" t="s">
-        <v>69</v>
-      </c>
-      <c r="T20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -3354,21 +3227,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -3380,10 +3253,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -3392,27 +3265,27 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="F2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G2" t="s">
         <v>32</v>
@@ -3435,22 +3308,22 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E3" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="F3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G3" t="s">
         <v>31</v>
@@ -3473,19 +3346,19 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
         <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F4" t="s">
         <v>22</v>
@@ -3511,22 +3384,22 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G5" t="s">
         <v>28</v>
@@ -3549,22 +3422,22 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B6" t="s">
         <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G6" t="s">
         <v>29</v>
@@ -3587,19 +3460,19 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F7" t="s">
         <v>25</v>
@@ -3625,22 +3498,22 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>77</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G8" t="s">
         <v>30</v>
@@ -3663,22 +3536,22 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F9" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G9" t="s">
         <v>17</v>
@@ -3701,19 +3574,19 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E10" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F10" t="s">
         <v>23</v>
@@ -3739,19 +3612,19 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B11" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F11" t="s">
         <v>25</v>
@@ -3777,22 +3650,22 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B12" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="F12" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G12" t="s">
         <v>27</v>
@@ -3815,107 +3688,107 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="C13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="E13" t="s">
-        <v>64</v>
+        <v>126</v>
       </c>
       <c r="F13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H13">
-        <v>22340</v>
+        <v>10640</v>
       </c>
       <c r="I13">
-        <v>2234000</v>
+        <v>7600000</v>
       </c>
       <c r="J13">
-        <v>10000</v>
+        <v>35000</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B14" t="s">
-        <v>77</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E14" t="s">
-        <v>130</v>
+        <v>62</v>
       </c>
       <c r="F14" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="G14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H14">
-        <v>10640</v>
+        <v>22340</v>
       </c>
       <c r="I14">
-        <v>7600000</v>
+        <v>2234000</v>
       </c>
       <c r="J14">
-        <v>35000</v>
+        <v>10000</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14">
-        <v>4</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="B15" t="s">
-        <v>80</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="D15" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="E15" t="s">
-        <v>64</v>
+        <v>127</v>
       </c>
       <c r="F15" t="s">
-        <v>87</v>
+        <v>22</v>
       </c>
       <c r="G15" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="H15">
-        <v>28960</v>
+        <v>22800</v>
       </c>
       <c r="I15">
-        <v>1810000</v>
+        <v>1500000</v>
       </c>
       <c r="J15">
         <v>16000</v>
@@ -3924,191 +3797,191 @@
         <v>0</v>
       </c>
       <c r="L15">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>78</v>
       </c>
       <c r="C16" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>102</v>
       </c>
       <c r="E16" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="F16" t="s">
-        <v>22</v>
+        <v>84</v>
       </c>
       <c r="G16" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="H16">
-        <v>22800</v>
+        <v>17400</v>
       </c>
       <c r="I16">
-        <v>1500000</v>
+        <v>7250000</v>
       </c>
       <c r="J16">
-        <v>16000</v>
+        <v>60000</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16">
-        <v>95</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="B17" t="s">
-        <v>79</v>
+        <v>24</v>
       </c>
       <c r="C17" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="D17" t="s">
-        <v>105</v>
+        <v>53</v>
       </c>
       <c r="E17" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F17" t="s">
-        <v>86</v>
+        <v>22</v>
       </c>
       <c r="G17" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="H17">
-        <v>17400</v>
+        <v>1200</v>
       </c>
       <c r="I17">
-        <v>7250000</v>
+        <v>1500000</v>
       </c>
       <c r="J17">
-        <v>60000</v>
+        <v>16000</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
       <c r="L17">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>78</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>55</v>
+        <v>102</v>
       </c>
       <c r="E18" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="F18" t="s">
-        <v>22</v>
+        <v>84</v>
       </c>
       <c r="G18" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="H18">
-        <v>1200</v>
+        <v>143550</v>
       </c>
       <c r="I18">
-        <v>1500000</v>
+        <v>7250000</v>
       </c>
       <c r="J18">
-        <v>16000</v>
+        <v>60000</v>
       </c>
       <c r="K18">
         <v>0</v>
       </c>
       <c r="L18">
-        <v>5</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B19" t="s">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="C19" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D19" t="s">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="E19" t="s">
-        <v>129</v>
+        <v>60</v>
       </c>
       <c r="F19" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="G19" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="H19">
-        <v>143550</v>
+        <v>15771</v>
       </c>
       <c r="I19">
-        <v>7250000</v>
+        <v>751000</v>
       </c>
       <c r="J19">
-        <v>60000</v>
+        <v>21000</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>33</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B20" t="s">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F20" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="G20" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="H20">
-        <v>15771</v>
+        <v>29700</v>
       </c>
       <c r="I20">
-        <v>751000</v>
+        <v>1350000</v>
       </c>
       <c r="J20">
-        <v>21000</v>
+        <v>22000</v>
       </c>
       <c r="K20">
         <v>0</v>
@@ -4119,34 +3992,34 @@
     </row>
     <row r="21" spans="1:12">
       <c r="A21" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C21" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="D21" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E21" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F21" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="G21" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="H21">
-        <v>29700</v>
+        <v>21700</v>
       </c>
       <c r="I21">
-        <v>1350000</v>
+        <v>1400000</v>
       </c>
       <c r="J21">
-        <v>22000</v>
+        <v>15500</v>
       </c>
       <c r="K21">
         <v>0</v>
@@ -4157,34 +4030,34 @@
     </row>
     <row r="22" spans="1:12">
       <c r="A22" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C22" t="s">
         <v>39</v>
       </c>
       <c r="D22" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E22" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F22" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G22" t="s">
         <v>21</v>
       </c>
       <c r="H22">
-        <v>21700</v>
+        <v>29000</v>
       </c>
       <c r="I22">
-        <v>1400000</v>
+        <v>1000000</v>
       </c>
       <c r="J22">
-        <v>15500</v>
+        <v>29000</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -4195,34 +4068,34 @@
     </row>
     <row r="23" spans="1:12">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B23" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C23" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D23" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E23" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F23" t="s">
-        <v>24</v>
+        <v>79</v>
       </c>
       <c r="G23" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H23">
-        <v>29000</v>
+        <v>13000</v>
       </c>
       <c r="I23">
         <v>1000000</v>
       </c>
       <c r="J23">
-        <v>29000</v>
+        <v>13000</v>
       </c>
       <c r="K23">
         <v>0</v>
@@ -4233,77 +4106,39 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B24" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="C24" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="D24" t="s">
-        <v>58</v>
+        <v>102</v>
       </c>
       <c r="E24" t="s">
-        <v>58</v>
+        <v>125</v>
       </c>
       <c r="F24" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G24" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H24">
-        <v>13000</v>
+        <v>143550</v>
       </c>
       <c r="I24">
-        <v>1000000</v>
+        <v>7250000</v>
       </c>
       <c r="J24">
-        <v>13000</v>
+        <v>60000</v>
       </c>
       <c r="K24">
         <v>0</v>
       </c>
       <c r="L24">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12">
-      <c r="A25" t="s">
-        <v>58</v>
-      </c>
-      <c r="B25" t="s">
-        <v>79</v>
-      </c>
-      <c r="C25" t="s">
-        <v>50</v>
-      </c>
-      <c r="D25" t="s">
-        <v>105</v>
-      </c>
-      <c r="E25" t="s">
-        <v>129</v>
-      </c>
-      <c r="F25" t="s">
-        <v>86</v>
-      </c>
-      <c r="G25" t="s">
-        <v>31</v>
-      </c>
-      <c r="H25">
-        <v>143550</v>
-      </c>
-      <c r="I25">
-        <v>7250000</v>
-      </c>
-      <c r="J25">
-        <v>60000</v>
-      </c>
-      <c r="K25">
-        <v>0</v>
-      </c>
-      <c r="L25">
         <v>33</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RPA datasets push 2024-08-31
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="132">
   <si>
     <t>상장일</t>
   </si>
@@ -69,6 +69,9 @@
     <t>총기관배정수량</t>
   </si>
   <si>
+    <t>2024-08-30</t>
+  </si>
+  <si>
     <t>2024-08-22</t>
   </si>
   <si>
@@ -117,6 +120,9 @@
     <t>2024-07-12</t>
   </si>
   <si>
+    <t>아이스크림미디어</t>
+  </si>
+  <si>
     <t>M83</t>
   </si>
   <si>
@@ -177,6 +183,9 @@
     <t>코스피</t>
   </si>
   <si>
+    <t>삼성</t>
+  </si>
+  <si>
     <t>신영</t>
   </si>
   <si>
@@ -204,9 +213,6 @@
     <t>교보</t>
   </si>
   <si>
-    <t>삼성</t>
-  </si>
-  <si>
     <t>SK</t>
   </si>
   <si>
@@ -255,6 +261,9 @@
     <t>2024-07-02</t>
   </si>
   <si>
+    <t>2024-08-26</t>
+  </si>
+  <si>
     <t>2024-08-14</t>
   </si>
   <si>
@@ -328,6 +337,9 @@
   </si>
   <si>
     <t>엘에스</t>
+  </si>
+  <si>
+    <t>12.89 : 1</t>
   </si>
   <si>
     <t>638.07 : 1</t>
@@ -757,7 +769,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -818,102 +830,102 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D2">
-        <v>240</v>
+        <v>787.2</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F2">
-        <v>228</v>
+        <v>787.2</v>
       </c>
       <c r="G2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M2">
-        <v>16000</v>
+        <v>32000</v>
       </c>
       <c r="N2">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="P2" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="Q2">
-        <v>2100000</v>
+        <v>1722000</v>
       </c>
     </row>
     <row r="3" spans="1:17">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D3">
         <v>240</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F3">
-        <v>12</v>
+        <v>228</v>
       </c>
       <c r="G3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="L3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M3">
         <v>16000</v>
       </c>
       <c r="N3">
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="O3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="P3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q3">
         <v>2100000</v>
@@ -924,52 +936,52 @@
         <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D4">
-        <v>239.7204</v>
+        <v>240</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F4">
-        <v>239.7204</v>
+        <v>12</v>
       </c>
       <c r="G4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="L4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M4">
-        <v>15300</v>
+        <v>16000</v>
       </c>
       <c r="N4">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="O4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="P4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q4">
-        <v>1156798</v>
+        <v>2100000</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -977,158 +989,158 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D5">
-        <v>130</v>
+        <v>239.7204</v>
       </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F5">
-        <v>130</v>
+        <v>239.7204</v>
       </c>
       <c r="G5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M5">
-        <v>13000</v>
+        <v>15300</v>
       </c>
       <c r="N5">
         <v>100</v>
       </c>
       <c r="O5" t="s">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="P5" t="s">
-        <v>79</v>
+        <v>23</v>
       </c>
       <c r="Q5">
-        <v>723700</v>
+        <v>1156798</v>
       </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D6">
         <v>130</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F6">
         <v>130</v>
       </c>
       <c r="G6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M6">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="N6">
         <v>100</v>
       </c>
       <c r="O6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="P6" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="Q6">
-        <v>4875000</v>
+        <v>723700</v>
       </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D7">
-        <v>507.81225</v>
+        <v>130</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F7">
-        <v>507.81225</v>
+        <v>130</v>
       </c>
       <c r="G7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M7">
-        <v>16500</v>
+        <v>2000</v>
       </c>
       <c r="N7">
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="P7" t="s">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="Q7">
-        <v>2078175</v>
+        <v>4875000</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -1136,105 +1148,105 @@
         <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D8">
-        <v>217</v>
+        <v>507.81225</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F8">
-        <v>217</v>
+        <v>507.81225</v>
       </c>
       <c r="G8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M8">
-        <v>15500</v>
+        <v>16500</v>
       </c>
       <c r="N8">
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="P8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q8">
-        <v>1050000</v>
+        <v>2078175</v>
       </c>
     </row>
     <row r="9" spans="1:17">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D9">
-        <v>290</v>
+        <v>217</v>
       </c>
       <c r="E9" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F9">
-        <v>290</v>
+        <v>217</v>
       </c>
       <c r="G9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M9">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="N9">
         <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P9" t="s">
         <v>24</v>
       </c>
       <c r="Q9">
-        <v>720000</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -1242,52 +1254,52 @@
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D10">
-        <v>157.71</v>
+        <v>290</v>
       </c>
       <c r="E10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F10">
-        <v>157.71</v>
+        <v>290</v>
       </c>
       <c r="G10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M10">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="N10">
         <v>100</v>
       </c>
       <c r="O10" t="s">
+        <v>74</v>
+      </c>
+      <c r="P10" t="s">
         <v>25</v>
       </c>
-      <c r="P10" t="s">
-        <v>70</v>
-      </c>
       <c r="Q10">
-        <v>540250</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -1295,52 +1307,52 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D11">
-        <v>116</v>
+        <v>157.71</v>
       </c>
       <c r="E11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F11">
-        <v>116</v>
+        <v>157.71</v>
       </c>
       <c r="G11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K11" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M11">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="N11">
         <v>100</v>
       </c>
       <c r="O11" t="s">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="P11" t="s">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="Q11">
-        <v>4350000</v>
+        <v>540250</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -1348,52 +1360,52 @@
         <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D12">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="E12" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F12">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="G12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K12" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M12">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N12">
         <v>100</v>
       </c>
       <c r="O12" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="P12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q12">
-        <v>1050000</v>
+        <v>4350000</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -1401,52 +1413,52 @@
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D13">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="E13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F13">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="G13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M13">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="N13">
         <v>100</v>
       </c>
       <c r="O13" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="P13" t="s">
-        <v>80</v>
+        <v>26</v>
       </c>
       <c r="Q13">
-        <v>1675500</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1454,52 +1466,52 @@
         <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D14">
-        <v>297</v>
+        <v>223.4</v>
       </c>
       <c r="E14" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F14">
-        <v>297</v>
+        <v>223.4</v>
       </c>
       <c r="G14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K14" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M14">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="N14">
         <v>100</v>
       </c>
       <c r="O14" t="s">
-        <v>74</v>
+        <v>30</v>
       </c>
       <c r="P14" t="s">
-        <v>29</v>
+        <v>83</v>
       </c>
       <c r="Q14">
-        <v>1012500</v>
+        <v>1675500</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1507,102 +1519,102 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D15">
-        <v>2660</v>
+        <v>297</v>
       </c>
       <c r="E15" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="F15">
-        <v>2553.6</v>
+        <v>297</v>
       </c>
       <c r="G15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K15" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M15">
-        <v>35000</v>
+        <v>22000</v>
       </c>
       <c r="N15">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="O15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="P15" t="s">
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="Q15">
-        <v>9340690</v>
+        <v>1012500</v>
       </c>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D16">
         <v>2660</v>
       </c>
       <c r="E16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F16">
-        <v>106.4</v>
+        <v>2553.6</v>
       </c>
       <c r="G16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K16" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="L16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M16">
         <v>35000</v>
       </c>
       <c r="N16">
-        <v>4</v>
+        <v>96</v>
       </c>
       <c r="O16" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="P16" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="Q16">
         <v>9340690</v>
@@ -1613,52 +1625,52 @@
         <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D17">
-        <v>120</v>
+        <v>2660</v>
       </c>
       <c r="E17" t="s">
         <v>55</v>
       </c>
       <c r="F17">
-        <v>120</v>
+        <v>106.4</v>
       </c>
       <c r="G17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K17" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="L17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M17">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="N17">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="O17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="P17" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q17">
-        <v>4500000</v>
+        <v>9340690</v>
       </c>
     </row>
     <row r="18" spans="1:17">
@@ -1666,37 +1678,37 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D18">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="E18" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="F18">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="G18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M18">
         <v>2000</v>
@@ -1705,13 +1717,13 @@
         <v>100</v>
       </c>
       <c r="O18" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="P18" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="Q18">
-        <v>3000000</v>
+        <v>4500000</v>
       </c>
     </row>
     <row r="19" spans="1:17">
@@ -1719,52 +1731,52 @@
         <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C19" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D19">
-        <v>161.8</v>
+        <v>80</v>
       </c>
       <c r="E19" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="F19">
-        <v>161.8</v>
+        <v>80</v>
       </c>
       <c r="G19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M19">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="N19">
         <v>100</v>
       </c>
       <c r="O19" t="s">
+        <v>31</v>
+      </c>
+      <c r="P19" t="s">
         <v>77</v>
       </c>
-      <c r="P19" t="s">
-        <v>83</v>
-      </c>
       <c r="Q19">
-        <v>1187900</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="20" spans="1:17">
@@ -1772,90 +1784,90 @@
         <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D20">
-        <v>4350</v>
+        <v>161.8</v>
       </c>
       <c r="E20" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F20">
-        <v>1435.5</v>
+        <v>161.8</v>
       </c>
       <c r="G20" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H20" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I20" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J20" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K20" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L20" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M20">
-        <v>60000</v>
+        <v>10000</v>
       </c>
       <c r="N20">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="O20" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="P20" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="Q20">
-        <v>21750000</v>
+        <v>1187900</v>
       </c>
     </row>
     <row r="21" spans="1:17">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D21">
         <v>4350</v>
       </c>
       <c r="E21" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="F21">
         <v>1435.5</v>
       </c>
       <c r="G21" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H21" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I21" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J21" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L21" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M21">
         <v>60000</v>
@@ -1864,10 +1876,10 @@
         <v>33</v>
       </c>
       <c r="O21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P21" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="Q21">
         <v>21750000</v>
@@ -1875,52 +1887,52 @@
     </row>
     <row r="22" spans="1:17">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C22" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D22">
         <v>4350</v>
       </c>
       <c r="E22" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="F22">
-        <v>1305</v>
+        <v>1435.5</v>
       </c>
       <c r="G22" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H22" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I22" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J22" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K22" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L22" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M22">
         <v>60000</v>
       </c>
       <c r="N22">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="O22" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P22" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="Q22">
         <v>21750000</v>
@@ -1928,52 +1940,52 @@
     </row>
     <row r="23" spans="1:17">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C23" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D23">
         <v>4350</v>
       </c>
       <c r="E23" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="F23">
-        <v>174</v>
+        <v>1305</v>
       </c>
       <c r="G23" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H23" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I23" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J23" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K23" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="L23" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M23">
         <v>60000</v>
       </c>
       <c r="N23">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="O23" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P23" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="Q23">
         <v>21750000</v>
@@ -1984,51 +1996,104 @@
         <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C24" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D24">
+        <v>4350</v>
+      </c>
+      <c r="E24" t="s">
+        <v>67</v>
+      </c>
+      <c r="F24">
+        <v>174</v>
+      </c>
+      <c r="G24" t="s">
+        <v>69</v>
+      </c>
+      <c r="H24" t="s">
+        <v>69</v>
+      </c>
+      <c r="I24" t="s">
+        <v>69</v>
+      </c>
+      <c r="J24" t="s">
+        <v>69</v>
+      </c>
+      <c r="K24" t="s">
+        <v>71</v>
+      </c>
+      <c r="L24" t="s">
+        <v>69</v>
+      </c>
+      <c r="M24">
+        <v>60000</v>
+      </c>
+      <c r="N24">
+        <v>4</v>
+      </c>
+      <c r="O24" t="s">
         <v>80</v>
       </c>
-      <c r="E24" t="s">
-        <v>66</v>
-      </c>
-      <c r="F24">
+      <c r="P24" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q24">
+        <v>21750000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17">
+      <c r="A25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" t="s">
+        <v>52</v>
+      </c>
+      <c r="C25" t="s">
+        <v>53</v>
+      </c>
+      <c r="D25">
         <v>80</v>
       </c>
-      <c r="G24" t="s">
-        <v>67</v>
-      </c>
-      <c r="H24" t="s">
-        <v>67</v>
-      </c>
-      <c r="I24" t="s">
-        <v>67</v>
-      </c>
-      <c r="J24" t="s">
-        <v>67</v>
-      </c>
-      <c r="K24" t="s">
+      <c r="E25" t="s">
         <v>68</v>
       </c>
-      <c r="L24" t="s">
-        <v>67</v>
-      </c>
-      <c r="M24">
+      <c r="F25">
+        <v>80</v>
+      </c>
+      <c r="G25" t="s">
+        <v>69</v>
+      </c>
+      <c r="H25" t="s">
+        <v>69</v>
+      </c>
+      <c r="I25" t="s">
+        <v>69</v>
+      </c>
+      <c r="J25" t="s">
+        <v>69</v>
+      </c>
+      <c r="K25" t="s">
+        <v>70</v>
+      </c>
+      <c r="L25" t="s">
+        <v>69</v>
+      </c>
+      <c r="M25">
         <v>2000</v>
       </c>
-      <c r="N24">
+      <c r="N25">
         <v>100</v>
       </c>
-      <c r="O24" t="s">
-        <v>78</v>
-      </c>
-      <c r="P24" t="s">
-        <v>84</v>
-      </c>
-      <c r="Q24">
+      <c r="O25" t="s">
+        <v>80</v>
+      </c>
+      <c r="P25" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q25">
         <v>3000000</v>
       </c>
     </row>
@@ -2039,7 +2104,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T19"/>
+  <dimension ref="A1:T20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -2047,10 +2112,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -2059,943 +2124,943 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
       </c>
       <c r="F2">
-        <v>24000000</v>
+        <v>78720000</v>
       </c>
       <c r="G2">
-        <v>1500000</v>
+        <v>2460000</v>
       </c>
       <c r="H2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I2">
-        <v>11000</v>
+        <v>32000</v>
       </c>
       <c r="J2">
-        <v>13000</v>
+        <v>40200</v>
       </c>
       <c r="K2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L2">
-        <v>16000</v>
+        <v>32000</v>
       </c>
       <c r="M2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="S2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E3" t="s">
         <v>18</v>
       </c>
       <c r="F3">
-        <v>23972040</v>
+        <v>24000000</v>
       </c>
       <c r="G3">
-        <v>1566800</v>
+        <v>1500000</v>
       </c>
       <c r="H3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I3">
-        <v>13600</v>
+        <v>11000</v>
       </c>
       <c r="J3">
-        <v>15300</v>
+        <v>13000</v>
       </c>
       <c r="K3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L3">
-        <v>15300</v>
+        <v>16000</v>
       </c>
       <c r="M3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="S3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>79</v>
+        <v>23</v>
       </c>
       <c r="E4" t="s">
         <v>19</v>
       </c>
       <c r="F4">
-        <v>13000000</v>
+        <v>23972040</v>
       </c>
       <c r="G4">
-        <v>1000000</v>
+        <v>1566800</v>
       </c>
       <c r="H4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I4">
-        <v>9500</v>
+        <v>13600</v>
       </c>
       <c r="J4">
-        <v>10700</v>
+        <v>15300</v>
       </c>
       <c r="K4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L4">
-        <v>13000</v>
+        <v>15300</v>
       </c>
       <c r="M4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O4">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R4" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="S4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F5">
         <v>13000000</v>
       </c>
       <c r="G5">
-        <v>6500000</v>
+        <v>1000000</v>
       </c>
       <c r="H5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I5">
-        <v>2000</v>
+        <v>9500</v>
       </c>
       <c r="J5">
-        <v>2000</v>
+        <v>10700</v>
       </c>
       <c r="K5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L5">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="M5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="P5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="S5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="E6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F6">
-        <v>50781225</v>
+        <v>13000000</v>
       </c>
       <c r="G6">
-        <v>3077650</v>
+        <v>6500000</v>
       </c>
       <c r="H6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I6">
-        <v>13800</v>
+        <v>2000</v>
       </c>
       <c r="J6">
-        <v>15700</v>
+        <v>2000</v>
       </c>
       <c r="K6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L6">
-        <v>16500</v>
+        <v>2000</v>
       </c>
       <c r="M6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O6">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R6" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="S6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E7" t="s">
         <v>21</v>
       </c>
       <c r="F7">
-        <v>21700000</v>
+        <v>50781225</v>
       </c>
       <c r="G7">
-        <v>1400000</v>
+        <v>3077650</v>
       </c>
       <c r="H7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I7">
-        <v>12500</v>
+        <v>13800</v>
       </c>
       <c r="J7">
-        <v>15500</v>
+        <v>15700</v>
       </c>
       <c r="K7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L7">
-        <v>15500</v>
+        <v>16500</v>
       </c>
       <c r="M7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R7" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="S7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D8" t="s">
         <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F8">
-        <v>29000000</v>
+        <v>21700000</v>
       </c>
       <c r="G8">
-        <v>1000000</v>
+        <v>1400000</v>
       </c>
       <c r="H8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I8">
-        <v>24000</v>
+        <v>12500</v>
       </c>
       <c r="J8">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="K8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L8">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="M8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R8" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="S8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" t="s">
         <v>25</v>
-      </c>
-      <c r="B9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" t="s">
-        <v>60</v>
-      </c>
-      <c r="D9" t="s">
-        <v>70</v>
       </c>
       <c r="E9" t="s">
         <v>22</v>
       </c>
       <c r="F9">
-        <v>15771000</v>
+        <v>29000000</v>
       </c>
       <c r="G9">
-        <v>751000</v>
+        <v>1000000</v>
       </c>
       <c r="H9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I9">
-        <v>18000</v>
+        <v>24000</v>
       </c>
       <c r="J9">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="K9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L9">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="M9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O9">
-        <v>72.87616511318242</v>
+        <v>0</v>
       </c>
       <c r="P9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R9" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="S9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="E10" t="s">
         <v>23</v>
       </c>
       <c r="F10">
-        <v>11600000</v>
+        <v>15771000</v>
       </c>
       <c r="G10">
-        <v>5800000</v>
+        <v>751000</v>
       </c>
       <c r="H10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I10">
-        <v>2000</v>
+        <v>18000</v>
       </c>
       <c r="J10">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="K10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L10">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="M10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O10">
-        <v>0</v>
+        <v>72.87616511318242</v>
       </c>
       <c r="P10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R10" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="S10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E11" t="s">
         <v>24</v>
       </c>
       <c r="F11">
-        <v>22400000</v>
+        <v>11600000</v>
       </c>
       <c r="G11">
-        <v>1400000</v>
+        <v>5800000</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I11">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="J11">
-        <v>19000</v>
+        <v>2000</v>
       </c>
       <c r="K11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L11">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="M11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O11">
         <v>0</v>
       </c>
       <c r="P11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R11" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="S11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>80</v>
+        <v>26</v>
       </c>
       <c r="E12" t="s">
         <v>25</v>
       </c>
       <c r="F12">
-        <v>22340000</v>
+        <v>22400000</v>
       </c>
       <c r="G12">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="H12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I12">
-        <v>7300</v>
+        <v>16000</v>
       </c>
       <c r="J12">
-        <v>8500</v>
+        <v>19000</v>
       </c>
       <c r="K12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L12">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="M12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O12">
         <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R12" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="S12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>74</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D13" t="s">
-        <v>29</v>
+        <v>83</v>
       </c>
       <c r="E13" t="s">
         <v>26</v>
       </c>
       <c r="F13">
-        <v>29700000</v>
+        <v>22340000</v>
       </c>
       <c r="G13">
-        <v>1350000</v>
+        <v>2234000</v>
       </c>
       <c r="H13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I13">
-        <v>14000</v>
+        <v>7300</v>
       </c>
       <c r="J13">
-        <v>17000</v>
+        <v>8500</v>
       </c>
       <c r="K13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L13">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="M13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O13">
         <v>0</v>
       </c>
       <c r="P13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R13" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="S13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C14" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D14" t="s">
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="E14" t="s">
         <v>27</v>
       </c>
       <c r="F14">
-        <v>266000000</v>
+        <v>29700000</v>
       </c>
       <c r="G14">
-        <v>7600000</v>
+        <v>1350000</v>
       </c>
       <c r="H14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I14">
-        <v>24000</v>
+        <v>14000</v>
       </c>
       <c r="J14">
-        <v>30000</v>
+        <v>17000</v>
       </c>
       <c r="K14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L14">
-        <v>35000</v>
+        <v>22000</v>
       </c>
       <c r="M14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O14">
-        <v>14.47368421052632</v>
+        <v>0</v>
       </c>
       <c r="P14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R14" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="S14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E15" t="s">
         <v>28</v>
       </c>
       <c r="F15">
-        <v>12000000</v>
+        <v>266000000</v>
       </c>
       <c r="G15">
-        <v>6000000</v>
+        <v>7600000</v>
       </c>
       <c r="H15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I15">
-        <v>2000</v>
+        <v>24000</v>
       </c>
       <c r="J15">
-        <v>2000</v>
+        <v>30000</v>
       </c>
       <c r="K15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L15">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="M15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O15">
-        <v>0</v>
+        <v>14.47368421052632</v>
       </c>
       <c r="P15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R15" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="S15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:20">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
       </c>
       <c r="F16">
-        <v>8000000</v>
+        <v>12000000</v>
       </c>
       <c r="G16">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="H16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I16">
         <v>2000</v>
@@ -3004,220 +3069,282 @@
         <v>2000</v>
       </c>
       <c r="K16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L16">
         <v>2000</v>
       </c>
       <c r="M16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O16">
         <v>0</v>
       </c>
       <c r="P16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R16" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="S16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:20">
       <c r="A17" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D17" t="s">
         <v>77</v>
-      </c>
-      <c r="B17" t="s">
-        <v>48</v>
-      </c>
-      <c r="C17" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" t="s">
-        <v>83</v>
       </c>
       <c r="E17" t="s">
         <v>30</v>
       </c>
       <c r="F17">
-        <v>16180000</v>
+        <v>8000000</v>
       </c>
       <c r="G17">
-        <v>1618000</v>
+        <v>4000000</v>
       </c>
       <c r="H17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I17">
-        <v>6200</v>
+        <v>2000</v>
       </c>
       <c r="J17">
-        <v>7700</v>
+        <v>2000</v>
       </c>
       <c r="K17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L17">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="M17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O17">
         <v>0</v>
       </c>
       <c r="P17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R17" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="S17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:20">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C18" t="s">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="D18" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E18" t="s">
         <v>31</v>
       </c>
       <c r="F18">
-        <v>435000000</v>
+        <v>16180000</v>
       </c>
       <c r="G18">
-        <v>7250000</v>
+        <v>1618000</v>
       </c>
       <c r="H18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I18">
-        <v>47000</v>
+        <v>6200</v>
       </c>
       <c r="J18">
-        <v>60000</v>
+        <v>7700</v>
       </c>
       <c r="K18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L18">
-        <v>60000</v>
+        <v>10000</v>
       </c>
       <c r="M18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O18">
         <v>0</v>
       </c>
       <c r="P18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R18" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="S18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:20">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D19" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E19" t="s">
         <v>32</v>
       </c>
       <c r="F19">
-        <v>8000000</v>
+        <v>435000000</v>
       </c>
       <c r="G19">
-        <v>4000000</v>
+        <v>7250000</v>
       </c>
       <c r="H19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I19">
-        <v>2000</v>
+        <v>47000</v>
       </c>
       <c r="J19">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="K19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L19">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="M19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O19">
         <v>0</v>
       </c>
       <c r="P19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="R19" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="S19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="T19" t="s">
-        <v>67</v>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20">
+      <c r="A20" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" t="s">
+        <v>106</v>
+      </c>
+      <c r="D20" t="s">
+        <v>87</v>
+      </c>
+      <c r="E20" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20">
+        <v>8000000</v>
+      </c>
+      <c r="G20">
+        <v>4000000</v>
+      </c>
+      <c r="H20" t="s">
+        <v>69</v>
+      </c>
+      <c r="I20">
+        <v>2000</v>
+      </c>
+      <c r="J20">
+        <v>2000</v>
+      </c>
+      <c r="K20" t="s">
+        <v>69</v>
+      </c>
+      <c r="L20">
+        <v>2000</v>
+      </c>
+      <c r="M20" t="s">
+        <v>69</v>
+      </c>
+      <c r="N20" t="s">
+        <v>69</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>69</v>
+      </c>
+      <c r="R20" t="s">
+        <v>125</v>
+      </c>
+      <c r="S20" t="s">
+        <v>69</v>
+      </c>
+      <c r="T20" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -3227,21 +3354,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -3253,10 +3380,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -3265,30 +3392,30 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="G2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H2">
         <v>8000</v>
@@ -3308,25 +3435,25 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E3" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="F3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="G3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H3">
         <v>130500</v>
@@ -3346,25 +3473,25 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H4">
         <v>23972.04</v>
@@ -3384,25 +3511,25 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H5">
         <v>12000</v>
@@ -3422,25 +3549,25 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G6" t="s">
         <v>30</v>
-      </c>
-      <c r="C6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F6" t="s">
-        <v>75</v>
-      </c>
-      <c r="G6" t="s">
-        <v>29</v>
       </c>
       <c r="H6">
         <v>8000</v>
@@ -3460,25 +3587,25 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D7" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E7" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H7">
         <v>11600</v>
@@ -3498,25 +3625,25 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F8" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="G8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H8">
         <v>16180</v>
@@ -3536,25 +3663,25 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F9" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H9">
         <v>13000</v>
@@ -3574,63 +3701,63 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E10" t="s">
-        <v>58</v>
+        <v>130</v>
       </c>
       <c r="F10" t="s">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="G10" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="H10">
-        <v>50781.225</v>
+        <v>255360</v>
       </c>
       <c r="I10">
-        <v>3077650</v>
+        <v>7600000</v>
       </c>
       <c r="J10">
-        <v>16500</v>
+        <v>35000</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B11" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F11" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" t="s">
         <v>25</v>
-      </c>
-      <c r="G11" t="s">
-        <v>24</v>
       </c>
       <c r="H11">
         <v>22400</v>
@@ -3650,329 +3777,329 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E12" t="s">
-        <v>126</v>
+        <v>61</v>
       </c>
       <c r="F12" t="s">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="G12" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="H12">
-        <v>255360</v>
+        <v>50781.225</v>
       </c>
       <c r="I12">
-        <v>7600000</v>
+        <v>3077650</v>
       </c>
       <c r="J12">
-        <v>35000</v>
+        <v>16500</v>
       </c>
       <c r="K12">
         <v>0</v>
       </c>
       <c r="L12">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
         <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E13" t="s">
-        <v>126</v>
+        <v>55</v>
       </c>
       <c r="F13" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H13">
-        <v>10640</v>
+        <v>22340</v>
       </c>
       <c r="I13">
-        <v>7600000</v>
+        <v>2234000</v>
       </c>
       <c r="J13">
-        <v>35000</v>
+        <v>10000</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
-        <v>4</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E14" t="s">
-        <v>62</v>
+        <v>130</v>
       </c>
       <c r="F14" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G14" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="H14">
-        <v>22340</v>
+        <v>10640</v>
       </c>
       <c r="I14">
-        <v>2234000</v>
+        <v>7600000</v>
       </c>
       <c r="J14">
-        <v>10000</v>
+        <v>35000</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D15" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E15" t="s">
-        <v>127</v>
+        <v>55</v>
       </c>
       <c r="F15" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="G15" t="s">
         <v>17</v>
       </c>
       <c r="H15">
-        <v>22800</v>
+        <v>78720</v>
       </c>
       <c r="I15">
-        <v>1500000</v>
+        <v>2460000</v>
       </c>
       <c r="J15">
-        <v>16000</v>
+        <v>32000</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="B16" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="C16" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="D16" t="s">
-        <v>102</v>
+        <v>56</v>
       </c>
       <c r="E16" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="F16" t="s">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="G16" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="H16">
-        <v>17400</v>
+        <v>22800</v>
       </c>
       <c r="I16">
-        <v>7250000</v>
+        <v>1500000</v>
       </c>
       <c r="J16">
-        <v>60000</v>
+        <v>16000</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16">
-        <v>4</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="D17" t="s">
-        <v>53</v>
+        <v>105</v>
       </c>
       <c r="E17" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F17" t="s">
-        <v>22</v>
+        <v>87</v>
       </c>
       <c r="G17" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="H17">
-        <v>1200</v>
+        <v>17400</v>
       </c>
       <c r="I17">
-        <v>1500000</v>
+        <v>7250000</v>
       </c>
       <c r="J17">
-        <v>16000</v>
+        <v>60000</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
       <c r="L17">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B18" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="D18" t="s">
-        <v>102</v>
+        <v>56</v>
       </c>
       <c r="E18" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="F18" t="s">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="G18" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="H18">
-        <v>143550</v>
+        <v>1200</v>
       </c>
       <c r="I18">
-        <v>7250000</v>
+        <v>1500000</v>
       </c>
       <c r="J18">
-        <v>60000</v>
+        <v>16000</v>
       </c>
       <c r="K18">
         <v>0</v>
       </c>
       <c r="L18">
-        <v>33</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>80</v>
       </c>
       <c r="C19" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>60</v>
+        <v>105</v>
       </c>
       <c r="E19" t="s">
-        <v>60</v>
+        <v>129</v>
       </c>
       <c r="F19" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="G19" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="H19">
-        <v>15771</v>
+        <v>143550</v>
       </c>
       <c r="I19">
-        <v>751000</v>
+        <v>7250000</v>
       </c>
       <c r="J19">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>100</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D20" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E20" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F20" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G20" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H20">
         <v>29700</v>
@@ -3992,34 +4119,34 @@
     </row>
     <row r="21" spans="1:12">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B21" t="s">
-        <v>71</v>
+        <v>26</v>
       </c>
       <c r="C21" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E21" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F21" t="s">
+        <v>72</v>
+      </c>
+      <c r="G21" t="s">
         <v>23</v>
       </c>
-      <c r="G21" t="s">
-        <v>21</v>
-      </c>
       <c r="H21">
-        <v>21700</v>
+        <v>15771</v>
       </c>
       <c r="I21">
-        <v>1400000</v>
+        <v>751000</v>
       </c>
       <c r="J21">
-        <v>15500</v>
+        <v>21000</v>
       </c>
       <c r="K21">
         <v>0</v>
@@ -4030,34 +4157,34 @@
     </row>
     <row r="22" spans="1:12">
       <c r="A22" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B22" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C22" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D22" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="E22" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F22" t="s">
         <v>24</v>
       </c>
       <c r="G22" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H22">
-        <v>29000</v>
+        <v>21700</v>
       </c>
       <c r="I22">
-        <v>1000000</v>
+        <v>1400000</v>
       </c>
       <c r="J22">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -4068,34 +4195,34 @@
     </row>
     <row r="23" spans="1:12">
       <c r="A23" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C23" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D23" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E23" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F23" t="s">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="G23" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="H23">
-        <v>13000</v>
+        <v>29000</v>
       </c>
       <c r="I23">
         <v>1000000</v>
       </c>
       <c r="J23">
-        <v>13000</v>
+        <v>29000</v>
       </c>
       <c r="K23">
         <v>0</v>
@@ -4106,39 +4233,77 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B24" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C24" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="D24" t="s">
-        <v>102</v>
+        <v>59</v>
       </c>
       <c r="E24" t="s">
-        <v>125</v>
+        <v>59</v>
       </c>
       <c r="F24" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G24" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H24">
-        <v>143550</v>
+        <v>13000</v>
       </c>
       <c r="I24">
-        <v>7250000</v>
+        <v>1000000</v>
       </c>
       <c r="J24">
-        <v>60000</v>
+        <v>13000</v>
       </c>
       <c r="K24">
         <v>0</v>
       </c>
       <c r="L24">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" t="s">
+        <v>59</v>
+      </c>
+      <c r="B25" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25" t="s">
+        <v>105</v>
+      </c>
+      <c r="E25" t="s">
+        <v>129</v>
+      </c>
+      <c r="F25" t="s">
+        <v>87</v>
+      </c>
+      <c r="G25" t="s">
+        <v>32</v>
+      </c>
+      <c r="H25">
+        <v>143550</v>
+      </c>
+      <c r="I25">
+        <v>7250000</v>
+      </c>
+      <c r="J25">
+        <v>60000</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
         <v>33</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-04
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="118">
   <si>
     <t>상장일</t>
   </si>
@@ -114,12 +114,6 @@
     <t>2024-07-15</t>
   </si>
   <si>
-    <t>2024-07-11</t>
-  </si>
-  <si>
-    <t>2024-07-12</t>
-  </si>
-  <si>
     <t>아이스크림미디어</t>
   </si>
   <si>
@@ -171,12 +165,6 @@
     <t>엑셀세라퓨틱스</t>
   </si>
   <si>
-    <t>시프트업</t>
-  </si>
-  <si>
-    <t>이베스트스팩6호</t>
-  </si>
-  <si>
     <t>코스닥</t>
   </si>
   <si>
@@ -216,15 +204,6 @@
     <t>SK</t>
   </si>
   <si>
-    <t>제이피모간회사</t>
-  </si>
-  <si>
-    <t>신한</t>
-  </si>
-  <si>
-    <t>LS</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -258,9 +237,6 @@
     <t>2024-07-03</t>
   </si>
   <si>
-    <t>2024-07-02</t>
-  </si>
-  <si>
     <t>2024-08-26</t>
   </si>
   <si>
@@ -279,9 +255,6 @@
     <t>2024-07-08</t>
   </si>
   <si>
-    <t>2024-07-05</t>
-  </si>
-  <si>
     <t>회사명</t>
   </si>
   <si>
@@ -333,12 +306,6 @@
     <t>수수료율</t>
   </si>
   <si>
-    <t>한국, 제이피모간회사 서울지점, NH</t>
-  </si>
-  <si>
-    <t>엘에스</t>
-  </si>
-  <si>
     <t>12.89 : 1</t>
   </si>
   <si>
@@ -390,12 +357,6 @@
     <t>517.7 : 1</t>
   </si>
   <si>
-    <t>341.24 : 1</t>
-  </si>
-  <si>
-    <t>107.32 : 1</t>
-  </si>
-  <si>
     <t>인수기관</t>
   </si>
   <si>
@@ -403,9 +364,6 @@
   </si>
   <si>
     <t>인수비율</t>
-  </si>
-  <si>
-    <t>한국, 제이피모간회사 서울지점, NH, 신한</t>
   </si>
   <si>
     <t>미래, 삼성</t>
@@ -769,7 +727,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -830,37 +788,37 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D2">
         <v>787.2</v>
       </c>
       <c r="E2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F2">
         <v>787.2</v>
       </c>
       <c r="G2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M2">
         <v>32000</v>
@@ -872,7 +830,7 @@
         <v>20</v>
       </c>
       <c r="P2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="Q2">
         <v>1722000</v>
@@ -883,37 +841,37 @@
         <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D3">
         <v>240</v>
       </c>
       <c r="E3" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F3">
         <v>228</v>
       </c>
       <c r="G3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K3" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M3">
         <v>16000</v>
@@ -936,37 +894,37 @@
         <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D4">
         <v>240</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F4">
         <v>12</v>
       </c>
       <c r="G4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K4" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="L4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M4">
         <v>16000</v>
@@ -989,37 +947,37 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D5">
         <v>239.7204</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F5">
         <v>239.7204</v>
       </c>
       <c r="G5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K5" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M5">
         <v>15300</v>
@@ -1042,37 +1000,37 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D6">
         <v>130</v>
       </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F6">
         <v>130</v>
       </c>
       <c r="G6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K6" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M6">
         <v>13000</v>
@@ -1081,10 +1039,10 @@
         <v>100</v>
       </c>
       <c r="O6" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="P6" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="Q6">
         <v>723700</v>
@@ -1095,37 +1053,37 @@
         <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D7">
         <v>130</v>
       </c>
       <c r="E7" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F7">
         <v>130</v>
       </c>
       <c r="G7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K7" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M7">
         <v>2000</v>
@@ -1134,10 +1092,10 @@
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="P7" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="Q7">
         <v>4875000</v>
@@ -1148,37 +1106,37 @@
         <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D8">
         <v>507.81225</v>
       </c>
       <c r="E8" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F8">
         <v>507.81225</v>
       </c>
       <c r="G8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K8" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M8">
         <v>16500</v>
@@ -1187,7 +1145,7 @@
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="P8" t="s">
         <v>24</v>
@@ -1201,37 +1159,37 @@
         <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D9">
         <v>217</v>
       </c>
       <c r="E9" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F9">
         <v>217</v>
       </c>
       <c r="G9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K9" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M9">
         <v>15500</v>
@@ -1240,7 +1198,7 @@
         <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="P9" t="s">
         <v>24</v>
@@ -1254,37 +1212,37 @@
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D10">
         <v>290</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F10">
         <v>290</v>
       </c>
       <c r="G10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K10" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M10">
         <v>29000</v>
@@ -1293,7 +1251,7 @@
         <v>100</v>
       </c>
       <c r="O10" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="P10" t="s">
         <v>25</v>
@@ -1307,37 +1265,37 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D11">
         <v>157.71</v>
       </c>
       <c r="E11" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F11">
         <v>157.71</v>
       </c>
       <c r="G11" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H11" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I11" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J11" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K11" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L11" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M11">
         <v>21000</v>
@@ -1349,7 +1307,7 @@
         <v>26</v>
       </c>
       <c r="P11" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="Q11">
         <v>540250</v>
@@ -1360,37 +1318,37 @@
         <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D12">
         <v>116</v>
       </c>
       <c r="E12" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F12">
         <v>116</v>
       </c>
       <c r="G12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K12" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M12">
         <v>2000</v>
@@ -1399,7 +1357,7 @@
         <v>100</v>
       </c>
       <c r="O12" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="P12" t="s">
         <v>26</v>
@@ -1413,37 +1371,37 @@
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D13">
         <v>224</v>
       </c>
       <c r="E13" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F13">
         <v>224</v>
       </c>
       <c r="G13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K13" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M13">
         <v>16000</v>
@@ -1452,7 +1410,7 @@
         <v>100</v>
       </c>
       <c r="O13" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="P13" t="s">
         <v>26</v>
@@ -1466,37 +1424,37 @@
         <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D14">
         <v>223.4</v>
       </c>
       <c r="E14" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F14">
         <v>223.4</v>
       </c>
       <c r="G14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K14" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M14">
         <v>10000</v>
@@ -1508,7 +1466,7 @@
         <v>30</v>
       </c>
       <c r="P14" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="Q14">
         <v>1675500</v>
@@ -1519,37 +1477,37 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D15">
         <v>297</v>
       </c>
       <c r="E15" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F15">
         <v>297</v>
       </c>
       <c r="G15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K15" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M15">
         <v>22000</v>
@@ -1558,7 +1516,7 @@
         <v>100</v>
       </c>
       <c r="O15" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="P15" t="s">
         <v>30</v>
@@ -1572,37 +1530,37 @@
         <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D16">
         <v>2660</v>
       </c>
       <c r="E16" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F16">
         <v>2553.6</v>
       </c>
       <c r="G16" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H16" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I16" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J16" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K16" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L16" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M16">
         <v>35000</v>
@@ -1611,10 +1569,10 @@
         <v>96</v>
       </c>
       <c r="O16" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="P16" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="Q16">
         <v>9340690</v>
@@ -1625,37 +1583,37 @@
         <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C17" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D17">
         <v>2660</v>
       </c>
       <c r="E17" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F17">
         <v>106.4</v>
       </c>
       <c r="G17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K17" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="L17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M17">
         <v>35000</v>
@@ -1664,10 +1622,10 @@
         <v>4</v>
       </c>
       <c r="O17" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="P17" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="Q17">
         <v>9340690</v>
@@ -1678,37 +1636,37 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D18">
         <v>120</v>
       </c>
       <c r="E18" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F18">
         <v>120</v>
       </c>
       <c r="G18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K18" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M18">
         <v>2000</v>
@@ -1717,10 +1675,10 @@
         <v>100</v>
       </c>
       <c r="O18" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="P18" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="Q18">
         <v>4500000</v>
@@ -1731,37 +1689,37 @@
         <v>30</v>
       </c>
       <c r="B19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" t="s">
         <v>49</v>
-      </c>
-      <c r="C19" t="s">
-        <v>53</v>
       </c>
       <c r="D19">
         <v>80</v>
       </c>
       <c r="E19" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F19">
         <v>80</v>
       </c>
       <c r="G19" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H19" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I19" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J19" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K19" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L19" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M19">
         <v>2000</v>
@@ -1773,7 +1731,7 @@
         <v>31</v>
       </c>
       <c r="P19" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="Q19">
         <v>3000000</v>
@@ -1784,37 +1742,37 @@
         <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C20" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D20">
         <v>161.8</v>
       </c>
       <c r="E20" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F20">
         <v>161.8</v>
       </c>
       <c r="G20" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H20" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I20" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J20" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K20" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L20" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M20">
         <v>10000</v>
@@ -1823,278 +1781,13 @@
         <v>100</v>
       </c>
       <c r="O20" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="P20" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="Q20">
         <v>1187900</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17">
-      <c r="A21" t="s">
-        <v>32</v>
-      </c>
-      <c r="B21" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" t="s">
-        <v>54</v>
-      </c>
-      <c r="D21">
-        <v>4350</v>
-      </c>
-      <c r="E21" t="s">
-        <v>59</v>
-      </c>
-      <c r="F21">
-        <v>1435.5</v>
-      </c>
-      <c r="G21" t="s">
-        <v>69</v>
-      </c>
-      <c r="H21" t="s">
-        <v>69</v>
-      </c>
-      <c r="I21" t="s">
-        <v>69</v>
-      </c>
-      <c r="J21" t="s">
-        <v>69</v>
-      </c>
-      <c r="K21" t="s">
-        <v>70</v>
-      </c>
-      <c r="L21" t="s">
-        <v>69</v>
-      </c>
-      <c r="M21">
-        <v>60000</v>
-      </c>
-      <c r="N21">
-        <v>33</v>
-      </c>
-      <c r="O21" t="s">
-        <v>80</v>
-      </c>
-      <c r="P21" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q21">
-        <v>21750000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17">
-      <c r="A22" t="s">
-        <v>32</v>
-      </c>
-      <c r="B22" t="s">
-        <v>51</v>
-      </c>
-      <c r="C22" t="s">
-        <v>54</v>
-      </c>
-      <c r="D22">
-        <v>4350</v>
-      </c>
-      <c r="E22" t="s">
-        <v>66</v>
-      </c>
-      <c r="F22">
-        <v>1435.5</v>
-      </c>
-      <c r="G22" t="s">
-        <v>69</v>
-      </c>
-      <c r="H22" t="s">
-        <v>69</v>
-      </c>
-      <c r="I22" t="s">
-        <v>69</v>
-      </c>
-      <c r="J22" t="s">
-        <v>69</v>
-      </c>
-      <c r="K22" t="s">
-        <v>70</v>
-      </c>
-      <c r="L22" t="s">
-        <v>69</v>
-      </c>
-      <c r="M22">
-        <v>60000</v>
-      </c>
-      <c r="N22">
-        <v>33</v>
-      </c>
-      <c r="O22" t="s">
-        <v>80</v>
-      </c>
-      <c r="P22" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q22">
-        <v>21750000</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17">
-      <c r="A23" t="s">
-        <v>32</v>
-      </c>
-      <c r="B23" t="s">
-        <v>51</v>
-      </c>
-      <c r="C23" t="s">
-        <v>54</v>
-      </c>
-      <c r="D23">
-        <v>4350</v>
-      </c>
-      <c r="E23" t="s">
-        <v>58</v>
-      </c>
-      <c r="F23">
-        <v>1305</v>
-      </c>
-      <c r="G23" t="s">
-        <v>69</v>
-      </c>
-      <c r="H23" t="s">
-        <v>69</v>
-      </c>
-      <c r="I23" t="s">
-        <v>69</v>
-      </c>
-      <c r="J23" t="s">
-        <v>69</v>
-      </c>
-      <c r="K23" t="s">
-        <v>70</v>
-      </c>
-      <c r="L23" t="s">
-        <v>69</v>
-      </c>
-      <c r="M23">
-        <v>60000</v>
-      </c>
-      <c r="N23">
-        <v>30</v>
-      </c>
-      <c r="O23" t="s">
-        <v>80</v>
-      </c>
-      <c r="P23" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q23">
-        <v>21750000</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17">
-      <c r="A24" t="s">
-        <v>32</v>
-      </c>
-      <c r="B24" t="s">
-        <v>51</v>
-      </c>
-      <c r="C24" t="s">
-        <v>54</v>
-      </c>
-      <c r="D24">
-        <v>4350</v>
-      </c>
-      <c r="E24" t="s">
-        <v>67</v>
-      </c>
-      <c r="F24">
-        <v>174</v>
-      </c>
-      <c r="G24" t="s">
-        <v>69</v>
-      </c>
-      <c r="H24" t="s">
-        <v>69</v>
-      </c>
-      <c r="I24" t="s">
-        <v>69</v>
-      </c>
-      <c r="J24" t="s">
-        <v>69</v>
-      </c>
-      <c r="K24" t="s">
-        <v>71</v>
-      </c>
-      <c r="L24" t="s">
-        <v>69</v>
-      </c>
-      <c r="M24">
-        <v>60000</v>
-      </c>
-      <c r="N24">
-        <v>4</v>
-      </c>
-      <c r="O24" t="s">
-        <v>80</v>
-      </c>
-      <c r="P24" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q24">
-        <v>21750000</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17">
-      <c r="A25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B25" t="s">
-        <v>52</v>
-      </c>
-      <c r="C25" t="s">
-        <v>53</v>
-      </c>
-      <c r="D25">
-        <v>80</v>
-      </c>
-      <c r="E25" t="s">
-        <v>68</v>
-      </c>
-      <c r="F25">
-        <v>80</v>
-      </c>
-      <c r="G25" t="s">
-        <v>69</v>
-      </c>
-      <c r="H25" t="s">
-        <v>69</v>
-      </c>
-      <c r="I25" t="s">
-        <v>69</v>
-      </c>
-      <c r="J25" t="s">
-        <v>69</v>
-      </c>
-      <c r="K25" t="s">
-        <v>70</v>
-      </c>
-      <c r="L25" t="s">
-        <v>69</v>
-      </c>
-      <c r="M25">
-        <v>2000</v>
-      </c>
-      <c r="N25">
-        <v>100</v>
-      </c>
-      <c r="O25" t="s">
-        <v>80</v>
-      </c>
-      <c r="P25" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q25">
-        <v>3000000</v>
       </c>
     </row>
   </sheetData>
@@ -2104,7 +1797,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:T18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -2112,10 +1805,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -2124,49 +1817,49 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:20">
@@ -2174,13 +1867,13 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
@@ -2192,7 +1885,7 @@
         <v>2460000</v>
       </c>
       <c r="H2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I2">
         <v>32000</v>
@@ -2201,34 +1894,34 @@
         <v>40200</v>
       </c>
       <c r="K2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L2">
         <v>32000</v>
       </c>
       <c r="M2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R2" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="S2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -2236,10 +1929,10 @@
         <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D3" t="s">
         <v>23</v>
@@ -2254,7 +1947,7 @@
         <v>1500000</v>
       </c>
       <c r="H3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I3">
         <v>11000</v>
@@ -2263,34 +1956,34 @@
         <v>13000</v>
       </c>
       <c r="K3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L3">
         <v>16000</v>
       </c>
       <c r="M3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R3" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="S3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T3" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -2298,10 +1991,10 @@
         <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D4" t="s">
         <v>23</v>
@@ -2316,7 +2009,7 @@
         <v>1566800</v>
       </c>
       <c r="H4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I4">
         <v>13600</v>
@@ -2325,48 +2018,48 @@
         <v>15300</v>
       </c>
       <c r="K4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L4">
         <v>15300</v>
       </c>
       <c r="M4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R4" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="S4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D5" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="E5" t="s">
         <v>20</v>
@@ -2378,7 +2071,7 @@
         <v>1000000</v>
       </c>
       <c r="H5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I5">
         <v>9500</v>
@@ -2387,48 +2080,48 @@
         <v>10700</v>
       </c>
       <c r="K5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L5">
         <v>13000</v>
       </c>
       <c r="M5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O5">
         <v>50</v>
       </c>
       <c r="P5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R5" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="S5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D6" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="E6" t="s">
         <v>18</v>
@@ -2440,7 +2133,7 @@
         <v>6500000</v>
       </c>
       <c r="H6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I6">
         <v>2000</v>
@@ -2449,45 +2142,45 @@
         <v>2000</v>
       </c>
       <c r="K6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L6">
         <v>2000</v>
       </c>
       <c r="M6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R6" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="S6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D7" t="s">
         <v>24</v>
@@ -2502,7 +2195,7 @@
         <v>3077650</v>
       </c>
       <c r="H7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I7">
         <v>13800</v>
@@ -2511,45 +2204,45 @@
         <v>15700</v>
       </c>
       <c r="K7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L7">
         <v>16500</v>
       </c>
       <c r="M7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O7">
         <v>100</v>
       </c>
       <c r="P7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R7" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="S7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D8" t="s">
         <v>24</v>
@@ -2564,7 +2257,7 @@
         <v>1400000</v>
       </c>
       <c r="H8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I8">
         <v>12500</v>
@@ -2573,45 +2266,45 @@
         <v>15500</v>
       </c>
       <c r="K8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L8">
         <v>15500</v>
       </c>
       <c r="M8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R8" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="S8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
         <v>25</v>
@@ -2626,7 +2319,7 @@
         <v>1000000</v>
       </c>
       <c r="H9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I9">
         <v>24000</v>
@@ -2635,34 +2328,34 @@
         <v>29000</v>
       </c>
       <c r="K9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L9">
         <v>29000</v>
       </c>
       <c r="M9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O9">
         <v>0</v>
       </c>
       <c r="P9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R9" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="S9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -2670,13 +2363,13 @@
         <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="E10" t="s">
         <v>23</v>
@@ -2688,7 +2381,7 @@
         <v>751000</v>
       </c>
       <c r="H10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I10">
         <v>18000</v>
@@ -2697,45 +2390,45 @@
         <v>21000</v>
       </c>
       <c r="K10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L10">
         <v>21000</v>
       </c>
       <c r="M10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O10">
         <v>72.87616511318242</v>
       </c>
       <c r="P10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R10" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="S10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D11" t="s">
         <v>26</v>
@@ -2750,7 +2443,7 @@
         <v>5800000</v>
       </c>
       <c r="H11" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I11">
         <v>2000</v>
@@ -2759,45 +2452,45 @@
         <v>2000</v>
       </c>
       <c r="K11" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L11">
         <v>2000</v>
       </c>
       <c r="M11" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N11" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O11">
         <v>0</v>
       </c>
       <c r="P11" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q11" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R11" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="S11" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T11" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D12" t="s">
         <v>26</v>
@@ -2812,7 +2505,7 @@
         <v>1400000</v>
       </c>
       <c r="H12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I12">
         <v>16000</v>
@@ -2821,34 +2514,34 @@
         <v>19000</v>
       </c>
       <c r="K12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L12">
         <v>16000</v>
       </c>
       <c r="M12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O12">
         <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R12" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="S12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T12" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -2856,13 +2549,13 @@
         <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D13" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="E13" t="s">
         <v>26</v>
@@ -2874,7 +2567,7 @@
         <v>2234000</v>
       </c>
       <c r="H13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I13">
         <v>7300</v>
@@ -2883,45 +2576,45 @@
         <v>8500</v>
       </c>
       <c r="K13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L13">
         <v>10000</v>
       </c>
       <c r="M13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O13">
         <v>0</v>
       </c>
       <c r="P13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R13" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="S13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D14" t="s">
         <v>30</v>
@@ -2936,7 +2629,7 @@
         <v>1350000</v>
       </c>
       <c r="H14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I14">
         <v>14000</v>
@@ -2945,48 +2638,48 @@
         <v>17000</v>
       </c>
       <c r="K14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L14">
         <v>22000</v>
       </c>
       <c r="M14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O14">
         <v>0</v>
       </c>
       <c r="P14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R14" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="S14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="B15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D15" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="E15" t="s">
         <v>28</v>
@@ -2998,7 +2691,7 @@
         <v>7600000</v>
       </c>
       <c r="H15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I15">
         <v>24000</v>
@@ -3007,48 +2700,48 @@
         <v>30000</v>
       </c>
       <c r="K15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L15">
         <v>35000</v>
       </c>
       <c r="M15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O15">
         <v>14.47368421052632</v>
       </c>
       <c r="P15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R15" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="S15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:20">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D16" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
@@ -3060,7 +2753,7 @@
         <v>6000000</v>
       </c>
       <c r="H16" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I16">
         <v>2000</v>
@@ -3069,34 +2762,34 @@
         <v>2000</v>
       </c>
       <c r="K16" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L16">
         <v>2000</v>
       </c>
       <c r="M16" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N16" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O16">
         <v>0</v>
       </c>
       <c r="P16" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q16" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R16" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="S16" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T16" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:20">
@@ -3104,13 +2797,13 @@
         <v>31</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="E17" t="s">
         <v>30</v>
@@ -3122,7 +2815,7 @@
         <v>4000000</v>
       </c>
       <c r="H17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I17">
         <v>2000</v>
@@ -3131,48 +2824,48 @@
         <v>2000</v>
       </c>
       <c r="K17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L17">
         <v>2000</v>
       </c>
       <c r="M17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O17">
         <v>0</v>
       </c>
       <c r="P17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R17" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="S17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T17" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:20">
       <c r="A18" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D18" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="E18" t="s">
         <v>31</v>
@@ -3184,7 +2877,7 @@
         <v>1618000</v>
       </c>
       <c r="H18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I18">
         <v>6200</v>
@@ -3193,158 +2886,34 @@
         <v>7700</v>
       </c>
       <c r="K18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L18">
         <v>10000</v>
       </c>
       <c r="M18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="N18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="O18">
         <v>0</v>
       </c>
       <c r="P18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="Q18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="R18" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="S18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="T18" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20">
-      <c r="A19" t="s">
-        <v>80</v>
-      </c>
-      <c r="B19" t="s">
-        <v>51</v>
-      </c>
-      <c r="C19" t="s">
-        <v>105</v>
-      </c>
-      <c r="D19" t="s">
-        <v>87</v>
-      </c>
-      <c r="E19" t="s">
-        <v>32</v>
-      </c>
-      <c r="F19">
-        <v>435000000</v>
-      </c>
-      <c r="G19">
-        <v>7250000</v>
-      </c>
-      <c r="H19" t="s">
-        <v>69</v>
-      </c>
-      <c r="I19">
-        <v>47000</v>
-      </c>
-      <c r="J19">
-        <v>60000</v>
-      </c>
-      <c r="K19" t="s">
-        <v>69</v>
-      </c>
-      <c r="L19">
-        <v>60000</v>
-      </c>
-      <c r="M19" t="s">
-        <v>69</v>
-      </c>
-      <c r="N19" t="s">
-        <v>69</v>
-      </c>
-      <c r="O19">
-        <v>0</v>
-      </c>
-      <c r="P19" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q19" t="s">
-        <v>69</v>
-      </c>
-      <c r="R19" t="s">
-        <v>124</v>
-      </c>
-      <c r="S19" t="s">
-        <v>69</v>
-      </c>
-      <c r="T19" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20">
-      <c r="A20" t="s">
-        <v>80</v>
-      </c>
-      <c r="B20" t="s">
-        <v>52</v>
-      </c>
-      <c r="C20" t="s">
-        <v>106</v>
-      </c>
-      <c r="D20" t="s">
-        <v>87</v>
-      </c>
-      <c r="E20" t="s">
-        <v>33</v>
-      </c>
-      <c r="F20">
-        <v>8000000</v>
-      </c>
-      <c r="G20">
-        <v>4000000</v>
-      </c>
-      <c r="H20" t="s">
-        <v>69</v>
-      </c>
-      <c r="I20">
-        <v>2000</v>
-      </c>
-      <c r="J20">
-        <v>2000</v>
-      </c>
-      <c r="K20" t="s">
-        <v>69</v>
-      </c>
-      <c r="L20">
-        <v>2000</v>
-      </c>
-      <c r="M20" t="s">
-        <v>69</v>
-      </c>
-      <c r="N20" t="s">
-        <v>69</v>
-      </c>
-      <c r="O20">
-        <v>0</v>
-      </c>
-      <c r="P20" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>69</v>
-      </c>
-      <c r="R20" t="s">
-        <v>125</v>
-      </c>
-      <c r="S20" t="s">
-        <v>69</v>
-      </c>
-      <c r="T20" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -3354,21 +2923,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -3380,10 +2949,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -3392,36 +2961,36 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>106</v>
+        <v>54</v>
       </c>
       <c r="E2" t="s">
-        <v>106</v>
+        <v>54</v>
       </c>
       <c r="F2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="G2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="H2">
-        <v>8000</v>
+        <v>12000</v>
       </c>
       <c r="I2">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="J2">
         <v>2000</v>
@@ -3435,72 +3004,72 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>105</v>
+        <v>54</v>
       </c>
       <c r="E3" t="s">
-        <v>129</v>
+        <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="H3">
-        <v>130500</v>
+        <v>23972.04</v>
       </c>
       <c r="I3">
-        <v>7250000</v>
+        <v>1566800</v>
       </c>
       <c r="J3">
-        <v>60000</v>
+        <v>15300</v>
       </c>
       <c r="K3">
         <v>0</v>
       </c>
       <c r="L3">
-        <v>30</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="D4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>70</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="H4">
-        <v>23972.04</v>
+        <v>8000</v>
       </c>
       <c r="I4">
-        <v>1566800</v>
+        <v>4000000</v>
       </c>
       <c r="J4">
-        <v>15300</v>
+        <v>2000</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -3511,31 +3080,31 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F5" t="s">
-        <v>85</v>
+        <v>26</v>
       </c>
       <c r="G5" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="H5">
-        <v>12000</v>
+        <v>11600</v>
       </c>
       <c r="I5">
-        <v>6000000</v>
+        <v>5800000</v>
       </c>
       <c r="J5">
         <v>2000</v>
@@ -3549,34 +3118,34 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="B6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G6" t="s">
         <v>31</v>
       </c>
-      <c r="C6" t="s">
-        <v>49</v>
-      </c>
-      <c r="D6" t="s">
-        <v>65</v>
-      </c>
-      <c r="E6" t="s">
-        <v>65</v>
-      </c>
-      <c r="F6" t="s">
-        <v>77</v>
-      </c>
-      <c r="G6" t="s">
-        <v>30</v>
-      </c>
       <c r="H6">
-        <v>8000</v>
+        <v>16180</v>
       </c>
       <c r="I6">
-        <v>4000000</v>
+        <v>1618000</v>
       </c>
       <c r="J6">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -3587,31 +3156,31 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="B7" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E7" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="F7" t="s">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="G7" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="H7">
-        <v>11600</v>
+        <v>13000</v>
       </c>
       <c r="I7">
-        <v>5800000</v>
+        <v>6500000</v>
       </c>
       <c r="J7">
         <v>2000</v>
@@ -3625,72 +3194,72 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D8" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>116</v>
       </c>
       <c r="F8" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="G8" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H8">
-        <v>16180</v>
+        <v>255360</v>
       </c>
       <c r="I8">
-        <v>1618000</v>
+        <v>7600000</v>
       </c>
       <c r="J8">
-        <v>10000</v>
+        <v>35000</v>
       </c>
       <c r="K8">
         <v>0</v>
       </c>
       <c r="L8">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F9" t="s">
-        <v>82</v>
+        <v>24</v>
       </c>
       <c r="G9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H9">
-        <v>13000</v>
+        <v>50781.225</v>
       </c>
       <c r="I9">
-        <v>6500000</v>
+        <v>3077650</v>
       </c>
       <c r="J9">
-        <v>2000</v>
+        <v>16500</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -3701,110 +3270,110 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E10" t="s">
-        <v>130</v>
+        <v>57</v>
       </c>
       <c r="F10" t="s">
-        <v>84</v>
+        <v>26</v>
       </c>
       <c r="G10" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H10">
-        <v>255360</v>
+        <v>22400</v>
       </c>
       <c r="I10">
-        <v>7600000</v>
+        <v>1400000</v>
       </c>
       <c r="J10">
-        <v>35000</v>
+        <v>16000</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B11" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D11" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E11" t="s">
-        <v>61</v>
+        <v>116</v>
       </c>
       <c r="F11" t="s">
-        <v>26</v>
+        <v>76</v>
       </c>
       <c r="G11" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="H11">
-        <v>22400</v>
+        <v>10640</v>
       </c>
       <c r="I11">
-        <v>1400000</v>
+        <v>7600000</v>
       </c>
       <c r="J11">
-        <v>16000</v>
+        <v>35000</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B12" t="s">
-        <v>73</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E12" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="F12" t="s">
-        <v>24</v>
+        <v>75</v>
       </c>
       <c r="G12" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="H12">
-        <v>50781.225</v>
+        <v>22340</v>
       </c>
       <c r="I12">
-        <v>3077650</v>
+        <v>2234000</v>
       </c>
       <c r="J12">
-        <v>16500</v>
+        <v>10000</v>
       </c>
       <c r="K12">
         <v>0</v>
@@ -3815,34 +3384,34 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E13" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F13" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="G13" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="H13">
-        <v>22340</v>
+        <v>78720</v>
       </c>
       <c r="I13">
-        <v>2234000</v>
+        <v>2460000</v>
       </c>
       <c r="J13">
-        <v>10000</v>
+        <v>32000</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -3853,458 +3422,268 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B14" t="s">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="D14" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E14" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="F14" t="s">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="G14" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="H14">
-        <v>10640</v>
+        <v>22800</v>
       </c>
       <c r="I14">
-        <v>7600000</v>
+        <v>1500000</v>
       </c>
       <c r="J14">
-        <v>35000</v>
+        <v>16000</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14">
-        <v>4</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B15" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D15" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E15" t="s">
-        <v>55</v>
+        <v>117</v>
       </c>
       <c r="F15" t="s">
-        <v>81</v>
+        <v>23</v>
       </c>
       <c r="G15" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H15">
-        <v>78720</v>
+        <v>1200</v>
       </c>
       <c r="I15">
-        <v>2460000</v>
+        <v>1500000</v>
       </c>
       <c r="J15">
-        <v>32000</v>
+        <v>16000</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>100</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B16" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="D16" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E16" t="s">
-        <v>131</v>
+        <v>59</v>
       </c>
       <c r="F16" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="G16" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="H16">
-        <v>22800</v>
+        <v>29700</v>
       </c>
       <c r="I16">
-        <v>1500000</v>
+        <v>1350000</v>
       </c>
       <c r="J16">
-        <v>16000</v>
+        <v>22000</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B17" t="s">
-        <v>80</v>
+        <v>26</v>
       </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="D17" t="s">
-        <v>105</v>
+        <v>59</v>
       </c>
       <c r="E17" t="s">
-        <v>129</v>
+        <v>59</v>
       </c>
       <c r="F17" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="G17" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="H17">
-        <v>17400</v>
+        <v>15771</v>
       </c>
       <c r="I17">
-        <v>7250000</v>
+        <v>751000</v>
       </c>
       <c r="J17">
-        <v>60000</v>
+        <v>21000</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
       <c r="L17">
-        <v>4</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="C18" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D18" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E18" t="s">
-        <v>131</v>
+        <v>58</v>
       </c>
       <c r="F18" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G18" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="H18">
-        <v>1200</v>
+        <v>21700</v>
       </c>
       <c r="I18">
-        <v>1500000</v>
+        <v>1400000</v>
       </c>
       <c r="J18">
-        <v>16000</v>
+        <v>15500</v>
       </c>
       <c r="K18">
         <v>0</v>
       </c>
       <c r="L18">
-        <v>5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="B19" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="C19" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="D19" t="s">
-        <v>105</v>
+        <v>55</v>
       </c>
       <c r="E19" t="s">
-        <v>129</v>
+        <v>55</v>
       </c>
       <c r="F19" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="G19" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="H19">
-        <v>143550</v>
+        <v>13000</v>
       </c>
       <c r="I19">
-        <v>7250000</v>
+        <v>1000000</v>
       </c>
       <c r="J19">
-        <v>60000</v>
+        <v>13000</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>33</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="C20" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="D20" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="E20" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="F20" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G20" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="H20">
-        <v>29700</v>
+        <v>29000</v>
       </c>
       <c r="I20">
-        <v>1350000</v>
+        <v>1000000</v>
       </c>
       <c r="J20">
-        <v>22000</v>
+        <v>29000</v>
       </c>
       <c r="K20">
         <v>0</v>
       </c>
       <c r="L20">
         <v>100</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12">
-      <c r="A21" t="s">
-        <v>63</v>
-      </c>
-      <c r="B21" t="s">
-        <v>26</v>
-      </c>
-      <c r="C21" t="s">
-        <v>42</v>
-      </c>
-      <c r="D21" t="s">
-        <v>63</v>
-      </c>
-      <c r="E21" t="s">
-        <v>63</v>
-      </c>
-      <c r="F21" t="s">
-        <v>72</v>
-      </c>
-      <c r="G21" t="s">
-        <v>23</v>
-      </c>
-      <c r="H21">
-        <v>15771</v>
-      </c>
-      <c r="I21">
-        <v>751000</v>
-      </c>
-      <c r="J21">
-        <v>21000</v>
-      </c>
-      <c r="K21">
-        <v>0</v>
-      </c>
-      <c r="L21">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12">
-      <c r="A22" t="s">
-        <v>62</v>
-      </c>
-      <c r="B22" t="s">
-        <v>73</v>
-      </c>
-      <c r="C22" t="s">
-        <v>40</v>
-      </c>
-      <c r="D22" t="s">
-        <v>62</v>
-      </c>
-      <c r="E22" t="s">
-        <v>62</v>
-      </c>
-      <c r="F22" t="s">
-        <v>24</v>
-      </c>
-      <c r="G22" t="s">
-        <v>22</v>
-      </c>
-      <c r="H22">
-        <v>21700</v>
-      </c>
-      <c r="I22">
-        <v>1400000</v>
-      </c>
-      <c r="J22">
-        <v>15500</v>
-      </c>
-      <c r="K22">
-        <v>0</v>
-      </c>
-      <c r="L22">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12">
-      <c r="A23" t="s">
-        <v>59</v>
-      </c>
-      <c r="B23" t="s">
-        <v>74</v>
-      </c>
-      <c r="C23" t="s">
-        <v>41</v>
-      </c>
-      <c r="D23" t="s">
-        <v>59</v>
-      </c>
-      <c r="E23" t="s">
-        <v>59</v>
-      </c>
-      <c r="F23" t="s">
-        <v>25</v>
-      </c>
-      <c r="G23" t="s">
-        <v>22</v>
-      </c>
-      <c r="H23">
-        <v>29000</v>
-      </c>
-      <c r="I23">
-        <v>1000000</v>
-      </c>
-      <c r="J23">
-        <v>29000</v>
-      </c>
-      <c r="K23">
-        <v>0</v>
-      </c>
-      <c r="L23">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12">
-      <c r="A24" t="s">
-        <v>59</v>
-      </c>
-      <c r="B24" t="s">
-        <v>72</v>
-      </c>
-      <c r="C24" t="s">
-        <v>37</v>
-      </c>
-      <c r="D24" t="s">
-        <v>59</v>
-      </c>
-      <c r="E24" t="s">
-        <v>59</v>
-      </c>
-      <c r="F24" t="s">
-        <v>82</v>
-      </c>
-      <c r="G24" t="s">
-        <v>20</v>
-      </c>
-      <c r="H24">
-        <v>13000</v>
-      </c>
-      <c r="I24">
-        <v>1000000</v>
-      </c>
-      <c r="J24">
-        <v>13000</v>
-      </c>
-      <c r="K24">
-        <v>0</v>
-      </c>
-      <c r="L24">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12">
-      <c r="A25" t="s">
-        <v>59</v>
-      </c>
-      <c r="B25" t="s">
-        <v>80</v>
-      </c>
-      <c r="C25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D25" t="s">
-        <v>105</v>
-      </c>
-      <c r="E25" t="s">
-        <v>129</v>
-      </c>
-      <c r="F25" t="s">
-        <v>87</v>
-      </c>
-      <c r="G25" t="s">
-        <v>32</v>
-      </c>
-      <c r="H25">
-        <v>143550</v>
-      </c>
-      <c r="I25">
-        <v>7250000</v>
-      </c>
-      <c r="J25">
-        <v>60000</v>
-      </c>
-      <c r="K25">
-        <v>0</v>
-      </c>
-      <c r="L25">
-        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-10
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="114">
   <si>
     <t>상장일</t>
   </si>
@@ -111,132 +111,126 @@
     <t>2024-07-25</t>
   </si>
   <si>
+    <t>아이스크림미디어</t>
+  </si>
+  <si>
+    <t>M83</t>
+  </si>
+  <si>
+    <t>이엔셀</t>
+  </si>
+  <si>
+    <t>티디에스팜</t>
+  </si>
+  <si>
+    <t>대신밸런스제18호스팩</t>
+  </si>
+  <si>
+    <t>전진건설로봇</t>
+  </si>
+  <si>
+    <t>케이쓰리아이</t>
+  </si>
+  <si>
+    <t>넥스트바이오메디컬</t>
+  </si>
+  <si>
+    <t>유라클</t>
+  </si>
+  <si>
+    <t>교보16호스팩</t>
+  </si>
+  <si>
+    <t>뱅크웨어글로벌</t>
+  </si>
+  <si>
+    <t>아이빔테크놀로지</t>
+  </si>
+  <si>
+    <t>피앤에스미캐닉스</t>
+  </si>
+  <si>
+    <t>산일전기</t>
+  </si>
+  <si>
+    <t>엔에이치스팩31호</t>
+  </si>
+  <si>
+    <t>SK증권제13호스팩</t>
+  </si>
+  <si>
+    <t>코스닥</t>
+  </si>
+  <si>
+    <t>코스피</t>
+  </si>
+  <si>
+    <t>삼성</t>
+  </si>
+  <si>
+    <t>신영</t>
+  </si>
+  <si>
+    <t>유진</t>
+  </si>
+  <si>
+    <t>NH</t>
+  </si>
+  <si>
+    <t>한국</t>
+  </si>
+  <si>
+    <t>대신</t>
+  </si>
+  <si>
+    <t>미래</t>
+  </si>
+  <si>
+    <t>하나</t>
+  </si>
+  <si>
+    <t>키움</t>
+  </si>
+  <si>
+    <t>교보</t>
+  </si>
+  <si>
+    <t>SK</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>대표</t>
+  </si>
+  <si>
+    <t>인수</t>
+  </si>
+  <si>
+    <t>2024-08-09</t>
+  </si>
+  <si>
+    <t>2024-08-08</t>
+  </si>
+  <si>
+    <t>2024-08-07</t>
+  </si>
+  <si>
+    <t>2024-08-01</t>
+  </si>
+  <si>
+    <t>2024-07-22</t>
+  </si>
+  <si>
+    <t>2024-07-18</t>
+  </si>
+  <si>
+    <t>2024-07-16</t>
+  </si>
+  <si>
     <t>2024-07-15</t>
   </si>
   <si>
-    <t>아이스크림미디어</t>
-  </si>
-  <si>
-    <t>M83</t>
-  </si>
-  <si>
-    <t>이엔셀</t>
-  </si>
-  <si>
-    <t>티디에스팜</t>
-  </si>
-  <si>
-    <t>대신밸런스제18호스팩</t>
-  </si>
-  <si>
-    <t>전진건설로봇</t>
-  </si>
-  <si>
-    <t>케이쓰리아이</t>
-  </si>
-  <si>
-    <t>넥스트바이오메디컬</t>
-  </si>
-  <si>
-    <t>유라클</t>
-  </si>
-  <si>
-    <t>교보16호스팩</t>
-  </si>
-  <si>
-    <t>뱅크웨어글로벌</t>
-  </si>
-  <si>
-    <t>아이빔테크놀로지</t>
-  </si>
-  <si>
-    <t>피앤에스미캐닉스</t>
-  </si>
-  <si>
-    <t>산일전기</t>
-  </si>
-  <si>
-    <t>엔에이치스팩31호</t>
-  </si>
-  <si>
-    <t>SK증권제13호스팩</t>
-  </si>
-  <si>
-    <t>엑셀세라퓨틱스</t>
-  </si>
-  <si>
-    <t>코스닥</t>
-  </si>
-  <si>
-    <t>코스피</t>
-  </si>
-  <si>
-    <t>삼성</t>
-  </si>
-  <si>
-    <t>신영</t>
-  </si>
-  <si>
-    <t>유진</t>
-  </si>
-  <si>
-    <t>NH</t>
-  </si>
-  <si>
-    <t>한국</t>
-  </si>
-  <si>
-    <t>대신</t>
-  </si>
-  <si>
-    <t>미래</t>
-  </si>
-  <si>
-    <t>하나</t>
-  </si>
-  <si>
-    <t>키움</t>
-  </si>
-  <si>
-    <t>교보</t>
-  </si>
-  <si>
-    <t>SK</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>대표</t>
-  </si>
-  <si>
-    <t>인수</t>
-  </si>
-  <si>
-    <t>2024-08-09</t>
-  </si>
-  <si>
-    <t>2024-08-08</t>
-  </si>
-  <si>
-    <t>2024-08-07</t>
-  </si>
-  <si>
-    <t>2024-08-01</t>
-  </si>
-  <si>
-    <t>2024-07-22</t>
-  </si>
-  <si>
-    <t>2024-07-18</t>
-  </si>
-  <si>
-    <t>2024-07-16</t>
-  </si>
-  <si>
-    <t>2024-07-03</t>
-  </si>
-  <si>
     <t>2024-08-26</t>
   </si>
   <si>
@@ -252,9 +246,6 @@
     <t>2024-07-19</t>
   </si>
   <si>
-    <t>2024-07-08</t>
-  </si>
-  <si>
     <t>회사명</t>
   </si>
   <si>
@@ -352,9 +343,6 @@
   </si>
   <si>
     <t>1654.28 : 1</t>
-  </si>
-  <si>
-    <t>517.7 : 1</t>
   </si>
   <si>
     <t>인수기관</t>
@@ -727,7 +715,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -788,37 +776,37 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D2">
         <v>787.2</v>
       </c>
       <c r="E2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F2">
         <v>787.2</v>
       </c>
       <c r="G2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M2">
         <v>32000</v>
@@ -830,7 +818,7 @@
         <v>20</v>
       </c>
       <c r="P2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="Q2">
         <v>1722000</v>
@@ -841,37 +829,37 @@
         <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D3">
         <v>240</v>
       </c>
       <c r="E3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F3">
         <v>228</v>
       </c>
       <c r="G3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M3">
         <v>16000</v>
@@ -894,37 +882,37 @@
         <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D4">
         <v>240</v>
       </c>
       <c r="E4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F4">
         <v>12</v>
       </c>
       <c r="G4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H4" t="s">
+        <v>60</v>
+      </c>
+      <c r="I4" t="s">
+        <v>60</v>
+      </c>
+      <c r="J4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K4" t="s">
         <v>62</v>
       </c>
-      <c r="H4" t="s">
-        <v>62</v>
-      </c>
-      <c r="I4" t="s">
-        <v>62</v>
-      </c>
-      <c r="J4" t="s">
-        <v>62</v>
-      </c>
-      <c r="K4" t="s">
-        <v>64</v>
-      </c>
       <c r="L4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M4">
         <v>16000</v>
@@ -947,37 +935,37 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D5">
         <v>239.7204</v>
       </c>
       <c r="E5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F5">
         <v>239.7204</v>
       </c>
       <c r="G5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M5">
         <v>15300</v>
@@ -1000,37 +988,37 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D6">
         <v>130</v>
       </c>
       <c r="E6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F6">
         <v>130</v>
       </c>
       <c r="G6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M6">
         <v>13000</v>
@@ -1039,10 +1027,10 @@
         <v>100</v>
       </c>
       <c r="O6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="P6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="Q6">
         <v>723700</v>
@@ -1053,37 +1041,37 @@
         <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D7">
         <v>130</v>
       </c>
       <c r="E7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F7">
         <v>130</v>
       </c>
       <c r="G7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M7">
         <v>2000</v>
@@ -1092,10 +1080,10 @@
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="P7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="Q7">
         <v>4875000</v>
@@ -1106,37 +1094,37 @@
         <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D8">
         <v>507.81225</v>
       </c>
       <c r="E8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F8">
         <v>507.81225</v>
       </c>
       <c r="G8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M8">
         <v>16500</v>
@@ -1145,7 +1133,7 @@
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="P8" t="s">
         <v>24</v>
@@ -1159,37 +1147,37 @@
         <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D9">
         <v>217</v>
       </c>
       <c r="E9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F9">
         <v>217</v>
       </c>
       <c r="G9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M9">
         <v>15500</v>
@@ -1198,7 +1186,7 @@
         <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="P9" t="s">
         <v>24</v>
@@ -1212,37 +1200,37 @@
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D10">
         <v>290</v>
       </c>
       <c r="E10" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F10">
         <v>290</v>
       </c>
       <c r="G10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M10">
         <v>29000</v>
@@ -1251,7 +1239,7 @@
         <v>100</v>
       </c>
       <c r="O10" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="P10" t="s">
         <v>25</v>
@@ -1265,37 +1253,37 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D11">
         <v>157.71</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F11">
         <v>157.71</v>
       </c>
       <c r="G11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M11">
         <v>21000</v>
@@ -1307,7 +1295,7 @@
         <v>26</v>
       </c>
       <c r="P11" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="Q11">
         <v>540250</v>
@@ -1318,37 +1306,37 @@
         <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D12">
         <v>116</v>
       </c>
       <c r="E12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F12">
         <v>116</v>
       </c>
       <c r="G12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K12" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M12">
         <v>2000</v>
@@ -1357,7 +1345,7 @@
         <v>100</v>
       </c>
       <c r="O12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="P12" t="s">
         <v>26</v>
@@ -1371,37 +1359,37 @@
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D13">
         <v>224</v>
       </c>
       <c r="E13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F13">
         <v>224</v>
       </c>
       <c r="G13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M13">
         <v>16000</v>
@@ -1410,7 +1398,7 @@
         <v>100</v>
       </c>
       <c r="O13" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="P13" t="s">
         <v>26</v>
@@ -1424,37 +1412,37 @@
         <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D14">
         <v>223.4</v>
       </c>
       <c r="E14" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F14">
         <v>223.4</v>
       </c>
       <c r="G14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K14" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M14">
         <v>10000</v>
@@ -1466,7 +1454,7 @@
         <v>30</v>
       </c>
       <c r="P14" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="Q14">
         <v>1675500</v>
@@ -1477,37 +1465,37 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D15">
         <v>297</v>
       </c>
       <c r="E15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F15">
         <v>297</v>
       </c>
       <c r="G15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K15" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M15">
         <v>22000</v>
@@ -1516,7 +1504,7 @@
         <v>100</v>
       </c>
       <c r="O15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="P15" t="s">
         <v>30</v>
@@ -1530,37 +1518,37 @@
         <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C16" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D16">
         <v>2660</v>
       </c>
       <c r="E16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F16">
         <v>2553.6</v>
       </c>
       <c r="G16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K16" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M16">
         <v>35000</v>
@@ -1569,10 +1557,10 @@
         <v>96</v>
       </c>
       <c r="O16" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="P16" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="Q16">
         <v>9340690</v>
@@ -1583,37 +1571,37 @@
         <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D17">
         <v>2660</v>
       </c>
       <c r="E17" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F17">
         <v>106.4</v>
       </c>
       <c r="G17" t="s">
+        <v>60</v>
+      </c>
+      <c r="H17" t="s">
+        <v>60</v>
+      </c>
+      <c r="I17" t="s">
+        <v>60</v>
+      </c>
+      <c r="J17" t="s">
+        <v>60</v>
+      </c>
+      <c r="K17" t="s">
         <v>62</v>
       </c>
-      <c r="H17" t="s">
-        <v>62</v>
-      </c>
-      <c r="I17" t="s">
-        <v>62</v>
-      </c>
-      <c r="J17" t="s">
-        <v>62</v>
-      </c>
-      <c r="K17" t="s">
-        <v>64</v>
-      </c>
       <c r="L17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M17">
         <v>35000</v>
@@ -1622,10 +1610,10 @@
         <v>4</v>
       </c>
       <c r="O17" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="P17" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="Q17">
         <v>9340690</v>
@@ -1636,37 +1624,37 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D18">
         <v>120</v>
       </c>
       <c r="E18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F18">
         <v>120</v>
       </c>
       <c r="G18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K18" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M18">
         <v>2000</v>
@@ -1675,10 +1663,10 @@
         <v>100</v>
       </c>
       <c r="O18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P18" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="Q18">
         <v>4500000</v>
@@ -1689,37 +1677,37 @@
         <v>30</v>
       </c>
       <c r="B19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" t="s">
         <v>47</v>
-      </c>
-      <c r="C19" t="s">
-        <v>49</v>
       </c>
       <c r="D19">
         <v>80</v>
       </c>
       <c r="E19" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F19">
         <v>80</v>
       </c>
       <c r="G19" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H19" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I19" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J19" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K19" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L19" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M19">
         <v>2000</v>
@@ -1728,66 +1716,13 @@
         <v>100</v>
       </c>
       <c r="O19" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="P19" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="Q19">
         <v>3000000</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17">
-      <c r="A20" t="s">
-        <v>31</v>
-      </c>
-      <c r="B20" t="s">
-        <v>48</v>
-      </c>
-      <c r="C20" t="s">
-        <v>49</v>
-      </c>
-      <c r="D20">
-        <v>161.8</v>
-      </c>
-      <c r="E20" t="s">
-        <v>56</v>
-      </c>
-      <c r="F20">
-        <v>161.8</v>
-      </c>
-      <c r="G20" t="s">
-        <v>62</v>
-      </c>
-      <c r="H20" t="s">
-        <v>62</v>
-      </c>
-      <c r="I20" t="s">
-        <v>62</v>
-      </c>
-      <c r="J20" t="s">
-        <v>62</v>
-      </c>
-      <c r="K20" t="s">
-        <v>63</v>
-      </c>
-      <c r="L20" t="s">
-        <v>62</v>
-      </c>
-      <c r="M20">
-        <v>10000</v>
-      </c>
-      <c r="N20">
-        <v>100</v>
-      </c>
-      <c r="O20" t="s">
-        <v>72</v>
-      </c>
-      <c r="P20" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q20">
-        <v>1187900</v>
       </c>
     </row>
   </sheetData>
@@ -1797,7 +1732,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T18"/>
+  <dimension ref="A1:T17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -1805,10 +1740,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -1817,49 +1752,49 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:20">
@@ -1867,13 +1802,13 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
@@ -1885,7 +1820,7 @@
         <v>2460000</v>
       </c>
       <c r="H2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I2">
         <v>32000</v>
@@ -1894,34 +1829,34 @@
         <v>40200</v>
       </c>
       <c r="K2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L2">
         <v>32000</v>
       </c>
       <c r="M2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="S2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1929,10 +1864,10 @@
         <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D3" t="s">
         <v>23</v>
@@ -1947,7 +1882,7 @@
         <v>1500000</v>
       </c>
       <c r="H3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I3">
         <v>11000</v>
@@ -1956,34 +1891,34 @@
         <v>13000</v>
       </c>
       <c r="K3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L3">
         <v>16000</v>
       </c>
       <c r="M3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="S3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1991,10 +1926,10 @@
         <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D4" t="s">
         <v>23</v>
@@ -2009,7 +1944,7 @@
         <v>1566800</v>
       </c>
       <c r="H4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I4">
         <v>13600</v>
@@ -2018,48 +1953,48 @@
         <v>15300</v>
       </c>
       <c r="K4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L4">
         <v>15300</v>
       </c>
       <c r="M4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R4" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="S4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E5" t="s">
         <v>20</v>
@@ -2071,7 +2006,7 @@
         <v>1000000</v>
       </c>
       <c r="H5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I5">
         <v>9500</v>
@@ -2080,48 +2015,48 @@
         <v>10700</v>
       </c>
       <c r="K5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L5">
         <v>13000</v>
       </c>
       <c r="M5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O5">
         <v>50</v>
       </c>
       <c r="P5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="S5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E6" t="s">
         <v>18</v>
@@ -2133,7 +2068,7 @@
         <v>6500000</v>
       </c>
       <c r="H6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I6">
         <v>2000</v>
@@ -2142,45 +2077,45 @@
         <v>2000</v>
       </c>
       <c r="K6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L6">
         <v>2000</v>
       </c>
       <c r="M6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="S6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D7" t="s">
         <v>24</v>
@@ -2195,7 +2130,7 @@
         <v>3077650</v>
       </c>
       <c r="H7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I7">
         <v>13800</v>
@@ -2204,45 +2139,45 @@
         <v>15700</v>
       </c>
       <c r="K7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L7">
         <v>16500</v>
       </c>
       <c r="M7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O7">
         <v>100</v>
       </c>
       <c r="P7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R7" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="S7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D8" t="s">
         <v>24</v>
@@ -2257,7 +2192,7 @@
         <v>1400000</v>
       </c>
       <c r="H8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I8">
         <v>12500</v>
@@ -2266,45 +2201,45 @@
         <v>15500</v>
       </c>
       <c r="K8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L8">
         <v>15500</v>
       </c>
       <c r="M8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R8" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="S8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D9" t="s">
         <v>25</v>
@@ -2319,7 +2254,7 @@
         <v>1000000</v>
       </c>
       <c r="H9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I9">
         <v>24000</v>
@@ -2328,34 +2263,34 @@
         <v>29000</v>
       </c>
       <c r="K9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L9">
         <v>29000</v>
       </c>
       <c r="M9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O9">
         <v>0</v>
       </c>
       <c r="P9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R9" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="S9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -2363,13 +2298,13 @@
         <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E10" t="s">
         <v>23</v>
@@ -2381,7 +2316,7 @@
         <v>751000</v>
       </c>
       <c r="H10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I10">
         <v>18000</v>
@@ -2390,45 +2325,45 @@
         <v>21000</v>
       </c>
       <c r="K10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L10">
         <v>21000</v>
       </c>
       <c r="M10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O10">
         <v>72.87616511318242</v>
       </c>
       <c r="P10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R10" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="S10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D11" t="s">
         <v>26</v>
@@ -2443,7 +2378,7 @@
         <v>5800000</v>
       </c>
       <c r="H11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I11">
         <v>2000</v>
@@ -2452,45 +2387,45 @@
         <v>2000</v>
       </c>
       <c r="K11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L11">
         <v>2000</v>
       </c>
       <c r="M11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O11">
         <v>0</v>
       </c>
       <c r="P11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R11" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="S11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D12" t="s">
         <v>26</v>
@@ -2505,7 +2440,7 @@
         <v>1400000</v>
       </c>
       <c r="H12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I12">
         <v>16000</v>
@@ -2514,34 +2449,34 @@
         <v>19000</v>
       </c>
       <c r="K12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L12">
         <v>16000</v>
       </c>
       <c r="M12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O12">
         <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R12" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="S12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -2549,13 +2484,13 @@
         <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D13" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E13" t="s">
         <v>26</v>
@@ -2567,7 +2502,7 @@
         <v>2234000</v>
       </c>
       <c r="H13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I13">
         <v>7300</v>
@@ -2576,45 +2511,45 @@
         <v>8500</v>
       </c>
       <c r="K13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L13">
         <v>10000</v>
       </c>
       <c r="M13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O13">
         <v>0</v>
       </c>
       <c r="P13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R13" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="S13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D14" t="s">
         <v>30</v>
@@ -2629,7 +2564,7 @@
         <v>1350000</v>
       </c>
       <c r="H14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I14">
         <v>14000</v>
@@ -2638,48 +2573,48 @@
         <v>17000</v>
       </c>
       <c r="K14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L14">
         <v>22000</v>
       </c>
       <c r="M14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O14">
         <v>0</v>
       </c>
       <c r="P14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R14" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="S14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D15" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E15" t="s">
         <v>28</v>
@@ -2691,7 +2626,7 @@
         <v>7600000</v>
       </c>
       <c r="H15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I15">
         <v>24000</v>
@@ -2700,48 +2635,48 @@
         <v>30000</v>
       </c>
       <c r="K15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L15">
         <v>35000</v>
       </c>
       <c r="M15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O15">
         <v>14.47368421052632</v>
       </c>
       <c r="P15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R15" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="S15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:20">
       <c r="A16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D16" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
@@ -2753,7 +2688,7 @@
         <v>6000000</v>
       </c>
       <c r="H16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I16">
         <v>2000</v>
@@ -2762,48 +2697,48 @@
         <v>2000</v>
       </c>
       <c r="K16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L16">
         <v>2000</v>
       </c>
       <c r="M16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O16">
         <v>0</v>
       </c>
       <c r="P16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R16" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="S16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:20">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D17" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E17" t="s">
         <v>30</v>
@@ -2815,7 +2750,7 @@
         <v>4000000</v>
       </c>
       <c r="H17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I17">
         <v>2000</v>
@@ -2824,96 +2759,34 @@
         <v>2000</v>
       </c>
       <c r="K17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L17">
         <v>2000</v>
       </c>
       <c r="M17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O17">
         <v>0</v>
       </c>
       <c r="P17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R17" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="S17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="T17" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20">
-      <c r="A18" t="s">
-        <v>72</v>
-      </c>
-      <c r="B18" t="s">
-        <v>48</v>
-      </c>
-      <c r="C18" t="s">
-        <v>56</v>
-      </c>
-      <c r="D18" t="s">
-        <v>78</v>
-      </c>
-      <c r="E18" t="s">
-        <v>31</v>
-      </c>
-      <c r="F18">
-        <v>16180000</v>
-      </c>
-      <c r="G18">
-        <v>1618000</v>
-      </c>
-      <c r="H18" t="s">
-        <v>62</v>
-      </c>
-      <c r="I18">
-        <v>6200</v>
-      </c>
-      <c r="J18">
-        <v>7700</v>
-      </c>
-      <c r="K18" t="s">
-        <v>62</v>
-      </c>
-      <c r="L18">
-        <v>10000</v>
-      </c>
-      <c r="M18" t="s">
-        <v>62</v>
-      </c>
-      <c r="N18" t="s">
-        <v>62</v>
-      </c>
-      <c r="O18">
-        <v>0</v>
-      </c>
-      <c r="P18" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>62</v>
-      </c>
-      <c r="R18" t="s">
-        <v>112</v>
-      </c>
-      <c r="S18" t="s">
-        <v>62</v>
-      </c>
-      <c r="T18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -2923,21 +2796,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -2949,10 +2822,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -2961,39 +2834,39 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>25</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
+        <v>23</v>
       </c>
       <c r="G2" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="H2">
-        <v>12000</v>
+        <v>23972.04</v>
       </c>
       <c r="I2">
-        <v>6000000</v>
+        <v>1566800</v>
       </c>
       <c r="J2">
-        <v>2000</v>
+        <v>15300</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -3004,34 +2877,34 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F3" t="s">
-        <v>23</v>
+        <v>75</v>
       </c>
       <c r="G3" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="H3">
-        <v>23972.04</v>
+        <v>12000</v>
       </c>
       <c r="I3">
-        <v>1566800</v>
+        <v>6000000</v>
       </c>
       <c r="J3">
-        <v>15300</v>
+        <v>2000</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -3042,22 +2915,22 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G4" t="s">
         <v>30</v>
@@ -3080,19 +2953,19 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F5" t="s">
         <v>26</v>
@@ -3118,34 +2991,34 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6" t="s">
         <v>72</v>
       </c>
-      <c r="C6" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" t="s">
-        <v>56</v>
-      </c>
-      <c r="E6" t="s">
-        <v>56</v>
-      </c>
-      <c r="F6" t="s">
-        <v>78</v>
-      </c>
       <c r="G6" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="H6">
-        <v>16180</v>
+        <v>13000</v>
       </c>
       <c r="I6">
-        <v>1618000</v>
+        <v>6500000</v>
       </c>
       <c r="J6">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -3156,110 +3029,110 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E7" t="s">
-        <v>56</v>
+        <v>112</v>
       </c>
       <c r="F7" t="s">
         <v>74</v>
       </c>
       <c r="G7" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H7">
-        <v>13000</v>
+        <v>255360</v>
       </c>
       <c r="I7">
-        <v>6500000</v>
+        <v>7600000</v>
       </c>
       <c r="J7">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E8" t="s">
-        <v>116</v>
+        <v>55</v>
       </c>
       <c r="F8" t="s">
-        <v>76</v>
+        <v>24</v>
       </c>
       <c r="G8" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="H8">
-        <v>255360</v>
+        <v>50781.225</v>
       </c>
       <c r="I8">
-        <v>7600000</v>
+        <v>3077650</v>
       </c>
       <c r="J8">
-        <v>35000</v>
+        <v>16500</v>
       </c>
       <c r="K8">
         <v>0</v>
       </c>
       <c r="L8">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
         <v>66</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G9" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H9">
-        <v>50781.225</v>
+        <v>22400</v>
       </c>
       <c r="I9">
-        <v>3077650</v>
+        <v>1400000</v>
       </c>
       <c r="J9">
-        <v>16500</v>
+        <v>16000</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -3270,110 +3143,110 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
         <v>68</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E10" t="s">
-        <v>57</v>
+        <v>112</v>
       </c>
       <c r="F10" t="s">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="G10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="H10">
-        <v>22400</v>
+        <v>10640</v>
       </c>
       <c r="I10">
-        <v>1400000</v>
+        <v>7600000</v>
       </c>
       <c r="J10">
-        <v>16000</v>
+        <v>35000</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E11" t="s">
-        <v>116</v>
+        <v>49</v>
       </c>
       <c r="F11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G11" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H11">
-        <v>10640</v>
+        <v>22340</v>
       </c>
       <c r="I11">
-        <v>7600000</v>
+        <v>2234000</v>
       </c>
       <c r="J11">
-        <v>35000</v>
+        <v>10000</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>4</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E12" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F12" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="G12" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="H12">
-        <v>22340</v>
+        <v>78720</v>
       </c>
       <c r="I12">
-        <v>2234000</v>
+        <v>2460000</v>
       </c>
       <c r="J12">
-        <v>10000</v>
+        <v>32000</v>
       </c>
       <c r="K12">
         <v>0</v>
@@ -3384,57 +3257,57 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C13" t="s">
         <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E13" t="s">
-        <v>51</v>
+        <v>113</v>
       </c>
       <c r="F13" t="s">
-        <v>73</v>
+        <v>23</v>
       </c>
       <c r="G13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H13">
-        <v>78720</v>
+        <v>22800</v>
       </c>
       <c r="I13">
-        <v>2460000</v>
+        <v>1500000</v>
       </c>
       <c r="J13">
-        <v>32000</v>
+        <v>16000</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s">
         <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D14" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E14" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F14" t="s">
         <v>23</v>
@@ -3443,7 +3316,7 @@
         <v>18</v>
       </c>
       <c r="H14">
-        <v>22800</v>
+        <v>1200</v>
       </c>
       <c r="I14">
         <v>1500000</v>
@@ -3455,77 +3328,77 @@
         <v>0</v>
       </c>
       <c r="L14">
-        <v>95</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="D15" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E15" t="s">
-        <v>117</v>
+        <v>57</v>
       </c>
       <c r="F15" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="G15" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="H15">
-        <v>1200</v>
+        <v>29700</v>
       </c>
       <c r="I15">
-        <v>1500000</v>
+        <v>1350000</v>
       </c>
       <c r="J15">
-        <v>16000</v>
+        <v>22000</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>26</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F16" t="s">
-        <v>30</v>
+        <v>63</v>
       </c>
       <c r="G16" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H16">
-        <v>29700</v>
+        <v>15771</v>
       </c>
       <c r="I16">
-        <v>1350000</v>
+        <v>751000</v>
       </c>
       <c r="J16">
-        <v>22000</v>
+        <v>21000</v>
       </c>
       <c r="K16">
         <v>0</v>
@@ -3536,34 +3409,34 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B17" t="s">
-        <v>26</v>
+        <v>64</v>
       </c>
       <c r="C17" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D17" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E17" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F17" t="s">
-        <v>65</v>
+        <v>24</v>
       </c>
       <c r="G17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H17">
-        <v>15771</v>
+        <v>21700</v>
       </c>
       <c r="I17">
-        <v>751000</v>
+        <v>1400000</v>
       </c>
       <c r="J17">
-        <v>21000</v>
+        <v>15500</v>
       </c>
       <c r="K17">
         <v>0</v>
@@ -3574,34 +3447,34 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B18" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C18" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E18" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="F18" t="s">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="G18" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H18">
-        <v>21700</v>
+        <v>13000</v>
       </c>
       <c r="I18">
-        <v>1400000</v>
+        <v>1000000</v>
       </c>
       <c r="J18">
-        <v>15500</v>
+        <v>13000</v>
       </c>
       <c r="K18">
         <v>0</v>
@@ -3612,77 +3485,39 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B19" t="s">
         <v>65</v>
       </c>
       <c r="C19" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D19" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E19" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F19" t="s">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="G19" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H19">
-        <v>13000</v>
+        <v>29000</v>
       </c>
       <c r="I19">
         <v>1000000</v>
       </c>
       <c r="J19">
-        <v>13000</v>
+        <v>29000</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12">
-      <c r="A20" t="s">
-        <v>55</v>
-      </c>
-      <c r="B20" t="s">
-        <v>67</v>
-      </c>
-      <c r="C20" t="s">
-        <v>39</v>
-      </c>
-      <c r="D20" t="s">
-        <v>55</v>
-      </c>
-      <c r="E20" t="s">
-        <v>55</v>
-      </c>
-      <c r="F20" t="s">
-        <v>25</v>
-      </c>
-      <c r="G20" t="s">
-        <v>22</v>
-      </c>
-      <c r="H20">
-        <v>29000</v>
-      </c>
-      <c r="I20">
-        <v>1000000</v>
-      </c>
-      <c r="J20">
-        <v>29000</v>
-      </c>
-      <c r="K20">
-        <v>0</v>
-      </c>
-      <c r="L20">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-12
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="119">
   <si>
     <t>상장일</t>
   </si>
@@ -69,6 +69,9 @@
     <t>총기관배정수량</t>
   </si>
   <si>
+    <t>2024-09-11</t>
+  </si>
+  <si>
     <t>2024-08-30</t>
   </si>
   <si>
@@ -111,6 +114,9 @@
     <t>2024-07-25</t>
   </si>
   <si>
+    <t>미래에셋비전스팩7호</t>
+  </si>
+  <si>
     <t>아이스크림미디어</t>
   </si>
   <si>
@@ -165,6 +171,9 @@
     <t>코스피</t>
   </si>
   <si>
+    <t>미래</t>
+  </si>
+  <si>
     <t>삼성</t>
   </si>
   <si>
@@ -183,9 +192,6 @@
     <t>대신</t>
   </si>
   <si>
-    <t>미래</t>
-  </si>
-  <si>
     <t>하나</t>
   </si>
   <si>
@@ -207,6 +213,9 @@
     <t>인수</t>
   </si>
   <si>
+    <t>2024-09-02</t>
+  </si>
+  <si>
     <t>2024-08-09</t>
   </si>
   <si>
@@ -231,6 +240,9 @@
     <t>2024-07-15</t>
   </si>
   <si>
+    <t>2024-09-05</t>
+  </si>
+  <si>
     <t>2024-08-26</t>
   </si>
   <si>
@@ -295,6 +307,9 @@
   </si>
   <si>
     <t>수수료율</t>
+  </si>
+  <si>
+    <t>1004 : 1</t>
   </si>
   <si>
     <t>12.89 : 1</t>
@@ -715,7 +730,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -776,52 +791,52 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D2">
-        <v>787.2</v>
+        <v>159</v>
       </c>
       <c r="E2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F2">
-        <v>787.2</v>
+        <v>159</v>
       </c>
       <c r="G2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M2">
-        <v>32000</v>
+        <v>2000</v>
       </c>
       <c r="N2">
         <v>100</v>
       </c>
       <c r="O2" t="s">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="P2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="Q2">
-        <v>1722000</v>
+        <v>5962500</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -829,102 +844,102 @@
         <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D3">
-        <v>240</v>
+        <v>787.2</v>
       </c>
       <c r="E3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F3">
-        <v>228</v>
+        <v>787.2</v>
       </c>
       <c r="G3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M3">
-        <v>16000</v>
+        <v>32000</v>
       </c>
       <c r="N3">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="P3" t="s">
-        <v>23</v>
+        <v>75</v>
       </c>
       <c r="Q3">
-        <v>2100000</v>
+        <v>1722000</v>
       </c>
     </row>
     <row r="4" spans="1:17">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D4">
         <v>240</v>
       </c>
       <c r="E4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F4">
-        <v>12</v>
+        <v>228</v>
       </c>
       <c r="G4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M4">
         <v>16000</v>
       </c>
       <c r="N4">
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="O4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q4">
         <v>2100000</v>
@@ -935,52 +950,52 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D5">
-        <v>239.7204</v>
+        <v>240</v>
       </c>
       <c r="E5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F5">
-        <v>239.7204</v>
+        <v>12</v>
       </c>
       <c r="G5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K5" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="L5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M5">
-        <v>15300</v>
+        <v>16000</v>
       </c>
       <c r="N5">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="O5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q5">
-        <v>1156798</v>
+        <v>2100000</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -988,158 +1003,158 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D6">
-        <v>130</v>
+        <v>239.7204</v>
       </c>
       <c r="E6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F6">
-        <v>130</v>
+        <v>239.7204</v>
       </c>
       <c r="G6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M6">
-        <v>13000</v>
+        <v>15300</v>
       </c>
       <c r="N6">
         <v>100</v>
       </c>
       <c r="O6" t="s">
-        <v>63</v>
+        <v>26</v>
       </c>
       <c r="P6" t="s">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="Q6">
-        <v>723700</v>
+        <v>1156798</v>
       </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D7">
         <v>130</v>
       </c>
       <c r="E7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F7">
         <v>130</v>
       </c>
       <c r="G7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M7">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="N7">
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="P7" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="Q7">
-        <v>4875000</v>
+        <v>723700</v>
       </c>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D8">
-        <v>507.81225</v>
+        <v>130</v>
       </c>
       <c r="E8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F8">
-        <v>507.81225</v>
+        <v>130</v>
       </c>
       <c r="G8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M8">
-        <v>16500</v>
+        <v>2000</v>
       </c>
       <c r="N8">
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="P8" t="s">
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="Q8">
-        <v>2078175</v>
+        <v>4875000</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -1147,105 +1162,105 @@
         <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D9">
-        <v>217</v>
+        <v>507.81225</v>
       </c>
       <c r="E9" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="F9">
-        <v>217</v>
+        <v>507.81225</v>
       </c>
       <c r="G9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M9">
-        <v>15500</v>
+        <v>16500</v>
       </c>
       <c r="N9">
         <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="P9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q9">
-        <v>1050000</v>
+        <v>2078175</v>
       </c>
     </row>
     <row r="10" spans="1:17">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D10">
-        <v>290</v>
+        <v>217</v>
       </c>
       <c r="E10" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F10">
-        <v>290</v>
+        <v>217</v>
       </c>
       <c r="G10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M10">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="N10">
         <v>100</v>
       </c>
       <c r="O10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="P10" t="s">
         <v>25</v>
       </c>
       <c r="Q10">
-        <v>720000</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -1253,52 +1268,52 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D11">
-        <v>157.71</v>
+        <v>290</v>
       </c>
       <c r="E11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F11">
-        <v>157.71</v>
+        <v>290</v>
       </c>
       <c r="G11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M11">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="N11">
         <v>100</v>
       </c>
       <c r="O11" t="s">
+        <v>68</v>
+      </c>
+      <c r="P11" t="s">
         <v>26</v>
       </c>
-      <c r="P11" t="s">
-        <v>63</v>
-      </c>
       <c r="Q11">
-        <v>540250</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -1306,52 +1321,52 @@
         <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D12">
-        <v>116</v>
+        <v>157.71</v>
       </c>
       <c r="E12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F12">
-        <v>116</v>
+        <v>157.71</v>
       </c>
       <c r="G12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M12">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="N12">
         <v>100</v>
       </c>
       <c r="O12" t="s">
+        <v>27</v>
+      </c>
+      <c r="P12" t="s">
         <v>66</v>
       </c>
-      <c r="P12" t="s">
-        <v>26</v>
-      </c>
       <c r="Q12">
-        <v>4350000</v>
+        <v>540250</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -1359,52 +1374,52 @@
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D13">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="E13" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="F13">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="G13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K13" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M13">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N13">
         <v>100</v>
       </c>
       <c r="O13" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="P13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q13">
-        <v>1050000</v>
+        <v>4350000</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1412,52 +1427,52 @@
         <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D14">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="E14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F14">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="G14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K14" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M14">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="N14">
         <v>100</v>
       </c>
       <c r="O14" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="P14" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="Q14">
-        <v>1675500</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1465,52 +1480,52 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D15">
-        <v>297</v>
+        <v>223.4</v>
       </c>
       <c r="E15" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F15">
-        <v>297</v>
+        <v>223.4</v>
       </c>
       <c r="G15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K15" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M15">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="N15">
         <v>100</v>
       </c>
       <c r="O15" t="s">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="P15" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="Q15">
-        <v>1012500</v>
+        <v>1675500</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -1518,102 +1533,102 @@
         <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D16">
-        <v>2660</v>
+        <v>297</v>
       </c>
       <c r="E16" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F16">
-        <v>2553.6</v>
+        <v>297</v>
       </c>
       <c r="G16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K16" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M16">
-        <v>35000</v>
+        <v>22000</v>
       </c>
       <c r="N16">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="O16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="P16" t="s">
-        <v>74</v>
+        <v>31</v>
       </c>
       <c r="Q16">
-        <v>9340690</v>
+        <v>1012500</v>
       </c>
     </row>
     <row r="17" spans="1:17">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D17">
         <v>2660</v>
       </c>
       <c r="E17" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F17">
-        <v>106.4</v>
+        <v>2553.6</v>
       </c>
       <c r="G17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M17">
         <v>35000</v>
       </c>
       <c r="N17">
-        <v>4</v>
+        <v>96</v>
       </c>
       <c r="O17" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="P17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="Q17">
         <v>9340690</v>
@@ -1624,52 +1639,52 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D18">
-        <v>120</v>
+        <v>2660</v>
       </c>
       <c r="E18" t="s">
         <v>52</v>
       </c>
       <c r="F18">
-        <v>120</v>
+        <v>106.4</v>
       </c>
       <c r="G18" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H18" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I18" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J18" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K18" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="L18" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M18">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="N18">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="O18" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="P18" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="Q18">
-        <v>4500000</v>
+        <v>9340690</v>
       </c>
     </row>
     <row r="19" spans="1:17">
@@ -1677,37 +1692,37 @@
         <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D19">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="E19" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F19">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="G19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K19" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M19">
         <v>2000</v>
@@ -1716,12 +1731,65 @@
         <v>100</v>
       </c>
       <c r="O19" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="P19" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="Q19">
+        <v>4500000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17">
+      <c r="A20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20">
+        <v>80</v>
+      </c>
+      <c r="E20" t="s">
+        <v>61</v>
+      </c>
+      <c r="F20">
+        <v>80</v>
+      </c>
+      <c r="G20" t="s">
+        <v>62</v>
+      </c>
+      <c r="H20" t="s">
+        <v>62</v>
+      </c>
+      <c r="I20" t="s">
+        <v>62</v>
+      </c>
+      <c r="J20" t="s">
+        <v>62</v>
+      </c>
+      <c r="K20" t="s">
+        <v>63</v>
+      </c>
+      <c r="L20" t="s">
+        <v>62</v>
+      </c>
+      <c r="M20">
+        <v>2000</v>
+      </c>
+      <c r="N20">
+        <v>100</v>
+      </c>
+      <c r="O20" t="s">
+        <v>73</v>
+      </c>
+      <c r="P20" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q20">
         <v>3000000</v>
       </c>
     </row>
@@ -1732,7 +1800,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T17"/>
+  <dimension ref="A1:T18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -1740,10 +1808,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -1752,1005 +1820,1005 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
       </c>
       <c r="F2">
-        <v>78720000</v>
+        <v>15900000</v>
       </c>
       <c r="G2">
-        <v>2460000</v>
+        <v>7950000</v>
       </c>
       <c r="H2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I2">
-        <v>32000</v>
+        <v>2000</v>
       </c>
       <c r="J2">
-        <v>40200</v>
+        <v>2000</v>
       </c>
       <c r="K2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L2">
-        <v>32000</v>
+        <v>2000</v>
       </c>
       <c r="M2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="S2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>75</v>
       </c>
       <c r="E3" t="s">
         <v>18</v>
       </c>
       <c r="F3">
-        <v>24000000</v>
+        <v>78720000</v>
       </c>
       <c r="G3">
-        <v>1500000</v>
+        <v>2460000</v>
       </c>
       <c r="H3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I3">
-        <v>11000</v>
+        <v>32000</v>
       </c>
       <c r="J3">
-        <v>13000</v>
+        <v>40200</v>
       </c>
       <c r="K3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L3">
-        <v>16000</v>
+        <v>32000</v>
       </c>
       <c r="M3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R3" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="S3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
         <v>19</v>
       </c>
       <c r="F4">
-        <v>23972040</v>
+        <v>24000000</v>
       </c>
       <c r="G4">
-        <v>1566800</v>
+        <v>1500000</v>
       </c>
       <c r="H4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I4">
-        <v>13600</v>
+        <v>11000</v>
       </c>
       <c r="J4">
-        <v>15300</v>
+        <v>13000</v>
       </c>
       <c r="K4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L4">
-        <v>15300</v>
+        <v>16000</v>
       </c>
       <c r="M4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R4" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="S4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D5" t="s">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
         <v>20</v>
       </c>
       <c r="F5">
-        <v>13000000</v>
+        <v>23972040</v>
       </c>
       <c r="G5">
-        <v>1000000</v>
+        <v>1566800</v>
       </c>
       <c r="H5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I5">
-        <v>9500</v>
+        <v>13600</v>
       </c>
       <c r="J5">
-        <v>10700</v>
+        <v>15300</v>
       </c>
       <c r="K5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L5">
-        <v>13000</v>
+        <v>15300</v>
       </c>
       <c r="M5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O5">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="S5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E6" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F6">
         <v>13000000</v>
       </c>
       <c r="G6">
-        <v>6500000</v>
+        <v>1000000</v>
       </c>
       <c r="H6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I6">
-        <v>2000</v>
+        <v>9500</v>
       </c>
       <c r="J6">
-        <v>2000</v>
+        <v>10700</v>
       </c>
       <c r="K6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L6">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="M6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="P6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R6" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="S6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="E7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F7">
-        <v>50781225</v>
+        <v>13000000</v>
       </c>
       <c r="G7">
-        <v>3077650</v>
+        <v>6500000</v>
       </c>
       <c r="H7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I7">
-        <v>13800</v>
+        <v>2000</v>
       </c>
       <c r="J7">
-        <v>15700</v>
+        <v>2000</v>
       </c>
       <c r="K7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L7">
-        <v>16500</v>
+        <v>2000</v>
       </c>
       <c r="M7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O7">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R7" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="S7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" t="s">
         <v>22</v>
       </c>
       <c r="F8">
-        <v>21700000</v>
+        <v>50781225</v>
       </c>
       <c r="G8">
-        <v>1400000</v>
+        <v>3077650</v>
       </c>
       <c r="H8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I8">
-        <v>12500</v>
+        <v>13800</v>
       </c>
       <c r="J8">
-        <v>15500</v>
+        <v>15700</v>
       </c>
       <c r="K8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L8">
-        <v>15500</v>
+        <v>16500</v>
       </c>
       <c r="M8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="S8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D9" t="s">
         <v>25</v>
       </c>
       <c r="E9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F9">
-        <v>29000000</v>
+        <v>21700000</v>
       </c>
       <c r="G9">
-        <v>1000000</v>
+        <v>1400000</v>
       </c>
       <c r="H9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I9">
-        <v>24000</v>
+        <v>12500</v>
       </c>
       <c r="J9">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="K9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L9">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="M9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O9">
         <v>0</v>
       </c>
       <c r="P9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R9" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="S9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" t="s">
         <v>26</v>
-      </c>
-      <c r="B10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" t="s">
-        <v>63</v>
       </c>
       <c r="E10" t="s">
         <v>23</v>
       </c>
       <c r="F10">
-        <v>15771000</v>
+        <v>29000000</v>
       </c>
       <c r="G10">
-        <v>751000</v>
+        <v>1000000</v>
       </c>
       <c r="H10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I10">
-        <v>18000</v>
+        <v>24000</v>
       </c>
       <c r="J10">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="K10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L10">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="M10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O10">
-        <v>72.87616511318242</v>
+        <v>0</v>
       </c>
       <c r="P10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R10" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="S10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" t="s">
         <v>66</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" t="s">
-        <v>26</v>
       </c>
       <c r="E11" t="s">
         <v>24</v>
       </c>
       <c r="F11">
-        <v>11600000</v>
+        <v>15771000</v>
       </c>
       <c r="G11">
-        <v>5800000</v>
+        <v>751000</v>
       </c>
       <c r="H11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I11">
-        <v>2000</v>
+        <v>18000</v>
       </c>
       <c r="J11">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="K11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L11">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="M11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O11">
-        <v>0</v>
+        <v>72.87616511318242</v>
       </c>
       <c r="P11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R11" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="S11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E12" t="s">
         <v>25</v>
       </c>
       <c r="F12">
-        <v>22400000</v>
+        <v>11600000</v>
       </c>
       <c r="G12">
-        <v>1400000</v>
+        <v>5800000</v>
       </c>
       <c r="H12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I12">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="J12">
-        <v>19000</v>
+        <v>2000</v>
       </c>
       <c r="K12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L12">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="M12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O12">
         <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R12" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="S12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D13" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="E13" t="s">
         <v>26</v>
       </c>
       <c r="F13">
-        <v>22340000</v>
+        <v>22400000</v>
       </c>
       <c r="G13">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="H13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I13">
-        <v>7300</v>
+        <v>16000</v>
       </c>
       <c r="J13">
-        <v>8500</v>
+        <v>19000</v>
       </c>
       <c r="K13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L13">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="M13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O13">
         <v>0</v>
       </c>
       <c r="P13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R13" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="S13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="E14" t="s">
         <v>27</v>
       </c>
       <c r="F14">
-        <v>29700000</v>
+        <v>22340000</v>
       </c>
       <c r="G14">
-        <v>1350000</v>
+        <v>2234000</v>
       </c>
       <c r="H14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I14">
-        <v>14000</v>
+        <v>7300</v>
       </c>
       <c r="J14">
-        <v>17000</v>
+        <v>8500</v>
       </c>
       <c r="K14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L14">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="M14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O14">
         <v>0</v>
       </c>
       <c r="P14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="S14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D15" t="s">
-        <v>74</v>
+        <v>31</v>
       </c>
       <c r="E15" t="s">
         <v>28</v>
       </c>
       <c r="F15">
-        <v>266000000</v>
+        <v>29700000</v>
       </c>
       <c r="G15">
-        <v>7600000</v>
+        <v>1350000</v>
       </c>
       <c r="H15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I15">
-        <v>24000</v>
+        <v>14000</v>
       </c>
       <c r="J15">
-        <v>30000</v>
+        <v>17000</v>
       </c>
       <c r="K15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L15">
-        <v>35000</v>
+        <v>22000</v>
       </c>
       <c r="M15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O15">
-        <v>14.47368421052632</v>
+        <v>0</v>
       </c>
       <c r="P15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R15" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="S15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:20">
       <c r="A16" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
       </c>
       <c r="F16">
-        <v>12000000</v>
+        <v>266000000</v>
       </c>
       <c r="G16">
-        <v>6000000</v>
+        <v>7600000</v>
       </c>
       <c r="H16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I16">
-        <v>2000</v>
+        <v>24000</v>
       </c>
       <c r="J16">
-        <v>2000</v>
+        <v>30000</v>
       </c>
       <c r="K16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L16">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="M16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O16">
-        <v>0</v>
+        <v>14.47368421052632</v>
       </c>
       <c r="P16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R16" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="S16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:20">
       <c r="A17" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D17" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="E17" t="s">
         <v>30</v>
       </c>
       <c r="F17">
-        <v>8000000</v>
+        <v>12000000</v>
       </c>
       <c r="G17">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="H17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I17">
         <v>2000</v>
@@ -2759,34 +2827,96 @@
         <v>2000</v>
       </c>
       <c r="K17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L17">
         <v>2000</v>
       </c>
       <c r="M17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="N17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O17">
         <v>0</v>
       </c>
       <c r="P17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="R17" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="S17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="T17" t="s">
-        <v>60</v>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20">
+      <c r="A18" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" t="s">
+        <v>61</v>
+      </c>
+      <c r="D18" t="s">
+        <v>71</v>
+      </c>
+      <c r="E18" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18">
+        <v>8000000</v>
+      </c>
+      <c r="G18">
+        <v>4000000</v>
+      </c>
+      <c r="H18" t="s">
+        <v>62</v>
+      </c>
+      <c r="I18">
+        <v>2000</v>
+      </c>
+      <c r="J18">
+        <v>2000</v>
+      </c>
+      <c r="K18" t="s">
+        <v>62</v>
+      </c>
+      <c r="L18">
+        <v>2000</v>
+      </c>
+      <c r="M18" t="s">
+        <v>62</v>
+      </c>
+      <c r="N18" t="s">
+        <v>62</v>
+      </c>
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>62</v>
+      </c>
+      <c r="R18" t="s">
+        <v>113</v>
+      </c>
+      <c r="S18" t="s">
+        <v>62</v>
+      </c>
+      <c r="T18" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -2796,21 +2926,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -2822,10 +2952,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -2834,30 +2964,30 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H2">
         <v>23972.04</v>
@@ -2877,25 +3007,25 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H3">
         <v>12000</v>
@@ -2915,25 +3045,25 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H4">
         <v>8000</v>
@@ -2953,25 +3083,25 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H5">
         <v>11600</v>
@@ -2991,25 +3121,25 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H6">
         <v>13000</v>
@@ -3029,25 +3159,25 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D7" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E7" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="F7" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H7">
         <v>255360</v>
@@ -3067,34 +3197,34 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D8" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G8" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="H8">
-        <v>50781.225</v>
+        <v>22400</v>
       </c>
       <c r="I8">
-        <v>3077650</v>
+        <v>1400000</v>
       </c>
       <c r="J8">
-        <v>16500</v>
+        <v>16000</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -3105,34 +3235,34 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E9" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F9" t="s">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="G9" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="H9">
-        <v>22400</v>
+        <v>15900</v>
       </c>
       <c r="I9">
-        <v>1400000</v>
+        <v>7950000</v>
       </c>
       <c r="J9">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -3143,63 +3273,63 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E10" t="s">
-        <v>112</v>
+        <v>51</v>
       </c>
       <c r="F10" t="s">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="G10" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="H10">
-        <v>10640</v>
+        <v>50781.225</v>
       </c>
       <c r="I10">
-        <v>7600000</v>
+        <v>3077650</v>
       </c>
       <c r="J10">
-        <v>35000</v>
+        <v>16500</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>4</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F11" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H11">
         <v>22340</v>
@@ -3219,25 +3349,25 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D12" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E12" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F12" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H12">
         <v>78720</v>
@@ -3257,66 +3387,66 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>71</v>
       </c>
       <c r="C13" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E13" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="F13" t="s">
-        <v>23</v>
+        <v>78</v>
       </c>
       <c r="G13" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="H13">
-        <v>22800</v>
+        <v>10640</v>
       </c>
       <c r="I13">
-        <v>1500000</v>
+        <v>7600000</v>
       </c>
       <c r="J13">
-        <v>16000</v>
+        <v>35000</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
-        <v>95</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D14" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E14" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="F14" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G14" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H14">
-        <v>1200</v>
+        <v>22800</v>
       </c>
       <c r="I14">
         <v>1500000</v>
@@ -3328,68 +3458,68 @@
         <v>0</v>
       </c>
       <c r="L14">
-        <v>5</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="C15" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E15" t="s">
-        <v>57</v>
+        <v>118</v>
       </c>
       <c r="F15" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G15" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H15">
-        <v>29700</v>
+        <v>1200</v>
       </c>
       <c r="I15">
-        <v>1350000</v>
+        <v>1500000</v>
       </c>
       <c r="J15">
-        <v>22000</v>
+        <v>16000</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>100</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C16" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E16" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F16" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H16">
         <v>15771</v>
@@ -3409,34 +3539,34 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B17" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C17" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D17" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E17" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F17" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="G17" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H17">
-        <v>21700</v>
+        <v>29700</v>
       </c>
       <c r="I17">
-        <v>1400000</v>
+        <v>1350000</v>
       </c>
       <c r="J17">
-        <v>15500</v>
+        <v>22000</v>
       </c>
       <c r="K17">
         <v>0</v>
@@ -3447,34 +3577,34 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B18" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="D18" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="E18" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F18" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="G18" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="H18">
-        <v>13000</v>
+        <v>21700</v>
       </c>
       <c r="I18">
-        <v>1000000</v>
+        <v>1400000</v>
       </c>
       <c r="J18">
-        <v>13000</v>
+        <v>15500</v>
       </c>
       <c r="K18">
         <v>0</v>
@@ -3485,39 +3615,77 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B19" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D19" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E19" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F19" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="G19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H19">
-        <v>29000</v>
+        <v>13000</v>
       </c>
       <c r="I19">
         <v>1000000</v>
       </c>
       <c r="J19">
-        <v>29000</v>
+        <v>13000</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" t="s">
+        <v>40</v>
+      </c>
+      <c r="D20" t="s">
+        <v>56</v>
+      </c>
+      <c r="E20" t="s">
+        <v>56</v>
+      </c>
+      <c r="F20" t="s">
+        <v>26</v>
+      </c>
+      <c r="G20" t="s">
+        <v>23</v>
+      </c>
+      <c r="H20">
+        <v>29000</v>
+      </c>
+      <c r="I20">
+        <v>1000000</v>
+      </c>
+      <c r="J20">
+        <v>29000</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-17
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="115">
   <si>
     <t>상장일</t>
   </si>
@@ -111,123 +111,117 @@
     <t>2024-07-26</t>
   </si>
   <si>
+    <t>미래에셋비전스팩7호</t>
+  </si>
+  <si>
+    <t>아이스크림미디어</t>
+  </si>
+  <si>
+    <t>M83</t>
+  </si>
+  <si>
+    <t>이엔셀</t>
+  </si>
+  <si>
+    <t>티디에스팜</t>
+  </si>
+  <si>
+    <t>대신밸런스제18호스팩</t>
+  </si>
+  <si>
+    <t>전진건설로봇</t>
+  </si>
+  <si>
+    <t>케이쓰리아이</t>
+  </si>
+  <si>
+    <t>넥스트바이오메디컬</t>
+  </si>
+  <si>
+    <t>유라클</t>
+  </si>
+  <si>
+    <t>교보16호스팩</t>
+  </si>
+  <si>
+    <t>뱅크웨어글로벌</t>
+  </si>
+  <si>
+    <t>아이빔테크놀로지</t>
+  </si>
+  <si>
+    <t>피앤에스미캐닉스</t>
+  </si>
+  <si>
+    <t>산일전기</t>
+  </si>
+  <si>
+    <t>엔에이치스팩31호</t>
+  </si>
+  <si>
+    <t>코스닥</t>
+  </si>
+  <si>
+    <t>코스피</t>
+  </si>
+  <si>
+    <t>미래</t>
+  </si>
+  <si>
+    <t>삼성</t>
+  </si>
+  <si>
+    <t>신영</t>
+  </si>
+  <si>
+    <t>유진</t>
+  </si>
+  <si>
+    <t>NH</t>
+  </si>
+  <si>
+    <t>한국</t>
+  </si>
+  <si>
+    <t>대신</t>
+  </si>
+  <si>
+    <t>하나</t>
+  </si>
+  <si>
+    <t>키움</t>
+  </si>
+  <si>
+    <t>교보</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>대표</t>
+  </si>
+  <si>
+    <t>인수</t>
+  </si>
+  <si>
+    <t>2024-09-02</t>
+  </si>
+  <si>
+    <t>2024-08-09</t>
+  </si>
+  <si>
+    <t>2024-08-08</t>
+  </si>
+  <si>
+    <t>2024-08-07</t>
+  </si>
+  <si>
+    <t>2024-08-01</t>
+  </si>
+  <si>
     <t>2024-07-25</t>
   </si>
   <si>
-    <t>미래에셋비전스팩7호</t>
-  </si>
-  <si>
-    <t>아이스크림미디어</t>
-  </si>
-  <si>
-    <t>M83</t>
-  </si>
-  <si>
-    <t>이엔셀</t>
-  </si>
-  <si>
-    <t>티디에스팜</t>
-  </si>
-  <si>
-    <t>대신밸런스제18호스팩</t>
-  </si>
-  <si>
-    <t>전진건설로봇</t>
-  </si>
-  <si>
-    <t>케이쓰리아이</t>
-  </si>
-  <si>
-    <t>넥스트바이오메디컬</t>
-  </si>
-  <si>
-    <t>유라클</t>
-  </si>
-  <si>
-    <t>교보16호스팩</t>
-  </si>
-  <si>
-    <t>뱅크웨어글로벌</t>
-  </si>
-  <si>
-    <t>아이빔테크놀로지</t>
-  </si>
-  <si>
-    <t>피앤에스미캐닉스</t>
-  </si>
-  <si>
-    <t>산일전기</t>
-  </si>
-  <si>
-    <t>엔에이치스팩31호</t>
-  </si>
-  <si>
-    <t>SK증권제13호스팩</t>
-  </si>
-  <si>
-    <t>코스닥</t>
-  </si>
-  <si>
-    <t>코스피</t>
-  </si>
-  <si>
-    <t>미래</t>
-  </si>
-  <si>
-    <t>삼성</t>
-  </si>
-  <si>
-    <t>신영</t>
-  </si>
-  <si>
-    <t>유진</t>
-  </si>
-  <si>
-    <t>NH</t>
-  </si>
-  <si>
-    <t>한국</t>
-  </si>
-  <si>
-    <t>대신</t>
-  </si>
-  <si>
-    <t>하나</t>
-  </si>
-  <si>
-    <t>키움</t>
-  </si>
-  <si>
-    <t>교보</t>
-  </si>
-  <si>
-    <t>SK</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>대표</t>
-  </si>
-  <si>
-    <t>인수</t>
-  </si>
-  <si>
-    <t>2024-09-02</t>
-  </si>
-  <si>
-    <t>2024-08-09</t>
-  </si>
-  <si>
-    <t>2024-08-08</t>
-  </si>
-  <si>
-    <t>2024-08-07</t>
-  </si>
-  <si>
-    <t>2024-08-01</t>
-  </si>
-  <si>
     <t>2024-07-22</t>
   </si>
   <si>
@@ -237,9 +231,6 @@
     <t>2024-07-16</t>
   </si>
   <si>
-    <t>2024-07-15</t>
-  </si>
-  <si>
     <t>2024-09-05</t>
   </si>
   <si>
@@ -355,9 +346,6 @@
   </si>
   <si>
     <t>1036 : 1</t>
-  </si>
-  <si>
-    <t>1654.28 : 1</t>
   </si>
   <si>
     <t>인수기관</t>
@@ -730,7 +718,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -791,37 +779,37 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D2">
         <v>159</v>
       </c>
       <c r="E2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F2">
         <v>159</v>
       </c>
       <c r="G2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M2">
         <v>2000</v>
@@ -830,10 +818,10 @@
         <v>100</v>
       </c>
       <c r="O2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="P2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="Q2">
         <v>5962500</v>
@@ -844,37 +832,37 @@
         <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D3">
         <v>787.2</v>
       </c>
       <c r="E3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F3">
         <v>787.2</v>
       </c>
       <c r="G3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M3">
         <v>32000</v>
@@ -886,7 +874,7 @@
         <v>21</v>
       </c>
       <c r="P3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="Q3">
         <v>1722000</v>
@@ -897,37 +885,37 @@
         <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D4">
         <v>240</v>
       </c>
       <c r="E4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F4">
         <v>228</v>
       </c>
       <c r="G4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M4">
         <v>16000</v>
@@ -950,37 +938,37 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D5">
         <v>240</v>
       </c>
       <c r="E5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F5">
         <v>12</v>
       </c>
       <c r="G5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K5" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="L5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M5">
         <v>16000</v>
@@ -1003,37 +991,37 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D6">
         <v>239.7204</v>
       </c>
       <c r="E6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F6">
         <v>239.7204</v>
       </c>
       <c r="G6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K6" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M6">
         <v>15300</v>
@@ -1056,37 +1044,37 @@
         <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D7">
         <v>130</v>
       </c>
       <c r="E7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F7">
         <v>130</v>
       </c>
       <c r="G7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M7">
         <v>13000</v>
@@ -1095,10 +1083,10 @@
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="P7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q7">
         <v>723700</v>
@@ -1109,37 +1097,37 @@
         <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D8">
         <v>130</v>
       </c>
       <c r="E8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F8">
         <v>130</v>
       </c>
       <c r="G8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K8" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M8">
         <v>2000</v>
@@ -1148,10 +1136,10 @@
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="P8" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="Q8">
         <v>4875000</v>
@@ -1162,37 +1150,37 @@
         <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D9">
         <v>507.81225</v>
       </c>
       <c r="E9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F9">
         <v>507.81225</v>
       </c>
       <c r="G9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K9" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M9">
         <v>16500</v>
@@ -1201,7 +1189,7 @@
         <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="P9" t="s">
         <v>25</v>
@@ -1215,37 +1203,37 @@
         <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D10">
         <v>217</v>
       </c>
       <c r="E10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F10">
         <v>217</v>
       </c>
       <c r="G10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K10" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M10">
         <v>15500</v>
@@ -1254,7 +1242,7 @@
         <v>100</v>
       </c>
       <c r="O10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="P10" t="s">
         <v>25</v>
@@ -1268,37 +1256,37 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D11">
         <v>290</v>
       </c>
       <c r="E11" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F11">
         <v>290</v>
       </c>
       <c r="G11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K11" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M11">
         <v>29000</v>
@@ -1307,7 +1295,7 @@
         <v>100</v>
       </c>
       <c r="O11" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="P11" t="s">
         <v>26</v>
@@ -1321,37 +1309,37 @@
         <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D12">
         <v>157.71</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F12">
         <v>157.71</v>
       </c>
       <c r="G12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K12" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M12">
         <v>21000</v>
@@ -1363,7 +1351,7 @@
         <v>27</v>
       </c>
       <c r="P12" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="Q12">
         <v>540250</v>
@@ -1374,37 +1362,37 @@
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D13">
         <v>116</v>
       </c>
       <c r="E13" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F13">
         <v>116</v>
       </c>
       <c r="G13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K13" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M13">
         <v>2000</v>
@@ -1413,7 +1401,7 @@
         <v>100</v>
       </c>
       <c r="O13" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="P13" t="s">
         <v>27</v>
@@ -1427,37 +1415,37 @@
         <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D14">
         <v>224</v>
       </c>
       <c r="E14" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F14">
         <v>224</v>
       </c>
       <c r="G14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K14" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M14">
         <v>16000</v>
@@ -1466,7 +1454,7 @@
         <v>100</v>
       </c>
       <c r="O14" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="P14" t="s">
         <v>27</v>
@@ -1480,37 +1468,37 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D15">
         <v>223.4</v>
       </c>
       <c r="E15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F15">
         <v>223.4</v>
       </c>
       <c r="G15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K15" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M15">
         <v>10000</v>
@@ -1519,10 +1507,10 @@
         <v>100</v>
       </c>
       <c r="O15" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="P15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Q15">
         <v>1675500</v>
@@ -1533,37 +1521,37 @@
         <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D16">
         <v>297</v>
       </c>
       <c r="E16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F16">
         <v>297</v>
       </c>
       <c r="G16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K16" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M16">
         <v>22000</v>
@@ -1572,10 +1560,10 @@
         <v>100</v>
       </c>
       <c r="O16" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="P16" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="Q16">
         <v>1012500</v>
@@ -1586,37 +1574,37 @@
         <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D17">
         <v>2660</v>
       </c>
       <c r="E17" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F17">
         <v>2553.6</v>
       </c>
       <c r="G17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K17" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M17">
         <v>35000</v>
@@ -1625,10 +1613,10 @@
         <v>96</v>
       </c>
       <c r="O17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P17" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="Q17">
         <v>9340690</v>
@@ -1639,37 +1627,37 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C18" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D18">
         <v>2660</v>
       </c>
       <c r="E18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F18">
         <v>106.4</v>
       </c>
       <c r="G18" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H18" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I18" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J18" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K18" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="L18" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M18">
         <v>35000</v>
@@ -1678,10 +1666,10 @@
         <v>4</v>
       </c>
       <c r="O18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P18" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="Q18">
         <v>9340690</v>
@@ -1692,37 +1680,37 @@
         <v>30</v>
       </c>
       <c r="B19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" t="s">
         <v>47</v>
-      </c>
-      <c r="C19" t="s">
-        <v>49</v>
       </c>
       <c r="D19">
         <v>120</v>
       </c>
       <c r="E19" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F19">
         <v>120</v>
       </c>
       <c r="G19" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H19" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I19" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J19" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K19" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L19" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M19">
         <v>2000</v>
@@ -1731,66 +1719,13 @@
         <v>100</v>
       </c>
       <c r="O19" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="P19" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="Q19">
         <v>4500000</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17">
-      <c r="A20" t="s">
-        <v>31</v>
-      </c>
-      <c r="B20" t="s">
-        <v>48</v>
-      </c>
-      <c r="C20" t="s">
-        <v>49</v>
-      </c>
-      <c r="D20">
-        <v>80</v>
-      </c>
-      <c r="E20" t="s">
-        <v>61</v>
-      </c>
-      <c r="F20">
-        <v>80</v>
-      </c>
-      <c r="G20" t="s">
-        <v>62</v>
-      </c>
-      <c r="H20" t="s">
-        <v>62</v>
-      </c>
-      <c r="I20" t="s">
-        <v>62</v>
-      </c>
-      <c r="J20" t="s">
-        <v>62</v>
-      </c>
-      <c r="K20" t="s">
-        <v>63</v>
-      </c>
-      <c r="L20" t="s">
-        <v>62</v>
-      </c>
-      <c r="M20">
-        <v>2000</v>
-      </c>
-      <c r="N20">
-        <v>100</v>
-      </c>
-      <c r="O20" t="s">
-        <v>73</v>
-      </c>
-      <c r="P20" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q20">
-        <v>3000000</v>
       </c>
     </row>
   </sheetData>
@@ -1800,7 +1735,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T18"/>
+  <dimension ref="A1:T17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -1808,10 +1743,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -1820,63 +1755,63 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
@@ -1888,7 +1823,7 @@
         <v>7950000</v>
       </c>
       <c r="H2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I2">
         <v>2000</v>
@@ -1897,34 +1832,34 @@
         <v>2000</v>
       </c>
       <c r="K2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L2">
         <v>2000</v>
       </c>
       <c r="M2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="S2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1932,13 +1867,13 @@
         <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E3" t="s">
         <v>18</v>
@@ -1950,7 +1885,7 @@
         <v>2460000</v>
       </c>
       <c r="H3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I3">
         <v>32000</v>
@@ -1959,34 +1894,34 @@
         <v>40200</v>
       </c>
       <c r="K3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L3">
         <v>32000</v>
       </c>
       <c r="M3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="S3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1994,10 +1929,10 @@
         <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D4" t="s">
         <v>24</v>
@@ -2012,7 +1947,7 @@
         <v>1500000</v>
       </c>
       <c r="H4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I4">
         <v>11000</v>
@@ -2021,34 +1956,34 @@
         <v>13000</v>
       </c>
       <c r="K4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L4">
         <v>16000</v>
       </c>
       <c r="M4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R4" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="S4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -2056,10 +1991,10 @@
         <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D5" t="s">
         <v>24</v>
@@ -2074,7 +2009,7 @@
         <v>1566800</v>
       </c>
       <c r="H5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I5">
         <v>13600</v>
@@ -2083,48 +2018,48 @@
         <v>15300</v>
       </c>
       <c r="K5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L5">
         <v>15300</v>
       </c>
       <c r="M5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R5" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="S5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E6" t="s">
         <v>21</v>
@@ -2136,7 +2071,7 @@
         <v>1000000</v>
       </c>
       <c r="H6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I6">
         <v>9500</v>
@@ -2145,48 +2080,48 @@
         <v>10700</v>
       </c>
       <c r="K6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L6">
         <v>13000</v>
       </c>
       <c r="M6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O6">
         <v>50</v>
       </c>
       <c r="P6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R6" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="S6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E7" t="s">
         <v>19</v>
@@ -2198,7 +2133,7 @@
         <v>6500000</v>
       </c>
       <c r="H7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I7">
         <v>2000</v>
@@ -2207,45 +2142,45 @@
         <v>2000</v>
       </c>
       <c r="K7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L7">
         <v>2000</v>
       </c>
       <c r="M7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="S7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
         <v>25</v>
@@ -2260,7 +2195,7 @@
         <v>3077650</v>
       </c>
       <c r="H8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I8">
         <v>13800</v>
@@ -2269,45 +2204,45 @@
         <v>15700</v>
       </c>
       <c r="K8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L8">
         <v>16500</v>
       </c>
       <c r="M8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O8">
         <v>100</v>
       </c>
       <c r="P8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R8" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="S8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D9" t="s">
         <v>25</v>
@@ -2322,7 +2257,7 @@
         <v>1400000</v>
       </c>
       <c r="H9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I9">
         <v>12500</v>
@@ -2331,45 +2266,45 @@
         <v>15500</v>
       </c>
       <c r="K9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L9">
         <v>15500</v>
       </c>
       <c r="M9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O9">
         <v>0</v>
       </c>
       <c r="P9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R9" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="S9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D10" t="s">
         <v>26</v>
@@ -2384,7 +2319,7 @@
         <v>1000000</v>
       </c>
       <c r="H10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I10">
         <v>24000</v>
@@ -2393,34 +2328,34 @@
         <v>29000</v>
       </c>
       <c r="K10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L10">
         <v>29000</v>
       </c>
       <c r="M10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O10">
         <v>0</v>
       </c>
       <c r="P10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R10" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="S10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -2428,13 +2363,13 @@
         <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D11" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E11" t="s">
         <v>24</v>
@@ -2446,7 +2381,7 @@
         <v>751000</v>
       </c>
       <c r="H11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I11">
         <v>18000</v>
@@ -2455,45 +2390,45 @@
         <v>21000</v>
       </c>
       <c r="K11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L11">
         <v>21000</v>
       </c>
       <c r="M11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O11">
         <v>72.87616511318242</v>
       </c>
       <c r="P11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R11" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="S11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D12" t="s">
         <v>27</v>
@@ -2508,7 +2443,7 @@
         <v>5800000</v>
       </c>
       <c r="H12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I12">
         <v>2000</v>
@@ -2517,45 +2452,45 @@
         <v>2000</v>
       </c>
       <c r="K12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L12">
         <v>2000</v>
       </c>
       <c r="M12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O12">
         <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R12" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="S12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D13" t="s">
         <v>27</v>
@@ -2570,7 +2505,7 @@
         <v>1400000</v>
       </c>
       <c r="H13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I13">
         <v>16000</v>
@@ -2579,48 +2514,48 @@
         <v>19000</v>
       </c>
       <c r="K13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L13">
         <v>16000</v>
       </c>
       <c r="M13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O13">
         <v>0</v>
       </c>
       <c r="P13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R13" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="S13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D14" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E14" t="s">
         <v>27</v>
@@ -2632,7 +2567,7 @@
         <v>2234000</v>
       </c>
       <c r="H14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I14">
         <v>7300</v>
@@ -2641,48 +2576,48 @@
         <v>8500</v>
       </c>
       <c r="K14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L14">
         <v>10000</v>
       </c>
       <c r="M14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O14">
         <v>0</v>
       </c>
       <c r="P14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R14" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="S14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D15" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="E15" t="s">
         <v>28</v>
@@ -2694,7 +2629,7 @@
         <v>1350000</v>
       </c>
       <c r="H15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I15">
         <v>14000</v>
@@ -2703,48 +2638,48 @@
         <v>17000</v>
       </c>
       <c r="K15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L15">
         <v>22000</v>
       </c>
       <c r="M15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O15">
         <v>0</v>
       </c>
       <c r="P15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R15" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="S15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:20">
       <c r="A16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D16" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
@@ -2756,7 +2691,7 @@
         <v>7600000</v>
       </c>
       <c r="H16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I16">
         <v>24000</v>
@@ -2765,48 +2700,48 @@
         <v>30000</v>
       </c>
       <c r="K16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L16">
         <v>35000</v>
       </c>
       <c r="M16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O16">
         <v>14.47368421052632</v>
       </c>
       <c r="P16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R16" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="S16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:20">
       <c r="A17" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D17" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E17" t="s">
         <v>30</v>
@@ -2818,7 +2753,7 @@
         <v>6000000</v>
       </c>
       <c r="H17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I17">
         <v>2000</v>
@@ -2827,96 +2762,34 @@
         <v>2000</v>
       </c>
       <c r="K17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L17">
         <v>2000</v>
       </c>
       <c r="M17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O17">
         <v>0</v>
       </c>
       <c r="P17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="Q17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="R17" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="S17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T17" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20">
-      <c r="A18" t="s">
-        <v>73</v>
-      </c>
-      <c r="B18" t="s">
-        <v>48</v>
-      </c>
-      <c r="C18" t="s">
-        <v>61</v>
-      </c>
-      <c r="D18" t="s">
-        <v>71</v>
-      </c>
-      <c r="E18" t="s">
-        <v>31</v>
-      </c>
-      <c r="F18">
-        <v>8000000</v>
-      </c>
-      <c r="G18">
-        <v>4000000</v>
-      </c>
-      <c r="H18" t="s">
-        <v>62</v>
-      </c>
-      <c r="I18">
-        <v>2000</v>
-      </c>
-      <c r="J18">
-        <v>2000</v>
-      </c>
-      <c r="K18" t="s">
-        <v>62</v>
-      </c>
-      <c r="L18">
-        <v>2000</v>
-      </c>
-      <c r="M18" t="s">
-        <v>62</v>
-      </c>
-      <c r="N18" t="s">
-        <v>62</v>
-      </c>
-      <c r="O18">
-        <v>0</v>
-      </c>
-      <c r="P18" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>62</v>
-      </c>
-      <c r="R18" t="s">
-        <v>113</v>
-      </c>
-      <c r="S18" t="s">
-        <v>62</v>
-      </c>
-      <c r="T18" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -2926,21 +2799,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -2952,10 +2825,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -2964,39 +2837,39 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>70</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F2" t="s">
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="G2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H2">
-        <v>23972.04</v>
+        <v>12000</v>
       </c>
       <c r="I2">
-        <v>1566800</v>
+        <v>6000000</v>
       </c>
       <c r="J2">
-        <v>15300</v>
+        <v>2000</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -3007,34 +2880,34 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F3" t="s">
-        <v>79</v>
+        <v>24</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H3">
-        <v>12000</v>
+        <v>23972.04</v>
       </c>
       <c r="I3">
-        <v>6000000</v>
+        <v>1566800</v>
       </c>
       <c r="J3">
-        <v>2000</v>
+        <v>15300</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -3045,31 +2918,31 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="F4" t="s">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="H4">
-        <v>8000</v>
+        <v>11600</v>
       </c>
       <c r="I4">
-        <v>4000000</v>
+        <v>5800000</v>
       </c>
       <c r="J4">
         <v>2000</v>
@@ -3083,31 +2956,31 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C5" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="G5" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H5">
-        <v>11600</v>
+        <v>13000</v>
       </c>
       <c r="I5">
-        <v>5800000</v>
+        <v>6500000</v>
       </c>
       <c r="J5">
         <v>2000</v>
@@ -3121,110 +2994,110 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D6" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>113</v>
       </c>
       <c r="F6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G6" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="H6">
-        <v>13000</v>
+        <v>255360</v>
       </c>
       <c r="I6">
-        <v>6500000</v>
+        <v>7600000</v>
       </c>
       <c r="J6">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="K6">
         <v>0</v>
       </c>
       <c r="L6">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
-        <v>117</v>
+        <v>49</v>
       </c>
       <c r="F7" t="s">
-        <v>78</v>
+        <v>27</v>
       </c>
       <c r="G7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H7">
-        <v>255360</v>
+        <v>22400</v>
       </c>
       <c r="I7">
-        <v>7600000</v>
+        <v>1400000</v>
       </c>
       <c r="J7">
-        <v>35000</v>
+        <v>16000</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G8" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H8">
-        <v>22400</v>
+        <v>50781.225</v>
       </c>
       <c r="I8">
-        <v>1400000</v>
+        <v>3077650</v>
       </c>
       <c r="J8">
-        <v>16000</v>
+        <v>16500</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -3235,22 +3108,22 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="G9" t="s">
         <v>17</v>
@@ -3273,60 +3146,60 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>51</v>
+        <v>113</v>
       </c>
       <c r="F10" t="s">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="G10" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="H10">
-        <v>50781.225</v>
+        <v>10640</v>
       </c>
       <c r="I10">
-        <v>3077650</v>
+        <v>7600000</v>
       </c>
       <c r="J10">
-        <v>16500</v>
+        <v>35000</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>100</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E11" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F11" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="G11" t="s">
         <v>27</v>
@@ -3349,22 +3222,22 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B12" t="s">
         <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E12" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F12" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="G12" t="s">
         <v>18</v>
@@ -3387,57 +3260,57 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B13" t="s">
-        <v>71</v>
+        <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="D13" t="s">
         <v>51</v>
       </c>
       <c r="E13" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F13" t="s">
-        <v>78</v>
+        <v>24</v>
       </c>
       <c r="G13" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="H13">
-        <v>10640</v>
+        <v>22800</v>
       </c>
       <c r="I13">
-        <v>7600000</v>
+        <v>1500000</v>
       </c>
       <c r="J13">
-        <v>35000</v>
+        <v>16000</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
-        <v>4</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B14" t="s">
         <v>26</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E14" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F14" t="s">
         <v>24</v>
@@ -3446,7 +3319,7 @@
         <v>19</v>
       </c>
       <c r="H14">
-        <v>22800</v>
+        <v>1200</v>
       </c>
       <c r="I14">
         <v>1500000</v>
@@ -3458,77 +3331,77 @@
         <v>0</v>
       </c>
       <c r="L14">
-        <v>95</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D15" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E15" t="s">
-        <v>118</v>
+        <v>57</v>
       </c>
       <c r="F15" t="s">
+        <v>63</v>
+      </c>
+      <c r="G15" t="s">
         <v>24</v>
       </c>
-      <c r="G15" t="s">
-        <v>19</v>
-      </c>
       <c r="H15">
-        <v>1200</v>
+        <v>15771</v>
       </c>
       <c r="I15">
-        <v>1500000</v>
+        <v>751000</v>
       </c>
       <c r="J15">
-        <v>16000</v>
+        <v>21000</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>68</v>
       </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F16" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G16" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="H16">
-        <v>15771</v>
+        <v>29700</v>
       </c>
       <c r="I16">
-        <v>751000</v>
+        <v>1350000</v>
       </c>
       <c r="J16">
-        <v>21000</v>
+        <v>22000</v>
       </c>
       <c r="K16">
         <v>0</v>
@@ -3539,34 +3412,34 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C17" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="D17" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E17" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F17" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="G17" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="H17">
-        <v>29700</v>
+        <v>21700</v>
       </c>
       <c r="I17">
-        <v>1350000</v>
+        <v>1400000</v>
       </c>
       <c r="J17">
-        <v>22000</v>
+        <v>15500</v>
       </c>
       <c r="K17">
         <v>0</v>
@@ -3577,34 +3450,34 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C18" t="s">
         <v>39</v>
       </c>
       <c r="D18" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E18" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F18" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G18" t="s">
         <v>23</v>
       </c>
       <c r="H18">
-        <v>21700</v>
+        <v>29000</v>
       </c>
       <c r="I18">
-        <v>1400000</v>
+        <v>1000000</v>
       </c>
       <c r="J18">
-        <v>15500</v>
+        <v>29000</v>
       </c>
       <c r="K18">
         <v>0</v>
@@ -3615,22 +3488,22 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B19" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D19" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E19" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F19" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G19" t="s">
         <v>21</v>
@@ -3648,44 +3521,6 @@
         <v>0</v>
       </c>
       <c r="L19">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12">
-      <c r="A20" t="s">
-        <v>56</v>
-      </c>
-      <c r="B20" t="s">
-        <v>68</v>
-      </c>
-      <c r="C20" t="s">
-        <v>40</v>
-      </c>
-      <c r="D20" t="s">
-        <v>56</v>
-      </c>
-      <c r="E20" t="s">
-        <v>56</v>
-      </c>
-      <c r="F20" t="s">
-        <v>26</v>
-      </c>
-      <c r="G20" t="s">
-        <v>23</v>
-      </c>
-      <c r="H20">
-        <v>29000</v>
-      </c>
-      <c r="I20">
-        <v>1000000</v>
-      </c>
-      <c r="J20">
-        <v>29000</v>
-      </c>
-      <c r="K20">
-        <v>0</v>
-      </c>
-      <c r="L20">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-18
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="110">
   <si>
     <t>상장일</t>
   </si>
@@ -108,9 +108,6 @@
     <t>2024-07-29</t>
   </si>
   <si>
-    <t>2024-07-26</t>
-  </si>
-  <si>
     <t>미래에셋비전스팩7호</t>
   </si>
   <si>
@@ -156,9 +153,6 @@
     <t>산일전기</t>
   </si>
   <si>
-    <t>엔에이치스팩31호</t>
-  </si>
-  <si>
     <t>코스닥</t>
   </si>
   <si>
@@ -228,9 +222,6 @@
     <t>2024-07-18</t>
   </si>
   <si>
-    <t>2024-07-16</t>
-  </si>
-  <si>
     <t>2024-09-05</t>
   </si>
   <si>
@@ -246,9 +237,6 @@
     <t>2024-07-23</t>
   </si>
   <si>
-    <t>2024-07-19</t>
-  </si>
-  <si>
     <t>회사명</t>
   </si>
   <si>
@@ -343,9 +331,6 @@
   </si>
   <si>
     <t>423.09 : 1</t>
-  </si>
-  <si>
-    <t>1036 : 1</t>
   </si>
   <si>
     <t>인수기관</t>
@@ -718,7 +703,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -779,37 +764,37 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D2">
         <v>159</v>
       </c>
       <c r="E2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F2">
         <v>159</v>
       </c>
       <c r="G2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M2">
         <v>2000</v>
@@ -818,10 +803,10 @@
         <v>100</v>
       </c>
       <c r="O2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="P2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="Q2">
         <v>5962500</v>
@@ -832,37 +817,37 @@
         <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D3">
         <v>787.2</v>
       </c>
       <c r="E3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F3">
         <v>787.2</v>
       </c>
       <c r="G3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M3">
         <v>32000</v>
@@ -874,7 +859,7 @@
         <v>21</v>
       </c>
       <c r="P3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="Q3">
         <v>1722000</v>
@@ -885,37 +870,37 @@
         <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D4">
         <v>240</v>
       </c>
       <c r="E4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F4">
         <v>228</v>
       </c>
       <c r="G4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M4">
         <v>16000</v>
@@ -938,37 +923,37 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D5">
         <v>240</v>
       </c>
       <c r="E5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F5">
         <v>12</v>
       </c>
       <c r="G5" t="s">
+        <v>57</v>
+      </c>
+      <c r="H5" t="s">
+        <v>57</v>
+      </c>
+      <c r="I5" t="s">
+        <v>57</v>
+      </c>
+      <c r="J5" t="s">
+        <v>57</v>
+      </c>
+      <c r="K5" t="s">
         <v>59</v>
       </c>
-      <c r="H5" t="s">
-        <v>59</v>
-      </c>
-      <c r="I5" t="s">
-        <v>59</v>
-      </c>
-      <c r="J5" t="s">
-        <v>59</v>
-      </c>
-      <c r="K5" t="s">
-        <v>61</v>
-      </c>
       <c r="L5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M5">
         <v>16000</v>
@@ -991,37 +976,37 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D6">
         <v>239.7204</v>
       </c>
       <c r="E6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F6">
         <v>239.7204</v>
       </c>
       <c r="G6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M6">
         <v>15300</v>
@@ -1044,37 +1029,37 @@
         <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D7">
         <v>130</v>
       </c>
       <c r="E7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F7">
         <v>130</v>
       </c>
       <c r="G7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M7">
         <v>13000</v>
@@ -1083,10 +1068,10 @@
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="P7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="Q7">
         <v>723700</v>
@@ -1097,37 +1082,37 @@
         <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D8">
         <v>130</v>
       </c>
       <c r="E8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F8">
         <v>130</v>
       </c>
       <c r="G8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M8">
         <v>2000</v>
@@ -1136,10 +1121,10 @@
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="P8" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="Q8">
         <v>4875000</v>
@@ -1150,37 +1135,37 @@
         <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D9">
         <v>507.81225</v>
       </c>
       <c r="E9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F9">
         <v>507.81225</v>
       </c>
       <c r="G9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M9">
         <v>16500</v>
@@ -1189,7 +1174,7 @@
         <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="P9" t="s">
         <v>25</v>
@@ -1203,37 +1188,37 @@
         <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D10">
         <v>217</v>
       </c>
       <c r="E10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F10">
         <v>217</v>
       </c>
       <c r="G10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K10" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M10">
         <v>15500</v>
@@ -1242,7 +1227,7 @@
         <v>100</v>
       </c>
       <c r="O10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="P10" t="s">
         <v>25</v>
@@ -1256,37 +1241,37 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D11">
         <v>290</v>
       </c>
       <c r="E11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F11">
         <v>290</v>
       </c>
       <c r="G11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K11" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M11">
         <v>29000</v>
@@ -1295,7 +1280,7 @@
         <v>100</v>
       </c>
       <c r="O11" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="P11" t="s">
         <v>26</v>
@@ -1309,37 +1294,37 @@
         <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D12">
         <v>157.71</v>
       </c>
       <c r="E12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F12">
         <v>157.71</v>
       </c>
       <c r="G12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M12">
         <v>21000</v>
@@ -1351,7 +1336,7 @@
         <v>27</v>
       </c>
       <c r="P12" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="Q12">
         <v>540250</v>
@@ -1362,37 +1347,37 @@
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D13">
         <v>116</v>
       </c>
       <c r="E13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F13">
         <v>116</v>
       </c>
       <c r="G13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K13" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M13">
         <v>2000</v>
@@ -1401,7 +1386,7 @@
         <v>100</v>
       </c>
       <c r="O13" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="P13" t="s">
         <v>27</v>
@@ -1415,37 +1400,37 @@
         <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D14">
         <v>224</v>
       </c>
       <c r="E14" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F14">
         <v>224</v>
       </c>
       <c r="G14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K14" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M14">
         <v>16000</v>
@@ -1454,7 +1439,7 @@
         <v>100</v>
       </c>
       <c r="O14" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="P14" t="s">
         <v>27</v>
@@ -1468,37 +1453,37 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D15">
         <v>223.4</v>
       </c>
       <c r="E15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F15">
         <v>223.4</v>
       </c>
       <c r="G15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K15" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M15">
         <v>10000</v>
@@ -1507,10 +1492,10 @@
         <v>100</v>
       </c>
       <c r="O15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="P15" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="Q15">
         <v>1675500</v>
@@ -1521,37 +1506,37 @@
         <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D16">
         <v>297</v>
       </c>
       <c r="E16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F16">
         <v>297</v>
       </c>
       <c r="G16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K16" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M16">
         <v>22000</v>
@@ -1560,10 +1545,10 @@
         <v>100</v>
       </c>
       <c r="O16" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="P16" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="Q16">
         <v>1012500</v>
@@ -1574,37 +1559,37 @@
         <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D17">
         <v>2660</v>
       </c>
       <c r="E17" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F17">
         <v>2553.6</v>
       </c>
       <c r="G17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K17" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M17">
         <v>35000</v>
@@ -1613,10 +1598,10 @@
         <v>96</v>
       </c>
       <c r="O17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="P17" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="Q17">
         <v>9340690</v>
@@ -1627,37 +1612,37 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C18" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D18">
         <v>2660</v>
       </c>
       <c r="E18" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F18">
         <v>106.4</v>
       </c>
       <c r="G18" t="s">
+        <v>57</v>
+      </c>
+      <c r="H18" t="s">
+        <v>57</v>
+      </c>
+      <c r="I18" t="s">
+        <v>57</v>
+      </c>
+      <c r="J18" t="s">
+        <v>57</v>
+      </c>
+      <c r="K18" t="s">
         <v>59</v>
       </c>
-      <c r="H18" t="s">
-        <v>59</v>
-      </c>
-      <c r="I18" t="s">
-        <v>59</v>
-      </c>
-      <c r="J18" t="s">
-        <v>59</v>
-      </c>
-      <c r="K18" t="s">
-        <v>61</v>
-      </c>
       <c r="L18" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M18">
         <v>35000</v>
@@ -1666,66 +1651,13 @@
         <v>4</v>
       </c>
       <c r="O18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="P18" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="Q18">
         <v>9340690</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17">
-      <c r="A19" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" t="s">
-        <v>46</v>
-      </c>
-      <c r="C19" t="s">
-        <v>47</v>
-      </c>
-      <c r="D19">
-        <v>120</v>
-      </c>
-      <c r="E19" t="s">
-        <v>53</v>
-      </c>
-      <c r="F19">
-        <v>120</v>
-      </c>
-      <c r="G19" t="s">
-        <v>59</v>
-      </c>
-      <c r="H19" t="s">
-        <v>59</v>
-      </c>
-      <c r="I19" t="s">
-        <v>59</v>
-      </c>
-      <c r="J19" t="s">
-        <v>59</v>
-      </c>
-      <c r="K19" t="s">
-        <v>60</v>
-      </c>
-      <c r="L19" t="s">
-        <v>59</v>
-      </c>
-      <c r="M19">
-        <v>2000</v>
-      </c>
-      <c r="N19">
-        <v>100</v>
-      </c>
-      <c r="O19" t="s">
-        <v>70</v>
-      </c>
-      <c r="P19" t="s">
-        <v>76</v>
-      </c>
-      <c r="Q19">
-        <v>4500000</v>
       </c>
     </row>
   </sheetData>
@@ -1735,7 +1667,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T17"/>
+  <dimension ref="A1:T16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -1743,10 +1675,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -1755,63 +1687,63 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
@@ -1823,7 +1755,7 @@
         <v>7950000</v>
       </c>
       <c r="H2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I2">
         <v>2000</v>
@@ -1832,34 +1764,34 @@
         <v>2000</v>
       </c>
       <c r="K2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L2">
         <v>2000</v>
       </c>
       <c r="M2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="S2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1867,13 +1799,13 @@
         <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E3" t="s">
         <v>18</v>
@@ -1885,7 +1817,7 @@
         <v>2460000</v>
       </c>
       <c r="H3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I3">
         <v>32000</v>
@@ -1894,34 +1826,34 @@
         <v>40200</v>
       </c>
       <c r="K3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L3">
         <v>32000</v>
       </c>
       <c r="M3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="S3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1929,10 +1861,10 @@
         <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
         <v>24</v>
@@ -1947,7 +1879,7 @@
         <v>1500000</v>
       </c>
       <c r="H4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I4">
         <v>11000</v>
@@ -1956,34 +1888,34 @@
         <v>13000</v>
       </c>
       <c r="K4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L4">
         <v>16000</v>
       </c>
       <c r="M4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="S4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -1991,10 +1923,10 @@
         <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D5" t="s">
         <v>24</v>
@@ -2009,7 +1941,7 @@
         <v>1566800</v>
       </c>
       <c r="H5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I5">
         <v>13600</v>
@@ -2018,48 +1950,48 @@
         <v>15300</v>
       </c>
       <c r="K5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L5">
         <v>15300</v>
       </c>
       <c r="M5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R5" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="S5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E6" t="s">
         <v>21</v>
@@ -2071,7 +2003,7 @@
         <v>1000000</v>
       </c>
       <c r="H6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I6">
         <v>9500</v>
@@ -2080,48 +2012,48 @@
         <v>10700</v>
       </c>
       <c r="K6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L6">
         <v>13000</v>
       </c>
       <c r="M6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O6">
         <v>50</v>
       </c>
       <c r="P6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R6" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="S6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E7" t="s">
         <v>19</v>
@@ -2133,7 +2065,7 @@
         <v>6500000</v>
       </c>
       <c r="H7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I7">
         <v>2000</v>
@@ -2142,45 +2074,45 @@
         <v>2000</v>
       </c>
       <c r="K7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L7">
         <v>2000</v>
       </c>
       <c r="M7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R7" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="S7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D8" t="s">
         <v>25</v>
@@ -2195,7 +2127,7 @@
         <v>3077650</v>
       </c>
       <c r="H8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I8">
         <v>13800</v>
@@ -2204,45 +2136,45 @@
         <v>15700</v>
       </c>
       <c r="K8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L8">
         <v>16500</v>
       </c>
       <c r="M8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O8">
         <v>100</v>
       </c>
       <c r="P8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R8" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="S8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D9" t="s">
         <v>25</v>
@@ -2257,7 +2189,7 @@
         <v>1400000</v>
       </c>
       <c r="H9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I9">
         <v>12500</v>
@@ -2266,45 +2198,45 @@
         <v>15500</v>
       </c>
       <c r="K9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L9">
         <v>15500</v>
       </c>
       <c r="M9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O9">
         <v>0</v>
       </c>
       <c r="P9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R9" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="S9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D10" t="s">
         <v>26</v>
@@ -2319,7 +2251,7 @@
         <v>1000000</v>
       </c>
       <c r="H10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I10">
         <v>24000</v>
@@ -2328,34 +2260,34 @@
         <v>29000</v>
       </c>
       <c r="K10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L10">
         <v>29000</v>
       </c>
       <c r="M10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O10">
         <v>0</v>
       </c>
       <c r="P10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R10" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="S10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -2363,13 +2295,13 @@
         <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E11" t="s">
         <v>24</v>
@@ -2381,7 +2313,7 @@
         <v>751000</v>
       </c>
       <c r="H11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I11">
         <v>18000</v>
@@ -2390,45 +2322,45 @@
         <v>21000</v>
       </c>
       <c r="K11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L11">
         <v>21000</v>
       </c>
       <c r="M11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O11">
         <v>72.87616511318242</v>
       </c>
       <c r="P11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R11" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="S11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D12" t="s">
         <v>27</v>
@@ -2443,7 +2375,7 @@
         <v>5800000</v>
       </c>
       <c r="H12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I12">
         <v>2000</v>
@@ -2452,45 +2384,45 @@
         <v>2000</v>
       </c>
       <c r="K12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L12">
         <v>2000</v>
       </c>
       <c r="M12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O12">
         <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R12" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="S12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D13" t="s">
         <v>27</v>
@@ -2505,7 +2437,7 @@
         <v>1400000</v>
       </c>
       <c r="H13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I13">
         <v>16000</v>
@@ -2514,48 +2446,48 @@
         <v>19000</v>
       </c>
       <c r="K13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L13">
         <v>16000</v>
       </c>
       <c r="M13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O13">
         <v>0</v>
       </c>
       <c r="P13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R13" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="S13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D14" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E14" t="s">
         <v>27</v>
@@ -2567,7 +2499,7 @@
         <v>2234000</v>
       </c>
       <c r="H14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I14">
         <v>7300</v>
@@ -2576,48 +2508,48 @@
         <v>8500</v>
       </c>
       <c r="K14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L14">
         <v>10000</v>
       </c>
       <c r="M14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O14">
         <v>0</v>
       </c>
       <c r="P14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R14" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="S14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E15" t="s">
         <v>28</v>
@@ -2629,7 +2561,7 @@
         <v>1350000</v>
       </c>
       <c r="H15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I15">
         <v>14000</v>
@@ -2638,48 +2570,48 @@
         <v>17000</v>
       </c>
       <c r="K15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L15">
         <v>22000</v>
       </c>
       <c r="M15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O15">
         <v>0</v>
       </c>
       <c r="P15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R15" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="S15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:20">
       <c r="A16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
@@ -2691,7 +2623,7 @@
         <v>7600000</v>
       </c>
       <c r="H16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I16">
         <v>24000</v>
@@ -2700,96 +2632,34 @@
         <v>30000</v>
       </c>
       <c r="K16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L16">
         <v>35000</v>
       </c>
       <c r="M16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O16">
         <v>14.47368421052632</v>
       </c>
       <c r="P16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="R16" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="S16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T16" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20">
-      <c r="A17" t="s">
-        <v>70</v>
-      </c>
-      <c r="B17" t="s">
-        <v>46</v>
-      </c>
-      <c r="C17" t="s">
-        <v>53</v>
-      </c>
-      <c r="D17" t="s">
-        <v>76</v>
-      </c>
-      <c r="E17" t="s">
-        <v>30</v>
-      </c>
-      <c r="F17">
-        <v>12000000</v>
-      </c>
-      <c r="G17">
-        <v>6000000</v>
-      </c>
-      <c r="H17" t="s">
-        <v>59</v>
-      </c>
-      <c r="I17">
-        <v>2000</v>
-      </c>
-      <c r="J17">
-        <v>2000</v>
-      </c>
-      <c r="K17" t="s">
-        <v>59</v>
-      </c>
-      <c r="L17">
-        <v>2000</v>
-      </c>
-      <c r="M17" t="s">
-        <v>59</v>
-      </c>
-      <c r="N17" t="s">
-        <v>59</v>
-      </c>
-      <c r="O17">
-        <v>0</v>
-      </c>
-      <c r="P17" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>59</v>
-      </c>
-      <c r="R17" t="s">
-        <v>109</v>
-      </c>
-      <c r="S17" t="s">
-        <v>59</v>
-      </c>
-      <c r="T17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -2799,21 +2669,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -2825,10 +2695,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -2837,39 +2707,39 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F2" t="s">
-        <v>76</v>
+        <v>24</v>
       </c>
       <c r="G2" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H2">
-        <v>12000</v>
+        <v>23972.04</v>
       </c>
       <c r="I2">
-        <v>6000000</v>
+        <v>1566800</v>
       </c>
       <c r="J2">
-        <v>2000</v>
+        <v>15300</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -2880,34 +2750,34 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H3">
-        <v>23972.04</v>
+        <v>11600</v>
       </c>
       <c r="I3">
-        <v>1566800</v>
+        <v>5800000</v>
       </c>
       <c r="J3">
-        <v>15300</v>
+        <v>2000</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -2918,31 +2788,31 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C4" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E4" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="F4" t="s">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="G4" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H4">
-        <v>11600</v>
+        <v>13000</v>
       </c>
       <c r="I4">
-        <v>5800000</v>
+        <v>6500000</v>
       </c>
       <c r="J4">
         <v>2000</v>
@@ -2956,31 +2826,31 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="F5" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="G5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="H5">
-        <v>13000</v>
+        <v>15900</v>
       </c>
       <c r="I5">
-        <v>6500000</v>
+        <v>7950000</v>
       </c>
       <c r="J5">
         <v>2000</v>
@@ -2994,95 +2864,95 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E6" t="s">
-        <v>113</v>
+        <v>47</v>
       </c>
       <c r="F6" t="s">
-        <v>75</v>
+        <v>27</v>
       </c>
       <c r="G6" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H6">
-        <v>255360</v>
+        <v>22400</v>
       </c>
       <c r="I6">
-        <v>7600000</v>
+        <v>1400000</v>
       </c>
       <c r="J6">
-        <v>35000</v>
+        <v>16000</v>
       </c>
       <c r="K6">
         <v>0</v>
       </c>
       <c r="L6">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>108</v>
       </c>
       <c r="F7" t="s">
-        <v>27</v>
+        <v>72</v>
       </c>
       <c r="G7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="H7">
-        <v>22400</v>
+        <v>255360</v>
       </c>
       <c r="I7">
-        <v>1400000</v>
+        <v>7600000</v>
       </c>
       <c r="J7">
-        <v>16000</v>
+        <v>35000</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F8" t="s">
         <v>25</v>
@@ -3108,34 +2978,34 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F9" t="s">
         <v>71</v>
       </c>
       <c r="G9" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="H9">
-        <v>15900</v>
+        <v>22340</v>
       </c>
       <c r="I9">
-        <v>7950000</v>
+        <v>2234000</v>
       </c>
       <c r="J9">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -3146,22 +3016,22 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E10" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="F10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="G10" t="s">
         <v>29</v>
@@ -3184,34 +3054,34 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B11" t="s">
-        <v>67</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F11" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="G11" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="H11">
-        <v>22340</v>
+        <v>78720</v>
       </c>
       <c r="I11">
-        <v>2234000</v>
+        <v>2460000</v>
       </c>
       <c r="J11">
-        <v>10000</v>
+        <v>32000</v>
       </c>
       <c r="K11">
         <v>0</v>
@@ -3222,57 +3092,57 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
         <v>32</v>
       </c>
       <c r="D12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E12" t="s">
-        <v>50</v>
+        <v>109</v>
       </c>
       <c r="F12" t="s">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="G12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H12">
-        <v>78720</v>
+        <v>22800</v>
       </c>
       <c r="I12">
-        <v>2460000</v>
+        <v>1500000</v>
       </c>
       <c r="J12">
-        <v>32000</v>
+        <v>16000</v>
       </c>
       <c r="K12">
         <v>0</v>
       </c>
       <c r="L12">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B13" t="s">
         <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E13" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="F13" t="s">
         <v>24</v>
@@ -3281,7 +3151,7 @@
         <v>19</v>
       </c>
       <c r="H13">
-        <v>22800</v>
+        <v>1200</v>
       </c>
       <c r="I13">
         <v>1500000</v>
@@ -3293,77 +3163,77 @@
         <v>0</v>
       </c>
       <c r="L13">
-        <v>95</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C14" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E14" t="s">
-        <v>114</v>
+        <v>55</v>
       </c>
       <c r="F14" t="s">
+        <v>61</v>
+      </c>
+      <c r="G14" t="s">
         <v>24</v>
       </c>
-      <c r="G14" t="s">
-        <v>19</v>
-      </c>
       <c r="H14">
-        <v>1200</v>
+        <v>15771</v>
       </c>
       <c r="I14">
-        <v>1500000</v>
+        <v>751000</v>
       </c>
       <c r="J14">
-        <v>16000</v>
+        <v>21000</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14">
-        <v>5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="C15" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F15" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G15" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="H15">
-        <v>15771</v>
+        <v>29700</v>
       </c>
       <c r="I15">
-        <v>751000</v>
+        <v>1350000</v>
       </c>
       <c r="J15">
-        <v>21000</v>
+        <v>22000</v>
       </c>
       <c r="K15">
         <v>0</v>
@@ -3374,34 +3244,34 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="D16" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E16" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F16" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="G16" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="H16">
-        <v>29700</v>
+        <v>21700</v>
       </c>
       <c r="I16">
-        <v>1350000</v>
+        <v>1400000</v>
       </c>
       <c r="J16">
-        <v>22000</v>
+        <v>15500</v>
       </c>
       <c r="K16">
         <v>0</v>
@@ -3412,34 +3282,34 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B17" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C17" t="s">
         <v>38</v>
       </c>
       <c r="D17" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E17" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G17" t="s">
         <v>23</v>
       </c>
       <c r="H17">
-        <v>21700</v>
+        <v>29000</v>
       </c>
       <c r="I17">
-        <v>1400000</v>
+        <v>1000000</v>
       </c>
       <c r="J17">
-        <v>15500</v>
+        <v>29000</v>
       </c>
       <c r="K17">
         <v>0</v>
@@ -3450,77 +3320,39 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B18" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C18" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F18" t="s">
-        <v>26</v>
+        <v>70</v>
       </c>
       <c r="G18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H18">
-        <v>29000</v>
+        <v>13000</v>
       </c>
       <c r="I18">
         <v>1000000</v>
       </c>
       <c r="J18">
-        <v>29000</v>
+        <v>13000</v>
       </c>
       <c r="K18">
         <v>0</v>
       </c>
       <c r="L18">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12">
-      <c r="A19" t="s">
-        <v>54</v>
-      </c>
-      <c r="B19" t="s">
-        <v>63</v>
-      </c>
-      <c r="C19" t="s">
-        <v>35</v>
-      </c>
-      <c r="D19" t="s">
-        <v>54</v>
-      </c>
-      <c r="E19" t="s">
-        <v>54</v>
-      </c>
-      <c r="F19" t="s">
-        <v>73</v>
-      </c>
-      <c r="G19" t="s">
-        <v>21</v>
-      </c>
-      <c r="H19">
-        <v>13000</v>
-      </c>
-      <c r="I19">
-        <v>1000000</v>
-      </c>
-      <c r="J19">
-        <v>13000</v>
-      </c>
-      <c r="K19">
-        <v>0</v>
-      </c>
-      <c r="L19">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-22
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="104">
   <si>
     <t>상장일</t>
   </si>
@@ -105,9 +105,6 @@
     <t>2024-07-31</t>
   </si>
   <si>
-    <t>2024-07-29</t>
-  </si>
-  <si>
     <t>미래에셋비전스팩7호</t>
   </si>
   <si>
@@ -150,9 +147,6 @@
     <t>피앤에스미캐닉스</t>
   </si>
   <si>
-    <t>산일전기</t>
-  </si>
-  <si>
     <t>코스닥</t>
   </si>
   <si>
@@ -219,9 +213,6 @@
     <t>2024-07-22</t>
   </si>
   <si>
-    <t>2024-07-18</t>
-  </si>
-  <si>
     <t>2024-09-05</t>
   </si>
   <si>
@@ -234,9 +225,6 @@
     <t>2024-07-30</t>
   </si>
   <si>
-    <t>2024-07-23</t>
-  </si>
-  <si>
     <t>회사명</t>
   </si>
   <si>
@@ -330,9 +318,6 @@
     <t>1585.92 : 1</t>
   </si>
   <si>
-    <t>423.09 : 1</t>
-  </si>
-  <si>
     <t>인수기관</t>
   </si>
   <si>
@@ -340,9 +325,6 @@
   </si>
   <si>
     <t>인수비율</t>
-  </si>
-  <si>
-    <t>미래, 삼성</t>
   </si>
   <si>
     <t>신영, 유진</t>
@@ -703,7 +685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -764,37 +746,37 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D2">
         <v>159</v>
       </c>
       <c r="E2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F2">
         <v>159</v>
       </c>
       <c r="G2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M2">
         <v>2000</v>
@@ -803,10 +785,10 @@
         <v>100</v>
       </c>
       <c r="O2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="P2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="Q2">
         <v>5962500</v>
@@ -817,37 +799,37 @@
         <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D3">
         <v>787.2</v>
       </c>
       <c r="E3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F3">
         <v>787.2</v>
       </c>
       <c r="G3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M3">
         <v>32000</v>
@@ -859,7 +841,7 @@
         <v>21</v>
       </c>
       <c r="P3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Q3">
         <v>1722000</v>
@@ -870,37 +852,37 @@
         <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D4">
         <v>240</v>
       </c>
       <c r="E4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F4">
         <v>228</v>
       </c>
       <c r="G4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M4">
         <v>16000</v>
@@ -923,37 +905,37 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D5">
         <v>240</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F5">
         <v>12</v>
       </c>
       <c r="G5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H5" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5" t="s">
+        <v>55</v>
+      </c>
+      <c r="J5" t="s">
+        <v>55</v>
+      </c>
+      <c r="K5" t="s">
         <v>57</v>
       </c>
-      <c r="H5" t="s">
-        <v>57</v>
-      </c>
-      <c r="I5" t="s">
-        <v>57</v>
-      </c>
-      <c r="J5" t="s">
-        <v>57</v>
-      </c>
-      <c r="K5" t="s">
-        <v>59</v>
-      </c>
       <c r="L5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M5">
         <v>16000</v>
@@ -976,37 +958,37 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D6">
         <v>239.7204</v>
       </c>
       <c r="E6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F6">
         <v>239.7204</v>
       </c>
       <c r="G6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M6">
         <v>15300</v>
@@ -1029,37 +1011,37 @@
         <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D7">
         <v>130</v>
       </c>
       <c r="E7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F7">
         <v>130</v>
       </c>
       <c r="G7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M7">
         <v>13000</v>
@@ -1068,10 +1050,10 @@
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="P7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="Q7">
         <v>723700</v>
@@ -1082,37 +1064,37 @@
         <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D8">
         <v>130</v>
       </c>
       <c r="E8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F8">
         <v>130</v>
       </c>
       <c r="G8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M8">
         <v>2000</v>
@@ -1121,10 +1103,10 @@
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="P8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="Q8">
         <v>4875000</v>
@@ -1135,37 +1117,37 @@
         <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D9">
         <v>507.81225</v>
       </c>
       <c r="E9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F9">
         <v>507.81225</v>
       </c>
       <c r="G9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M9">
         <v>16500</v>
@@ -1174,7 +1156,7 @@
         <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="P9" t="s">
         <v>25</v>
@@ -1188,37 +1170,37 @@
         <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D10">
         <v>217</v>
       </c>
       <c r="E10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F10">
         <v>217</v>
       </c>
       <c r="G10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M10">
         <v>15500</v>
@@ -1227,7 +1209,7 @@
         <v>100</v>
       </c>
       <c r="O10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="P10" t="s">
         <v>25</v>
@@ -1241,37 +1223,37 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D11">
         <v>290</v>
       </c>
       <c r="E11" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F11">
         <v>290</v>
       </c>
       <c r="G11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M11">
         <v>29000</v>
@@ -1280,7 +1262,7 @@
         <v>100</v>
       </c>
       <c r="O11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="P11" t="s">
         <v>26</v>
@@ -1294,37 +1276,37 @@
         <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D12">
         <v>157.71</v>
       </c>
       <c r="E12" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F12">
         <v>157.71</v>
       </c>
       <c r="G12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M12">
         <v>21000</v>
@@ -1336,7 +1318,7 @@
         <v>27</v>
       </c>
       <c r="P12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="Q12">
         <v>540250</v>
@@ -1347,37 +1329,37 @@
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D13">
         <v>116</v>
       </c>
       <c r="E13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F13">
         <v>116</v>
       </c>
       <c r="G13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M13">
         <v>2000</v>
@@ -1386,7 +1368,7 @@
         <v>100</v>
       </c>
       <c r="O13" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="P13" t="s">
         <v>27</v>
@@ -1400,37 +1382,37 @@
         <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D14">
         <v>224</v>
       </c>
       <c r="E14" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F14">
         <v>224</v>
       </c>
       <c r="G14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K14" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M14">
         <v>16000</v>
@@ -1439,7 +1421,7 @@
         <v>100</v>
       </c>
       <c r="O14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="P14" t="s">
         <v>27</v>
@@ -1453,37 +1435,37 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C15" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D15">
         <v>223.4</v>
       </c>
       <c r="E15" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F15">
         <v>223.4</v>
       </c>
       <c r="G15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K15" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M15">
         <v>10000</v>
@@ -1492,10 +1474,10 @@
         <v>100</v>
       </c>
       <c r="O15" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="P15" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="Q15">
         <v>1675500</v>
@@ -1506,37 +1488,37 @@
         <v>28</v>
       </c>
       <c r="B16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" t="s">
         <v>43</v>
-      </c>
-      <c r="C16" t="s">
-        <v>45</v>
       </c>
       <c r="D16">
         <v>297</v>
       </c>
       <c r="E16" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F16">
         <v>297</v>
       </c>
       <c r="G16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K16" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M16">
         <v>22000</v>
@@ -1545,119 +1527,13 @@
         <v>100</v>
       </c>
       <c r="O16" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="P16" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="Q16">
         <v>1012500</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17">
-      <c r="A17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C17" t="s">
-        <v>46</v>
-      </c>
-      <c r="D17">
-        <v>2660</v>
-      </c>
-      <c r="E17" t="s">
-        <v>47</v>
-      </c>
-      <c r="F17">
-        <v>2553.6</v>
-      </c>
-      <c r="G17" t="s">
-        <v>57</v>
-      </c>
-      <c r="H17" t="s">
-        <v>57</v>
-      </c>
-      <c r="I17" t="s">
-        <v>57</v>
-      </c>
-      <c r="J17" t="s">
-        <v>57</v>
-      </c>
-      <c r="K17" t="s">
-        <v>58</v>
-      </c>
-      <c r="L17" t="s">
-        <v>57</v>
-      </c>
-      <c r="M17">
-        <v>35000</v>
-      </c>
-      <c r="N17">
-        <v>96</v>
-      </c>
-      <c r="O17" t="s">
-        <v>67</v>
-      </c>
-      <c r="P17" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q17">
-        <v>9340690</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17">
-      <c r="A18" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" t="s">
-        <v>46</v>
-      </c>
-      <c r="D18">
-        <v>2660</v>
-      </c>
-      <c r="E18" t="s">
-        <v>48</v>
-      </c>
-      <c r="F18">
-        <v>106.4</v>
-      </c>
-      <c r="G18" t="s">
-        <v>57</v>
-      </c>
-      <c r="H18" t="s">
-        <v>57</v>
-      </c>
-      <c r="I18" t="s">
-        <v>57</v>
-      </c>
-      <c r="J18" t="s">
-        <v>57</v>
-      </c>
-      <c r="K18" t="s">
-        <v>59</v>
-      </c>
-      <c r="L18" t="s">
-        <v>57</v>
-      </c>
-      <c r="M18">
-        <v>35000</v>
-      </c>
-      <c r="N18">
-        <v>4</v>
-      </c>
-      <c r="O18" t="s">
-        <v>67</v>
-      </c>
-      <c r="P18" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q18">
-        <v>9340690</v>
       </c>
     </row>
   </sheetData>
@@ -1667,7 +1543,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T16"/>
+  <dimension ref="A1:T15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -1675,10 +1551,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -1687,63 +1563,63 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
@@ -1755,7 +1631,7 @@
         <v>7950000</v>
       </c>
       <c r="H2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I2">
         <v>2000</v>
@@ -1764,34 +1640,34 @@
         <v>2000</v>
       </c>
       <c r="K2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L2">
         <v>2000</v>
       </c>
       <c r="M2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R2" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="S2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1799,13 +1675,13 @@
         <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E3" t="s">
         <v>18</v>
@@ -1817,7 +1693,7 @@
         <v>2460000</v>
       </c>
       <c r="H3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I3">
         <v>32000</v>
@@ -1826,34 +1702,34 @@
         <v>40200</v>
       </c>
       <c r="K3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L3">
         <v>32000</v>
       </c>
       <c r="M3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R3" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="S3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1861,10 +1737,10 @@
         <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D4" t="s">
         <v>24</v>
@@ -1879,7 +1755,7 @@
         <v>1500000</v>
       </c>
       <c r="H4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I4">
         <v>11000</v>
@@ -1888,34 +1764,34 @@
         <v>13000</v>
       </c>
       <c r="K4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L4">
         <v>16000</v>
       </c>
       <c r="M4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R4" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="S4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -1923,10 +1799,10 @@
         <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D5" t="s">
         <v>24</v>
@@ -1941,7 +1817,7 @@
         <v>1566800</v>
       </c>
       <c r="H5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I5">
         <v>13600</v>
@@ -1950,48 +1826,48 @@
         <v>15300</v>
       </c>
       <c r="K5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L5">
         <v>15300</v>
       </c>
       <c r="M5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R5" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="S5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E6" t="s">
         <v>21</v>
@@ -2003,7 +1879,7 @@
         <v>1000000</v>
       </c>
       <c r="H6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I6">
         <v>9500</v>
@@ -2012,48 +1888,48 @@
         <v>10700</v>
       </c>
       <c r="K6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L6">
         <v>13000</v>
       </c>
       <c r="M6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O6">
         <v>50</v>
       </c>
       <c r="P6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R6" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="S6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E7" t="s">
         <v>19</v>
@@ -2065,7 +1941,7 @@
         <v>6500000</v>
       </c>
       <c r="H7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I7">
         <v>2000</v>
@@ -2074,45 +1950,45 @@
         <v>2000</v>
       </c>
       <c r="K7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L7">
         <v>2000</v>
       </c>
       <c r="M7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R7" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="S7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D8" t="s">
         <v>25</v>
@@ -2127,7 +2003,7 @@
         <v>3077650</v>
       </c>
       <c r="H8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I8">
         <v>13800</v>
@@ -2136,45 +2012,45 @@
         <v>15700</v>
       </c>
       <c r="K8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L8">
         <v>16500</v>
       </c>
       <c r="M8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O8">
         <v>100</v>
       </c>
       <c r="P8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R8" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="S8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D9" t="s">
         <v>25</v>
@@ -2189,7 +2065,7 @@
         <v>1400000</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I9">
         <v>12500</v>
@@ -2198,45 +2074,45 @@
         <v>15500</v>
       </c>
       <c r="K9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L9">
         <v>15500</v>
       </c>
       <c r="M9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O9">
         <v>0</v>
       </c>
       <c r="P9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R9" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="S9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D10" t="s">
         <v>26</v>
@@ -2251,7 +2127,7 @@
         <v>1000000</v>
       </c>
       <c r="H10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I10">
         <v>24000</v>
@@ -2260,34 +2136,34 @@
         <v>29000</v>
       </c>
       <c r="K10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L10">
         <v>29000</v>
       </c>
       <c r="M10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O10">
         <v>0</v>
       </c>
       <c r="P10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R10" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="S10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -2295,13 +2171,13 @@
         <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E11" t="s">
         <v>24</v>
@@ -2313,7 +2189,7 @@
         <v>751000</v>
       </c>
       <c r="H11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I11">
         <v>18000</v>
@@ -2322,45 +2198,45 @@
         <v>21000</v>
       </c>
       <c r="K11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L11">
         <v>21000</v>
       </c>
       <c r="M11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O11">
         <v>72.87616511318242</v>
       </c>
       <c r="P11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R11" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="S11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D12" t="s">
         <v>27</v>
@@ -2375,7 +2251,7 @@
         <v>5800000</v>
       </c>
       <c r="H12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I12">
         <v>2000</v>
@@ -2384,45 +2260,45 @@
         <v>2000</v>
       </c>
       <c r="K12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L12">
         <v>2000</v>
       </c>
       <c r="M12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O12">
         <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R12" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="S12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
         <v>27</v>
@@ -2437,7 +2313,7 @@
         <v>1400000</v>
       </c>
       <c r="H13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I13">
         <v>16000</v>
@@ -2446,48 +2322,48 @@
         <v>19000</v>
       </c>
       <c r="K13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L13">
         <v>16000</v>
       </c>
       <c r="M13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O13">
         <v>0</v>
       </c>
       <c r="P13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R13" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="S13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E14" t="s">
         <v>27</v>
@@ -2499,7 +2375,7 @@
         <v>2234000</v>
       </c>
       <c r="H14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I14">
         <v>7300</v>
@@ -2508,48 +2384,48 @@
         <v>8500</v>
       </c>
       <c r="K14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L14">
         <v>10000</v>
       </c>
       <c r="M14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O14">
         <v>0</v>
       </c>
       <c r="P14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R14" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="S14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D15" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E15" t="s">
         <v>28</v>
@@ -2561,7 +2437,7 @@
         <v>1350000</v>
       </c>
       <c r="H15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I15">
         <v>14000</v>
@@ -2570,96 +2446,34 @@
         <v>17000</v>
       </c>
       <c r="K15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L15">
         <v>22000</v>
       </c>
       <c r="M15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O15">
         <v>0</v>
       </c>
       <c r="P15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="R15" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="S15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="T15" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20">
-      <c r="A16" t="s">
-        <v>67</v>
-      </c>
-      <c r="B16" t="s">
-        <v>44</v>
-      </c>
-      <c r="C16" t="s">
-        <v>47</v>
-      </c>
-      <c r="D16" t="s">
-        <v>72</v>
-      </c>
-      <c r="E16" t="s">
-        <v>29</v>
-      </c>
-      <c r="F16">
-        <v>266000000</v>
-      </c>
-      <c r="G16">
-        <v>7600000</v>
-      </c>
-      <c r="H16" t="s">
-        <v>57</v>
-      </c>
-      <c r="I16">
-        <v>24000</v>
-      </c>
-      <c r="J16">
-        <v>30000</v>
-      </c>
-      <c r="K16" t="s">
-        <v>57</v>
-      </c>
-      <c r="L16">
-        <v>35000</v>
-      </c>
-      <c r="M16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N16" t="s">
-        <v>57</v>
-      </c>
-      <c r="O16">
-        <v>14.47368421052632</v>
-      </c>
-      <c r="P16" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q16" t="s">
-        <v>57</v>
-      </c>
-      <c r="R16" t="s">
-        <v>104</v>
-      </c>
-      <c r="S16" t="s">
-        <v>57</v>
-      </c>
-      <c r="T16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -2669,21 +2483,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -2695,10 +2509,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -2707,24 +2521,24 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
         <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F2" t="s">
         <v>24</v>
@@ -2750,19 +2564,19 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F3" t="s">
         <v>27</v>
@@ -2788,22 +2602,22 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G4" t="s">
         <v>19</v>
@@ -2826,22 +2640,22 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="G5" t="s">
         <v>17</v>
@@ -2864,34 +2678,34 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G6" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H6">
-        <v>22400</v>
+        <v>50781.225</v>
       </c>
       <c r="I6">
-        <v>1400000</v>
+        <v>3077650</v>
       </c>
       <c r="J6">
-        <v>16000</v>
+        <v>16500</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -2902,72 +2716,72 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>108</v>
+        <v>45</v>
       </c>
       <c r="F7" t="s">
-        <v>72</v>
+        <v>27</v>
       </c>
       <c r="G7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H7">
-        <v>255360</v>
+        <v>22400</v>
       </c>
       <c r="I7">
-        <v>7600000</v>
+        <v>1400000</v>
       </c>
       <c r="J7">
-        <v>35000</v>
+        <v>16000</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F8" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="G8" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H8">
-        <v>50781.225</v>
+        <v>78720</v>
       </c>
       <c r="I8">
-        <v>3077650</v>
+        <v>2460000</v>
       </c>
       <c r="J8">
-        <v>16500</v>
+        <v>32000</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -2978,22 +2792,22 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="G9" t="s">
         <v>27</v>
@@ -3016,40 +2830,40 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="D10" t="s">
         <v>47</v>
       </c>
       <c r="E10" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F10" t="s">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="G10" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="H10">
-        <v>10640</v>
+        <v>22800</v>
       </c>
       <c r="I10">
-        <v>7600000</v>
+        <v>1500000</v>
       </c>
       <c r="J10">
-        <v>35000</v>
+        <v>16000</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>4</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -3057,145 +2871,145 @@
         <v>48</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C11" t="s">
         <v>31</v>
       </c>
       <c r="D11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E11" t="s">
-        <v>48</v>
+        <v>103</v>
       </c>
       <c r="F11" t="s">
-        <v>69</v>
+        <v>24</v>
       </c>
       <c r="G11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H11">
-        <v>78720</v>
+        <v>1200</v>
       </c>
       <c r="I11">
-        <v>2460000</v>
+        <v>1500000</v>
       </c>
       <c r="J11">
-        <v>32000</v>
+        <v>16000</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>100</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="E12" t="s">
-        <v>109</v>
+        <v>53</v>
       </c>
       <c r="F12" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" t="s">
         <v>24</v>
       </c>
-      <c r="G12" t="s">
-        <v>19</v>
-      </c>
       <c r="H12">
-        <v>22800</v>
+        <v>15771</v>
       </c>
       <c r="I12">
-        <v>1500000</v>
+        <v>751000</v>
       </c>
       <c r="J12">
-        <v>16000</v>
+        <v>21000</v>
       </c>
       <c r="K12">
         <v>0</v>
       </c>
       <c r="L12">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>64</v>
       </c>
       <c r="C13" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="E13" t="s">
-        <v>109</v>
+        <v>53</v>
       </c>
       <c r="F13" t="s">
-        <v>24</v>
+        <v>63</v>
       </c>
       <c r="G13" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="H13">
-        <v>1200</v>
+        <v>29700</v>
       </c>
       <c r="I13">
-        <v>1500000</v>
+        <v>1350000</v>
       </c>
       <c r="J13">
-        <v>16000</v>
+        <v>22000</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
-        <v>5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E14" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F14" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="G14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H14">
-        <v>15771</v>
+        <v>21700</v>
       </c>
       <c r="I14">
-        <v>751000</v>
+        <v>1400000</v>
       </c>
       <c r="J14">
-        <v>21000</v>
+        <v>15500</v>
       </c>
       <c r="K14">
         <v>0</v>
@@ -3206,34 +3020,34 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C15" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D15" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E15" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G15" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="H15">
-        <v>29700</v>
+        <v>13000</v>
       </c>
       <c r="I15">
-        <v>1350000</v>
+        <v>1000000</v>
       </c>
       <c r="J15">
-        <v>22000</v>
+        <v>13000</v>
       </c>
       <c r="K15">
         <v>0</v>
@@ -3244,115 +3058,39 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C16" t="s">
         <v>37</v>
       </c>
       <c r="D16" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E16" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G16" t="s">
         <v>23</v>
       </c>
       <c r="H16">
-        <v>21700</v>
+        <v>29000</v>
       </c>
       <c r="I16">
-        <v>1400000</v>
+        <v>1000000</v>
       </c>
       <c r="J16">
-        <v>15500</v>
+        <v>29000</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12">
-      <c r="A17" t="s">
-        <v>52</v>
-      </c>
-      <c r="B17" t="s">
-        <v>63</v>
-      </c>
-      <c r="C17" t="s">
-        <v>38</v>
-      </c>
-      <c r="D17" t="s">
-        <v>52</v>
-      </c>
-      <c r="E17" t="s">
-        <v>52</v>
-      </c>
-      <c r="F17" t="s">
-        <v>26</v>
-      </c>
-      <c r="G17" t="s">
-        <v>23</v>
-      </c>
-      <c r="H17">
-        <v>29000</v>
-      </c>
-      <c r="I17">
-        <v>1000000</v>
-      </c>
-      <c r="J17">
-        <v>29000</v>
-      </c>
-      <c r="K17">
-        <v>0</v>
-      </c>
-      <c r="L17">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12">
-      <c r="A18" t="s">
-        <v>52</v>
-      </c>
-      <c r="B18" t="s">
-        <v>61</v>
-      </c>
-      <c r="C18" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" t="s">
-        <v>52</v>
-      </c>
-      <c r="E18" t="s">
-        <v>52</v>
-      </c>
-      <c r="F18" t="s">
-        <v>70</v>
-      </c>
-      <c r="G18" t="s">
-        <v>21</v>
-      </c>
-      <c r="H18">
-        <v>13000</v>
-      </c>
-      <c r="I18">
-        <v>1000000</v>
-      </c>
-      <c r="J18">
-        <v>13000</v>
-      </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-24
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="105">
   <si>
     <t>상장일</t>
   </si>
@@ -69,6 +69,9 @@
     <t>총기관배정수량</t>
   </si>
   <si>
+    <t>2024-09-23</t>
+  </si>
+  <si>
     <t>2024-09-11</t>
   </si>
   <si>
@@ -102,7 +105,7 @@
     <t>2024-08-06</t>
   </si>
   <si>
-    <t>2024-07-31</t>
+    <t>아이언디바이스</t>
   </si>
   <si>
     <t>미래에셋비전스팩7호</t>
@@ -144,15 +147,15 @@
     <t>아이빔테크놀로지</t>
   </si>
   <si>
-    <t>피앤에스미캐닉스</t>
-  </si>
-  <si>
     <t>코스닥</t>
   </si>
   <si>
     <t>코스피</t>
   </si>
   <si>
+    <t>대신</t>
+  </si>
+  <si>
     <t>미래</t>
   </si>
   <si>
@@ -171,9 +174,6 @@
     <t>한국</t>
   </si>
   <si>
-    <t>대신</t>
-  </si>
-  <si>
     <t>하나</t>
   </si>
   <si>
@@ -192,6 +192,9 @@
     <t>인수</t>
   </si>
   <si>
+    <t>2024-09-09</t>
+  </si>
+  <si>
     <t>2024-09-02</t>
   </si>
   <si>
@@ -210,7 +213,7 @@
     <t>2024-07-25</t>
   </si>
   <si>
-    <t>2024-07-22</t>
+    <t>2024-09-12</t>
   </si>
   <si>
     <t>2024-09-05</t>
@@ -276,6 +279,9 @@
     <t>수수료율</t>
   </si>
   <si>
+    <t>1965.03 : 1</t>
+  </si>
+  <si>
     <t>1004 : 1</t>
   </si>
   <si>
@@ -313,9 +319,6 @@
   </si>
   <si>
     <t>1094.66 : 1</t>
-  </si>
-  <si>
-    <t>1585.92 : 1</t>
   </si>
   <si>
     <t>인수기관</t>
@@ -752,13 +755,13 @@
         <v>43</v>
       </c>
       <c r="D2">
-        <v>159</v>
+        <v>210</v>
       </c>
       <c r="E2" t="s">
         <v>45</v>
       </c>
       <c r="F2">
-        <v>159</v>
+        <v>210</v>
       </c>
       <c r="G2" t="s">
         <v>55</v>
@@ -779,7 +782,7 @@
         <v>55</v>
       </c>
       <c r="M2">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="N2">
         <v>100</v>
@@ -791,7 +794,7 @@
         <v>65</v>
       </c>
       <c r="Q2">
-        <v>5962500</v>
+        <v>2187000</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -805,13 +808,13 @@
         <v>43</v>
       </c>
       <c r="D3">
-        <v>787.2</v>
+        <v>159</v>
       </c>
       <c r="E3" t="s">
         <v>46</v>
       </c>
       <c r="F3">
-        <v>787.2</v>
+        <v>159</v>
       </c>
       <c r="G3" t="s">
         <v>55</v>
@@ -832,19 +835,19 @@
         <v>55</v>
       </c>
       <c r="M3">
-        <v>32000</v>
+        <v>2000</v>
       </c>
       <c r="N3">
         <v>100</v>
       </c>
       <c r="O3" t="s">
-        <v>21</v>
+        <v>59</v>
       </c>
       <c r="P3" t="s">
         <v>66</v>
       </c>
       <c r="Q3">
-        <v>1722000</v>
+        <v>5962500</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -858,13 +861,13 @@
         <v>43</v>
       </c>
       <c r="D4">
-        <v>240</v>
+        <v>787.2</v>
       </c>
       <c r="E4" t="s">
         <v>47</v>
       </c>
       <c r="F4">
-        <v>228</v>
+        <v>787.2</v>
       </c>
       <c r="G4" t="s">
         <v>55</v>
@@ -885,27 +888,27 @@
         <v>55</v>
       </c>
       <c r="M4">
-        <v>16000</v>
+        <v>32000</v>
       </c>
       <c r="N4">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="P4" t="s">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="Q4">
-        <v>2100000</v>
+        <v>1722000</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
         <v>43</v>
@@ -917,7 +920,7 @@
         <v>48</v>
       </c>
       <c r="F5">
-        <v>12</v>
+        <v>228</v>
       </c>
       <c r="G5" t="s">
         <v>55</v>
@@ -932,7 +935,7 @@
         <v>55</v>
       </c>
       <c r="K5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L5" t="s">
         <v>55</v>
@@ -941,13 +944,13 @@
         <v>16000</v>
       </c>
       <c r="N5">
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="O5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q5">
         <v>2100000</v>
@@ -964,13 +967,13 @@
         <v>43</v>
       </c>
       <c r="D6">
-        <v>239.7204</v>
+        <v>240</v>
       </c>
       <c r="E6" t="s">
         <v>49</v>
       </c>
       <c r="F6">
-        <v>239.7204</v>
+        <v>12</v>
       </c>
       <c r="G6" t="s">
         <v>55</v>
@@ -985,25 +988,25 @@
         <v>55</v>
       </c>
       <c r="K6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L6" t="s">
         <v>55</v>
       </c>
       <c r="M6">
-        <v>15300</v>
+        <v>16000</v>
       </c>
       <c r="N6">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="O6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q6">
-        <v>1156798</v>
+        <v>2100000</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -1017,13 +1020,13 @@
         <v>43</v>
       </c>
       <c r="D7">
-        <v>130</v>
+        <v>239.7204</v>
       </c>
       <c r="E7" t="s">
         <v>50</v>
       </c>
       <c r="F7">
-        <v>130</v>
+        <v>239.7204</v>
       </c>
       <c r="G7" t="s">
         <v>55</v>
@@ -1044,24 +1047,24 @@
         <v>55</v>
       </c>
       <c r="M7">
-        <v>13000</v>
+        <v>15300</v>
       </c>
       <c r="N7">
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="P7" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="Q7">
-        <v>723700</v>
+        <v>1156798</v>
       </c>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
         <v>34</v>
@@ -1097,39 +1100,39 @@
         <v>55</v>
       </c>
       <c r="M8">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="N8">
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="P8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q8">
-        <v>4875000</v>
+        <v>723700</v>
       </c>
     </row>
     <row r="9" spans="1:17">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B9" t="s">
         <v>35</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D9">
-        <v>507.81225</v>
+        <v>130</v>
       </c>
       <c r="E9" t="s">
         <v>45</v>
       </c>
       <c r="F9">
-        <v>507.81225</v>
+        <v>130</v>
       </c>
       <c r="G9" t="s">
         <v>55</v>
@@ -1150,7 +1153,7 @@
         <v>55</v>
       </c>
       <c r="M9">
-        <v>16500</v>
+        <v>2000</v>
       </c>
       <c r="N9">
         <v>100</v>
@@ -1159,10 +1162,10 @@
         <v>60</v>
       </c>
       <c r="P9" t="s">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="Q9">
-        <v>2078175</v>
+        <v>4875000</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -1173,16 +1176,16 @@
         <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D10">
-        <v>217</v>
+        <v>507.81225</v>
       </c>
       <c r="E10" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="F10">
-        <v>217</v>
+        <v>507.81225</v>
       </c>
       <c r="G10" t="s">
         <v>55</v>
@@ -1203,24 +1206,24 @@
         <v>55</v>
       </c>
       <c r="M10">
-        <v>15500</v>
+        <v>16500</v>
       </c>
       <c r="N10">
         <v>100</v>
       </c>
       <c r="O10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="P10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q10">
-        <v>1050000</v>
+        <v>2078175</v>
       </c>
     </row>
     <row r="11" spans="1:17">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
         <v>37</v>
@@ -1229,13 +1232,13 @@
         <v>43</v>
       </c>
       <c r="D11">
-        <v>290</v>
+        <v>217</v>
       </c>
       <c r="E11" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F11">
-        <v>290</v>
+        <v>217</v>
       </c>
       <c r="G11" t="s">
         <v>55</v>
@@ -1256,7 +1259,7 @@
         <v>55</v>
       </c>
       <c r="M11">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="N11">
         <v>100</v>
@@ -1268,7 +1271,7 @@
         <v>26</v>
       </c>
       <c r="Q11">
-        <v>720000</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -1282,13 +1285,13 @@
         <v>43</v>
       </c>
       <c r="D12">
-        <v>157.71</v>
+        <v>290</v>
       </c>
       <c r="E12" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F12">
-        <v>157.71</v>
+        <v>290</v>
       </c>
       <c r="G12" t="s">
         <v>55</v>
@@ -1309,19 +1312,19 @@
         <v>55</v>
       </c>
       <c r="M12">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="N12">
         <v>100</v>
       </c>
       <c r="O12" t="s">
+        <v>62</v>
+      </c>
+      <c r="P12" t="s">
         <v>27</v>
       </c>
-      <c r="P12" t="s">
-        <v>59</v>
-      </c>
       <c r="Q12">
-        <v>540250</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -1335,13 +1338,13 @@
         <v>43</v>
       </c>
       <c r="D13">
-        <v>116</v>
+        <v>157.71</v>
       </c>
       <c r="E13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F13">
-        <v>116</v>
+        <v>157.71</v>
       </c>
       <c r="G13" t="s">
         <v>55</v>
@@ -1362,19 +1365,19 @@
         <v>55</v>
       </c>
       <c r="M13">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="N13">
         <v>100</v>
       </c>
       <c r="O13" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="P13" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="Q13">
-        <v>4350000</v>
+        <v>540250</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1388,13 +1391,13 @@
         <v>43</v>
       </c>
       <c r="D14">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="E14" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="F14">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="G14" t="s">
         <v>55</v>
@@ -1415,19 +1418,19 @@
         <v>55</v>
       </c>
       <c r="M14">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N14">
         <v>100</v>
       </c>
       <c r="O14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q14">
-        <v>1050000</v>
+        <v>4350000</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1441,13 +1444,13 @@
         <v>43</v>
       </c>
       <c r="D15">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="E15" t="s">
         <v>46</v>
       </c>
       <c r="F15">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="G15" t="s">
         <v>55</v>
@@ -1468,7 +1471,7 @@
         <v>55</v>
       </c>
       <c r="M15">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="N15">
         <v>100</v>
@@ -1477,10 +1480,10 @@
         <v>63</v>
       </c>
       <c r="P15" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="Q15">
-        <v>1675500</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -1494,13 +1497,13 @@
         <v>43</v>
       </c>
       <c r="D16">
-        <v>297</v>
+        <v>223.4</v>
       </c>
       <c r="E16" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="F16">
-        <v>297</v>
+        <v>223.4</v>
       </c>
       <c r="G16" t="s">
         <v>55</v>
@@ -1521,7 +1524,7 @@
         <v>55</v>
       </c>
       <c r="M16">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="N16">
         <v>100</v>
@@ -1530,10 +1533,10 @@
         <v>64</v>
       </c>
       <c r="P16" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="Q16">
-        <v>1012500</v>
+        <v>1675500</v>
       </c>
     </row>
   </sheetData>
@@ -1551,10 +1554,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -1563,49 +1566,49 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:20">
@@ -1625,25 +1628,25 @@
         <v>17</v>
       </c>
       <c r="F2">
-        <v>15900000</v>
+        <v>21000000</v>
       </c>
       <c r="G2">
-        <v>7950000</v>
+        <v>3000000</v>
       </c>
       <c r="H2" t="s">
         <v>55</v>
       </c>
       <c r="I2">
-        <v>2000</v>
+        <v>4900</v>
       </c>
       <c r="J2">
-        <v>2000</v>
+        <v>5700</v>
       </c>
       <c r="K2" t="s">
         <v>55</v>
       </c>
       <c r="L2">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="M2" t="s">
         <v>55</v>
@@ -1661,7 +1664,7 @@
         <v>55</v>
       </c>
       <c r="R2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S2" t="s">
         <v>55</v>
@@ -1672,7 +1675,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>59</v>
       </c>
       <c r="B3" t="s">
         <v>30</v>
@@ -1687,25 +1690,25 @@
         <v>18</v>
       </c>
       <c r="F3">
-        <v>78720000</v>
+        <v>15900000</v>
       </c>
       <c r="G3">
-        <v>2460000</v>
+        <v>7950000</v>
       </c>
       <c r="H3" t="s">
         <v>55</v>
       </c>
       <c r="I3">
-        <v>32000</v>
+        <v>2000</v>
       </c>
       <c r="J3">
-        <v>40200</v>
+        <v>2000</v>
       </c>
       <c r="K3" t="s">
         <v>55</v>
       </c>
       <c r="L3">
-        <v>32000</v>
+        <v>2000</v>
       </c>
       <c r="M3" t="s">
         <v>55</v>
@@ -1723,7 +1726,7 @@
         <v>55</v>
       </c>
       <c r="R3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="S3" t="s">
         <v>55</v>
@@ -1734,7 +1737,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
         <v>31</v>
@@ -1743,31 +1746,31 @@
         <v>47</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="E4" t="s">
         <v>19</v>
       </c>
       <c r="F4">
-        <v>24000000</v>
+        <v>78720000</v>
       </c>
       <c r="G4">
-        <v>1500000</v>
+        <v>2460000</v>
       </c>
       <c r="H4" t="s">
         <v>55</v>
       </c>
       <c r="I4">
-        <v>11000</v>
+        <v>32000</v>
       </c>
       <c r="J4">
-        <v>13000</v>
+        <v>40200</v>
       </c>
       <c r="K4" t="s">
         <v>55</v>
       </c>
       <c r="L4">
-        <v>16000</v>
+        <v>32000</v>
       </c>
       <c r="M4" t="s">
         <v>55</v>
@@ -1785,7 +1788,7 @@
         <v>55</v>
       </c>
       <c r="R4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="S4" t="s">
         <v>55</v>
@@ -1796,40 +1799,40 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
         <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" t="s">
         <v>20</v>
       </c>
       <c r="F5">
-        <v>23972040</v>
+        <v>24000000</v>
       </c>
       <c r="G5">
-        <v>1566800</v>
+        <v>1500000</v>
       </c>
       <c r="H5" t="s">
         <v>55</v>
       </c>
       <c r="I5">
-        <v>13600</v>
+        <v>11000</v>
       </c>
       <c r="J5">
-        <v>15300</v>
+        <v>13000</v>
       </c>
       <c r="K5" t="s">
         <v>55</v>
       </c>
       <c r="L5">
-        <v>15300</v>
+        <v>16000</v>
       </c>
       <c r="M5" t="s">
         <v>55</v>
@@ -1847,7 +1850,7 @@
         <v>55</v>
       </c>
       <c r="R5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="S5" t="s">
         <v>55</v>
@@ -1858,7 +1861,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
         <v>33</v>
@@ -1867,31 +1870,31 @@
         <v>50</v>
       </c>
       <c r="D6" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
         <v>21</v>
       </c>
       <c r="F6">
-        <v>13000000</v>
+        <v>23972040</v>
       </c>
       <c r="G6">
-        <v>1000000</v>
+        <v>1566800</v>
       </c>
       <c r="H6" t="s">
         <v>55</v>
       </c>
       <c r="I6">
-        <v>9500</v>
+        <v>13600</v>
       </c>
       <c r="J6">
-        <v>10700</v>
+        <v>15300</v>
       </c>
       <c r="K6" t="s">
         <v>55</v>
       </c>
       <c r="L6">
-        <v>13000</v>
+        <v>15300</v>
       </c>
       <c r="M6" t="s">
         <v>55</v>
@@ -1900,7 +1903,7 @@
         <v>55</v>
       </c>
       <c r="O6">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P6" t="s">
         <v>55</v>
@@ -1909,7 +1912,7 @@
         <v>55</v>
       </c>
       <c r="R6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="S6" t="s">
         <v>55</v>
@@ -1920,7 +1923,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B7" t="s">
         <v>34</v>
@@ -1929,31 +1932,31 @@
         <v>51</v>
       </c>
       <c r="D7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F7">
         <v>13000000</v>
       </c>
       <c r="G7">
-        <v>6500000</v>
+        <v>1000000</v>
       </c>
       <c r="H7" t="s">
         <v>55</v>
       </c>
       <c r="I7">
-        <v>2000</v>
+        <v>9500</v>
       </c>
       <c r="J7">
-        <v>2000</v>
+        <v>10700</v>
       </c>
       <c r="K7" t="s">
         <v>55</v>
       </c>
       <c r="L7">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="M7" t="s">
         <v>55</v>
@@ -1962,7 +1965,7 @@
         <v>55</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="P7" t="s">
         <v>55</v>
@@ -1971,7 +1974,7 @@
         <v>55</v>
       </c>
       <c r="R7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="S7" t="s">
         <v>55</v>
@@ -1991,31 +1994,31 @@
         <v>45</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="E8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F8">
-        <v>50781225</v>
+        <v>13000000</v>
       </c>
       <c r="G8">
-        <v>3077650</v>
+        <v>6500000</v>
       </c>
       <c r="H8" t="s">
         <v>55</v>
       </c>
       <c r="I8">
-        <v>13800</v>
+        <v>2000</v>
       </c>
       <c r="J8">
-        <v>15700</v>
+        <v>2000</v>
       </c>
       <c r="K8" t="s">
         <v>55</v>
       </c>
       <c r="L8">
-        <v>16500</v>
+        <v>2000</v>
       </c>
       <c r="M8" t="s">
         <v>55</v>
@@ -2024,7 +2027,7 @@
         <v>55</v>
       </c>
       <c r="O8">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P8" t="s">
         <v>55</v>
@@ -2033,7 +2036,7 @@
         <v>55</v>
       </c>
       <c r="R8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="S8" t="s">
         <v>55</v>
@@ -2044,40 +2047,40 @@
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B9" t="s">
         <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E9" t="s">
         <v>23</v>
       </c>
       <c r="F9">
-        <v>21700000</v>
+        <v>50781225</v>
       </c>
       <c r="G9">
-        <v>1400000</v>
+        <v>3077650</v>
       </c>
       <c r="H9" t="s">
         <v>55</v>
       </c>
       <c r="I9">
-        <v>12500</v>
+        <v>13800</v>
       </c>
       <c r="J9">
-        <v>15500</v>
+        <v>15700</v>
       </c>
       <c r="K9" t="s">
         <v>55</v>
       </c>
       <c r="L9">
-        <v>15500</v>
+        <v>16500</v>
       </c>
       <c r="M9" t="s">
         <v>55</v>
@@ -2086,7 +2089,7 @@
         <v>55</v>
       </c>
       <c r="O9">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P9" t="s">
         <v>55</v>
@@ -2095,7 +2098,7 @@
         <v>55</v>
       </c>
       <c r="R9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="S9" t="s">
         <v>55</v>
@@ -2112,34 +2115,34 @@
         <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D10" t="s">
         <v>26</v>
       </c>
       <c r="E10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F10">
-        <v>29000000</v>
+        <v>21700000</v>
       </c>
       <c r="G10">
-        <v>1000000</v>
+        <v>1400000</v>
       </c>
       <c r="H10" t="s">
         <v>55</v>
       </c>
       <c r="I10">
-        <v>24000</v>
+        <v>12500</v>
       </c>
       <c r="J10">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="K10" t="s">
         <v>55</v>
       </c>
       <c r="L10">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="M10" t="s">
         <v>55</v>
@@ -2157,7 +2160,7 @@
         <v>55</v>
       </c>
       <c r="R10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S10" t="s">
         <v>55</v>
@@ -2168,40 +2171,40 @@
     </row>
     <row r="11" spans="1:20">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="B11" t="s">
         <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D11" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E11" t="s">
         <v>24</v>
       </c>
       <c r="F11">
-        <v>15771000</v>
+        <v>29000000</v>
       </c>
       <c r="G11">
-        <v>751000</v>
+        <v>1000000</v>
       </c>
       <c r="H11" t="s">
         <v>55</v>
       </c>
       <c r="I11">
-        <v>18000</v>
+        <v>24000</v>
       </c>
       <c r="J11">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="K11" t="s">
         <v>55</v>
       </c>
       <c r="L11">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="M11" t="s">
         <v>55</v>
@@ -2210,7 +2213,7 @@
         <v>55</v>
       </c>
       <c r="O11">
-        <v>72.87616511318242</v>
+        <v>0</v>
       </c>
       <c r="P11" t="s">
         <v>55</v>
@@ -2219,7 +2222,7 @@
         <v>55</v>
       </c>
       <c r="R11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="S11" t="s">
         <v>55</v>
@@ -2230,40 +2233,40 @@
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
         <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="E12" t="s">
         <v>25</v>
       </c>
       <c r="F12">
-        <v>11600000</v>
+        <v>15771000</v>
       </c>
       <c r="G12">
-        <v>5800000</v>
+        <v>751000</v>
       </c>
       <c r="H12" t="s">
         <v>55</v>
       </c>
       <c r="I12">
-        <v>2000</v>
+        <v>18000</v>
       </c>
       <c r="J12">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="K12" t="s">
         <v>55</v>
       </c>
       <c r="L12">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="M12" t="s">
         <v>55</v>
@@ -2272,7 +2275,7 @@
         <v>55</v>
       </c>
       <c r="O12">
-        <v>0</v>
+        <v>72.87616511318242</v>
       </c>
       <c r="P12" t="s">
         <v>55</v>
@@ -2281,7 +2284,7 @@
         <v>55</v>
       </c>
       <c r="R12" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="S12" t="s">
         <v>55</v>
@@ -2292,40 +2295,40 @@
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B13" t="s">
         <v>40</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="D13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E13" t="s">
         <v>26</v>
       </c>
       <c r="F13">
-        <v>22400000</v>
+        <v>11600000</v>
       </c>
       <c r="G13">
-        <v>1400000</v>
+        <v>5800000</v>
       </c>
       <c r="H13" t="s">
         <v>55</v>
       </c>
       <c r="I13">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="J13">
-        <v>19000</v>
+        <v>2000</v>
       </c>
       <c r="K13" t="s">
         <v>55</v>
       </c>
       <c r="L13">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="M13" t="s">
         <v>55</v>
@@ -2343,7 +2346,7 @@
         <v>55</v>
       </c>
       <c r="R13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="S13" t="s">
         <v>55</v>
@@ -2363,31 +2366,31 @@
         <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="E14" t="s">
         <v>27</v>
       </c>
       <c r="F14">
-        <v>22340000</v>
+        <v>22400000</v>
       </c>
       <c r="G14">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="H14" t="s">
         <v>55</v>
       </c>
       <c r="I14">
-        <v>7300</v>
+        <v>16000</v>
       </c>
       <c r="J14">
-        <v>8500</v>
+        <v>19000</v>
       </c>
       <c r="K14" t="s">
         <v>55</v>
       </c>
       <c r="L14">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="M14" t="s">
         <v>55</v>
@@ -2405,7 +2408,7 @@
         <v>55</v>
       </c>
       <c r="R14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="S14" t="s">
         <v>55</v>
@@ -2422,34 +2425,34 @@
         <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="E15" t="s">
         <v>28</v>
       </c>
       <c r="F15">
-        <v>29700000</v>
+        <v>22340000</v>
       </c>
       <c r="G15">
-        <v>1350000</v>
+        <v>2234000</v>
       </c>
       <c r="H15" t="s">
         <v>55</v>
       </c>
       <c r="I15">
-        <v>14000</v>
+        <v>7300</v>
       </c>
       <c r="J15">
-        <v>17000</v>
+        <v>8500</v>
       </c>
       <c r="K15" t="s">
         <v>55</v>
       </c>
       <c r="L15">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="M15" t="s">
         <v>55</v>
@@ -2467,7 +2470,7 @@
         <v>55</v>
       </c>
       <c r="R15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="S15" t="s">
         <v>55</v>
@@ -2488,16 +2491,16 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -2509,10 +2512,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -2521,30 +2524,30 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H2">
         <v>23972.04</v>
@@ -2567,10 +2570,10 @@
         <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D3" t="s">
         <v>54</v>
@@ -2579,10 +2582,10 @@
         <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H3">
         <v>11600</v>
@@ -2602,34 +2605,34 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="F4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="H4">
-        <v>13000</v>
+        <v>21000</v>
       </c>
       <c r="I4">
-        <v>6500000</v>
+        <v>3000000</v>
       </c>
       <c r="J4">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -2643,10 +2646,10 @@
         <v>45</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
         <v>45</v>
@@ -2655,16 +2658,16 @@
         <v>45</v>
       </c>
       <c r="F5" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H5">
-        <v>15900</v>
+        <v>13000</v>
       </c>
       <c r="I5">
-        <v>7950000</v>
+        <v>6500000</v>
       </c>
       <c r="J5">
         <v>2000</v>
@@ -2678,34 +2681,34 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="G6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H6">
-        <v>50781.225</v>
+        <v>15900</v>
       </c>
       <c r="I6">
-        <v>3077650</v>
+        <v>7950000</v>
       </c>
       <c r="J6">
-        <v>16500</v>
+        <v>2000</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -2716,34 +2719,34 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C7" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G7" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="H7">
-        <v>22400</v>
+        <v>50781.225</v>
       </c>
       <c r="I7">
-        <v>1400000</v>
+        <v>3077650</v>
       </c>
       <c r="J7">
-        <v>16000</v>
+        <v>16500</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -2757,10 +2760,10 @@
         <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>63</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
         <v>46</v>
@@ -2769,19 +2772,19 @@
         <v>46</v>
       </c>
       <c r="F8" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="G8" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="H8">
-        <v>78720</v>
+        <v>22400</v>
       </c>
       <c r="I8">
-        <v>2460000</v>
+        <v>1400000</v>
       </c>
       <c r="J8">
-        <v>32000</v>
+        <v>16000</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -2792,34 +2795,34 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G9" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H9">
-        <v>22340</v>
+        <v>78720</v>
       </c>
       <c r="I9">
-        <v>2234000</v>
+        <v>2460000</v>
       </c>
       <c r="J9">
-        <v>10000</v>
+        <v>32000</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -2833,37 +2836,37 @@
         <v>47</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
         <v>47</v>
       </c>
       <c r="E10" t="s">
-        <v>103</v>
+        <v>47</v>
       </c>
       <c r="F10" t="s">
-        <v>24</v>
+        <v>69</v>
       </c>
       <c r="G10" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="H10">
-        <v>22800</v>
+        <v>22340</v>
       </c>
       <c r="I10">
-        <v>1500000</v>
+        <v>2234000</v>
       </c>
       <c r="J10">
-        <v>16000</v>
+        <v>10000</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -2871,25 +2874,25 @@
         <v>48</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H11">
-        <v>1200</v>
+        <v>22800</v>
       </c>
       <c r="I11">
         <v>1500000</v>
@@ -2901,45 +2904,45 @@
         <v>0</v>
       </c>
       <c r="L11">
-        <v>5</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B12" t="s">
         <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D12" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E12" t="s">
-        <v>53</v>
+        <v>104</v>
       </c>
       <c r="F12" t="s">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="G12" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H12">
-        <v>15771</v>
+        <v>1200</v>
       </c>
       <c r="I12">
-        <v>751000</v>
+        <v>1500000</v>
       </c>
       <c r="J12">
-        <v>21000</v>
+        <v>16000</v>
       </c>
       <c r="K12">
         <v>0</v>
       </c>
       <c r="L12">
-        <v>100</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -2947,10 +2950,10 @@
         <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D13" t="s">
         <v>53</v>
@@ -2959,19 +2962,19 @@
         <v>53</v>
       </c>
       <c r="F13" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G13" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H13">
-        <v>29700</v>
+        <v>15771</v>
       </c>
       <c r="I13">
-        <v>1350000</v>
+        <v>751000</v>
       </c>
       <c r="J13">
-        <v>22000</v>
+        <v>21000</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -2985,10 +2988,10 @@
         <v>52</v>
       </c>
       <c r="B14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D14" t="s">
         <v>52</v>
@@ -2997,10 +3000,10 @@
         <v>52</v>
       </c>
       <c r="F14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G14" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H14">
         <v>21700</v>
@@ -3020,25 +3023,25 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G15" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H15">
         <v>13000</v>
@@ -3058,25 +3061,25 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H16">
         <v>29000</v>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-26
</commit_message>
<xml_diff>
--- a/datasets/corporate-finance-data.xlsx
+++ b/datasets/corporate-finance-data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="111">
   <si>
     <t>상장일</t>
   </si>
@@ -69,6 +69,9 @@
     <t>총기관배정수량</t>
   </si>
   <si>
+    <t>2024-09-25</t>
+  </si>
+  <si>
     <t>2024-09-23</t>
   </si>
   <si>
@@ -105,6 +108,9 @@
     <t>2024-08-06</t>
   </si>
   <si>
+    <t>KB제30호스팩</t>
+  </si>
+  <si>
     <t>아이언디바이스</t>
   </si>
   <si>
@@ -153,6 +159,9 @@
     <t>코스피</t>
   </si>
   <si>
+    <t>KB</t>
+  </si>
+  <si>
     <t>대신</t>
   </si>
   <si>
@@ -192,6 +201,9 @@
     <t>인수</t>
   </si>
   <si>
+    <t>2024-09-10</t>
+  </si>
+  <si>
     <t>2024-09-09</t>
   </si>
   <si>
@@ -213,6 +225,9 @@
     <t>2024-07-25</t>
   </si>
   <si>
+    <t>2024-09-13</t>
+  </si>
+  <si>
     <t>2024-09-12</t>
   </si>
   <si>
@@ -277,6 +292,9 @@
   </si>
   <si>
     <t>수수료율</t>
+  </si>
+  <si>
+    <t>619.62 : 1</t>
   </si>
   <si>
     <t>1965.03 : 1</t>
@@ -688,7 +706,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -749,52 +767,52 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D2">
-        <v>210</v>
+        <v>100</v>
       </c>
       <c r="E2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F2">
-        <v>210</v>
+        <v>100</v>
       </c>
       <c r="G2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M2">
-        <v>7000</v>
+        <v>2000</v>
       </c>
       <c r="N2">
         <v>100</v>
       </c>
       <c r="O2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="P2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="Q2">
-        <v>2187000</v>
+        <v>3750000</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -802,52 +820,52 @@
         <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D3">
-        <v>159</v>
+        <v>210</v>
       </c>
       <c r="E3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F3">
-        <v>159</v>
+        <v>210</v>
       </c>
       <c r="G3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M3">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="N3">
         <v>100</v>
       </c>
       <c r="O3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="P3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="Q3">
-        <v>5962500</v>
+        <v>2187000</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -855,52 +873,52 @@
         <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D4">
-        <v>787.2</v>
+        <v>159</v>
       </c>
       <c r="E4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F4">
-        <v>787.2</v>
+        <v>159</v>
       </c>
       <c r="G4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M4">
-        <v>32000</v>
+        <v>2000</v>
       </c>
       <c r="N4">
         <v>100</v>
       </c>
       <c r="O4" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="P4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="Q4">
-        <v>1722000</v>
+        <v>5962500</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -908,102 +926,102 @@
         <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D5">
-        <v>240</v>
+        <v>787.2</v>
       </c>
       <c r="E5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F5">
-        <v>228</v>
+        <v>787.2</v>
       </c>
       <c r="G5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M5">
-        <v>16000</v>
+        <v>32000</v>
       </c>
       <c r="N5">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O5" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="P5" t="s">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="Q5">
-        <v>2100000</v>
+        <v>1722000</v>
       </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D6">
         <v>240</v>
       </c>
       <c r="E6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F6">
-        <v>12</v>
+        <v>228</v>
       </c>
       <c r="G6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M6">
         <v>16000</v>
       </c>
       <c r="N6">
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="O6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q6">
         <v>2100000</v>
@@ -1014,52 +1032,52 @@
         <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D7">
-        <v>239.7204</v>
+        <v>240</v>
       </c>
       <c r="E7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F7">
-        <v>239.7204</v>
+        <v>12</v>
       </c>
       <c r="G7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="L7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M7">
-        <v>15300</v>
+        <v>16000</v>
       </c>
       <c r="N7">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="O7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q7">
-        <v>1156798</v>
+        <v>2100000</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -1067,158 +1085,158 @@
         <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D8">
-        <v>130</v>
+        <v>239.7204</v>
       </c>
       <c r="E8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F8">
-        <v>130</v>
+        <v>239.7204</v>
       </c>
       <c r="G8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M8">
-        <v>13000</v>
+        <v>15300</v>
       </c>
       <c r="N8">
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="P8" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="Q8">
-        <v>723700</v>
+        <v>1156798</v>
       </c>
     </row>
     <row r="9" spans="1:17">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D9">
         <v>130</v>
       </c>
       <c r="E9" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="F9">
         <v>130</v>
       </c>
       <c r="G9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K9" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M9">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="N9">
         <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="P9" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="Q9">
-        <v>4875000</v>
+        <v>723700</v>
       </c>
     </row>
     <row r="10" spans="1:17">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D10">
-        <v>507.81225</v>
+        <v>130</v>
       </c>
       <c r="E10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F10">
-        <v>507.81225</v>
+        <v>130</v>
       </c>
       <c r="G10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K10" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M10">
-        <v>16500</v>
+        <v>2000</v>
       </c>
       <c r="N10">
         <v>100</v>
       </c>
       <c r="O10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="P10" t="s">
-        <v>26</v>
+        <v>73</v>
       </c>
       <c r="Q10">
-        <v>2078175</v>
+        <v>4875000</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -1226,105 +1244,105 @@
         <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D11">
-        <v>217</v>
+        <v>507.81225</v>
       </c>
       <c r="E11" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F11">
-        <v>217</v>
+        <v>507.81225</v>
       </c>
       <c r="G11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K11" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M11">
-        <v>15500</v>
+        <v>16500</v>
       </c>
       <c r="N11">
         <v>100</v>
       </c>
       <c r="O11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="P11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q11">
-        <v>1050000</v>
+        <v>2078175</v>
       </c>
     </row>
     <row r="12" spans="1:17">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D12">
-        <v>290</v>
+        <v>217</v>
       </c>
       <c r="E12" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F12">
-        <v>290</v>
+        <v>217</v>
       </c>
       <c r="G12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K12" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M12">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="N12">
         <v>100</v>
       </c>
       <c r="O12" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="P12" t="s">
         <v>27</v>
       </c>
       <c r="Q12">
-        <v>720000</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -1332,52 +1350,52 @@
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D13">
-        <v>157.71</v>
+        <v>290</v>
       </c>
       <c r="E13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F13">
-        <v>157.71</v>
+        <v>290</v>
       </c>
       <c r="G13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K13" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M13">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="N13">
         <v>100</v>
       </c>
       <c r="O13" t="s">
+        <v>66</v>
+      </c>
+      <c r="P13" t="s">
         <v>28</v>
       </c>
-      <c r="P13" t="s">
-        <v>60</v>
-      </c>
       <c r="Q13">
-        <v>540250</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1385,52 +1403,52 @@
         <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D14">
-        <v>116</v>
+        <v>157.71</v>
       </c>
       <c r="E14" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F14">
-        <v>116</v>
+        <v>157.71</v>
       </c>
       <c r="G14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K14" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M14">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="N14">
         <v>100</v>
       </c>
       <c r="O14" t="s">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="P14" t="s">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="Q14">
-        <v>4350000</v>
+        <v>540250</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1438,52 +1456,52 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D15">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="E15" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="F15">
-        <v>224</v>
+        <v>116</v>
       </c>
       <c r="G15" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H15" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I15" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J15" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K15" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L15" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M15">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N15">
         <v>100</v>
       </c>
       <c r="O15" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="P15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q15">
-        <v>1050000</v>
+        <v>4350000</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -1491,51 +1509,104 @@
         <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D16">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="E16" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F16">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="G16" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H16" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I16" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J16" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K16" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L16" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M16">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="N16">
         <v>100</v>
       </c>
       <c r="O16" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="P16" t="s">
-        <v>69</v>
+        <v>29</v>
       </c>
       <c r="Q16">
+        <v>1050000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17">
+      <c r="A17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17">
+        <v>223.4</v>
+      </c>
+      <c r="E17" t="s">
+        <v>50</v>
+      </c>
+      <c r="F17">
+        <v>223.4</v>
+      </c>
+      <c r="G17" t="s">
+        <v>58</v>
+      </c>
+      <c r="H17" t="s">
+        <v>58</v>
+      </c>
+      <c r="I17" t="s">
+        <v>58</v>
+      </c>
+      <c r="J17" t="s">
+        <v>58</v>
+      </c>
+      <c r="K17" t="s">
+        <v>59</v>
+      </c>
+      <c r="L17" t="s">
+        <v>58</v>
+      </c>
+      <c r="M17">
+        <v>10000</v>
+      </c>
+      <c r="N17">
+        <v>100</v>
+      </c>
+      <c r="O17" t="s">
+        <v>68</v>
+      </c>
+      <c r="P17" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q17">
         <v>1675500</v>
       </c>
     </row>
@@ -1546,7 +1617,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T15"/>
+  <dimension ref="A1:T16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -1554,10 +1625,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>15</v>
@@ -1566,917 +1637,979 @@
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
       </c>
       <c r="F2">
-        <v>21000000</v>
+        <v>10000000</v>
       </c>
       <c r="G2">
-        <v>3000000</v>
+        <v>5000000</v>
       </c>
       <c r="H2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I2">
-        <v>4900</v>
+        <v>2000</v>
       </c>
       <c r="J2">
-        <v>5700</v>
+        <v>2000</v>
       </c>
       <c r="K2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L2">
-        <v>7000</v>
+        <v>2000</v>
       </c>
       <c r="M2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R2" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="S2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="E3" t="s">
         <v>18</v>
       </c>
       <c r="F3">
-        <v>15900000</v>
+        <v>21000000</v>
       </c>
       <c r="G3">
-        <v>7950000</v>
+        <v>3000000</v>
       </c>
       <c r="H3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I3">
-        <v>2000</v>
+        <v>4900</v>
       </c>
       <c r="J3">
-        <v>2000</v>
+        <v>5700</v>
       </c>
       <c r="K3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L3">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="M3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R3" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="S3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E4" t="s">
         <v>19</v>
       </c>
       <c r="F4">
-        <v>78720000</v>
+        <v>15900000</v>
       </c>
       <c r="G4">
-        <v>2460000</v>
+        <v>7950000</v>
       </c>
       <c r="H4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I4">
-        <v>32000</v>
+        <v>2000</v>
       </c>
       <c r="J4">
-        <v>40200</v>
+        <v>2000</v>
       </c>
       <c r="K4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L4">
-        <v>32000</v>
+        <v>2000</v>
       </c>
       <c r="M4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R4" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="S4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="E5" t="s">
         <v>20</v>
       </c>
       <c r="F5">
-        <v>24000000</v>
+        <v>78720000</v>
       </c>
       <c r="G5">
-        <v>1500000</v>
+        <v>2460000</v>
       </c>
       <c r="H5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I5">
-        <v>11000</v>
+        <v>32000</v>
       </c>
       <c r="J5">
-        <v>13000</v>
+        <v>40200</v>
       </c>
       <c r="K5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L5">
-        <v>16000</v>
+        <v>32000</v>
       </c>
       <c r="M5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R5" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="S5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E6" t="s">
         <v>21</v>
       </c>
       <c r="F6">
-        <v>23972040</v>
+        <v>24000000</v>
       </c>
       <c r="G6">
-        <v>1566800</v>
+        <v>1500000</v>
       </c>
       <c r="H6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I6">
-        <v>13600</v>
+        <v>11000</v>
       </c>
       <c r="J6">
-        <v>15300</v>
+        <v>13000</v>
       </c>
       <c r="K6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L6">
-        <v>15300</v>
+        <v>16000</v>
       </c>
       <c r="M6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R6" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="S6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D7" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s">
         <v>22</v>
       </c>
       <c r="F7">
-        <v>13000000</v>
+        <v>23972040</v>
       </c>
       <c r="G7">
-        <v>1000000</v>
+        <v>1566800</v>
       </c>
       <c r="H7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I7">
-        <v>9500</v>
+        <v>13600</v>
       </c>
       <c r="J7">
-        <v>10700</v>
+        <v>15300</v>
       </c>
       <c r="K7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L7">
-        <v>13000</v>
+        <v>15300</v>
       </c>
       <c r="M7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O7">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="S7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="D8" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E8" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F8">
         <v>13000000</v>
       </c>
       <c r="G8">
-        <v>6500000</v>
+        <v>1000000</v>
       </c>
       <c r="H8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I8">
-        <v>2000</v>
+        <v>9500</v>
       </c>
       <c r="J8">
-        <v>2000</v>
+        <v>10700</v>
       </c>
       <c r="K8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L8">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="M8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="P8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R8" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="S8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
+        <v>73</v>
       </c>
       <c r="E9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F9">
-        <v>50781225</v>
+        <v>13000000</v>
       </c>
       <c r="G9">
-        <v>3077650</v>
+        <v>6500000</v>
       </c>
       <c r="H9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I9">
-        <v>13800</v>
+        <v>2000</v>
       </c>
       <c r="J9">
-        <v>15700</v>
+        <v>2000</v>
       </c>
       <c r="K9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L9">
-        <v>16500</v>
+        <v>2000</v>
       </c>
       <c r="M9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O9">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R9" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="S9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E10" t="s">
         <v>24</v>
       </c>
       <c r="F10">
-        <v>21700000</v>
+        <v>50781225</v>
       </c>
       <c r="G10">
-        <v>1400000</v>
+        <v>3077650</v>
       </c>
       <c r="H10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I10">
-        <v>12500</v>
+        <v>13800</v>
       </c>
       <c r="J10">
-        <v>15500</v>
+        <v>15700</v>
       </c>
       <c r="K10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L10">
-        <v>15500</v>
+        <v>16500</v>
       </c>
       <c r="M10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O10">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R10" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="S10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D11" t="s">
         <v>27</v>
       </c>
       <c r="E11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F11">
-        <v>29000000</v>
+        <v>21700000</v>
       </c>
       <c r="G11">
-        <v>1000000</v>
+        <v>1400000</v>
       </c>
       <c r="H11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I11">
-        <v>24000</v>
+        <v>12500</v>
       </c>
       <c r="J11">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="K11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L11">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="M11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O11">
         <v>0</v>
       </c>
       <c r="P11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R11" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="S11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" t="s">
         <v>28</v>
-      </c>
-      <c r="B12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" t="s">
-        <v>53</v>
-      </c>
-      <c r="D12" t="s">
-        <v>60</v>
       </c>
       <c r="E12" t="s">
         <v>25</v>
       </c>
       <c r="F12">
-        <v>15771000</v>
+        <v>29000000</v>
       </c>
       <c r="G12">
-        <v>751000</v>
+        <v>1000000</v>
       </c>
       <c r="H12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I12">
-        <v>18000</v>
+        <v>24000</v>
       </c>
       <c r="J12">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="K12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L12">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="M12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O12">
-        <v>72.87616511318242</v>
+        <v>0</v>
       </c>
       <c r="P12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R12" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="S12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E13" t="s">
         <v>26</v>
       </c>
       <c r="F13">
-        <v>11600000</v>
+        <v>15771000</v>
       </c>
       <c r="G13">
-        <v>5800000</v>
+        <v>751000</v>
       </c>
       <c r="H13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I13">
-        <v>2000</v>
+        <v>18000</v>
       </c>
       <c r="J13">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="K13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L13">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="M13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O13">
-        <v>0</v>
+        <v>72.87616511318242</v>
       </c>
       <c r="P13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R13" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="S13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:20">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E14" t="s">
         <v>27</v>
       </c>
       <c r="F14">
-        <v>22400000</v>
+        <v>11600000</v>
       </c>
       <c r="G14">
-        <v>1400000</v>
+        <v>5800000</v>
       </c>
       <c r="H14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I14">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="J14">
-        <v>19000</v>
+        <v>2000</v>
       </c>
       <c r="K14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L14">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="M14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O14">
         <v>0</v>
       </c>
       <c r="P14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R14" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="S14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C15" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D15" t="s">
-        <v>69</v>
+        <v>29</v>
       </c>
       <c r="E15" t="s">
         <v>28</v>
       </c>
       <c r="F15">
-        <v>22340000</v>
+        <v>22400000</v>
       </c>
       <c r="G15">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="H15" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I15">
-        <v>7300</v>
+        <v>16000</v>
       </c>
       <c r="J15">
-        <v>8500</v>
+        <v>19000</v>
       </c>
       <c r="K15" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L15">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="M15" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N15" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="O15">
         <v>0</v>
       </c>
       <c r="P15" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q15" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R15" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="S15" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T15" t="s">
-        <v>55</v>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20">
+      <c r="A16" t="s">
+        <v>68</v>
+      </c>
+      <c r="B16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" t="s">
+        <v>74</v>
+      </c>
+      <c r="E16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16">
+        <v>22340000</v>
+      </c>
+      <c r="G16">
+        <v>2234000</v>
+      </c>
+      <c r="H16" t="s">
+        <v>58</v>
+      </c>
+      <c r="I16">
+        <v>7300</v>
+      </c>
+      <c r="J16">
+        <v>8500</v>
+      </c>
+      <c r="K16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L16">
+        <v>10000</v>
+      </c>
+      <c r="M16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N16" t="s">
+        <v>58</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>58</v>
+      </c>
+      <c r="R16" t="s">
+        <v>106</v>
+      </c>
+      <c r="S16" t="s">
+        <v>58</v>
+      </c>
+      <c r="T16" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -2486,21 +2619,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -2512,10 +2645,10 @@
         <v>0</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>12</v>
@@ -2524,39 +2657,39 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>61</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F2" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="G2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="H2">
-        <v>23972.04</v>
+        <v>10000</v>
       </c>
       <c r="I2">
-        <v>1566800</v>
+        <v>5000000</v>
       </c>
       <c r="J2">
-        <v>15300</v>
+        <v>2000</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -2567,34 +2700,34 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H3">
-        <v>11600</v>
+        <v>23972.04</v>
       </c>
       <c r="I3">
-        <v>5800000</v>
+        <v>1566800</v>
       </c>
       <c r="J3">
-        <v>2000</v>
+        <v>15300</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -2605,34 +2738,34 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="C4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F4" t="s">
         <v>29</v>
       </c>
-      <c r="D4" t="s">
-        <v>45</v>
-      </c>
-      <c r="E4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F4" t="s">
-        <v>65</v>
-      </c>
       <c r="G4" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="H4">
-        <v>21000</v>
+        <v>11600</v>
       </c>
       <c r="I4">
-        <v>3000000</v>
+        <v>5800000</v>
       </c>
       <c r="J4">
-        <v>7000</v>
+        <v>2000</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -2643,34 +2776,34 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H5">
-        <v>13000</v>
+        <v>21000</v>
       </c>
       <c r="I5">
-        <v>6500000</v>
+        <v>3000000</v>
       </c>
       <c r="J5">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="K5">
         <v>0</v>
@@ -2681,31 +2814,31 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="G6" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H6">
-        <v>15900</v>
+        <v>13000</v>
       </c>
       <c r="I6">
-        <v>7950000</v>
+        <v>6500000</v>
       </c>
       <c r="J6">
         <v>2000</v>
@@ -2719,34 +2852,34 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F7" t="s">
-        <v>26</v>
+        <v>71</v>
       </c>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="H7">
-        <v>50781.225</v>
+        <v>15900</v>
       </c>
       <c r="I7">
-        <v>3077650</v>
+        <v>7950000</v>
       </c>
       <c r="J7">
-        <v>16500</v>
+        <v>2000</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -2757,34 +2890,34 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G8" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H8">
-        <v>22400</v>
+        <v>50781.225</v>
       </c>
       <c r="I8">
-        <v>1400000</v>
+        <v>3077650</v>
       </c>
       <c r="J8">
-        <v>16000</v>
+        <v>16500</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -2795,34 +2928,34 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F9" t="s">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="G9" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="H9">
-        <v>78720</v>
+        <v>22400</v>
       </c>
       <c r="I9">
-        <v>2460000</v>
+        <v>1400000</v>
       </c>
       <c r="J9">
-        <v>32000</v>
+        <v>16000</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -2833,34 +2966,34 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>64</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F10" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G10" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="H10">
-        <v>22340</v>
+        <v>78720</v>
       </c>
       <c r="I10">
-        <v>2234000</v>
+        <v>2460000</v>
       </c>
       <c r="J10">
-        <v>10000</v>
+        <v>32000</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -2871,66 +3004,66 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>68</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="D11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E11" t="s">
-        <v>104</v>
+        <v>50</v>
       </c>
       <c r="F11" t="s">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="G11" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="H11">
-        <v>22800</v>
+        <v>22340</v>
       </c>
       <c r="I11">
-        <v>1500000</v>
+        <v>2234000</v>
       </c>
       <c r="J11">
-        <v>16000</v>
+        <v>10000</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E12" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H12">
-        <v>1200</v>
+        <v>22800</v>
       </c>
       <c r="I12">
         <v>1500000</v>
@@ -2942,77 +3075,77 @@
         <v>0</v>
       </c>
       <c r="L12">
-        <v>5</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B13" t="s">
         <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E13" t="s">
-        <v>53</v>
+        <v>110</v>
       </c>
       <c r="F13" t="s">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="G13" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="H13">
-        <v>15771</v>
+        <v>1200</v>
       </c>
       <c r="I13">
-        <v>751000</v>
+        <v>1500000</v>
       </c>
       <c r="J13">
-        <v>21000</v>
+        <v>16000</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
-        <v>100</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D14" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E14" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F14" t="s">
+        <v>64</v>
+      </c>
+      <c r="G14" t="s">
         <v>26</v>
       </c>
-      <c r="G14" t="s">
-        <v>24</v>
-      </c>
       <c r="H14">
-        <v>21700</v>
+        <v>15771</v>
       </c>
       <c r="I14">
-        <v>1400000</v>
+        <v>751000</v>
       </c>
       <c r="J14">
-        <v>15500</v>
+        <v>21000</v>
       </c>
       <c r="K14">
         <v>0</v>
@@ -3023,34 +3156,34 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B15" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="D15" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E15" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F15" t="s">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="G15" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H15">
-        <v>13000</v>
+        <v>21700</v>
       </c>
       <c r="I15">
-        <v>1000000</v>
+        <v>1400000</v>
       </c>
       <c r="J15">
-        <v>13000</v>
+        <v>15500</v>
       </c>
       <c r="K15">
         <v>0</v>
@@ -3061,39 +3194,77 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D16" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E16" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F16" t="s">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="G16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H16">
-        <v>29000</v>
+        <v>13000</v>
       </c>
       <c r="I16">
         <v>1000000</v>
       </c>
       <c r="J16">
-        <v>29000</v>
+        <v>13000</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" t="s">
+        <v>54</v>
+      </c>
+      <c r="F17" t="s">
+        <v>28</v>
+      </c>
+      <c r="G17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H17">
+        <v>29000</v>
+      </c>
+      <c r="I17">
+        <v>1000000</v>
+      </c>
+      <c r="J17">
+        <v>29000</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
         <v>100</v>
       </c>
     </row>

</xml_diff>